<commit_message>
Auto update scanner reports
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1255,7 +1255,7 @@
         <v>116</v>
       </c>
       <c r="W2" t="n">
-        <v>1385.37</v>
+        <v>1385.36</v>
       </c>
       <c r="X2" t="n">
         <v>2.03</v>
@@ -1476,11 +1476,11 @@
       </c>
       <c r="CQ2" t="inlineStr">
         <is>
-          <t>20260729_191046</t>
+          <t>20260729_201524</t>
         </is>
       </c>
       <c r="CR2" s="2" t="n">
-        <v>46232.7991485242</v>
+        <v>46232.84402826882</v>
       </c>
     </row>
   </sheetData>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02068046438157106</v>
+        <v>0.02068046468277598</v>
       </c>
     </row>
     <row r="6">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3282921945057972</v>
+        <v>0.328292199287277</v>
       </c>
     </row>
     <row r="7">
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04360851252576205</v>
+        <v>0.04360850604479853</v>
       </c>
     </row>
     <row r="13">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-29 19:10:46.467285+05:30</t>
+          <t>2026-07-29 20:15:24.074896+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-30 12:02 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1408,7 +1408,7 @@
         <v>0.248</v>
       </c>
       <c r="BT2" t="n">
-        <v>1385.36</v>
+        <v>1385.37</v>
       </c>
       <c r="BU2" t="n">
         <v>-14.17</v>
@@ -1485,11 +1485,11 @@
       </c>
       <c r="CR2" t="inlineStr">
         <is>
-          <t>20260730_135416</t>
+          <t>20260730_173254</t>
         </is>
       </c>
       <c r="CS2" s="2" t="n">
-        <v>46233.57935683676</v>
+        <v>46233.73119120294</v>
       </c>
     </row>
   </sheetData>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46233.57935185185</v>
+        <v>46233.73118055556</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46203</v>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02068046435822286</v>
+        <v>0.02068046106278525</v>
       </c>
     </row>
     <row r="6">
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.328292194135156</v>
+        <v>0.3282921418217057</v>
       </c>
     </row>
     <row r="7">
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02915034011916945</v>
+        <v>0.02915031460181465</v>
       </c>
     </row>
     <row r="12">
@@ -1952,7 +1952,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04360851743837789</v>
+        <v>0.04360849350454595</v>
       </c>
     </row>
     <row r="13">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-30 13:54:16.453111+05:30</t>
+          <t>2026-07-30 17:32:54.948815+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 06:00 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1198,19 +1198,19 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="H2" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1243,10 +1243,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.92</v>
+        <v>13.03</v>
       </c>
       <c r="R2" t="n">
-        <v>17.88</v>
+        <v>19.54</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1257,49 +1257,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1500.3</v>
+        <v>1785</v>
       </c>
       <c r="V2" t="n">
-        <v>1522.4</v>
+        <v>1825</v>
       </c>
       <c r="W2" t="n">
-        <v>1485</v>
+        <v>1785</v>
       </c>
       <c r="X2" t="n">
-        <v>1517.4</v>
+        <v>1817.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>1517.4</v>
+        <v>1817.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>3274608</v>
+        <v>1405833</v>
       </c>
       <c r="AA2" t="n">
-        <v>2372338</v>
+        <v>2255234</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.38</v>
+        <v>0.62</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.14</v>
+        <v>2.03</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="AE2" t="n">
-        <v>37.4</v>
+        <v>40</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.46</v>
+        <v>2.2</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.12</v>
+        <v>46.18</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.12</v>
+        <v>46.18</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.51</v>
+        <v>2.54</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1308,71 +1308,71 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>6.58</v>
+        <v>14.32</v>
       </c>
       <c r="AM2" t="n">
-        <v>14.83</v>
+        <v>22.37</v>
       </c>
       <c r="AN2" t="n">
-        <v>40.77</v>
+        <v>57.34</v>
       </c>
       <c r="AO2" t="n">
-        <v>72.78</v>
+        <v>81.76000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>10.24</v>
+        <v>16.68</v>
       </c>
       <c r="AQ2" t="n">
-        <v>53.01</v>
+        <v>55.97</v>
       </c>
       <c r="AR2" t="n">
-        <v>1517.4</v>
+        <v>1817.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>1669.14</v>
+        <v>1999.14</v>
       </c>
       <c r="AT2" t="n">
-        <v>1441.16</v>
+        <v>1725.05</v>
       </c>
       <c r="AU2" t="n">
-        <v>1517.400024414062</v>
+        <v>1817.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AX2" t="n">
         <v>10</v>
       </c>
       <c r="AY2" t="n">
-        <v>151.74</v>
+        <v>181.74</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.02</v>
+        <v>5.08</v>
       </c>
       <c r="BA2" t="n">
-        <v>76.23999999999999</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>1.99</v>
+        <v>1.97</v>
       </c>
       <c r="BC2" t="n">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.3</v>
+        <v>33.4</v>
       </c>
       <c r="BE2" t="n">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.9</v>
+        <v>48.4</v>
       </c>
       <c r="BG2" t="n">
         <v>116</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.7</v>
+        <v>18.1</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -1387,40 +1387,40 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>619</v>
+        <v>640</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.4</v>
+        <v>50.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.24</v>
+        <v>2.41</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.75</v>
+        <v>8.92</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.38</v>
+        <v>-4.35</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.248</v>
+        <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1385.37</v>
+        <v>1543.51</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.17</v>
+        <v>-12.91</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.03</v>
+        <v>2.13</v>
       </c>
       <c r="BW2" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>-0.88</v>
+        <v>-0.84</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -1429,14 +1429,14 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.5y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.6y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
@@ -1485,11 +1485,11 @@
       </c>
       <c r="CR2" t="inlineStr">
         <is>
-          <t>20260730_173254</t>
+          <t>20260731_113036</t>
         </is>
       </c>
       <c r="CS2" s="2" t="n">
-        <v>46233.73119120294</v>
+        <v>46234.47959107105</v>
       </c>
     </row>
   </sheetData>
@@ -1527,7 +1527,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -1710,13 +1710,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46233.73118055556</v>
+        <v>46234.47958333333</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46218</v>
+        <v>46248</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.92</v>
+        <v>13.03</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1744,58 +1744,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1517.4</v>
+        <v>1817.4</v>
       </c>
       <c r="L2" t="n">
-        <v>1500.3</v>
+        <v>1785</v>
       </c>
       <c r="M2" t="n">
-        <v>1522.4</v>
+        <v>1825</v>
       </c>
       <c r="N2" t="n">
-        <v>1485</v>
+        <v>1785</v>
       </c>
       <c r="O2" t="n">
-        <v>1517.4</v>
+        <v>1817.4</v>
       </c>
       <c r="P2" t="n">
-        <v>3274608</v>
+        <v>1405833</v>
       </c>
       <c r="Q2" t="n">
-        <v>1517.4</v>
+        <v>1817.4</v>
       </c>
       <c r="R2" t="n">
-        <v>1669.14</v>
+        <v>1999.14</v>
       </c>
       <c r="S2" t="n">
-        <v>1441.16</v>
+        <v>1725.05</v>
       </c>
       <c r="T2" t="n">
         <v>10</v>
       </c>
       <c r="U2" t="n">
-        <v>151.74</v>
+        <v>181.74</v>
       </c>
       <c r="V2" t="n">
-        <v>5.024383814419402</v>
+        <v>5.081435017057342</v>
       </c>
       <c r="W2" t="n">
-        <v>76.24000000000001</v>
+        <v>92.35000000000014</v>
       </c>
       <c r="X2" t="n">
-        <v>1.990293809024134</v>
+        <v>1.967948023822412</v>
       </c>
       <c r="Y2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB2" t="n">
         <v>0</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>200</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -1807,11 +1807,11 @@
         <v>10</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.024383814419402</v>
+        <v>5.081435017057342</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>TIME EXIT</t>
+          <t>ACTIVE</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02068046106278525</v>
+        <v>0.02072211868828375</v>
       </c>
     </row>
     <row r="6">
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3282921418217057</v>
+        <v>0.3289534361253768</v>
       </c>
     </row>
     <row r="7">
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02915031460181465</v>
+        <v>0.02912455342062642</v>
       </c>
     </row>
     <row r="12">
@@ -1952,7 +1952,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04360849350454595</v>
+        <v>0.0433135169498943</v>
       </c>
     </row>
     <row r="13">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.74</v>
+        <v>38.68</v>
       </c>
     </row>
     <row r="16">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-30 17:32:54.948815+05:30</t>
+          <t>2026-07-31 11:30:36.692979+05:30</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 1, 'average_expected_return_pct': 10.0, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9902938090241342}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.0, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9679480238224119}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 06:26 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1260,43 +1260,43 @@
         <v>1785</v>
       </c>
       <c r="V2" t="n">
-        <v>1826.5</v>
+        <v>1826.6</v>
       </c>
       <c r="W2" t="n">
         <v>1785</v>
       </c>
       <c r="X2" t="n">
-        <v>1823.7</v>
+        <v>1824.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>1823.7</v>
+        <v>1824.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>1531536</v>
+        <v>1577332</v>
       </c>
       <c r="AA2" t="n">
-        <v>2261519</v>
+        <v>2263809</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.38</v>
+        <v>2.43</v>
       </c>
       <c r="AD2" t="n">
         <v>0.21</v>
       </c>
       <c r="AE2" t="n">
-        <v>41.5</v>
+        <v>41.6</v>
       </c>
       <c r="AF2" t="n">
         <v>2.28</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.28</v>
+        <v>46.29</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.28</v>
+        <v>46.29</v>
       </c>
       <c r="AI2" t="n">
         <v>2.54</v>
@@ -1308,34 +1308,34 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>14.69</v>
+        <v>14.74</v>
       </c>
       <c r="AM2" t="n">
-        <v>22.78</v>
+        <v>22.83</v>
       </c>
       <c r="AN2" t="n">
-        <v>57.88</v>
+        <v>57.95</v>
       </c>
       <c r="AO2" t="n">
-        <v>82.04000000000001</v>
+        <v>82.08</v>
       </c>
       <c r="AP2" t="n">
-        <v>17.08</v>
+        <v>17.14</v>
       </c>
       <c r="AQ2" t="n">
-        <v>56.51</v>
+        <v>56.58</v>
       </c>
       <c r="AR2" t="n">
-        <v>1823.7</v>
+        <v>1824.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2006.07</v>
+        <v>2006.95</v>
       </c>
       <c r="AT2" t="n">
-        <v>1731.13</v>
+        <v>1731.92</v>
       </c>
       <c r="AU2" t="n">
-        <v>1823.699951171875</v>
+        <v>1824.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
@@ -1345,13 +1345,13 @@
         <v>10</v>
       </c>
       <c r="AY2" t="n">
-        <v>182.37</v>
+        <v>182.45</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.08</v>
+        <v>5.07</v>
       </c>
       <c r="BA2" t="n">
-        <v>92.56999999999999</v>
+        <v>92.58</v>
       </c>
       <c r="BB2" t="n">
         <v>1.97</v>
@@ -1408,10 +1408,10 @@
         <v>0.269</v>
       </c>
       <c r="BT2" t="n">
-        <v>1548.6</v>
+        <v>1549.25</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.85</v>
+        <v>-12.84</v>
       </c>
       <c r="BV2" t="n">
         <v>2.13</v>
@@ -1485,11 +1485,11 @@
       </c>
       <c r="CR2" t="inlineStr">
         <is>
-          <t>20260731_114724</t>
+          <t>20260731_115629</t>
         </is>
       </c>
       <c r="CS2" s="2" t="n">
-        <v>46234.49125598947</v>
+        <v>46234.49756057575</v>
       </c>
     </row>
   </sheetData>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.49125</v>
+        <v>46234.49755787037</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -1744,46 +1744,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1823.7</v>
+        <v>1824.5</v>
       </c>
       <c r="L2" t="n">
         <v>1785</v>
       </c>
       <c r="M2" t="n">
-        <v>1826.5</v>
+        <v>1826.6</v>
       </c>
       <c r="N2" t="n">
         <v>1785</v>
       </c>
       <c r="O2" t="n">
-        <v>1823.7</v>
+        <v>1824.5</v>
       </c>
       <c r="P2" t="n">
-        <v>1531536</v>
+        <v>1577332</v>
       </c>
       <c r="Q2" t="n">
-        <v>1823.7</v>
+        <v>1824.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2006.07</v>
+        <v>2006.95</v>
       </c>
       <c r="S2" t="n">
-        <v>1731.13</v>
+        <v>1731.92</v>
       </c>
       <c r="T2" t="n">
-        <v>9.999999999999993</v>
+        <v>10</v>
       </c>
       <c r="U2" t="n">
-        <v>182.3699999999999</v>
+        <v>182.45</v>
       </c>
       <c r="V2" t="n">
-        <v>5.075944508416951</v>
+        <v>5.074266922444502</v>
       </c>
       <c r="W2" t="n">
-        <v>92.56999999999994</v>
+        <v>92.57999999999993</v>
       </c>
       <c r="X2" t="n">
-        <v>1.970076698714486</v>
+        <v>1.970728019010588</v>
       </c>
       <c r="Y2" t="n">
         <v>14</v>
@@ -1804,10 +1804,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.999999999999993</v>
+        <v>10</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.075944508416951</v>
+        <v>5.074266922444502</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0207271525277319</v>
+        <v>0.02072785608434918</v>
       </c>
     </row>
     <row r="6">
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3290333458492946</v>
+        <v>0.32904451446435</v>
       </c>
     </row>
     <row r="7">
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02912455360790231</v>
+        <v>0.02912455342062642</v>
       </c>
     </row>
     <row r="12">
@@ -1952,7 +1952,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331352831328317</v>
+        <v>0.04331352038086517</v>
       </c>
     </row>
     <row r="13">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 11:47:24.546876+05:30</t>
+          <t>2026-07-31 11:56:29.265305+05:30</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.999999999999993, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9700766987144864}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.000000000000002, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9707280190105876}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 07:01 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -22,7 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -52,8 +57,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -437,6 +444,142 @@
           <t>Value</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Portfolio Holdings</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total Weight</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Invested Weight</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cash Weight</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Largest Position</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Smallest Position</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Average Position</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Median Position</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sector Count</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Largest Sector</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Largest Sector Weight</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Expected Return</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Portfolio Beta</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Portfolio Volatility</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -449,23 +592,904 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:CS2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="14" customWidth="1" min="37" max="37"/>
+    <col width="16" customWidth="1" min="38" max="38"/>
+    <col width="16" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="19" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="18" customWidth="1" min="49" max="49"/>
+    <col width="21" customWidth="1" min="50" max="50"/>
+    <col width="24" customWidth="1" min="51" max="51"/>
+    <col width="12" customWidth="1" min="52" max="52"/>
+    <col width="13" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="13" customWidth="1" min="55" max="55"/>
+    <col width="16" customWidth="1" min="56" max="56"/>
+    <col width="12" customWidth="1" min="57" max="57"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
+    <col width="13" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
+    <col width="12" customWidth="1" min="63" max="63"/>
+    <col width="12" customWidth="1" min="64" max="64"/>
+    <col width="13" customWidth="1" min="65" max="65"/>
+    <col width="12" customWidth="1" min="66" max="66"/>
+    <col width="12" customWidth="1" min="67" max="67"/>
+    <col width="12" customWidth="1" min="68" max="68"/>
+    <col width="12" customWidth="1" min="69" max="69"/>
+    <col width="12" customWidth="1" min="70" max="70"/>
+    <col width="15" customWidth="1" min="71" max="71"/>
+    <col width="20" customWidth="1" min="72" max="72"/>
+    <col width="12" customWidth="1" min="73" max="73"/>
+    <col width="15" customWidth="1" min="74" max="74"/>
+    <col width="19" customWidth="1" min="75" max="75"/>
+    <col width="17" customWidth="1" min="76" max="76"/>
+    <col width="16" customWidth="1" min="77" max="77"/>
+    <col width="24" customWidth="1" min="78" max="78"/>
+    <col width="12" customWidth="1" min="79" max="79"/>
+    <col width="12" customWidth="1" min="80" max="80"/>
+    <col width="40" customWidth="1" min="81" max="81"/>
+    <col width="17" customWidth="1" min="82" max="82"/>
+    <col width="17" customWidth="1" min="83" max="83"/>
+    <col width="24" customWidth="1" min="84" max="84"/>
+    <col width="17" customWidth="1" min="85" max="85"/>
+    <col width="15" customWidth="1" min="86" max="86"/>
+    <col width="20" customWidth="1" min="87" max="87"/>
+    <col width="12" customWidth="1" min="88" max="88"/>
+    <col width="12" customWidth="1" min="89" max="89"/>
+    <col width="18" customWidth="1" min="90" max="90"/>
+    <col width="16" customWidth="1" min="91" max="91"/>
+    <col width="15" customWidth="1" min="92" max="92"/>
+    <col width="15" customWidth="1" min="93" max="93"/>
+    <col width="18" customWidth="1" min="94" max="94"/>
+    <col width="12" customWidth="1" min="95" max="95"/>
+    <col width="17" customWidth="1" min="96" max="96"/>
+    <col width="28" customWidth="1" min="97" max="97"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>yahoo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>scan_date</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>signal_date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>bt_from</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>bt_to</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>exchange</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>subsector</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>trade_status</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>signals_today</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>rank_score</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>portfolio_rank</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>regime_today</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>close</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>cmp</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>avg20_volume</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>volume_ratio</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>day_chg_%</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>gap_%</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>candle_range</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>candle_range_%</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>atr</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>atr_points</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>atr_pct</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>above_50dma</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>above_200dma</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>pct_from_20dma</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>pct_from_50dma</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>pct_from_200dma</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>rsi</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>roc</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>relative_strength</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>entry</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>stop_loss</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>entry_ref</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>limit_price</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>target_hold_days</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>expected_return_pct</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>expected_return_points</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>risk_pct</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>risk_points</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>risk_reward</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>target_hits</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>target_hit_pct</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>stop_hits</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>stop_hit_pct</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>trail_exits</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>trail_pct</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>time_exits</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>time_pct</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>time_win</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>time_loss</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>hist_trades</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>win_rate</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>expectancy</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>avg_win_%</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>avg_loss_%</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>avg_days</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>exp_per_day_%</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>total_return_sum_%</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>cagr_%</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>reward_risk_ratio</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>recovery_factor</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>max_drawdown_%</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>max_consecutive_losses</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>seq_trades</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>cut_exits</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>confidence_norm</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>rank_score_norm</t>
+        </is>
+      </c>
+      <c r="CF1" t="inlineStr">
+        <is>
+          <t>relative_strength_norm</t>
+        </is>
+      </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>expectancy_norm</t>
+        </is>
+      </c>
+      <c r="CH1" t="inlineStr">
+        <is>
+          <t>win_rate_norm</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr">
+        <is>
+          <t>portfolio_score</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>weight</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr">
+        <is>
+          <t>weight_pct</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr">
+        <is>
+          <t>capital_fraction</t>
+        </is>
+      </c>
+      <c r="CM1" t="inlineStr">
+        <is>
+          <t>current_weight</t>
+        </is>
+      </c>
+      <c r="CN1" t="inlineStr">
+        <is>
+          <t>target_weight</t>
+        </is>
+      </c>
+      <c r="CO1" t="inlineStr">
+        <is>
+          <t>weight_change</t>
+        </is>
+      </c>
+      <c r="CP1" t="inlineStr">
+        <is>
+          <t>rebalance_action</t>
+        </is>
+      </c>
+      <c r="CQ1" t="inlineStr">
+        <is>
+          <t>turnover</t>
+        </is>
+      </c>
+      <c r="CR1" t="inlineStr">
+        <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="CS1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>43101</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>PASS_combined</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>13.03</v>
+      </c>
+      <c r="R2" t="n">
+        <v>19.54</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>1785</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1826.6</v>
+      </c>
+      <c r="W2" t="n">
+        <v>1785</v>
+      </c>
+      <c r="X2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1758227</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2272854</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>46.29</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>46.29</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="AJ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>14.21</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>22.24</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>81.68000000000001</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>16.56</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>2000.66</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>1722.92</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="n">
+        <v>14</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>185.16</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>92.58</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>214</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>310</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>116</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>640</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>-4.35</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>9</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>1541.98</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>-12.93</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>-0.84</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>-80.69</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>8</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>131</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>limited history: 8.6y (&lt;10y) - lower confidence</t>
+        </is>
+      </c>
+      <c r="CD2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>100</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="CQ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR2" t="inlineStr">
+        <is>
+          <t>20260731_123131</t>
+        </is>
+      </c>
+      <c r="CS2" s="2" t="n">
+        <v>46234.52189789173</v>
       </c>
     </row>
   </sheetData>
@@ -479,9 +1503,319 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="19" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="30" max="30"/>
+    <col width="24" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scan_date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>signal_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>expected_exit_date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>subsector</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>regime_today</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>cmp</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>close</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>entry</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>stop_loss</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>expected_return_pct</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>expected_return_points</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>risk_pct</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>risk_points</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>risk_reward</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>target_hold_days</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>days_since_signal</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>days_remaining</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>holding_progress_pct</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>current_return_pct</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>target_progress_pct</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>distance_to_target_pct</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>distance_to_stop_pct</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>trade_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46234.52188657408</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PASS_combined</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>13.03</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1785</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1826.6</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1785</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1758227</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1815.5</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2000.66</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1722.92</v>
+      </c>
+      <c r="T2" t="n">
+        <v>10.19884329385845</v>
+      </c>
+      <c r="U2" t="n">
+        <v>185.1600000000001</v>
+      </c>
+      <c r="V2" t="n">
+        <v>5.099421646929216</v>
+      </c>
+      <c r="W2" t="n">
+        <v>92.57999999999993</v>
+      </c>
+      <c r="X2" t="n">
+        <v>2.000000000000003</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>10.19884329385845</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>5.099421646929216</v>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -492,11 +1826,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,7 +1852,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -528,7 +1862,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -538,7 +1872,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -548,7 +1882,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.02072077631158337</v>
       </c>
     </row>
     <row r="6">
@@ -558,7 +1892,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>0.3289321265558869</v>
       </c>
     </row>
     <row r="7">
@@ -568,7 +1902,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -578,7 +1912,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -588,7 +1922,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -598,7 +1932,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -608,7 +1942,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>0.02912454722856361</v>
       </c>
     </row>
     <row r="12">
@@ -618,7 +1952,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>0.0433135164490069</v>
       </c>
     </row>
     <row r="13">
@@ -628,7 +1962,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -638,7 +1972,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -647,7 +1981,21 @@
           <t>Overall Risk Score</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="n">
+        <v>38.69</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Risk Rating</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -760,10 +2108,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -778,6 +2126,102 @@
           <t>Value</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Expected Portfolio Return</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Benchmark Return</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Portfolio Beta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Portfolio Volatility</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sharpe Ratio</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sortino Ratio</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Maximum Drawdown</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CAGR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Win Rate</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Information Ratio</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -817,7 +2261,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 12:25:25.755826+05:30</t>
+          <t>2026-07-31 12:31:32.008568+05:30</t>
         </is>
       </c>
     </row>
@@ -829,7 +2273,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 0, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': nan, 'average_current_return_pct': nan, 'average_risk_reward': nan}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.198843293858447, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 08:35 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1375,10 +1375,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.03</v>
+        <v>13.06</v>
       </c>
       <c r="R2" t="n">
-        <v>50.33</v>
+        <v>50.37</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1398,22 +1398,22 @@
         <v>1785</v>
       </c>
       <c r="X2" t="n">
-        <v>1819</v>
+        <v>1817.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1819</v>
+        <v>1817.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>1876142</v>
+        <v>1976572</v>
       </c>
       <c r="AA2" t="n">
-        <v>2278750</v>
+        <v>2237177</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.82</v>
+        <v>0.88</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.12</v>
+        <v>2.02</v>
       </c>
       <c r="AD2" t="n">
         <v>0.21</v>
@@ -1425,13 +1425,13 @@
         <v>2.29</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.29</v>
+        <v>44.91</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.29</v>
+        <v>44.91</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.54</v>
+        <v>2.47</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1440,50 +1440,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>14.42</v>
+        <v>13.46</v>
       </c>
       <c r="AM2" t="n">
-        <v>22.47</v>
+        <v>21.64</v>
       </c>
       <c r="AN2" t="n">
-        <v>57.48</v>
+        <v>56.71</v>
       </c>
       <c r="AO2" t="n">
-        <v>81.83</v>
+        <v>81.88</v>
       </c>
       <c r="AP2" t="n">
-        <v>16.78</v>
+        <v>18.79</v>
       </c>
       <c r="AQ2" t="n">
-        <v>56.11</v>
+        <v>56.27</v>
       </c>
       <c r="AR2" t="n">
-        <v>1819</v>
+        <v>1817.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>2004.16</v>
+        <v>1996.95</v>
       </c>
       <c r="AT2" t="n">
-        <v>1726.42</v>
+        <v>1727.47</v>
       </c>
       <c r="AU2" t="n">
-        <v>1819</v>
+        <v>1817.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>14</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.18</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>185.16</v>
+        <v>179.65</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.09</v>
+        <v>4.94</v>
       </c>
       <c r="BA2" t="n">
-        <v>92.58</v>
+        <v>89.83</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1501,10 +1501,10 @@
         <v>48.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.1</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -1519,16 +1519,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.9</v>
+        <v>51</v>
       </c>
       <c r="BO2" t="n">
         <v>2.41</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.93</v>
+        <v>8.9</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.35</v>
@@ -1540,10 +1540,10 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1544.8</v>
+        <v>1544.72</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.9</v>
+        <v>-12.91</v>
       </c>
       <c r="BV2" t="n">
         <v>2.13</v>
@@ -1581,7 +1581,7 @@
         <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -1605,7 +1605,7 @@
         <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>41.2</v>
+        <v>44.2</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -1683,11 +1683,11 @@
       </c>
       <c r="DN2" t="inlineStr">
         <is>
-          <t>20260731_132934</t>
+          <t>20260731_140529</t>
         </is>
       </c>
       <c r="DO2" s="2" t="n">
-        <v>46234.56220268775</v>
+        <v>46234.58714782468</v>
       </c>
     </row>
   </sheetData>
@@ -1725,7 +1725,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -1908,7 +1908,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.56219907408</v>
+        <v>46234.5871412037</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.03</v>
+        <v>13.06</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1819</v>
+        <v>1817.3</v>
       </c>
       <c r="L2" t="n">
         <v>1785</v>
@@ -1954,34 +1954,34 @@
         <v>1785</v>
       </c>
       <c r="O2" t="n">
-        <v>1819</v>
+        <v>1817.3</v>
       </c>
       <c r="P2" t="n">
-        <v>1876142</v>
+        <v>1976572</v>
       </c>
       <c r="Q2" t="n">
-        <v>1819</v>
+        <v>1817.3</v>
       </c>
       <c r="R2" t="n">
-        <v>2004.16</v>
+        <v>1996.95</v>
       </c>
       <c r="S2" t="n">
-        <v>1726.42</v>
+        <v>1727.47</v>
       </c>
       <c r="T2" t="n">
-        <v>10.17921935129192</v>
+        <v>9.885544489077208</v>
       </c>
       <c r="U2" t="n">
-        <v>185.1600000000001</v>
+        <v>179.6500000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.089609675645955</v>
+        <v>4.943047377978315</v>
       </c>
       <c r="W2" t="n">
-        <v>92.57999999999993</v>
+        <v>89.82999999999993</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000003</v>
+        <v>1.999888678615165</v>
       </c>
       <c r="Y2" t="n">
         <v>14</v>
@@ -2002,10 +2002,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.17921935129192</v>
+        <v>9.885544489077208</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.089609675645955</v>
+        <v>4.943047377978315</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02072330906136154</v>
+        <v>0.02070656716351207</v>
       </c>
     </row>
     <row r="6">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.328972332712164</v>
+        <v>0.3287065633230544</v>
       </c>
     </row>
     <row r="7">
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02912455342062642</v>
+        <v>0.02911166025863079</v>
       </c>
     </row>
     <row r="12">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331351364655098</v>
+        <v>0.04331351785731263</v>
       </c>
     </row>
     <row r="13">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.68</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="16">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 13:29:34.343557+05:30</t>
+          <t>2026-07-31 14:05:29.603336+05:30</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.179219351291923, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.885544489077208, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998886786151646}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 11:35 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DO2"/>
+  <dimension ref="A1:FL2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -698,22 +698,71 @@
     <col width="19" customWidth="1" min="101" max="101"/>
     <col width="20" customWidth="1" min="102" max="102"/>
     <col width="20" customWidth="1" min="103" max="103"/>
-    <col width="17" customWidth="1" min="104" max="104"/>
-    <col width="17" customWidth="1" min="105" max="105"/>
-    <col width="24" customWidth="1" min="106" max="106"/>
-    <col width="17" customWidth="1" min="107" max="107"/>
-    <col width="15" customWidth="1" min="108" max="108"/>
+    <col width="22" customWidth="1" min="104" max="104"/>
+    <col width="20" customWidth="1" min="105" max="105"/>
+    <col width="23" customWidth="1" min="106" max="106"/>
+    <col width="20" customWidth="1" min="107" max="107"/>
+    <col width="18" customWidth="1" min="108" max="108"/>
     <col width="20" customWidth="1" min="109" max="109"/>
-    <col width="12" customWidth="1" min="110" max="110"/>
-    <col width="12" customWidth="1" min="111" max="111"/>
-    <col width="18" customWidth="1" min="112" max="112"/>
-    <col width="16" customWidth="1" min="113" max="113"/>
-    <col width="15" customWidth="1" min="114" max="114"/>
-    <col width="15" customWidth="1" min="115" max="115"/>
-    <col width="18" customWidth="1" min="116" max="116"/>
-    <col width="12" customWidth="1" min="117" max="117"/>
-    <col width="17" customWidth="1" min="118" max="118"/>
-    <col width="28" customWidth="1" min="119" max="119"/>
+    <col width="24" customWidth="1" min="110" max="110"/>
+    <col width="28" customWidth="1" min="111" max="111"/>
+    <col width="21" customWidth="1" min="112" max="112"/>
+    <col width="18" customWidth="1" min="113" max="113"/>
+    <col width="19" customWidth="1" min="114" max="114"/>
+    <col width="23" customWidth="1" min="115" max="115"/>
+    <col width="28" customWidth="1" min="116" max="116"/>
+    <col width="19" customWidth="1" min="117" max="117"/>
+    <col width="21" customWidth="1" min="118" max="118"/>
+    <col width="22" customWidth="1" min="119" max="119"/>
+    <col width="23" customWidth="1" min="120" max="120"/>
+    <col width="18" customWidth="1" min="121" max="121"/>
+    <col width="12" customWidth="1" min="122" max="122"/>
+    <col width="15" customWidth="1" min="123" max="123"/>
+    <col width="13" customWidth="1" min="124" max="124"/>
+    <col width="17" customWidth="1" min="125" max="125"/>
+    <col width="16" customWidth="1" min="126" max="126"/>
+    <col width="22" customWidth="1" min="127" max="127"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="129" max="129"/>
+    <col width="18" customWidth="1" min="130" max="130"/>
+    <col width="16" customWidth="1" min="131" max="131"/>
+    <col width="14" customWidth="1" min="132" max="132"/>
+    <col width="14" customWidth="1" min="133" max="133"/>
+    <col width="14" customWidth="1" min="134" max="134"/>
+    <col width="23" customWidth="1" min="135" max="135"/>
+    <col width="22" customWidth="1" min="136" max="136"/>
+    <col width="17" customWidth="1" min="137" max="137"/>
+    <col width="21" customWidth="1" min="138" max="138"/>
+    <col width="19" customWidth="1" min="139" max="139"/>
+    <col width="19" customWidth="1" min="140" max="140"/>
+    <col width="22" customWidth="1" min="141" max="141"/>
+    <col width="29" customWidth="1" min="142" max="142"/>
+    <col width="20" customWidth="1" min="143" max="143"/>
+    <col width="19" customWidth="1" min="144" max="144"/>
+    <col width="18" customWidth="1" min="145" max="145"/>
+    <col width="14" customWidth="1" min="146" max="146"/>
+    <col width="13" customWidth="1" min="147" max="147"/>
+    <col width="17" customWidth="1" min="148" max="148"/>
+    <col width="15" customWidth="1" min="149" max="149"/>
+    <col width="20" customWidth="1" min="150" max="150"/>
+    <col width="16" customWidth="1" min="151" max="151"/>
+    <col width="14" customWidth="1" min="152" max="152"/>
+    <col width="17" customWidth="1" min="153" max="153"/>
+    <col width="17" customWidth="1" min="154" max="154"/>
+    <col width="24" customWidth="1" min="155" max="155"/>
+    <col width="17" customWidth="1" min="156" max="156"/>
+    <col width="15" customWidth="1" min="157" max="157"/>
+    <col width="20" customWidth="1" min="158" max="158"/>
+    <col width="12" customWidth="1" min="159" max="159"/>
+    <col width="12" customWidth="1" min="160" max="160"/>
+    <col width="18" customWidth="1" min="161" max="161"/>
+    <col width="16" customWidth="1" min="162" max="162"/>
+    <col width="15" customWidth="1" min="163" max="163"/>
+    <col width="15" customWidth="1" min="164" max="164"/>
+    <col width="18" customWidth="1" min="165" max="165"/>
+    <col width="12" customWidth="1" min="166" max="166"/>
+    <col width="17" customWidth="1" min="167" max="167"/>
+    <col width="28" customWidth="1" min="168" max="168"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1234,80 +1283,325 @@
       </c>
       <c r="CZ1" t="inlineStr">
         <is>
+          <t>remaining_upside_pct</t>
+        </is>
+      </c>
+      <c r="DA1" t="inlineStr">
+        <is>
+          <t>entry_distance_pct</t>
+        </is>
+      </c>
+      <c r="DB1" t="inlineStr">
+        <is>
+          <t>target_completion_pct</t>
+        </is>
+      </c>
+      <c r="DC1" t="inlineStr">
+        <is>
+          <t>return_per_day_pct</t>
+        </is>
+      </c>
+      <c r="DD1" t="inlineStr">
+        <is>
+          <t>risk_per_day_pct</t>
+        </is>
+      </c>
+      <c r="DE1" t="inlineStr">
+        <is>
+          <t>capital_efficiency</t>
+        </is>
+      </c>
+      <c r="DF1" t="inlineStr">
+        <is>
+          <t>opportunity_efficiency</t>
+        </is>
+      </c>
+      <c r="DG1" t="inlineStr">
+        <is>
+          <t>confidence_weighted_return</t>
+        </is>
+      </c>
+      <c r="DH1" t="inlineStr">
+        <is>
+          <t>atr_adjusted_return</t>
+        </is>
+      </c>
+      <c r="DI1" t="inlineStr">
+        <is>
+          <t>stop_cushion_pct</t>
+        </is>
+      </c>
+      <c r="DJ1" t="inlineStr">
+        <is>
+          <t>opportunity_score</t>
+        </is>
+      </c>
+      <c r="DK1" t="inlineStr">
+        <is>
+          <t>downside_exposure_pct</t>
+        </is>
+      </c>
+      <c r="DL1" t="inlineStr">
+        <is>
+          <t>target_stop_distance_ratio</t>
+        </is>
+      </c>
+      <c r="DM1" t="inlineStr">
+        <is>
+          <t>atr_risk_multiple</t>
+        </is>
+      </c>
+      <c r="DN1" t="inlineStr">
+        <is>
+          <t>return_to_atr_ratio</t>
+        </is>
+      </c>
+      <c r="DO1" t="inlineStr">
+        <is>
+          <t>risk_adjusted_return</t>
+        </is>
+      </c>
+      <c r="DP1" t="inlineStr">
+        <is>
+          <t>volatility_efficiency</t>
+        </is>
+      </c>
+      <c r="DQ1" t="inlineStr">
+        <is>
+          <t>stop_loss_buffer</t>
+        </is>
+      </c>
+      <c r="DR1" t="inlineStr">
+        <is>
+          <t>risk_score</t>
+        </is>
+      </c>
+      <c r="DS1" t="inlineStr">
+        <is>
+          <t>risk_quintile</t>
+        </is>
+      </c>
+      <c r="DT1" t="inlineStr">
+        <is>
+          <t>risk_decile</t>
+        </is>
+      </c>
+      <c r="DU1" t="inlineStr">
+        <is>
+          <t>trend_alignment</t>
+        </is>
+      </c>
+      <c r="DV1" t="inlineStr">
+        <is>
+          <t>trend_strength</t>
+        </is>
+      </c>
+      <c r="DW1" t="inlineStr">
+        <is>
+          <t>momentum_trend_ratio</t>
+        </is>
+      </c>
+      <c r="DX1" t="inlineStr">
+        <is>
+          <t>rsi_trend_score</t>
+        </is>
+      </c>
+      <c r="DY1" t="inlineStr">
+        <is>
+          <t>breakout_strength</t>
+        </is>
+      </c>
+      <c r="DZ1" t="inlineStr">
+        <is>
+          <t>trend_conviction</t>
+        </is>
+      </c>
+      <c r="EA1" t="inlineStr">
+        <is>
+          <t>trend_quintile</t>
+        </is>
+      </c>
+      <c r="EB1" t="inlineStr">
+        <is>
+          <t>trend_decile</t>
+        </is>
+      </c>
+      <c r="EC1" t="inlineStr">
+        <is>
+          <t>roc_strength</t>
+        </is>
+      </c>
+      <c r="ED1" t="inlineStr">
+        <is>
+          <t>rsi_strength</t>
+        </is>
+      </c>
+      <c r="EE1" t="inlineStr">
+        <is>
+          <t>momentum_acceleration</t>
+        </is>
+      </c>
+      <c r="EF1" t="inlineStr">
+        <is>
+          <t>momentum_persistence</t>
+        </is>
+      </c>
+      <c r="EG1" t="inlineStr">
+        <is>
+          <t>volume_strength</t>
+        </is>
+      </c>
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t>participation_score</t>
+        </is>
+      </c>
+      <c r="EI1" t="inlineStr">
+        <is>
+          <t>volume_conviction</t>
+        </is>
+      </c>
+      <c r="EJ1" t="inlineStr">
+        <is>
+          <t>volume_efficiency</t>
+        </is>
+      </c>
+      <c r="EK1" t="inlineStr">
+        <is>
+          <t>liquidity_efficiency</t>
+        </is>
+      </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t>institutional_participation</t>
+        </is>
+      </c>
+      <c r="EM1" t="inlineStr">
+        <is>
+          <t>accumulation_score</t>
+        </is>
+      </c>
+      <c r="EN1" t="inlineStr">
+        <is>
+          <t>distribution_risk</t>
+        </is>
+      </c>
+      <c r="EO1" t="inlineStr">
+        <is>
+          <t>turnover_quality</t>
+        </is>
+      </c>
+      <c r="EP1" t="inlineStr">
+        <is>
+          <t>volume_score</t>
+        </is>
+      </c>
+      <c r="EQ1" t="inlineStr">
+        <is>
+          <t>volume_band</t>
+        </is>
+      </c>
+      <c r="ER1" t="inlineStr">
+        <is>
+          <t>volume_quintile</t>
+        </is>
+      </c>
+      <c r="ES1" t="inlineStr">
+        <is>
+          <t>volume_decile</t>
+        </is>
+      </c>
+      <c r="ET1" t="inlineStr">
+        <is>
+          <t>confidence_quality</t>
+        </is>
+      </c>
+      <c r="EU1" t="inlineStr">
+        <is>
+          <t>reward_quality</t>
+        </is>
+      </c>
+      <c r="EV1" t="inlineStr">
+        <is>
+          <t>risk_quality</t>
+        </is>
+      </c>
+      <c r="EW1" t="inlineStr">
+        <is>
           <t>confidence_norm</t>
         </is>
       </c>
-      <c r="DA1" t="inlineStr">
+      <c r="EX1" t="inlineStr">
         <is>
           <t>rank_score_norm</t>
         </is>
       </c>
-      <c r="DB1" t="inlineStr">
+      <c r="EY1" t="inlineStr">
         <is>
           <t>relative_strength_norm</t>
         </is>
       </c>
-      <c r="DC1" t="inlineStr">
+      <c r="EZ1" t="inlineStr">
         <is>
           <t>expectancy_norm</t>
         </is>
       </c>
-      <c r="DD1" t="inlineStr">
+      <c r="FA1" t="inlineStr">
         <is>
           <t>win_rate_norm</t>
         </is>
       </c>
-      <c r="DE1" t="inlineStr">
+      <c r="FB1" t="inlineStr">
         <is>
           <t>portfolio_score</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="FC1" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="DG1" t="inlineStr">
+      <c r="FD1" t="inlineStr">
         <is>
           <t>weight_pct</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="FE1" t="inlineStr">
         <is>
           <t>capital_fraction</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="FF1" t="inlineStr">
         <is>
           <t>current_weight</t>
         </is>
       </c>
-      <c r="DJ1" t="inlineStr">
+      <c r="FG1" t="inlineStr">
         <is>
           <t>target_weight</t>
         </is>
       </c>
-      <c r="DK1" t="inlineStr">
+      <c r="FH1" t="inlineStr">
         <is>
           <t>weight_change</t>
         </is>
       </c>
-      <c r="DL1" t="inlineStr">
+      <c r="FI1" t="inlineStr">
         <is>
           <t>rebalance_action</t>
         </is>
       </c>
-      <c r="DM1" t="inlineStr">
+      <c r="FJ1" t="inlineStr">
         <is>
           <t>turnover</t>
         </is>
       </c>
-      <c r="DN1" t="inlineStr">
+      <c r="FK1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="DO1" t="inlineStr">
+      <c r="FL1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
@@ -1378,7 +1672,7 @@
         <v>13.06</v>
       </c>
       <c r="R2" t="n">
-        <v>50.37</v>
+        <v>50.46</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1398,22 +1692,22 @@
         <v>1785</v>
       </c>
       <c r="X2" t="n">
-        <v>1817.3</v>
+        <v>1816.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1817.3</v>
+        <v>1816.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1976572</v>
+        <v>2502212</v>
       </c>
       <c r="AA2" t="n">
-        <v>2237177</v>
+        <v>2263459</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.88</v>
+        <v>1.11</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.02</v>
+        <v>1.96</v>
       </c>
       <c r="AD2" t="n">
         <v>0.21</v>
@@ -1440,34 +1734,34 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>13.46</v>
+        <v>13.4</v>
       </c>
       <c r="AM2" t="n">
-        <v>21.64</v>
+        <v>21.57</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.71</v>
+        <v>56.62</v>
       </c>
       <c r="AO2" t="n">
-        <v>81.88</v>
+        <v>81.83</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.79</v>
+        <v>18.72</v>
       </c>
       <c r="AQ2" t="n">
-        <v>56.27</v>
+        <v>56.17</v>
       </c>
       <c r="AR2" t="n">
-        <v>1817.3</v>
+        <v>1816.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>1996.95</v>
+        <v>1995.85</v>
       </c>
       <c r="AT2" t="n">
-        <v>1727.47</v>
+        <v>1726.37</v>
       </c>
       <c r="AU2" t="n">
-        <v>1817.300048828125</v>
+        <v>1816.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
@@ -1480,7 +1774,7 @@
         <v>179.65</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.94</v>
+        <v>4.95</v>
       </c>
       <c r="BA2" t="n">
         <v>89.83</v>
@@ -1540,10 +1834,10 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1544.72</v>
+        <v>1543.79</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.91</v>
+        <v>-12.92</v>
       </c>
       <c r="BV2" t="n">
         <v>2.13</v>
@@ -1552,7 +1846,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>-0.84</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -1602,10 +1896,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>100</v>
+        <v>99.31</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.2</v>
+        <v>47.66</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -1638,56 +1932,205 @@
         <v>92.27</v>
       </c>
       <c r="CZ2" t="n">
+        <v>9.891500000000001</v>
+      </c>
+      <c r="DA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DC2" t="n">
+        <v>0.7064</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>0.3536</v>
+      </c>
+      <c r="DE2" t="n">
+        <v>0.0989</v>
+      </c>
+      <c r="DF2" t="n">
+        <v>1.998</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.2916</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.946</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.946</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>1.9999</v>
+      </c>
+      <c r="DM2" t="n">
+        <v>2.004</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>4.004</v>
+      </c>
+      <c r="DO2" t="n">
+        <v>1.9977</v>
+      </c>
+      <c r="DP2" t="n">
+        <v>0.8089</v>
+      </c>
+      <c r="DQ2" t="n">
+        <v>89.83</v>
+      </c>
+      <c r="DR2" t="n">
+        <v>42.74</v>
+      </c>
+      <c r="DS2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DT2" t="n">
+        <v>6</v>
+      </c>
+      <c r="DU2" t="n">
+        <v>2</v>
+      </c>
+      <c r="DV2" t="n">
+        <v>100</v>
+      </c>
+      <c r="DW2" t="n">
+        <v>7.5789</v>
+      </c>
+      <c r="DX2" t="n">
+        <v>45.425</v>
+      </c>
+      <c r="DY2" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="DZ2" t="n">
+        <v>98.038</v>
+      </c>
+      <c r="EA2" t="n">
+        <v>5</v>
+      </c>
+      <c r="EB2" t="n">
+        <v>10</v>
+      </c>
+      <c r="EC2" t="n">
+        <v>100</v>
+      </c>
+      <c r="ED2" t="n">
+        <v>26.69</v>
+      </c>
+      <c r="EE2" t="n">
+        <v>7.5789</v>
+      </c>
+      <c r="EF2" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="EG2" t="n">
+        <v>80.38</v>
+      </c>
+      <c r="EH2" t="n">
+        <v>10.4976</v>
+      </c>
+      <c r="EI2" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="EJ2" t="n">
+        <v>8.9099</v>
+      </c>
+      <c r="EK2" t="n">
+        <v>11.5245</v>
+      </c>
+      <c r="EL2" t="n">
+        <v>63.953</v>
+      </c>
+      <c r="EM2" t="n">
+        <v>20.7792</v>
+      </c>
+      <c r="EN2" t="n">
+        <v>1.1706</v>
+      </c>
+      <c r="EO2" t="n">
+        <v>79.8254</v>
+      </c>
+      <c r="EP2" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="EQ2" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="ER2" t="n">
+        <v>5</v>
+      </c>
+      <c r="ES2" t="n">
+        <v>10</v>
+      </c>
+      <c r="ET2" t="n">
+        <v>69.25</v>
+      </c>
+      <c r="EU2" t="n">
+        <v>29.62</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>73.61</v>
+      </c>
+      <c r="EW2" t="n">
         <v>1</v>
       </c>
-      <c r="DA2" t="n">
+      <c r="EX2" t="n">
         <v>1</v>
       </c>
-      <c r="DB2" t="n">
+      <c r="EY2" t="n">
         <v>1</v>
       </c>
-      <c r="DC2" t="n">
+      <c r="EZ2" t="n">
         <v>1</v>
       </c>
-      <c r="DD2" t="n">
+      <c r="FA2" t="n">
         <v>1</v>
       </c>
-      <c r="DE2" t="n">
+      <c r="FB2" t="n">
         <v>0.9999999999999999</v>
       </c>
-      <c r="DF2" t="n">
+      <c r="FC2" t="n">
         <v>1</v>
       </c>
-      <c r="DG2" t="n">
+      <c r="FD2" t="n">
         <v>100</v>
       </c>
-      <c r="DH2" t="n">
+      <c r="FE2" t="n">
         <v>1</v>
       </c>
-      <c r="DI2" t="n">
+      <c r="FF2" t="n">
         <v>0</v>
       </c>
-      <c r="DJ2" t="n">
+      <c r="FG2" t="n">
         <v>1</v>
       </c>
-      <c r="DK2" t="n">
+      <c r="FH2" t="n">
         <v>1</v>
       </c>
-      <c r="DL2" t="inlineStr">
+      <c r="FI2" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="DM2" t="n">
+      <c r="FJ2" t="n">
         <v>1</v>
       </c>
-      <c r="DN2" t="inlineStr">
-        <is>
-          <t>20260731_140529</t>
-        </is>
-      </c>
-      <c r="DO2" s="2" t="n">
-        <v>46234.58714782468</v>
+      <c r="FK2" t="inlineStr">
+        <is>
+          <t>20260731_170504</t>
+        </is>
+      </c>
+      <c r="FL2" s="2" t="n">
+        <v>46234.71185617313</v>
       </c>
     </row>
   </sheetData>
@@ -1725,9 +2168,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -1908,7 +2351,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.5871412037</v>
+        <v>46234.71185185185</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -1942,7 +2385,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1817.3</v>
+        <v>1816.2</v>
       </c>
       <c r="L2" t="n">
         <v>1785</v>
@@ -1954,34 +2397,34 @@
         <v>1785</v>
       </c>
       <c r="O2" t="n">
-        <v>1817.3</v>
+        <v>1816.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1976572</v>
+        <v>2502212</v>
       </c>
       <c r="Q2" t="n">
-        <v>1817.3</v>
+        <v>1816.2</v>
       </c>
       <c r="R2" t="n">
-        <v>1996.95</v>
+        <v>1995.85</v>
       </c>
       <c r="S2" t="n">
-        <v>1727.47</v>
+        <v>1726.37</v>
       </c>
       <c r="T2" t="n">
-        <v>9.885544489077208</v>
+        <v>9.891531769628887</v>
       </c>
       <c r="U2" t="n">
-        <v>179.6500000000001</v>
+        <v>179.6499999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.943047377978315</v>
+        <v>4.94604118489154</v>
       </c>
       <c r="W2" t="n">
-        <v>89.82999999999993</v>
+        <v>89.83000000000015</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999888678615165</v>
+        <v>1.999888678615157</v>
       </c>
       <c r="Y2" t="n">
         <v>14</v>
@@ -2002,10 +2445,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.885544489077208</v>
+        <v>9.891531769628887</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.943047377978315</v>
+        <v>4.94604118489154</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2080,7 +2523,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02070656716351207</v>
+        <v>0.02070578403168969</v>
       </c>
     </row>
     <row r="6">
@@ -2090,7 +2533,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3287065633230544</v>
+        <v>0.3286941314907796</v>
       </c>
     </row>
     <row r="7">
@@ -2140,7 +2583,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911166025863079</v>
+        <v>0.02911165397293003</v>
       </c>
     </row>
     <row r="12">
@@ -2150,7 +2593,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331351785731263</v>
+        <v>0.04331350751157916</v>
       </c>
     </row>
     <row r="13">
@@ -2160,7 +2603,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2459,7 +2902,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 14:05:29.603336+05:30</t>
+          <t>2026-07-31 17:05:04.409389+05:30</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2914,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.885544489077208, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998886786151646}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.891531769628887, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999888678615157}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 11:41 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FL2"/>
+  <dimension ref="A1:GR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -731,38 +731,70 @@
     <col width="14" customWidth="1" min="134" max="134"/>
     <col width="23" customWidth="1" min="135" max="135"/>
     <col width="22" customWidth="1" min="136" max="136"/>
-    <col width="17" customWidth="1" min="137" max="137"/>
+    <col width="19" customWidth="1" min="137" max="137"/>
     <col width="21" customWidth="1" min="138" max="138"/>
-    <col width="19" customWidth="1" min="139" max="139"/>
-    <col width="19" customWidth="1" min="140" max="140"/>
-    <col width="22" customWidth="1" min="141" max="141"/>
-    <col width="29" customWidth="1" min="142" max="142"/>
-    <col width="20" customWidth="1" min="143" max="143"/>
-    <col width="19" customWidth="1" min="144" max="144"/>
-    <col width="18" customWidth="1" min="145" max="145"/>
-    <col width="14" customWidth="1" min="146" max="146"/>
-    <col width="13" customWidth="1" min="147" max="147"/>
-    <col width="17" customWidth="1" min="148" max="148"/>
-    <col width="15" customWidth="1" min="149" max="149"/>
-    <col width="20" customWidth="1" min="150" max="150"/>
-    <col width="16" customWidth="1" min="151" max="151"/>
-    <col width="14" customWidth="1" min="152" max="152"/>
-    <col width="17" customWidth="1" min="153" max="153"/>
-    <col width="17" customWidth="1" min="154" max="154"/>
-    <col width="24" customWidth="1" min="155" max="155"/>
+    <col width="21" customWidth="1" min="139" max="139"/>
+    <col width="18" customWidth="1" min="140" max="140"/>
+    <col width="16" customWidth="1" min="141" max="141"/>
+    <col width="15" customWidth="1" min="142" max="142"/>
+    <col width="19" customWidth="1" min="143" max="143"/>
+    <col width="17" customWidth="1" min="144" max="144"/>
+    <col width="17" customWidth="1" min="145" max="145"/>
+    <col width="21" customWidth="1" min="146" max="146"/>
+    <col width="19" customWidth="1" min="147" max="147"/>
+    <col width="19" customWidth="1" min="148" max="148"/>
+    <col width="22" customWidth="1" min="149" max="149"/>
+    <col width="29" customWidth="1" min="150" max="150"/>
+    <col width="20" customWidth="1" min="151" max="151"/>
+    <col width="19" customWidth="1" min="152" max="152"/>
+    <col width="18" customWidth="1" min="153" max="153"/>
+    <col width="14" customWidth="1" min="154" max="154"/>
+    <col width="13" customWidth="1" min="155" max="155"/>
     <col width="17" customWidth="1" min="156" max="156"/>
     <col width="15" customWidth="1" min="157" max="157"/>
     <col width="20" customWidth="1" min="158" max="158"/>
-    <col width="12" customWidth="1" min="159" max="159"/>
-    <col width="12" customWidth="1" min="160" max="160"/>
-    <col width="18" customWidth="1" min="161" max="161"/>
-    <col width="16" customWidth="1" min="162" max="162"/>
-    <col width="15" customWidth="1" min="163" max="163"/>
-    <col width="15" customWidth="1" min="164" max="164"/>
-    <col width="18" customWidth="1" min="165" max="165"/>
-    <col width="12" customWidth="1" min="166" max="166"/>
-    <col width="17" customWidth="1" min="167" max="167"/>
-    <col width="28" customWidth="1" min="168" max="168"/>
+    <col width="16" customWidth="1" min="159" max="159"/>
+    <col width="14" customWidth="1" min="160" max="160"/>
+    <col width="15" customWidth="1" min="161" max="161"/>
+    <col width="19" customWidth="1" min="162" max="162"/>
+    <col width="19" customWidth="1" min="163" max="163"/>
+    <col width="21" customWidth="1" min="164" max="164"/>
+    <col width="21" customWidth="1" min="165" max="165"/>
+    <col width="15" customWidth="1" min="166" max="166"/>
+    <col width="14" customWidth="1" min="167" max="167"/>
+    <col width="18" customWidth="1" min="168" max="168"/>
+    <col width="16" customWidth="1" min="169" max="169"/>
+    <col width="21" customWidth="1" min="170" max="170"/>
+    <col width="13" customWidth="1" min="171" max="171"/>
+    <col width="17" customWidth="1" min="172" max="172"/>
+    <col width="21" customWidth="1" min="173" max="173"/>
+    <col width="17" customWidth="1" min="174" max="174"/>
+    <col width="26" customWidth="1" min="175" max="175"/>
+    <col width="24" customWidth="1" min="176" max="176"/>
+    <col width="22" customWidth="1" min="177" max="177"/>
+    <col width="21" customWidth="1" min="178" max="178"/>
+    <col width="22" customWidth="1" min="179" max="179"/>
+    <col width="21" customWidth="1" min="180" max="180"/>
+    <col width="12" customWidth="1" min="181" max="181"/>
+    <col width="14" customWidth="1" min="182" max="182"/>
+    <col width="16" customWidth="1" min="183" max="183"/>
+    <col width="19" customWidth="1" min="184" max="184"/>
+    <col width="17" customWidth="1" min="185" max="185"/>
+    <col width="17" customWidth="1" min="186" max="186"/>
+    <col width="24" customWidth="1" min="187" max="187"/>
+    <col width="17" customWidth="1" min="188" max="188"/>
+    <col width="15" customWidth="1" min="189" max="189"/>
+    <col width="20" customWidth="1" min="190" max="190"/>
+    <col width="12" customWidth="1" min="191" max="191"/>
+    <col width="12" customWidth="1" min="192" max="192"/>
+    <col width="18" customWidth="1" min="193" max="193"/>
+    <col width="16" customWidth="1" min="194" max="194"/>
+    <col width="15" customWidth="1" min="195" max="195"/>
+    <col width="15" customWidth="1" min="196" max="196"/>
+    <col width="18" customWidth="1" min="197" max="197"/>
+    <col width="12" customWidth="1" min="198" max="198"/>
+    <col width="17" customWidth="1" min="199" max="199"/>
+    <col width="28" customWidth="1" min="200" max="200"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1448,160 +1480,320 @@
       </c>
       <c r="EG1" t="inlineStr">
         <is>
+          <t>relative_momentum</t>
+        </is>
+      </c>
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t>momentum_efficiency</t>
+        </is>
+      </c>
+      <c r="EI1" t="inlineStr">
+        <is>
+          <t>conviction_momentum</t>
+        </is>
+      </c>
+      <c r="EJ1" t="inlineStr">
+        <is>
+          <t>momentum_quality</t>
+        </is>
+      </c>
+      <c r="EK1" t="inlineStr">
+        <is>
+          <t>momentum_score</t>
+        </is>
+      </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t>momentum_band</t>
+        </is>
+      </c>
+      <c r="EM1" t="inlineStr">
+        <is>
+          <t>momentum_quintile</t>
+        </is>
+      </c>
+      <c r="EN1" t="inlineStr">
+        <is>
+          <t>momentum_decile</t>
+        </is>
+      </c>
+      <c r="EO1" t="inlineStr">
+        <is>
           <t>volume_strength</t>
         </is>
       </c>
-      <c r="EH1" t="inlineStr">
+      <c r="EP1" t="inlineStr">
         <is>
           <t>participation_score</t>
         </is>
       </c>
-      <c r="EI1" t="inlineStr">
+      <c r="EQ1" t="inlineStr">
         <is>
           <t>volume_conviction</t>
         </is>
       </c>
-      <c r="EJ1" t="inlineStr">
+      <c r="ER1" t="inlineStr">
         <is>
           <t>volume_efficiency</t>
         </is>
       </c>
-      <c r="EK1" t="inlineStr">
+      <c r="ES1" t="inlineStr">
         <is>
           <t>liquidity_efficiency</t>
         </is>
       </c>
-      <c r="EL1" t="inlineStr">
+      <c r="ET1" t="inlineStr">
         <is>
           <t>institutional_participation</t>
         </is>
       </c>
-      <c r="EM1" t="inlineStr">
+      <c r="EU1" t="inlineStr">
         <is>
           <t>accumulation_score</t>
         </is>
       </c>
-      <c r="EN1" t="inlineStr">
+      <c r="EV1" t="inlineStr">
         <is>
           <t>distribution_risk</t>
         </is>
       </c>
-      <c r="EO1" t="inlineStr">
+      <c r="EW1" t="inlineStr">
         <is>
           <t>turnover_quality</t>
         </is>
       </c>
-      <c r="EP1" t="inlineStr">
+      <c r="EX1" t="inlineStr">
         <is>
           <t>volume_score</t>
         </is>
       </c>
-      <c r="EQ1" t="inlineStr">
+      <c r="EY1" t="inlineStr">
         <is>
           <t>volume_band</t>
         </is>
       </c>
-      <c r="ER1" t="inlineStr">
+      <c r="EZ1" t="inlineStr">
         <is>
           <t>volume_quintile</t>
         </is>
       </c>
-      <c r="ES1" t="inlineStr">
+      <c r="FA1" t="inlineStr">
         <is>
           <t>volume_decile</t>
         </is>
       </c>
-      <c r="ET1" t="inlineStr">
+      <c r="FB1" t="inlineStr">
         <is>
           <t>confidence_quality</t>
         </is>
       </c>
-      <c r="EU1" t="inlineStr">
+      <c r="FC1" t="inlineStr">
         <is>
           <t>reward_quality</t>
         </is>
       </c>
-      <c r="EV1" t="inlineStr">
+      <c r="FD1" t="inlineStr">
         <is>
           <t>risk_quality</t>
         </is>
       </c>
-      <c r="EW1" t="inlineStr">
+      <c r="FE1" t="inlineStr">
+        <is>
+          <t>trend_quality</t>
+        </is>
+      </c>
+      <c r="FF1" t="inlineStr">
+        <is>
+          <t>liquidity_quality</t>
+        </is>
+      </c>
+      <c r="FG1" t="inlineStr">
+        <is>
+          <t>stability_quality</t>
+        </is>
+      </c>
+      <c r="FH1" t="inlineStr">
+        <is>
+          <t>consistency_quality</t>
+        </is>
+      </c>
+      <c r="FI1" t="inlineStr">
+        <is>
+          <t>opportunity_quality</t>
+        </is>
+      </c>
+      <c r="FJ1" t="inlineStr">
+        <is>
+          <t>quality_score</t>
+        </is>
+      </c>
+      <c r="FK1" t="inlineStr">
+        <is>
+          <t>quality_band</t>
+        </is>
+      </c>
+      <c r="FL1" t="inlineStr">
+        <is>
+          <t>quality_quintile</t>
+        </is>
+      </c>
+      <c r="FM1" t="inlineStr">
+        <is>
+          <t>quality_decile</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
+        <is>
+          <t>institutional_score</t>
+        </is>
+      </c>
+      <c r="FO1" t="inlineStr">
+        <is>
+          <t>alpha_score</t>
+        </is>
+      </c>
+      <c r="FP1" t="inlineStr">
+        <is>
+          <t>execution_score</t>
+        </is>
+      </c>
+      <c r="FQ1" t="inlineStr">
+        <is>
+          <t>portfolio_fit_score</t>
+        </is>
+      </c>
+      <c r="FR1" t="inlineStr">
+        <is>
+          <t>composite_score</t>
+        </is>
+      </c>
+      <c r="FS1" t="inlineStr">
+        <is>
+          <t>institutional_percentile</t>
+        </is>
+      </c>
+      <c r="FT1" t="inlineStr">
+        <is>
+          <t>institutional_quintile</t>
+        </is>
+      </c>
+      <c r="FU1" t="inlineStr">
+        <is>
+          <t>institutional_decile</t>
+        </is>
+      </c>
+      <c r="FV1" t="inlineStr">
+        <is>
+          <t>institutional_grade</t>
+        </is>
+      </c>
+      <c r="FW1" t="inlineStr">
+        <is>
+          <t>recommendation_score</t>
+        </is>
+      </c>
+      <c r="FX1" t="inlineStr">
+        <is>
+          <t>recommendation_band</t>
+        </is>
+      </c>
+      <c r="FY1" t="inlineStr">
+        <is>
+          <t>top_decile</t>
+        </is>
+      </c>
+      <c r="FZ1" t="inlineStr">
+        <is>
+          <t>top_quintile</t>
+        </is>
+      </c>
+      <c r="GA1" t="inlineStr">
+        <is>
+          <t>top_10_percent</t>
+        </is>
+      </c>
+      <c r="GB1" t="inlineStr">
+        <is>
+          <t>bottom_10_percent</t>
+        </is>
+      </c>
+      <c r="GC1" t="inlineStr">
         <is>
           <t>confidence_norm</t>
         </is>
       </c>
-      <c r="EX1" t="inlineStr">
+      <c r="GD1" t="inlineStr">
         <is>
           <t>rank_score_norm</t>
         </is>
       </c>
-      <c r="EY1" t="inlineStr">
+      <c r="GE1" t="inlineStr">
         <is>
           <t>relative_strength_norm</t>
         </is>
       </c>
-      <c r="EZ1" t="inlineStr">
+      <c r="GF1" t="inlineStr">
         <is>
           <t>expectancy_norm</t>
         </is>
       </c>
-      <c r="FA1" t="inlineStr">
+      <c r="GG1" t="inlineStr">
         <is>
           <t>win_rate_norm</t>
         </is>
       </c>
-      <c r="FB1" t="inlineStr">
+      <c r="GH1" t="inlineStr">
         <is>
           <t>portfolio_score</t>
         </is>
       </c>
-      <c r="FC1" t="inlineStr">
+      <c r="GI1" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="FD1" t="inlineStr">
+      <c r="GJ1" t="inlineStr">
         <is>
           <t>weight_pct</t>
         </is>
       </c>
-      <c r="FE1" t="inlineStr">
+      <c r="GK1" t="inlineStr">
         <is>
           <t>capital_fraction</t>
         </is>
       </c>
-      <c r="FF1" t="inlineStr">
+      <c r="GL1" t="inlineStr">
         <is>
           <t>current_weight</t>
         </is>
       </c>
-      <c r="FG1" t="inlineStr">
+      <c r="GM1" t="inlineStr">
         <is>
           <t>target_weight</t>
         </is>
       </c>
-      <c r="FH1" t="inlineStr">
+      <c r="GN1" t="inlineStr">
         <is>
           <t>weight_change</t>
         </is>
       </c>
-      <c r="FI1" t="inlineStr">
+      <c r="GO1" t="inlineStr">
         <is>
           <t>rebalance_action</t>
         </is>
       </c>
-      <c r="FJ1" t="inlineStr">
+      <c r="GP1" t="inlineStr">
         <is>
           <t>turnover</t>
         </is>
       </c>
-      <c r="FK1" t="inlineStr">
+      <c r="GQ1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="FL1" t="inlineStr">
+      <c r="GR1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
@@ -1834,7 +2026,7 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1543.79</v>
+        <v>1543.78</v>
       </c>
       <c r="BU2" t="n">
         <v>-12.92</v>
@@ -1929,7 +2121,7 @@
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>92.27</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
         <v>9.891500000000001</v>
@@ -2031,106 +2223,210 @@
         <v>1.11</v>
       </c>
       <c r="EG2" t="n">
+        <v>2.4448</v>
+      </c>
+      <c r="EH2" t="n">
+        <v>4.0047</v>
+      </c>
+      <c r="EI2" t="n">
+        <v>0.3193</v>
+      </c>
+      <c r="EJ2" t="n">
+        <v>0.6731</v>
+      </c>
+      <c r="EK2" t="n">
+        <v>76.08</v>
+      </c>
+      <c r="EL2" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="EM2" t="n">
+        <v>5</v>
+      </c>
+      <c r="EN2" t="n">
+        <v>10</v>
+      </c>
+      <c r="EO2" t="n">
         <v>80.38</v>
       </c>
-      <c r="EH2" t="n">
+      <c r="EP2" t="n">
         <v>10.4976</v>
       </c>
-      <c r="EI2" t="n">
+      <c r="EQ2" t="n">
         <v>0.145</v>
       </c>
-      <c r="EJ2" t="n">
+      <c r="ER2" t="n">
         <v>8.9099</v>
       </c>
-      <c r="EK2" t="n">
+      <c r="ES2" t="n">
         <v>11.5245</v>
       </c>
-      <c r="EL2" t="n">
+      <c r="ET2" t="n">
         <v>63.953</v>
       </c>
-      <c r="EM2" t="n">
+      <c r="EU2" t="n">
         <v>20.7792</v>
       </c>
-      <c r="EN2" t="n">
+      <c r="EV2" t="n">
         <v>1.1706</v>
       </c>
-      <c r="EO2" t="n">
+      <c r="EW2" t="n">
         <v>79.8254</v>
       </c>
-      <c r="EP2" t="n">
+      <c r="EX2" t="n">
         <v>60.55</v>
       </c>
-      <c r="EQ2" t="inlineStr">
+      <c r="EY2" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="ER2" t="n">
+      <c r="EZ2" t="n">
         <v>5</v>
       </c>
-      <c r="ES2" t="n">
+      <c r="FA2" t="n">
         <v>10</v>
       </c>
-      <c r="ET2" t="n">
+      <c r="FB2" t="n">
         <v>69.25</v>
       </c>
-      <c r="EU2" t="n">
+      <c r="FC2" t="n">
         <v>29.62</v>
       </c>
-      <c r="EV2" t="n">
+      <c r="FD2" t="n">
         <v>73.61</v>
       </c>
-      <c r="EW2" t="n">
-        <v>1</v>
-      </c>
-      <c r="EX2" t="n">
-        <v>1</v>
-      </c>
-      <c r="EY2" t="n">
-        <v>1</v>
-      </c>
-      <c r="EZ2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FA2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FB2" t="n">
+      <c r="FE2" t="n">
+        <v>87.69499999999999</v>
+      </c>
+      <c r="FF2" t="n">
+        <v>54.105</v>
+      </c>
+      <c r="FG2" t="n">
+        <v>28.6196</v>
+      </c>
+      <c r="FH2" t="n">
+        <v>76.52800000000001</v>
+      </c>
+      <c r="FI2" t="n">
+        <v>41.365</v>
+      </c>
+      <c r="FJ2" t="n">
+        <v>60.34</v>
+      </c>
+      <c r="FK2" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="FL2" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM2" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN2" t="n">
+        <v>60.98</v>
+      </c>
+      <c r="FO2" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="FP2" t="n">
+        <v>55.55</v>
+      </c>
+      <c r="FQ2" t="n">
+        <v>48.96</v>
+      </c>
+      <c r="FR2" t="n">
+        <v>58.95</v>
+      </c>
+      <c r="FS2" t="n">
+        <v>100</v>
+      </c>
+      <c r="FT2" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU2" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW2" t="n">
+        <v>53.9525</v>
+      </c>
+      <c r="FX2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY2" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GD2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GE2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GF2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GH2" t="n">
         <v>0.9999999999999999</v>
       </c>
-      <c r="FC2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FD2" t="n">
+      <c r="GI2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GJ2" t="n">
         <v>100</v>
       </c>
-      <c r="FE2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FF2" t="n">
+      <c r="GK2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GL2" t="n">
         <v>0</v>
       </c>
-      <c r="FG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FH2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FI2" t="inlineStr">
+      <c r="GM2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GO2" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="FJ2" t="n">
-        <v>1</v>
-      </c>
-      <c r="FK2" t="inlineStr">
-        <is>
-          <t>20260731_170504</t>
-        </is>
-      </c>
-      <c r="FL2" s="2" t="n">
-        <v>46234.71185617313</v>
+      <c r="GP2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GQ2" t="inlineStr">
+        <is>
+          <t>20260731_171116</t>
+        </is>
+      </c>
+      <c r="GR2" s="2" t="n">
+        <v>46234.71615986427</v>
       </c>
     </row>
   </sheetData>
@@ -2351,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.71185185185</v>
+        <v>46234.71615740741</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -2523,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02070578403168969</v>
+        <v>0.02070578242158459</v>
       </c>
     </row>
     <row r="6">
@@ -2533,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3286941314907796</v>
+        <v>0.3286941059311535</v>
       </c>
     </row>
     <row r="7">
@@ -2583,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911165397293003</v>
+        <v>0.02911165716259938</v>
       </c>
     </row>
     <row r="12">
@@ -2593,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331350751157916</v>
+        <v>0.04331351622743339</v>
       </c>
     </row>
     <row r="13">
@@ -2603,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347617</v>
       </c>
     </row>
     <row r="14">
@@ -2902,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 17:05:04.409389+05:30</t>
+          <t>2026-07-31 17:11:16.242987+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 12:08 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2178,7 +2178,7 @@
         <v>89.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.74</v>
+        <v>42.79</v>
       </c>
       <c r="DS2" t="n">
         <v>3</v>
@@ -2311,7 +2311,7 @@
         <v>76.52800000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.365</v>
+        <v>41.39</v>
       </c>
       <c r="FJ2" t="n">
         <v>60.34</v>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>60.98</v>
+        <v>60.99</v>
       </c>
       <c r="FO2" t="n">
         <v>66.81</v>
       </c>
       <c r="FP2" t="n">
-        <v>55.55</v>
+        <v>55.56</v>
       </c>
       <c r="FQ2" t="n">
-        <v>48.96</v>
+        <v>48.97</v>
       </c>
       <c r="FR2" t="n">
-        <v>58.95</v>
+        <v>58.96</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>53.9525</v>
+        <v>53.965</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260731_171116</t>
+          <t>20260731_173817</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46234.71615986427</v>
+        <v>46234.73492532277</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.71615740741</v>
+        <v>46234.73491898148</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02070578242158459</v>
+        <v>0.02070578395742099</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3286941059311535</v>
+        <v>0.3286941303118006</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911165716259938</v>
+        <v>0.02911166025863079</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331351622743339</v>
+        <v>0.04331351341998324</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347617</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 17:11:16.242987+05:30</t>
+          <t>2026-07-31 17:38:17.584506+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 12:14 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1543.78</v>
+        <v>1543.79</v>
       </c>
       <c r="BU2" t="n">
         <v>-12.92</v>
@@ -2178,7 +2178,7 @@
         <v>89.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.79</v>
+        <v>42.74</v>
       </c>
       <c r="DS2" t="n">
         <v>3</v>
@@ -2311,7 +2311,7 @@
         <v>76.52800000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.39</v>
+        <v>41.365</v>
       </c>
       <c r="FJ2" t="n">
         <v>60.34</v>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>60.99</v>
+        <v>60.98</v>
       </c>
       <c r="FO2" t="n">
         <v>66.81</v>
       </c>
       <c r="FP2" t="n">
-        <v>55.56</v>
+        <v>55.55</v>
       </c>
       <c r="FQ2" t="n">
-        <v>48.97</v>
+        <v>48.96</v>
       </c>
       <c r="FR2" t="n">
-        <v>58.96</v>
+        <v>58.95</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>53.965</v>
+        <v>53.9525</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260731_173817</t>
+          <t>20260731_174431</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46234.73492532277</v>
+        <v>46234.73925388121</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.73491898148</v>
+        <v>46234.73924768518</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02070578395742099</v>
+        <v>0.02070578490075779</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3286941303118006</v>
+        <v>0.328694145286808</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911166025863079</v>
+        <v>0.0291116633546618</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331351341998324</v>
+        <v>0.04331352249973785</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645465</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 17:38:17.584506+05:30</t>
+          <t>2026-07-31 17:44:31.569855+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 13:08 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GD11"/>
+  <dimension ref="A1:GR11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -717,70 +717,84 @@
     <col width="23" customWidth="1" min="120" max="120"/>
     <col width="18" customWidth="1" min="121" max="121"/>
     <col width="12" customWidth="1" min="122" max="122"/>
-    <col width="17" customWidth="1" min="123" max="123"/>
-    <col width="16" customWidth="1" min="124" max="124"/>
-    <col width="22" customWidth="1" min="125" max="125"/>
-    <col width="20" customWidth="1" min="126" max="126"/>
-    <col width="19" customWidth="1" min="127" max="127"/>
-    <col width="18" customWidth="1" min="128" max="128"/>
-    <col width="16" customWidth="1" min="129" max="129"/>
-    <col width="14" customWidth="1" min="130" max="130"/>
-    <col width="14" customWidth="1" min="131" max="131"/>
+    <col width="15" customWidth="1" min="123" max="123"/>
+    <col width="13" customWidth="1" min="124" max="124"/>
+    <col width="17" customWidth="1" min="125" max="125"/>
+    <col width="16" customWidth="1" min="126" max="126"/>
+    <col width="22" customWidth="1" min="127" max="127"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="129" max="129"/>
+    <col width="18" customWidth="1" min="130" max="130"/>
+    <col width="16" customWidth="1" min="131" max="131"/>
     <col width="14" customWidth="1" min="132" max="132"/>
-    <col width="23" customWidth="1" min="133" max="133"/>
-    <col width="22" customWidth="1" min="134" max="134"/>
-    <col width="19" customWidth="1" min="135" max="135"/>
-    <col width="21" customWidth="1" min="136" max="136"/>
-    <col width="21" customWidth="1" min="137" max="137"/>
-    <col width="18" customWidth="1" min="138" max="138"/>
-    <col width="16" customWidth="1" min="139" max="139"/>
-    <col width="15" customWidth="1" min="140" max="140"/>
-    <col width="19" customWidth="1" min="141" max="141"/>
-    <col width="17" customWidth="1" min="142" max="142"/>
-    <col width="17" customWidth="1" min="143" max="143"/>
-    <col width="21" customWidth="1" min="144" max="144"/>
-    <col width="19" customWidth="1" min="145" max="145"/>
-    <col width="19" customWidth="1" min="146" max="146"/>
-    <col width="22" customWidth="1" min="147" max="147"/>
-    <col width="29" customWidth="1" min="148" max="148"/>
-    <col width="20" customWidth="1" min="149" max="149"/>
-    <col width="19" customWidth="1" min="150" max="150"/>
-    <col width="18" customWidth="1" min="151" max="151"/>
-    <col width="14" customWidth="1" min="152" max="152"/>
-    <col width="13" customWidth="1" min="153" max="153"/>
-    <col width="17" customWidth="1" min="154" max="154"/>
-    <col width="15" customWidth="1" min="155" max="155"/>
-    <col width="20" customWidth="1" min="156" max="156"/>
-    <col width="16" customWidth="1" min="157" max="157"/>
-    <col width="14" customWidth="1" min="158" max="158"/>
-    <col width="15" customWidth="1" min="159" max="159"/>
-    <col width="19" customWidth="1" min="160" max="160"/>
-    <col width="19" customWidth="1" min="161" max="161"/>
-    <col width="21" customWidth="1" min="162" max="162"/>
-    <col width="21" customWidth="1" min="163" max="163"/>
-    <col width="15" customWidth="1" min="164" max="164"/>
-    <col width="14" customWidth="1" min="165" max="165"/>
-    <col width="21" customWidth="1" min="166" max="166"/>
-    <col width="13" customWidth="1" min="167" max="167"/>
-    <col width="17" customWidth="1" min="168" max="168"/>
-    <col width="21" customWidth="1" min="169" max="169"/>
-    <col width="17" customWidth="1" min="170" max="170"/>
-    <col width="21" customWidth="1" min="171" max="171"/>
-    <col width="21" customWidth="1" min="172" max="172"/>
-    <col width="24" customWidth="1" min="173" max="173"/>
-    <col width="22" customWidth="1" min="174" max="174"/>
-    <col width="21" customWidth="1" min="175" max="175"/>
-    <col width="21" customWidth="1" min="176" max="176"/>
-    <col width="21" customWidth="1" min="177" max="177"/>
-    <col width="19" customWidth="1" min="178" max="178"/>
-    <col width="21" customWidth="1" min="179" max="179"/>
-    <col width="16" customWidth="1" min="180" max="180"/>
-    <col width="21" customWidth="1" min="181" max="181"/>
-    <col width="21" customWidth="1" min="182" max="182"/>
-    <col width="18" customWidth="1" min="183" max="183"/>
-    <col width="21" customWidth="1" min="184" max="184"/>
-    <col width="17" customWidth="1" min="185" max="185"/>
-    <col width="28" customWidth="1" min="186" max="186"/>
+    <col width="14" customWidth="1" min="133" max="133"/>
+    <col width="14" customWidth="1" min="134" max="134"/>
+    <col width="23" customWidth="1" min="135" max="135"/>
+    <col width="22" customWidth="1" min="136" max="136"/>
+    <col width="19" customWidth="1" min="137" max="137"/>
+    <col width="21" customWidth="1" min="138" max="138"/>
+    <col width="21" customWidth="1" min="139" max="139"/>
+    <col width="18" customWidth="1" min="140" max="140"/>
+    <col width="16" customWidth="1" min="141" max="141"/>
+    <col width="15" customWidth="1" min="142" max="142"/>
+    <col width="19" customWidth="1" min="143" max="143"/>
+    <col width="17" customWidth="1" min="144" max="144"/>
+    <col width="17" customWidth="1" min="145" max="145"/>
+    <col width="21" customWidth="1" min="146" max="146"/>
+    <col width="19" customWidth="1" min="147" max="147"/>
+    <col width="19" customWidth="1" min="148" max="148"/>
+    <col width="22" customWidth="1" min="149" max="149"/>
+    <col width="29" customWidth="1" min="150" max="150"/>
+    <col width="20" customWidth="1" min="151" max="151"/>
+    <col width="19" customWidth="1" min="152" max="152"/>
+    <col width="18" customWidth="1" min="153" max="153"/>
+    <col width="14" customWidth="1" min="154" max="154"/>
+    <col width="13" customWidth="1" min="155" max="155"/>
+    <col width="17" customWidth="1" min="156" max="156"/>
+    <col width="15" customWidth="1" min="157" max="157"/>
+    <col width="20" customWidth="1" min="158" max="158"/>
+    <col width="16" customWidth="1" min="159" max="159"/>
+    <col width="14" customWidth="1" min="160" max="160"/>
+    <col width="15" customWidth="1" min="161" max="161"/>
+    <col width="19" customWidth="1" min="162" max="162"/>
+    <col width="19" customWidth="1" min="163" max="163"/>
+    <col width="21" customWidth="1" min="164" max="164"/>
+    <col width="21" customWidth="1" min="165" max="165"/>
+    <col width="15" customWidth="1" min="166" max="166"/>
+    <col width="14" customWidth="1" min="167" max="167"/>
+    <col width="18" customWidth="1" min="168" max="168"/>
+    <col width="16" customWidth="1" min="169" max="169"/>
+    <col width="21" customWidth="1" min="170" max="170"/>
+    <col width="13" customWidth="1" min="171" max="171"/>
+    <col width="17" customWidth="1" min="172" max="172"/>
+    <col width="21" customWidth="1" min="173" max="173"/>
+    <col width="17" customWidth="1" min="174" max="174"/>
+    <col width="26" customWidth="1" min="175" max="175"/>
+    <col width="24" customWidth="1" min="176" max="176"/>
+    <col width="22" customWidth="1" min="177" max="177"/>
+    <col width="21" customWidth="1" min="178" max="178"/>
+    <col width="22" customWidth="1" min="179" max="179"/>
+    <col width="21" customWidth="1" min="180" max="180"/>
+    <col width="12" customWidth="1" min="181" max="181"/>
+    <col width="14" customWidth="1" min="182" max="182"/>
+    <col width="16" customWidth="1" min="183" max="183"/>
+    <col width="19" customWidth="1" min="184" max="184"/>
+    <col width="21" customWidth="1" min="185" max="185"/>
+    <col width="21" customWidth="1" min="186" max="186"/>
+    <col width="24" customWidth="1" min="187" max="187"/>
+    <col width="22" customWidth="1" min="188" max="188"/>
+    <col width="21" customWidth="1" min="189" max="189"/>
+    <col width="21" customWidth="1" min="190" max="190"/>
+    <col width="21" customWidth="1" min="191" max="191"/>
+    <col width="19" customWidth="1" min="192" max="192"/>
+    <col width="21" customWidth="1" min="193" max="193"/>
+    <col width="16" customWidth="1" min="194" max="194"/>
+    <col width="21" customWidth="1" min="195" max="195"/>
+    <col width="21" customWidth="1" min="196" max="196"/>
+    <col width="18" customWidth="1" min="197" max="197"/>
+    <col width="21" customWidth="1" min="198" max="198"/>
+    <col width="17" customWidth="1" min="199" max="199"/>
+    <col width="28" customWidth="1" min="200" max="200"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1396,320 +1410,390 @@
       </c>
       <c r="DS1" t="inlineStr">
         <is>
+          <t>risk_quintile</t>
+        </is>
+      </c>
+      <c r="DT1" t="inlineStr">
+        <is>
+          <t>risk_decile</t>
+        </is>
+      </c>
+      <c r="DU1" t="inlineStr">
+        <is>
           <t>trend_alignment</t>
         </is>
       </c>
-      <c r="DT1" t="inlineStr">
+      <c r="DV1" t="inlineStr">
         <is>
           <t>trend_strength</t>
         </is>
       </c>
-      <c r="DU1" t="inlineStr">
+      <c r="DW1" t="inlineStr">
         <is>
           <t>momentum_trend_ratio</t>
         </is>
       </c>
-      <c r="DV1" t="inlineStr">
+      <c r="DX1" t="inlineStr">
         <is>
           <t>rsi_trend_score</t>
         </is>
       </c>
-      <c r="DW1" t="inlineStr">
+      <c r="DY1" t="inlineStr">
         <is>
           <t>breakout_strength</t>
         </is>
       </c>
-      <c r="DX1" t="inlineStr">
+      <c r="DZ1" t="inlineStr">
         <is>
           <t>trend_conviction</t>
         </is>
       </c>
-      <c r="DY1" t="inlineStr">
+      <c r="EA1" t="inlineStr">
         <is>
           <t>trend_quintile</t>
         </is>
       </c>
-      <c r="DZ1" t="inlineStr">
+      <c r="EB1" t="inlineStr">
         <is>
           <t>trend_decile</t>
         </is>
       </c>
-      <c r="EA1" t="inlineStr">
+      <c r="EC1" t="inlineStr">
         <is>
           <t>roc_strength</t>
         </is>
       </c>
-      <c r="EB1" t="inlineStr">
+      <c r="ED1" t="inlineStr">
         <is>
           <t>rsi_strength</t>
         </is>
       </c>
-      <c r="EC1" t="inlineStr">
+      <c r="EE1" t="inlineStr">
         <is>
           <t>momentum_acceleration</t>
         </is>
       </c>
-      <c r="ED1" t="inlineStr">
+      <c r="EF1" t="inlineStr">
         <is>
           <t>momentum_persistence</t>
         </is>
       </c>
-      <c r="EE1" t="inlineStr">
+      <c r="EG1" t="inlineStr">
         <is>
           <t>relative_momentum</t>
         </is>
       </c>
-      <c r="EF1" t="inlineStr">
+      <c r="EH1" t="inlineStr">
         <is>
           <t>momentum_efficiency</t>
         </is>
       </c>
-      <c r="EG1" t="inlineStr">
+      <c r="EI1" t="inlineStr">
         <is>
           <t>conviction_momentum</t>
         </is>
       </c>
-      <c r="EH1" t="inlineStr">
+      <c r="EJ1" t="inlineStr">
         <is>
           <t>momentum_quality</t>
         </is>
       </c>
-      <c r="EI1" t="inlineStr">
+      <c r="EK1" t="inlineStr">
         <is>
           <t>momentum_score</t>
         </is>
       </c>
-      <c r="EJ1" t="inlineStr">
+      <c r="EL1" t="inlineStr">
         <is>
           <t>momentum_band</t>
         </is>
       </c>
-      <c r="EK1" t="inlineStr">
+      <c r="EM1" t="inlineStr">
         <is>
           <t>momentum_quintile</t>
         </is>
       </c>
-      <c r="EL1" t="inlineStr">
+      <c r="EN1" t="inlineStr">
         <is>
           <t>momentum_decile</t>
         </is>
       </c>
-      <c r="EM1" t="inlineStr">
+      <c r="EO1" t="inlineStr">
         <is>
           <t>volume_strength</t>
         </is>
       </c>
-      <c r="EN1" t="inlineStr">
+      <c r="EP1" t="inlineStr">
         <is>
           <t>participation_score</t>
         </is>
       </c>
-      <c r="EO1" t="inlineStr">
+      <c r="EQ1" t="inlineStr">
         <is>
           <t>volume_conviction</t>
         </is>
       </c>
-      <c r="EP1" t="inlineStr">
+      <c r="ER1" t="inlineStr">
         <is>
           <t>volume_efficiency</t>
         </is>
       </c>
-      <c r="EQ1" t="inlineStr">
+      <c r="ES1" t="inlineStr">
         <is>
           <t>liquidity_efficiency</t>
         </is>
       </c>
-      <c r="ER1" t="inlineStr">
+      <c r="ET1" t="inlineStr">
         <is>
           <t>institutional_participation</t>
         </is>
       </c>
-      <c r="ES1" t="inlineStr">
+      <c r="EU1" t="inlineStr">
         <is>
           <t>accumulation_score</t>
         </is>
       </c>
-      <c r="ET1" t="inlineStr">
+      <c r="EV1" t="inlineStr">
         <is>
           <t>distribution_risk</t>
         </is>
       </c>
-      <c r="EU1" t="inlineStr">
+      <c r="EW1" t="inlineStr">
         <is>
           <t>turnover_quality</t>
         </is>
       </c>
-      <c r="EV1" t="inlineStr">
+      <c r="EX1" t="inlineStr">
         <is>
           <t>volume_score</t>
         </is>
       </c>
-      <c r="EW1" t="inlineStr">
+      <c r="EY1" t="inlineStr">
         <is>
           <t>volume_band</t>
         </is>
       </c>
-      <c r="EX1" t="inlineStr">
+      <c r="EZ1" t="inlineStr">
         <is>
           <t>volume_quintile</t>
         </is>
       </c>
-      <c r="EY1" t="inlineStr">
+      <c r="FA1" t="inlineStr">
         <is>
           <t>volume_decile</t>
         </is>
       </c>
-      <c r="EZ1" t="inlineStr">
+      <c r="FB1" t="inlineStr">
         <is>
           <t>confidence_quality</t>
         </is>
       </c>
-      <c r="FA1" t="inlineStr">
+      <c r="FC1" t="inlineStr">
         <is>
           <t>reward_quality</t>
         </is>
       </c>
-      <c r="FB1" t="inlineStr">
+      <c r="FD1" t="inlineStr">
         <is>
           <t>risk_quality</t>
         </is>
       </c>
-      <c r="FC1" t="inlineStr">
+      <c r="FE1" t="inlineStr">
         <is>
           <t>trend_quality</t>
         </is>
       </c>
-      <c r="FD1" t="inlineStr">
+      <c r="FF1" t="inlineStr">
         <is>
           <t>liquidity_quality</t>
         </is>
       </c>
-      <c r="FE1" t="inlineStr">
+      <c r="FG1" t="inlineStr">
         <is>
           <t>stability_quality</t>
         </is>
       </c>
-      <c r="FF1" t="inlineStr">
+      <c r="FH1" t="inlineStr">
         <is>
           <t>consistency_quality</t>
         </is>
       </c>
-      <c r="FG1" t="inlineStr">
+      <c r="FI1" t="inlineStr">
         <is>
           <t>opportunity_quality</t>
         </is>
       </c>
-      <c r="FH1" t="inlineStr">
+      <c r="FJ1" t="inlineStr">
         <is>
           <t>quality_score</t>
         </is>
       </c>
-      <c r="FI1" t="inlineStr">
+      <c r="FK1" t="inlineStr">
         <is>
           <t>quality_band</t>
         </is>
       </c>
-      <c r="FJ1" t="inlineStr">
+      <c r="FL1" t="inlineStr">
+        <is>
+          <t>quality_quintile</t>
+        </is>
+      </c>
+      <c r="FM1" t="inlineStr">
+        <is>
+          <t>quality_decile</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
         <is>
           <t>institutional_score</t>
         </is>
       </c>
-      <c r="FK1" t="inlineStr">
+      <c r="FO1" t="inlineStr">
         <is>
           <t>alpha_score</t>
         </is>
       </c>
-      <c r="FL1" t="inlineStr">
+      <c r="FP1" t="inlineStr">
         <is>
           <t>execution_score</t>
         </is>
       </c>
-      <c r="FM1" t="inlineStr">
+      <c r="FQ1" t="inlineStr">
         <is>
           <t>portfolio_fit_score</t>
         </is>
       </c>
-      <c r="FN1" t="inlineStr">
+      <c r="FR1" t="inlineStr">
         <is>
           <t>composite_score</t>
         </is>
       </c>
-      <c r="FO1" t="inlineStr">
+      <c r="FS1" t="inlineStr">
+        <is>
+          <t>institutional_percentile</t>
+        </is>
+      </c>
+      <c r="FT1" t="inlineStr">
+        <is>
+          <t>institutional_quintile</t>
+        </is>
+      </c>
+      <c r="FU1" t="inlineStr">
+        <is>
+          <t>institutional_decile</t>
+        </is>
+      </c>
+      <c r="FV1" t="inlineStr">
+        <is>
+          <t>institutional_grade</t>
+        </is>
+      </c>
+      <c r="FW1" t="inlineStr">
+        <is>
+          <t>recommendation_score</t>
+        </is>
+      </c>
+      <c r="FX1" t="inlineStr">
+        <is>
+          <t>recommendation_band</t>
+        </is>
+      </c>
+      <c r="FY1" t="inlineStr">
+        <is>
+          <t>top_decile</t>
+        </is>
+      </c>
+      <c r="FZ1" t="inlineStr">
+        <is>
+          <t>top_quintile</t>
+        </is>
+      </c>
+      <c r="GA1" t="inlineStr">
+        <is>
+          <t>top_10_percent</t>
+        </is>
+      </c>
+      <c r="GB1" t="inlineStr">
+        <is>
+          <t>bottom_10_percent</t>
+        </is>
+      </c>
+      <c r="GC1" t="inlineStr">
         <is>
           <t>confidence_norm</t>
         </is>
       </c>
-      <c r="FP1" t="inlineStr">
+      <c r="GD1" t="inlineStr">
         <is>
           <t>rank_score_norm</t>
         </is>
       </c>
-      <c r="FQ1" t="inlineStr">
+      <c r="GE1" t="inlineStr">
         <is>
           <t>relative_strength_norm</t>
         </is>
       </c>
-      <c r="FR1" t="inlineStr">
+      <c r="GF1" t="inlineStr">
         <is>
           <t>expectancy_norm</t>
         </is>
       </c>
-      <c r="FS1" t="inlineStr">
+      <c r="GG1" t="inlineStr">
         <is>
           <t>win_rate_norm</t>
         </is>
       </c>
-      <c r="FT1" t="inlineStr">
+      <c r="GH1" t="inlineStr">
         <is>
           <t>portfolio_score</t>
         </is>
       </c>
-      <c r="FU1" t="inlineStr">
+      <c r="GI1" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="FV1" t="inlineStr">
+      <c r="GJ1" t="inlineStr">
         <is>
           <t>weight_pct</t>
         </is>
       </c>
-      <c r="FW1" t="inlineStr">
+      <c r="GK1" t="inlineStr">
         <is>
           <t>capital_fraction</t>
         </is>
       </c>
-      <c r="FX1" t="inlineStr">
+      <c r="GL1" t="inlineStr">
         <is>
           <t>current_weight</t>
         </is>
       </c>
-      <c r="FY1" t="inlineStr">
+      <c r="GM1" t="inlineStr">
         <is>
           <t>target_weight</t>
         </is>
       </c>
-      <c r="FZ1" t="inlineStr">
+      <c r="GN1" t="inlineStr">
         <is>
           <t>weight_change</t>
         </is>
       </c>
-      <c r="GA1" t="inlineStr">
+      <c r="GO1" t="inlineStr">
         <is>
           <t>rebalance_action</t>
         </is>
       </c>
-      <c r="GB1" t="inlineStr">
+      <c r="GP1" t="inlineStr">
         <is>
           <t>turnover</t>
         </is>
       </c>
-      <c r="GC1" t="inlineStr">
+      <c r="GQ1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="GD1" t="inlineStr">
+      <c r="GR1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
@@ -1765,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1942,7 +2026,7 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1543.78</v>
+        <v>1543.79</v>
       </c>
       <c r="BU2" t="n">
         <v>-12.92</v>
@@ -2037,7 +2121,7 @@
         <v>53.41614906832298</v>
       </c>
       <c r="CY2" t="n">
-        <v>94.06999999999999</v>
+        <v>13</v>
       </c>
       <c r="CZ2" t="n">
         <v>9.891500000000001</v>
@@ -2097,206 +2181,252 @@
         <v>41.83</v>
       </c>
       <c r="DS2" t="n">
+        <v>5</v>
+      </c>
+      <c r="DT2" t="n">
+        <v>9</v>
+      </c>
+      <c r="DU2" t="n">
         <v>2</v>
       </c>
-      <c r="DT2" t="n">
+      <c r="DV2" t="n">
         <v>100</v>
       </c>
-      <c r="DU2" t="n">
+      <c r="DW2" t="n">
         <v>7.5789</v>
       </c>
-      <c r="DV2" t="n">
+      <c r="DX2" t="n">
         <v>45.425</v>
       </c>
-      <c r="DW2" t="n">
+      <c r="DY2" t="n">
         <v>55.5</v>
       </c>
-      <c r="DX2" t="n">
+      <c r="DZ2" t="n">
         <v>91.61199999999999</v>
       </c>
-      <c r="DY2" t="n">
+      <c r="EA2" t="n">
         <v>5</v>
       </c>
-      <c r="DZ2" t="n">
+      <c r="EB2" t="n">
         <v>10</v>
       </c>
-      <c r="EA2" t="n">
+      <c r="EC2" t="n">
         <v>100</v>
       </c>
-      <c r="EB2" t="n">
+      <c r="ED2" t="n">
         <v>28.57</v>
       </c>
-      <c r="EC2" t="n">
+      <c r="EE2" t="n">
         <v>7.5789</v>
       </c>
-      <c r="ED2" t="n">
+      <c r="EF2" t="n">
         <v>1.11</v>
       </c>
-      <c r="EE2" t="n">
+      <c r="EG2" t="n">
         <v>2.4448</v>
       </c>
-      <c r="EF2" t="n">
+      <c r="EH2" t="n">
         <v>4.0047</v>
       </c>
-      <c r="EG2" t="n">
+      <c r="EI2" t="n">
         <v>0.3193</v>
       </c>
-      <c r="EH2" t="n">
+      <c r="EJ2" t="n">
         <v>0.6731</v>
       </c>
-      <c r="EI2" t="n">
+      <c r="EK2" t="n">
         <v>68.73999999999999</v>
       </c>
-      <c r="EJ2" t="inlineStr">
+      <c r="EL2" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EK2" t="n">
+      <c r="EM2" t="n">
         <v>5</v>
       </c>
-      <c r="EL2" t="n">
+      <c r="EN2" t="n">
         <v>10</v>
       </c>
-      <c r="EM2" t="n">
+      <c r="EO2" t="n">
         <v>16.12</v>
       </c>
-      <c r="EN2" t="n">
+      <c r="EP2" t="n">
         <v>2.1053</v>
       </c>
-      <c r="EO2" t="n">
+      <c r="EQ2" t="n">
         <v>0.145</v>
       </c>
-      <c r="EP2" t="n">
+      <c r="ER2" t="n">
         <v>8.9099</v>
       </c>
-      <c r="EQ2" t="n">
+      <c r="ES2" t="n">
         <v>12.3314</v>
       </c>
-      <c r="ER2" t="n">
+      <c r="ET2" t="n">
         <v>60.88</v>
       </c>
-      <c r="ES2" t="n">
+      <c r="EU2" t="n">
         <v>20.7792</v>
       </c>
-      <c r="ET2" t="n">
+      <c r="EV2" t="n">
         <v>1.1706</v>
       </c>
-      <c r="EU2" t="n">
+      <c r="EW2" t="n">
         <v>13.5489</v>
       </c>
-      <c r="EV2" t="n">
+      <c r="EX2" t="n">
         <v>64.29000000000001</v>
       </c>
-      <c r="EW2" t="inlineStr">
+      <c r="EY2" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EX2" t="n">
+      <c r="EZ2" t="n">
         <v>5</v>
       </c>
-      <c r="EY2" t="n">
+      <c r="FA2" t="n">
         <v>10</v>
       </c>
-      <c r="EZ2" t="n">
+      <c r="FB2" t="n">
         <v>100</v>
       </c>
-      <c r="FA2" t="n">
+      <c r="FC2" t="n">
         <v>36.01</v>
       </c>
-      <c r="FB2" t="n">
+      <c r="FD2" t="n">
         <v>75.88</v>
       </c>
-      <c r="FC2" t="n">
+      <c r="FE2" t="n">
         <v>76.395</v>
       </c>
-      <c r="FD2" t="n">
+      <c r="FF2" t="n">
         <v>64.7</v>
       </c>
-      <c r="FE2" t="n">
+      <c r="FG2" t="n">
         <v>24.2219</v>
       </c>
-      <c r="FF2" t="n">
+      <c r="FH2" t="n">
         <v>88.07299999999999</v>
       </c>
-      <c r="FG2" t="n">
+      <c r="FI2" t="n">
         <v>42.31</v>
       </c>
-      <c r="FH2" t="n">
+      <c r="FJ2" t="n">
         <v>67.45</v>
       </c>
-      <c r="FI2" t="inlineStr">
+      <c r="FK2" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="FJ2" t="n">
+      <c r="FL2" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM2" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN2" t="n">
         <v>59.76</v>
       </c>
-      <c r="FK2" t="n">
+      <c r="FO2" t="n">
         <v>61.66</v>
       </c>
-      <c r="FL2" t="n">
+      <c r="FP2" t="n">
         <v>62.97</v>
       </c>
-      <c r="FM2" t="n">
+      <c r="FQ2" t="n">
         <v>52.37</v>
       </c>
-      <c r="FN2" t="n">
+      <c r="FR2" t="n">
         <v>59.4</v>
       </c>
-      <c r="FO2" t="n">
+      <c r="FS2" t="n">
+        <v>97.5104</v>
+      </c>
+      <c r="FT2" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU2" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW2" t="n">
+        <v>55.883</v>
+      </c>
+      <c r="FX2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY2" t="b">
         <v>1</v>
       </c>
-      <c r="FP2" t="n">
+      <c r="FZ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="GD2" t="n">
         <v>0.6449489963803883</v>
       </c>
-      <c r="FQ2" t="n">
+      <c r="GE2" t="n">
         <v>1</v>
       </c>
-      <c r="FR2" t="n">
+      <c r="GF2" t="n">
         <v>1</v>
       </c>
-      <c r="FS2" t="n">
+      <c r="GG2" t="n">
         <v>0.3909774436090226</v>
       </c>
-      <c r="FT2" t="n">
+      <c r="GH2" t="n">
         <v>0.8325824432750187</v>
       </c>
-      <c r="FU2" t="n">
+      <c r="GI2" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FV2" t="n">
+      <c r="GJ2" t="n">
         <v>10.47423883705045</v>
       </c>
-      <c r="FW2" t="n">
+      <c r="GK2" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FX2" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY2" t="n">
+      <c r="GL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM2" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FZ2" t="n">
+      <c r="GN2" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GA2" t="inlineStr">
+      <c r="GO2" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB2" t="n">
+      <c r="GP2" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GC2" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD2" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ2" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR2" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="3">
@@ -2615,7 +2745,7 @@
         <v>3.519668737060042</v>
       </c>
       <c r="CY3" t="n">
-        <v>87.42</v>
+        <v>10</v>
       </c>
       <c r="CZ3" t="n">
         <v>15.619</v>
@@ -2678,203 +2808,249 @@
         <v>2</v>
       </c>
       <c r="DT3" t="n">
+        <v>4</v>
+      </c>
+      <c r="DU3" t="n">
+        <v>2</v>
+      </c>
+      <c r="DV3" t="n">
         <v>100</v>
       </c>
-      <c r="DU3" t="n">
+      <c r="DW3" t="n">
         <v>0.1231</v>
       </c>
-      <c r="DV3" t="n">
+      <c r="DX3" t="n">
         <v>68.625</v>
       </c>
-      <c r="DW3" t="n">
+      <c r="DY3" t="n">
         <v>30</v>
       </c>
-      <c r="DX3" t="n">
+      <c r="DZ3" t="n">
         <v>63.105</v>
       </c>
-      <c r="DY3" t="n">
+      <c r="EA3" t="n">
         <v>4</v>
       </c>
-      <c r="DZ3" t="n">
+      <c r="EB3" t="n">
         <v>7</v>
       </c>
-      <c r="EA3" t="n">
+      <c r="EC3" t="n">
         <v>49.61</v>
       </c>
-      <c r="EB3" t="n">
+      <c r="ED3" t="n">
         <v>59.05</v>
       </c>
-      <c r="EC3" t="n">
+      <c r="EE3" t="n">
         <v>0.1231</v>
       </c>
-      <c r="ED3" t="n">
+      <c r="EF3" t="n">
         <v>0.6</v>
       </c>
-      <c r="EE3" t="n">
+      <c r="EG3" t="n">
         <v>0.0505</v>
       </c>
-      <c r="EF3" t="n">
+      <c r="EH3" t="n">
         <v>4.0049</v>
       </c>
-      <c r="EG3" t="n">
+      <c r="EI3" t="n">
         <v>0.0053</v>
       </c>
-      <c r="EH3" t="n">
+      <c r="EJ3" t="n">
         <v>0.4546</v>
       </c>
-      <c r="EI3" t="n">
+      <c r="EK3" t="n">
         <v>45.66</v>
       </c>
-      <c r="EJ3" t="inlineStr">
+      <c r="EL3" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EK3" t="n">
+      <c r="EM3" t="n">
         <v>2</v>
       </c>
-      <c r="EL3" t="n">
+      <c r="EN3" t="n">
         <v>4</v>
       </c>
-      <c r="EM3" t="n">
+      <c r="EO3" t="n">
         <v>7.28</v>
       </c>
-      <c r="EN3" t="n">
+      <c r="EP3" t="n">
         <v>0.7665999999999999</v>
       </c>
-      <c r="EO3" t="n">
+      <c r="EQ3" t="n">
         <v>0.06320000000000001</v>
       </c>
-      <c r="EP3" t="n">
+      <c r="ER3" t="n">
         <v>26.0333</v>
       </c>
-      <c r="EQ3" t="n">
+      <c r="ES3" t="n">
         <v>20.4082</v>
       </c>
-      <c r="ER3" t="n">
+      <c r="ET3" t="n">
         <v>43.931</v>
       </c>
-      <c r="ES3" t="n">
+      <c r="EU3" t="n">
         <v>0.288</v>
       </c>
-      <c r="ET3" t="n">
+      <c r="EV3" t="n">
         <v>2.4375</v>
       </c>
-      <c r="EU3" t="n">
+      <c r="EW3" t="n">
         <v>4.6461</v>
       </c>
-      <c r="EV3" t="n">
+      <c r="EX3" t="n">
         <v>36.3</v>
       </c>
-      <c r="EW3" t="inlineStr">
+      <c r="EY3" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX3" t="n">
+      <c r="EZ3" t="n">
         <v>5</v>
       </c>
-      <c r="EY3" t="n">
+      <c r="FA3" t="n">
         <v>9</v>
       </c>
-      <c r="EZ3" t="n">
+      <c r="FB3" t="n">
         <v>83.84999999999999</v>
       </c>
-      <c r="FA3" t="n">
+      <c r="FC3" t="n">
         <v>96</v>
       </c>
-      <c r="FB3" t="n">
+      <c r="FD3" t="n">
         <v>44.57</v>
       </c>
-      <c r="FC3" t="n">
+      <c r="FE3" t="n">
         <v>54.74</v>
       </c>
-      <c r="FD3" t="n">
+      <c r="FF3" t="n">
         <v>38.89</v>
       </c>
-      <c r="FE3" t="n">
+      <c r="FG3" t="n">
         <v>13.0245</v>
       </c>
-      <c r="FF3" t="n">
+      <c r="FH3" t="n">
         <v>68.331</v>
       </c>
-      <c r="FG3" t="n">
+      <c r="FI3" t="n">
         <v>64.72</v>
       </c>
-      <c r="FH3" t="n">
+      <c r="FJ3" t="n">
         <v>60.14</v>
       </c>
-      <c r="FI3" t="inlineStr">
+      <c r="FK3" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="FJ3" t="n">
+      <c r="FL3" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM3" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN3" t="n">
         <v>57.97</v>
       </c>
-      <c r="FK3" t="n">
+      <c r="FO3" t="n">
         <v>75.56</v>
       </c>
-      <c r="FL3" t="n">
+      <c r="FP3" t="n">
         <v>41.76</v>
       </c>
-      <c r="FM3" t="n">
+      <c r="FQ3" t="n">
         <v>62.89</v>
       </c>
-      <c r="FN3" t="n">
+      <c r="FR3" t="n">
         <v>60.11</v>
       </c>
-      <c r="FO3" t="n">
+      <c r="FS3" t="n">
+        <v>98.1328</v>
+      </c>
+      <c r="FT3" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU3" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="FW3" t="n">
+        <v>61.499</v>
+      </c>
+      <c r="FX3" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="FY3" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ3" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA3" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB3" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC3" t="n">
         <v>0.6809583858764185</v>
       </c>
-      <c r="FP3" t="n">
+      <c r="GD3" t="n">
         <v>1</v>
       </c>
-      <c r="FQ3" t="n">
+      <c r="GE3" t="n">
         <v>0.2458309911935544</v>
       </c>
-      <c r="FR3" t="n">
+      <c r="GF3" t="n">
         <v>0.6462585034013604</v>
       </c>
-      <c r="FS3" t="n">
+      <c r="GG3" t="n">
         <v>1</v>
       </c>
-      <c r="FT3" t="n">
+      <c r="GH3" t="n">
         <v>0.7398359340759155</v>
       </c>
-      <c r="FU3" t="n">
+      <c r="GI3" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FV3" t="n">
+      <c r="GJ3" t="n">
         <v>10.47423883705045</v>
       </c>
-      <c r="FW3" t="n">
+      <c r="GK3" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FX3" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY3" t="n">
+      <c r="GL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM3" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FZ3" t="n">
+      <c r="GN3" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GA3" t="inlineStr">
+      <c r="GO3" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB3" t="n">
+      <c r="GP3" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GC3" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD3" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ3" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR3" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="4">
@@ -3193,7 +3369,7 @@
         <v>39.33747412008282</v>
       </c>
       <c r="CY4" t="n">
-        <v>87.67</v>
+        <v>3</v>
       </c>
       <c r="CZ4" t="n">
         <v>13.8536</v>
@@ -3253,206 +3429,252 @@
         <v>38.39</v>
       </c>
       <c r="DS4" t="n">
+        <v>4</v>
+      </c>
+      <c r="DT4" t="n">
+        <v>8</v>
+      </c>
+      <c r="DU4" t="n">
         <v>2</v>
       </c>
-      <c r="DT4" t="n">
+      <c r="DV4" t="n">
         <v>100</v>
       </c>
-      <c r="DU4" t="n">
+      <c r="DW4" t="n">
         <v>4.1503</v>
       </c>
-      <c r="DV4" t="n">
+      <c r="DX4" t="n">
         <v>72.95000000000002</v>
       </c>
-      <c r="DW4" t="n">
+      <c r="DY4" t="n">
         <v>46.5</v>
       </c>
-      <c r="DX4" t="n">
+      <c r="DZ4" t="n">
         <v>87.858</v>
       </c>
-      <c r="DY4" t="n">
+      <c r="EA4" t="n">
         <v>5</v>
       </c>
-      <c r="DZ4" t="n">
+      <c r="EB4" t="n">
         <v>10</v>
       </c>
-      <c r="EA4" t="n">
+      <c r="EC4" t="n">
         <v>97.73999999999999</v>
       </c>
-      <c r="EB4" t="n">
+      <c r="ED4" t="n">
         <v>64.73</v>
       </c>
-      <c r="EC4" t="n">
+      <c r="EE4" t="n">
         <v>4.1503</v>
       </c>
-      <c r="ED4" t="n">
+      <c r="EF4" t="n">
         <v>0.93</v>
       </c>
-      <c r="EE4" t="n">
+      <c r="EG4" t="n">
         <v>1.1919</v>
       </c>
-      <c r="EF4" t="n">
+      <c r="EH4" t="n">
         <v>4.0039</v>
       </c>
-      <c r="EG4" t="n">
+      <c r="EI4" t="n">
         <v>0.0989</v>
       </c>
-      <c r="EH4" t="n">
+      <c r="EJ4" t="n">
         <v>0.5049</v>
       </c>
-      <c r="EI4" t="n">
+      <c r="EK4" t="n">
         <v>68.14</v>
       </c>
-      <c r="EJ4" t="inlineStr">
+      <c r="EL4" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EK4" t="n">
+      <c r="EM4" t="n">
         <v>5</v>
       </c>
-      <c r="EL4" t="n">
+      <c r="EN4" t="n">
         <v>9</v>
       </c>
-      <c r="EM4" t="n">
+      <c r="EO4" t="n">
         <v>13</v>
       </c>
-      <c r="EN4" t="n">
+      <c r="EP4" t="n">
         <v>1.079</v>
       </c>
-      <c r="EO4" t="n">
+      <c r="EQ4" t="n">
         <v>0.0772</v>
       </c>
-      <c r="EP4" t="n">
+      <c r="ER4" t="n">
         <v>14.8925</v>
       </c>
-      <c r="EQ4" t="n">
+      <c r="ES4" t="n">
         <v>18.213</v>
       </c>
-      <c r="ER4" t="n">
+      <c r="ET4" t="n">
         <v>51.194</v>
       </c>
-      <c r="ES4" t="n">
+      <c r="EU4" t="n">
         <v>13.3548</v>
       </c>
-      <c r="ET4" t="n">
+      <c r="EV4" t="n">
         <v>1.7927</v>
       </c>
-      <c r="EU4" t="n">
+      <c r="EW4" t="n">
         <v>10.5144</v>
       </c>
-      <c r="EV4" t="n">
+      <c r="EX4" t="n">
         <v>47.3</v>
       </c>
-      <c r="EW4" t="inlineStr">
+      <c r="EY4" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EX4" t="n">
+      <c r="EZ4" t="n">
         <v>5</v>
       </c>
-      <c r="EY4" t="n">
+      <c r="FA4" t="n">
         <v>10</v>
       </c>
-      <c r="EZ4" t="n">
+      <c r="FB4" t="n">
         <v>66.09999999999999</v>
       </c>
-      <c r="FA4" t="n">
+      <c r="FC4" t="n">
         <v>77.47</v>
       </c>
-      <c r="FB4" t="n">
+      <c r="FD4" t="n">
         <v>74.92</v>
       </c>
-      <c r="FC4" t="n">
+      <c r="FE4" t="n">
         <v>74.51000000000001</v>
       </c>
-      <c r="FD4" t="n">
+      <c r="FF4" t="n">
         <v>57.98</v>
       </c>
-      <c r="FE4" t="n">
+      <c r="FG4" t="n">
         <v>18.1345</v>
       </c>
-      <c r="FF4" t="n">
+      <c r="FH4" t="n">
         <v>66.774</v>
       </c>
-      <c r="FG4" t="n">
+      <c r="FI4" t="n">
         <v>59.81</v>
       </c>
-      <c r="FH4" t="n">
+      <c r="FJ4" t="n">
         <v>64.94</v>
       </c>
-      <c r="FI4" t="inlineStr">
+      <c r="FK4" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="FJ4" t="n">
+      <c r="FL4" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM4" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN4" t="n">
         <v>64</v>
       </c>
-      <c r="FK4" t="n">
+      <c r="FO4" t="n">
         <v>77.84999999999999</v>
       </c>
-      <c r="FL4" t="n">
+      <c r="FP4" t="n">
         <v>49.05</v>
       </c>
-      <c r="FM4" t="n">
+      <c r="FQ4" t="n">
         <v>61.86</v>
       </c>
-      <c r="FN4" t="n">
+      <c r="FR4" t="n">
         <v>64.04000000000001</v>
       </c>
-      <c r="FO4" t="n">
+      <c r="FS4" t="n">
+        <v>99.5851</v>
+      </c>
+      <c r="FT4" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU4" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="FW4" t="n">
+        <v>62.951</v>
+      </c>
+      <c r="FX4" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="FY4" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ4" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA4" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC4" t="n">
         <v>0.3997477931904162</v>
       </c>
-      <c r="FP4" t="n">
+      <c r="GD4" t="n">
         <v>0.4781178019085225</v>
       </c>
-      <c r="FQ4" t="n">
+      <c r="GE4" t="n">
         <v>0.8390481543938542</v>
       </c>
-      <c r="FR4" t="n">
+      <c r="GF4" t="n">
         <v>0.6326530612244898</v>
       </c>
-      <c r="FS4" t="n">
+      <c r="GG4" t="n">
         <v>0.112781954887218</v>
       </c>
-      <c r="FT4" t="n">
+      <c r="GH4" t="n">
         <v>0.4837477929594513</v>
       </c>
-      <c r="FU4" t="n">
+      <c r="GI4" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FV4" t="n">
+      <c r="GJ4" t="n">
         <v>10.47423883705045</v>
       </c>
-      <c r="FW4" t="n">
+      <c r="GK4" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FX4" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY4" t="n">
+      <c r="GL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM4" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FZ4" t="n">
+      <c r="GN4" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GA4" t="inlineStr">
+      <c r="GO4" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB4" t="n">
+      <c r="GP4" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GC4" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD4" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ4" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR4" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="5">
@@ -3503,7 +3725,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -3771,7 +3993,7 @@
         <v>77.01863354037268</v>
       </c>
       <c r="CY5" t="n">
-        <v>81.84999999999999</v>
+        <v>42</v>
       </c>
       <c r="CZ5" t="n">
         <v>12.0377</v>
@@ -3831,206 +4053,252 @@
         <v>39.9</v>
       </c>
       <c r="DS5" t="n">
+        <v>4</v>
+      </c>
+      <c r="DT5" t="n">
+        <v>8</v>
+      </c>
+      <c r="DU5" t="n">
         <v>1</v>
       </c>
-      <c r="DT5" t="n">
+      <c r="DV5" t="n">
         <v>50</v>
       </c>
-      <c r="DU5" t="n">
+      <c r="DW5" t="n">
         <v>-0.5947</v>
       </c>
-      <c r="DV5" t="n">
+      <c r="DX5" t="n">
         <v>59.55</v>
       </c>
-      <c r="DW5" t="n">
+      <c r="DY5" t="n">
         <v>36.25</v>
       </c>
-      <c r="DX5" t="n">
+      <c r="DZ5" t="n">
         <v>40.705</v>
       </c>
-      <c r="DY5" t="n">
+      <c r="EA5" t="n">
         <v>2</v>
       </c>
-      <c r="DZ5" t="n">
+      <c r="EB5" t="n">
         <v>4</v>
       </c>
-      <c r="EA5" t="n">
+      <c r="EC5" t="n">
         <v>41.74</v>
       </c>
-      <c r="EB5" t="n">
+      <c r="ED5" t="n">
         <v>47.13</v>
       </c>
-      <c r="EC5" t="n">
+      <c r="EE5" t="n">
         <v>-0.5947</v>
       </c>
-      <c r="ED5" t="n">
+      <c r="EF5" t="n">
         <v>0.725</v>
       </c>
-      <c r="EE5" t="n">
+      <c r="EG5" t="n">
         <v>-0.2064</v>
       </c>
-      <c r="EF5" t="n">
+      <c r="EH5" t="n">
         <v>3.9992</v>
       </c>
-      <c r="EG5" t="n">
+      <c r="EI5" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="EH5" t="n">
+      <c r="EJ5" t="n">
         <v>0.5697</v>
       </c>
-      <c r="EI5" t="n">
+      <c r="EK5" t="n">
         <v>44</v>
       </c>
-      <c r="EJ5" t="inlineStr">
+      <c r="EL5" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EK5" t="n">
+      <c r="EM5" t="n">
         <v>2</v>
       </c>
-      <c r="EL5" t="n">
+      <c r="EN5" t="n">
         <v>3</v>
       </c>
-      <c r="EM5" t="n">
+      <c r="EO5" t="n">
         <v>22.01</v>
       </c>
-      <c r="EN5" t="n">
+      <c r="EP5" t="n">
         <v>2.5378</v>
       </c>
-      <c r="EO5" t="n">
+      <c r="EQ5" t="n">
         <v>0.1672</v>
       </c>
-      <c r="EP5" t="n">
+      <c r="ER5" t="n">
         <v>8.3034</v>
       </c>
-      <c r="EQ5" t="n">
+      <c r="ES5" t="n">
         <v>16.1471</v>
       </c>
-      <c r="ER5" t="n">
+      <c r="ET5" t="n">
         <v>52.937</v>
       </c>
-      <c r="ES5" t="n">
+      <c r="EU5" t="n">
         <v>-2.5955</v>
       </c>
-      <c r="ET5" t="n">
+      <c r="EV5" t="n">
         <v>1.2286</v>
       </c>
-      <c r="EU5" t="n">
+      <c r="EW5" t="n">
         <v>8.240500000000001</v>
       </c>
-      <c r="EV5" t="n">
+      <c r="EX5" t="n">
         <v>62.03</v>
       </c>
-      <c r="EW5" t="inlineStr">
+      <c r="EY5" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EX5" t="n">
+      <c r="EZ5" t="n">
         <v>5</v>
       </c>
-      <c r="EY5" t="n">
+      <c r="FA5" t="n">
         <v>10</v>
       </c>
-      <c r="EZ5" t="n">
+      <c r="FB5" t="n">
         <v>91.81999999999999</v>
       </c>
-      <c r="FA5" t="n">
+      <c r="FC5" t="n">
         <v>58.52</v>
       </c>
-      <c r="FB5" t="n">
+      <c r="FD5" t="n">
         <v>66.25</v>
       </c>
-      <c r="FC5" t="n">
+      <c r="FE5" t="n">
         <v>40.72</v>
       </c>
-      <c r="FD5" t="n">
+      <c r="FF5" t="n">
         <v>54.5</v>
       </c>
-      <c r="FE5" t="n">
+      <c r="FG5" t="n">
         <v>9.3367</v>
       </c>
-      <c r="FF5" t="n">
+      <c r="FH5" t="n">
         <v>69.548</v>
       </c>
-      <c r="FG5" t="n">
+      <c r="FI5" t="n">
         <v>52.325</v>
       </c>
-      <c r="FH5" t="n">
+      <c r="FJ5" t="n">
         <v>58.98</v>
       </c>
-      <c r="FI5" t="inlineStr">
+      <c r="FK5" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ5" t="n">
+      <c r="FL5" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM5" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN5" t="n">
         <v>51.14</v>
       </c>
-      <c r="FK5" t="n">
+      <c r="FO5" t="n">
         <v>51.37</v>
       </c>
-      <c r="FL5" t="n">
+      <c r="FP5" t="n">
         <v>58.73</v>
       </c>
-      <c r="FM5" t="n">
+      <c r="FQ5" t="n">
         <v>54.99</v>
       </c>
-      <c r="FN5" t="n">
+      <c r="FR5" t="n">
         <v>53.49</v>
       </c>
-      <c r="FO5" t="n">
+      <c r="FS5" t="n">
+        <v>91.49379999999999</v>
+      </c>
+      <c r="FT5" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU5" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW5" t="n">
+        <v>54.2385</v>
+      </c>
+      <c r="FX5" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY5" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ5" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA5" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB5" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC5" t="n">
         <v>0.8070617906683479</v>
       </c>
-      <c r="FP5" t="n">
+      <c r="GD5" t="n">
         <v>0.3445212240868706</v>
       </c>
-      <c r="FQ5" t="n">
+      <c r="GE5" t="n">
         <v>0.06651676972081692</v>
       </c>
-      <c r="FR5" t="n">
+      <c r="GF5" t="n">
         <v>0.5510204081632653</v>
       </c>
-      <c r="FS5" t="n">
+      <c r="GG5" t="n">
         <v>0.1278195488721806</v>
       </c>
-      <c r="FT5" t="n">
+      <c r="GH5" t="n">
         <v>0.46368950512165</v>
       </c>
-      <c r="FU5" t="n">
+      <c r="GI5" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FV5" t="n">
+      <c r="GJ5" t="n">
         <v>10.47423883705045</v>
       </c>
-      <c r="FW5" t="n">
+      <c r="GK5" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FX5" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY5" t="n">
+      <c r="GL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM5" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FZ5" t="n">
+      <c r="GN5" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GA5" t="inlineStr">
+      <c r="GO5" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB5" t="n">
+      <c r="GP5" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GC5" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD5" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ5" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR5" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="6">
@@ -4083,7 +4351,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -4355,7 +4623,7 @@
         <v>6.625258799171843</v>
       </c>
       <c r="CY6" t="n">
-        <v>89.20999999999999</v>
+        <v>111</v>
       </c>
       <c r="CZ6" t="n">
         <v>8.3043</v>
@@ -4415,206 +4683,252 @@
         <v>52.02</v>
       </c>
       <c r="DS6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DT6" t="n">
+        <v>10</v>
+      </c>
+      <c r="DU6" t="n">
         <v>2</v>
       </c>
-      <c r="DT6" t="n">
+      <c r="DV6" t="n">
         <v>100</v>
       </c>
-      <c r="DU6" t="n">
+      <c r="DW6" t="n">
         <v>4.9615</v>
       </c>
-      <c r="DV6" t="n">
+      <c r="DX6" t="n">
         <v>63.125</v>
       </c>
-      <c r="DW6" t="n">
+      <c r="DY6" t="n">
         <v>21.5</v>
       </c>
-      <c r="DX6" t="n">
+      <c r="DZ6" t="n">
         <v>84.426</v>
       </c>
-      <c r="DY6" t="n">
+      <c r="EA6" t="n">
         <v>5</v>
       </c>
-      <c r="DZ6" t="n">
+      <c r="EB6" t="n">
         <v>10</v>
       </c>
-      <c r="EA6" t="n">
+      <c r="EC6" t="n">
         <v>83.73</v>
       </c>
-      <c r="EB6" t="n">
+      <c r="ED6" t="n">
         <v>51.83</v>
       </c>
-      <c r="EC6" t="n">
+      <c r="EE6" t="n">
         <v>4.9615</v>
       </c>
-      <c r="ED6" t="n">
+      <c r="EF6" t="n">
         <v>0.43</v>
       </c>
-      <c r="EE6" t="n">
+      <c r="EG6" t="n">
         <v>0.6522</v>
       </c>
-      <c r="EF6" t="n">
+      <c r="EH6" t="n">
         <v>3.9925</v>
       </c>
-      <c r="EG6" t="n">
+      <c r="EI6" t="n">
         <v>0.0412</v>
       </c>
-      <c r="EH6" t="n">
+      <c r="EJ6" t="n">
         <v>0.7752</v>
       </c>
-      <c r="EI6" t="n">
+      <c r="EK6" t="n">
         <v>71.25</v>
       </c>
-      <c r="EJ6" t="inlineStr">
+      <c r="EL6" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EK6" t="n">
+      <c r="EM6" t="n">
         <v>5</v>
       </c>
-      <c r="EL6" t="n">
+      <c r="EN6" t="n">
         <v>10</v>
       </c>
-      <c r="EM6" t="n">
+      <c r="EO6" t="n">
         <v>4.33</v>
       </c>
-      <c r="EN6" t="n">
+      <c r="EP6" t="n">
         <v>0.2737</v>
       </c>
-      <c r="EO6" t="n">
+      <c r="EQ6" t="n">
         <v>0.0272</v>
       </c>
-      <c r="EP6" t="n">
+      <c r="ER6" t="n">
         <v>19.3023</v>
       </c>
-      <c r="EQ6" t="n">
+      <c r="ES6" t="n">
         <v>7.1104</v>
       </c>
-      <c r="ER6" t="n">
+      <c r="ET6" t="n">
         <v>30.838</v>
       </c>
-      <c r="ES6" t="n">
+      <c r="EU6" t="n">
         <v>4.4376</v>
       </c>
-      <c r="ET6" t="n">
+      <c r="EV6" t="n">
         <v>1.4545</v>
       </c>
-      <c r="EU6" t="n">
+      <c r="EW6" t="n">
         <v>3.4294</v>
       </c>
-      <c r="EV6" t="n">
+      <c r="EX6" t="n">
         <v>22.7</v>
       </c>
-      <c r="EW6" t="inlineStr">
+      <c r="EY6" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX6" t="n">
+      <c r="EZ6" t="n">
         <v>3</v>
       </c>
-      <c r="EY6" t="n">
+      <c r="FA6" t="n">
         <v>6</v>
       </c>
-      <c r="EZ6" t="n">
+      <c r="FB6" t="n">
         <v>50.33</v>
       </c>
-      <c r="FA6" t="n">
+      <c r="FC6" t="n">
         <v>19.37</v>
       </c>
-      <c r="FB6" t="n">
+      <c r="FD6" t="n">
         <v>79.25</v>
       </c>
-      <c r="FC6" t="n">
+      <c r="FE6" t="n">
         <v>75.22499999999999</v>
       </c>
-      <c r="FD6" t="n">
+      <c r="FF6" t="n">
         <v>29.4</v>
       </c>
-      <c r="FE6" t="n">
+      <c r="FG6" t="n">
         <v>25.7143</v>
       </c>
-      <c r="FF6" t="n">
+      <c r="FH6" t="n">
         <v>53.465</v>
       </c>
-      <c r="FG6" t="n">
+      <c r="FI6" t="n">
         <v>36.96</v>
       </c>
-      <c r="FH6" t="n">
+      <c r="FJ6" t="n">
         <v>50.14</v>
       </c>
-      <c r="FI6" t="inlineStr">
+      <c r="FK6" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ6" t="n">
+      <c r="FL6" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM6" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN6" t="n">
         <v>49.65</v>
       </c>
-      <c r="FK6" t="n">
+      <c r="FO6" t="n">
         <v>51.43</v>
       </c>
-      <c r="FL6" t="n">
+      <c r="FP6" t="n">
         <v>36.65</v>
       </c>
-      <c r="FM6" t="n">
+      <c r="FQ6" t="n">
         <v>42.23</v>
       </c>
-      <c r="FN6" t="n">
+      <c r="FR6" t="n">
         <v>46.01</v>
       </c>
-      <c r="FO6" t="n">
+      <c r="FS6" t="n">
+        <v>76.14109999999999</v>
+      </c>
+      <c r="FT6" t="n">
+        <v>4</v>
+      </c>
+      <c r="FU6" t="n">
+        <v>8</v>
+      </c>
+      <c r="FV6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW6" t="n">
+        <v>44.121</v>
+      </c>
+      <c r="FX6" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY6" t="b">
+        <v>0</v>
+      </c>
+      <c r="FZ6" t="b">
+        <v>0</v>
+      </c>
+      <c r="GA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="GB6" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC6" t="n">
         <v>0.150063051702396</v>
       </c>
-      <c r="FP6" t="n">
+      <c r="GD6" t="n">
         <v>0.6742349457058243</v>
       </c>
-      <c r="FQ6" t="n">
+      <c r="GE6" t="n">
         <v>0.2527637249391043</v>
       </c>
-      <c r="FR6" t="n">
+      <c r="GF6" t="n">
         <v>0.2653061224489797</v>
       </c>
-      <c r="FS6" t="n">
+      <c r="GG6" t="n">
         <v>0.150375939849624</v>
       </c>
-      <c r="FT6" t="n">
+      <c r="GH6" t="n">
         <v>0.3342753167783119</v>
       </c>
-      <c r="FU6" t="n">
+      <c r="GI6" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FV6" t="n">
+      <c r="GJ6" t="n">
         <v>10.47423883705045</v>
       </c>
-      <c r="FW6" t="n">
+      <c r="GK6" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FX6" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY6" t="n">
+      <c r="GL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM6" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FZ6" t="n">
+      <c r="GN6" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GA6" t="inlineStr">
+      <c r="GO6" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB6" t="n">
+      <c r="GP6" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GC6" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD6" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ6" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR6" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="7">
@@ -4665,7 +4979,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -4921,7 +5235,7 @@
         <v>50.72463768115942</v>
       </c>
       <c r="CU7" t="n">
-        <v>94.20289855072464</v>
+        <v>94.40993788819875</v>
       </c>
       <c r="CV7" t="n">
         <v>7.246376811594203</v>
@@ -4933,7 +5247,7 @@
         <v>55.48654244306418</v>
       </c>
       <c r="CY7" t="n">
-        <v>72.52</v>
+        <v>279</v>
       </c>
       <c r="CZ7" t="n">
         <v>10.8228</v>
@@ -4993,206 +5307,252 @@
         <v>27</v>
       </c>
       <c r="DS7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="DT7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="DU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW7" t="n">
         <v>-1.3469</v>
       </c>
-      <c r="DV7" t="n">
+      <c r="DX7" t="n">
         <v>58.62500000000001</v>
       </c>
-      <c r="DW7" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX7" t="n">
+      <c r="DY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ7" t="n">
         <v>17.091</v>
       </c>
-      <c r="DY7" t="n">
+      <c r="EA7" t="n">
         <v>1</v>
       </c>
-      <c r="DZ7" t="n">
+      <c r="EB7" t="n">
         <v>1</v>
       </c>
-      <c r="EA7" t="n">
+      <c r="EC7" t="n">
         <v>35.29</v>
       </c>
-      <c r="EB7" t="n">
+      <c r="ED7" t="n">
         <v>45.91</v>
       </c>
-      <c r="EC7" t="n">
+      <c r="EE7" t="n">
         <v>-1.3469</v>
       </c>
-      <c r="ED7" t="n">
-        <v>0</v>
-      </c>
-      <c r="EE7" t="n">
+      <c r="EF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="EG7" t="n">
         <v>-0.2489</v>
       </c>
-      <c r="EF7" t="n">
+      <c r="EH7" t="n">
         <v>3.9937</v>
       </c>
-      <c r="EG7" t="n">
+      <c r="EI7" t="n">
         <v>-0.017</v>
       </c>
-      <c r="EH7" t="n">
+      <c r="EJ7" t="n">
         <v>0.6221</v>
       </c>
-      <c r="EI7" t="n">
+      <c r="EK7" t="n">
         <v>41.17</v>
       </c>
-      <c r="EJ7" t="inlineStr">
+      <c r="EL7" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EK7" t="n">
+      <c r="EM7" t="n">
         <v>2</v>
       </c>
-      <c r="EL7" t="n">
+      <c r="EN7" t="n">
         <v>3</v>
       </c>
-      <c r="EM7" t="n">
+      <c r="EO7" t="n">
         <v>6.76</v>
       </c>
-      <c r="EN7" t="n">
+      <c r="EP7" t="n">
         <v>0.461</v>
       </c>
-      <c r="EO7" t="n">
+      <c r="EQ7" t="n">
         <v>0.0389</v>
       </c>
-      <c r="EP7" t="n">
+      <c r="ER7" t="n">
         <v>18.9825</v>
       </c>
-      <c r="EQ7" t="n">
+      <c r="ES7" t="n">
         <v>13.0243</v>
       </c>
-      <c r="ER7" t="n">
+      <c r="ET7" t="n">
         <v>48.309</v>
       </c>
-      <c r="ES7" t="n">
+      <c r="EU7" t="n">
         <v>-2.0805</v>
       </c>
-      <c r="ET7" t="n">
+      <c r="EV7" t="n">
         <v>1.7261</v>
       </c>
-      <c r="EU7" t="n">
+      <c r="EW7" t="n">
         <v>0.5043</v>
       </c>
-      <c r="EV7" t="n">
+      <c r="EX7" t="n">
         <v>38</v>
       </c>
-      <c r="EW7" t="inlineStr">
+      <c r="EY7" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX7" t="n">
+      <c r="EZ7" t="n">
         <v>5</v>
       </c>
-      <c r="EY7" t="n">
+      <c r="FA7" t="n">
         <v>10</v>
       </c>
-      <c r="EZ7" t="n">
+      <c r="FB7" t="n">
         <v>54.31</v>
       </c>
-      <c r="FA7" t="n">
+      <c r="FC7" t="n">
         <v>45.75</v>
       </c>
-      <c r="FB7" t="n">
+      <c r="FD7" t="n">
         <v>51.8</v>
       </c>
-      <c r="FC7" t="n">
+      <c r="FE7" t="n">
         <v>24.315</v>
       </c>
-      <c r="FD7" t="n">
+      <c r="FF7" t="n">
         <v>56.485</v>
       </c>
-      <c r="FE7" t="n">
+      <c r="FG7" t="n">
         <v>2.0108</v>
       </c>
-      <c r="FF7" t="n">
+      <c r="FH7" t="n">
         <v>36.993</v>
       </c>
-      <c r="FG7" t="n">
+      <c r="FI7" t="n">
         <v>37.66</v>
       </c>
-      <c r="FH7" t="n">
+      <c r="FJ7" t="n">
         <v>41.31</v>
       </c>
-      <c r="FI7" t="inlineStr">
+      <c r="FK7" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ7" t="n">
+      <c r="FL7" t="n">
+        <v>4</v>
+      </c>
+      <c r="FM7" t="n">
+        <v>8</v>
+      </c>
+      <c r="FN7" t="n">
         <v>34.42</v>
       </c>
-      <c r="FK7" t="n">
+      <c r="FO7" t="n">
         <v>34.27</v>
       </c>
-      <c r="FL7" t="n">
+      <c r="FP7" t="n">
         <v>39.92</v>
       </c>
-      <c r="FM7" t="n">
+      <c r="FQ7" t="n">
         <v>39.12</v>
       </c>
-      <c r="FN7" t="n">
+      <c r="FR7" t="n">
         <v>36.42</v>
       </c>
-      <c r="FO7" t="n">
+      <c r="FS7" t="n">
+        <v>37.3444</v>
+      </c>
+      <c r="FT7" t="n">
+        <v>2</v>
+      </c>
+      <c r="FU7" t="n">
+        <v>4</v>
+      </c>
+      <c r="FV7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="FW7" t="n">
+        <v>37.77</v>
+      </c>
+      <c r="FX7" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="FY7" t="b">
+        <v>0</v>
+      </c>
+      <c r="FZ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="GA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="GB7" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC7" t="n">
         <v>0.2131147540983607</v>
       </c>
-      <c r="FP7" t="n">
-        <v>0</v>
-      </c>
-      <c r="FQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="FR7" t="n">
+      <c r="GD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="GE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="GF7" t="n">
         <v>0.1292517006802721</v>
       </c>
-      <c r="FS7" t="n">
+      <c r="GG7" t="n">
         <v>0.2180451127819552</v>
       </c>
-      <c r="FT7" t="n">
+      <c r="GH7" t="n">
         <v>0.109319845280649</v>
       </c>
-      <c r="FU7" t="n">
+      <c r="GI7" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FV7" t="n">
+      <c r="GJ7" t="n">
         <v>10.47423883705045</v>
       </c>
-      <c r="FW7" t="n">
+      <c r="GK7" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FX7" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY7" t="n">
+      <c r="GL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM7" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="FZ7" t="n">
+      <c r="GN7" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GA7" t="inlineStr">
+      <c r="GO7" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB7" t="n">
+      <c r="GP7" t="n">
         <v>0.1047423883705045</v>
       </c>
-      <c r="GC7" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD7" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ7" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR7" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="8">
@@ -5243,7 +5603,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -5487,7 +5847,7 @@
         <v>92.96066252587993</v>
       </c>
       <c r="CQ8" t="n">
-        <v>94.20289855072464</v>
+        <v>94.30641821946169</v>
       </c>
       <c r="CR8" t="n">
         <v>73.70600414078675</v>
@@ -5511,7 +5871,7 @@
         <v>25.05175983436853</v>
       </c>
       <c r="CY8" t="n">
-        <v>86.59</v>
+        <v>45</v>
       </c>
       <c r="CZ8" t="n">
         <v>12.868</v>
@@ -5571,206 +5931,252 @@
         <v>38.71</v>
       </c>
       <c r="DS8" t="n">
+        <v>4</v>
+      </c>
+      <c r="DT8" t="n">
+        <v>8</v>
+      </c>
+      <c r="DU8" t="n">
         <v>2</v>
       </c>
-      <c r="DT8" t="n">
+      <c r="DV8" t="n">
         <v>100</v>
       </c>
-      <c r="DU8" t="n">
+      <c r="DW8" t="n">
         <v>-0.6056</v>
       </c>
-      <c r="DV8" t="n">
+      <c r="DX8" t="n">
         <v>99.97500000000001</v>
       </c>
-      <c r="DW8" t="n">
+      <c r="DY8" t="n">
         <v>48</v>
       </c>
-      <c r="DX8" t="n">
+      <c r="DZ8" t="n">
         <v>66.43600000000001</v>
       </c>
-      <c r="DY8" t="n">
+      <c r="EA8" t="n">
         <v>4</v>
       </c>
-      <c r="DZ8" t="n">
+      <c r="EB8" t="n">
         <v>7</v>
       </c>
-      <c r="EA8" t="n">
+      <c r="EC8" t="n">
         <v>41.18</v>
       </c>
-      <c r="EB8" t="n">
+      <c r="ED8" t="n">
         <v>100</v>
       </c>
-      <c r="EC8" t="n">
+      <c r="EE8" t="n">
         <v>-0.6056</v>
       </c>
-      <c r="ED8" t="n">
+      <c r="EF8" t="n">
         <v>0.96</v>
       </c>
-      <c r="EE8" t="n">
+      <c r="EG8" t="n">
         <v>-0.1203</v>
       </c>
-      <c r="EF8" t="n">
+      <c r="EH8" t="n">
         <v>3.9963</v>
       </c>
-      <c r="EG8" t="n">
+      <c r="EI8" t="n">
         <v>-0.0074</v>
       </c>
-      <c r="EH8" t="n">
+      <c r="EJ8" t="n">
         <v>0.5379</v>
       </c>
-      <c r="EI8" t="n">
+      <c r="EK8" t="n">
         <v>53.78</v>
       </c>
-      <c r="EJ8" t="inlineStr">
+      <c r="EL8" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EK8" t="n">
+      <c r="EM8" t="n">
         <v>3</v>
       </c>
-      <c r="EL8" t="n">
+      <c r="EN8" t="n">
         <v>6</v>
       </c>
-      <c r="EM8" t="n">
+      <c r="EO8" t="n">
         <v>13.52</v>
       </c>
-      <c r="EN8" t="n">
+      <c r="EP8" t="n">
         <v>0.8342000000000001</v>
       </c>
-      <c r="EO8" t="n">
+      <c r="EQ8" t="n">
         <v>0.0592</v>
       </c>
-      <c r="EP8" t="n">
+      <c r="ER8" t="n">
         <v>13.4062</v>
       </c>
-      <c r="EQ8" t="n">
+      <c r="ES8" t="n">
         <v>16.3697</v>
       </c>
-      <c r="ER8" t="n">
+      <c r="ET8" t="n">
         <v>38.359</v>
       </c>
-      <c r="ES8" t="n">
+      <c r="EU8" t="n">
         <v>-1.872</v>
       </c>
-      <c r="ET8" t="n">
+      <c r="EV8" t="n">
         <v>1.6429</v>
       </c>
-      <c r="EU8" t="n">
+      <c r="EW8" t="n">
         <v>8.801500000000001</v>
       </c>
-      <c r="EV8" t="n">
+      <c r="EX8" t="n">
         <v>35.38</v>
       </c>
-      <c r="EW8" t="inlineStr">
+      <c r="EY8" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX8" t="n">
+      <c r="EZ8" t="n">
         <v>5</v>
       </c>
-      <c r="EY8" t="n">
+      <c r="FA8" t="n">
         <v>9</v>
       </c>
-      <c r="EZ8" t="n">
+      <c r="FB8" t="n">
         <v>49.13</v>
       </c>
-      <c r="FA8" t="n">
+      <c r="FC8" t="n">
         <v>67.20999999999999</v>
       </c>
-      <c r="FB8" t="n">
+      <c r="FD8" t="n">
         <v>52.76</v>
       </c>
-      <c r="FC8" t="n">
+      <c r="FE8" t="n">
         <v>59.44</v>
       </c>
-      <c r="FD8" t="n">
+      <c r="FF8" t="n">
         <v>42.145</v>
       </c>
-      <c r="FE8" t="n">
+      <c r="FG8" t="n">
         <v>15.4265</v>
       </c>
-      <c r="FF8" t="n">
+      <c r="FH8" t="n">
         <v>51.171</v>
       </c>
-      <c r="FG8" t="n">
+      <c r="FI8" t="n">
         <v>53.895</v>
       </c>
-      <c r="FH8" t="n">
+      <c r="FJ8" t="n">
         <v>50.39</v>
       </c>
-      <c r="FI8" t="inlineStr">
+      <c r="FK8" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ8" t="n">
+      <c r="FL8" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM8" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN8" t="n">
         <v>53.01</v>
       </c>
-      <c r="FK8" t="n">
+      <c r="FO8" t="n">
         <v>64.06</v>
       </c>
-      <c r="FL8" t="n">
+      <c r="FP8" t="n">
         <v>39.46</v>
       </c>
-      <c r="FM8" t="n">
+      <c r="FQ8" t="n">
         <v>52.49</v>
       </c>
-      <c r="FN8" t="n">
+      <c r="FR8" t="n">
         <v>52.96</v>
       </c>
-      <c r="FO8" t="n">
+      <c r="FS8" t="n">
+        <v>90.6639</v>
+      </c>
+      <c r="FT8" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU8" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW8" t="n">
+        <v>52.7265</v>
+      </c>
+      <c r="FX8" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY8" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ8" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA8" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB8" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC8" t="n">
         <v>0.1311475409836066</v>
       </c>
-      <c r="FP8" t="n">
+      <c r="GD8" t="n">
         <v>0.2546890424481738</v>
       </c>
-      <c r="FQ8" t="n">
+      <c r="GE8" t="n">
         <v>0.4131534569983136</v>
       </c>
-      <c r="FR8" t="n">
+      <c r="GF8" t="n">
         <v>0.1088435374149661</v>
       </c>
-      <c r="FS8" t="n">
+      <c r="GG8" t="n">
         <v>0.2406015037593986</v>
       </c>
-      <c r="FT8" t="n">
+      <c r="GH8" t="n">
         <v>0.2192258747458979</v>
       </c>
-      <c r="FU8" t="n">
+      <c r="GI8" t="n">
         <v>0.1022952602643429</v>
       </c>
-      <c r="FV8" t="n">
+      <c r="GJ8" t="n">
         <v>10.22952602643429</v>
       </c>
-      <c r="FW8" t="n">
+      <c r="GK8" t="n">
         <v>0.1022952602643429</v>
       </c>
-      <c r="FX8" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY8" t="n">
+      <c r="GL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM8" t="n">
         <v>0.1022952602643429</v>
       </c>
-      <c r="FZ8" t="n">
+      <c r="GN8" t="n">
         <v>0.1022952602643429</v>
       </c>
-      <c r="GA8" t="inlineStr">
+      <c r="GO8" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB8" t="n">
+      <c r="GP8" t="n">
         <v>0.1022952602643429</v>
       </c>
-      <c r="GC8" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD8" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ8" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR8" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="9">
@@ -5821,7 +6227,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -6089,7 +6495,7 @@
         <v>45.13457556935818</v>
       </c>
       <c r="CY9" t="n">
-        <v>80.73</v>
+        <v>59</v>
       </c>
       <c r="CZ9" t="n">
         <v>10.5036</v>
@@ -6149,206 +6555,252 @@
         <v>43.18</v>
       </c>
       <c r="DS9" t="n">
+        <v>5</v>
+      </c>
+      <c r="DT9" t="n">
+        <v>9</v>
+      </c>
+      <c r="DU9" t="n">
         <v>2</v>
       </c>
-      <c r="DT9" t="n">
+      <c r="DV9" t="n">
         <v>100</v>
       </c>
-      <c r="DU9" t="n">
+      <c r="DW9" t="n">
         <v>2.924</v>
       </c>
-      <c r="DV9" t="n">
+      <c r="DX9" t="n">
         <v>92.15000000000001</v>
       </c>
-      <c r="DW9" t="n">
+      <c r="DY9" t="n">
         <v>26.5</v>
       </c>
-      <c r="DX9" t="n">
+      <c r="DZ9" t="n">
         <v>77.024</v>
       </c>
-      <c r="DY9" t="n">
+      <c r="EA9" t="n">
         <v>5</v>
       </c>
-      <c r="DZ9" t="n">
+      <c r="EB9" t="n">
         <v>9</v>
       </c>
-      <c r="EA9" t="n">
+      <c r="EC9" t="n">
         <v>74.61</v>
       </c>
-      <c r="EB9" t="n">
+      <c r="ED9" t="n">
         <v>89.95999999999999</v>
       </c>
-      <c r="EC9" t="n">
+      <c r="EE9" t="n">
         <v>2.924</v>
       </c>
-      <c r="ED9" t="n">
+      <c r="EF9" t="n">
         <v>0.53</v>
       </c>
-      <c r="EE9" t="n">
+      <c r="EG9" t="n">
         <v>0.4422</v>
       </c>
-      <c r="EF9" t="n">
+      <c r="EH9" t="n">
         <v>3.9938</v>
       </c>
-      <c r="EG9" t="n">
+      <c r="EI9" t="n">
         <v>0.0254</v>
       </c>
-      <c r="EH9" t="n">
+      <c r="EJ9" t="n">
         <v>0.639</v>
       </c>
-      <c r="EI9" t="n">
+      <c r="EK9" t="n">
         <v>68.81</v>
       </c>
-      <c r="EJ9" t="inlineStr">
+      <c r="EL9" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EK9" t="n">
+      <c r="EM9" t="n">
         <v>5</v>
       </c>
-      <c r="EL9" t="n">
+      <c r="EN9" t="n">
         <v>10</v>
       </c>
-      <c r="EM9" t="n">
+      <c r="EO9" t="n">
         <v>6.07</v>
       </c>
-      <c r="EN9" t="n">
+      <c r="EP9" t="n">
         <v>0.349</v>
       </c>
-      <c r="EO9" t="n">
+      <c r="EQ9" t="n">
         <v>0.0305</v>
       </c>
-      <c r="EP9" t="n">
+      <c r="ER9" t="n">
         <v>19.8113</v>
       </c>
-      <c r="EQ9" t="n">
+      <c r="ES9" t="n">
         <v>12.2011</v>
       </c>
-      <c r="ER9" t="n">
+      <c r="ET9" t="n">
         <v>43.666</v>
       </c>
-      <c r="ES9" t="n">
+      <c r="EU9" t="n">
         <v>4.0757</v>
       </c>
-      <c r="ET9" t="n">
+      <c r="EV9" t="n">
         <v>1.719</v>
       </c>
-      <c r="EU9" t="n">
+      <c r="EW9" t="n">
         <v>4.4554</v>
       </c>
-      <c r="EV9" t="n">
+      <c r="EX9" t="n">
         <v>34.7</v>
       </c>
-      <c r="EW9" t="inlineStr">
+      <c r="EY9" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX9" t="n">
+      <c r="EZ9" t="n">
         <v>5</v>
       </c>
-      <c r="EY9" t="n">
+      <c r="FA9" t="n">
         <v>9</v>
       </c>
-      <c r="EZ9" t="n">
+      <c r="FB9" t="n">
         <v>45.79</v>
       </c>
-      <c r="FA9" t="n">
+      <c r="FC9" t="n">
         <v>42.4</v>
       </c>
-      <c r="FB9" t="n">
+      <c r="FD9" t="n">
         <v>58.54</v>
       </c>
-      <c r="FC9" t="n">
+      <c r="FE9" t="n">
         <v>71.105</v>
       </c>
-      <c r="FD9" t="n">
+      <c r="FF9" t="n">
         <v>52.485</v>
       </c>
-      <c r="FE9" t="n">
+      <c r="FG9" t="n">
         <v>20.2204</v>
       </c>
-      <c r="FF9" t="n">
+      <c r="FH9" t="n">
         <v>51.855</v>
       </c>
-      <c r="FG9" t="n">
+      <c r="FI9" t="n">
         <v>43.735</v>
       </c>
-      <c r="FH9" t="n">
+      <c r="FJ9" t="n">
         <v>49.94</v>
       </c>
-      <c r="FI9" t="inlineStr">
+      <c r="FK9" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ9" t="n">
+      <c r="FL9" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM9" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN9" t="n">
         <v>52.28</v>
       </c>
-      <c r="FK9" t="n">
+      <c r="FO9" t="n">
         <v>59.15</v>
       </c>
-      <c r="FL9" t="n">
+      <c r="FP9" t="n">
         <v>41.58</v>
       </c>
-      <c r="FM9" t="n">
+      <c r="FQ9" t="n">
         <v>46.22</v>
       </c>
-      <c r="FN9" t="n">
+      <c r="FR9" t="n">
         <v>50.65</v>
       </c>
-      <c r="FO9" t="n">
+      <c r="FS9" t="n">
+        <v>87.7593</v>
+      </c>
+      <c r="FT9" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU9" t="n">
+        <v>9</v>
+      </c>
+      <c r="FV9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW9" t="n">
+        <v>48.4335</v>
+      </c>
+      <c r="FX9" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY9" t="b">
+        <v>0</v>
+      </c>
+      <c r="FZ9" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="GB9" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC9" t="n">
         <v>0.07818411097099623</v>
       </c>
-      <c r="FP9" t="n">
+      <c r="GD9" t="n">
         <v>0.1013491280026324</v>
       </c>
-      <c r="FQ9" t="n">
+      <c r="GE9" t="n">
         <v>0.04609331084879145</v>
       </c>
-      <c r="FR9" t="n">
+      <c r="GF9" t="n">
         <v>0.07482993197278917</v>
       </c>
-      <c r="FS9" t="n">
+      <c r="GG9" t="n">
         <v>0.03007518796992523</v>
       </c>
-      <c r="FT9" t="n">
+      <c r="GH9" t="n">
         <v>0.07517368586222856</v>
       </c>
-      <c r="FU9" t="n">
+      <c r="GI9" t="n">
         <v>0.0953318876045335</v>
       </c>
-      <c r="FV9" t="n">
+      <c r="GJ9" t="n">
         <v>9.533188760453349</v>
       </c>
-      <c r="FW9" t="n">
+      <c r="GK9" t="n">
         <v>0.0953318876045335</v>
       </c>
-      <c r="FX9" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY9" t="n">
+      <c r="GL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM9" t="n">
         <v>0.0953318876045335</v>
       </c>
-      <c r="FZ9" t="n">
+      <c r="GN9" t="n">
         <v>0.0953318876045335</v>
       </c>
-      <c r="GA9" t="inlineStr">
+      <c r="GO9" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB9" t="n">
+      <c r="GP9" t="n">
         <v>0.0953318876045335</v>
       </c>
-      <c r="GC9" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD9" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ9" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR9" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="10">
@@ -6399,7 +6851,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -6572,7 +7024,7 @@
         <v>0.123</v>
       </c>
       <c r="BT10" t="n">
-        <v>577.6799999999999</v>
+        <v>577.67</v>
       </c>
       <c r="BU10" t="n">
         <v>-17.65</v>
@@ -6667,7 +7119,7 @@
         <v>63.97515527950311</v>
       </c>
       <c r="CY10" t="n">
-        <v>84.13</v>
+        <v>31</v>
       </c>
       <c r="CZ10" t="n">
         <v>14.0241</v>
@@ -6727,206 +7179,252 @@
         <v>34.65</v>
       </c>
       <c r="DS10" t="n">
+        <v>3</v>
+      </c>
+      <c r="DT10" t="n">
+        <v>6</v>
+      </c>
+      <c r="DU10" t="n">
         <v>2</v>
       </c>
-      <c r="DT10" t="n">
+      <c r="DV10" t="n">
         <v>100</v>
       </c>
-      <c r="DU10" t="n">
+      <c r="DW10" t="n">
         <v>2.3932</v>
       </c>
-      <c r="DV10" t="n">
+      <c r="DX10" t="n">
         <v>95.72499999999999</v>
       </c>
-      <c r="DW10" t="n">
+      <c r="DY10" t="n">
         <v>20</v>
       </c>
-      <c r="DX10" t="n">
+      <c r="DZ10" t="n">
         <v>76.94</v>
       </c>
-      <c r="DY10" t="n">
+      <c r="EA10" t="n">
         <v>5</v>
       </c>
-      <c r="DZ10" t="n">
+      <c r="EB10" t="n">
         <v>9</v>
       </c>
-      <c r="EA10" t="n">
+      <c r="EC10" t="n">
         <v>77.06999999999999</v>
       </c>
-      <c r="EB10" t="n">
+      <c r="ED10" t="n">
         <v>94.66</v>
       </c>
-      <c r="EC10" t="n">
+      <c r="EE10" t="n">
         <v>2.3932</v>
       </c>
-      <c r="ED10" t="n">
+      <c r="EF10" t="n">
         <v>0.4</v>
       </c>
-      <c r="EE10" t="n">
+      <c r="EG10" t="n">
         <v>0.4502</v>
       </c>
-      <c r="EF10" t="n">
+      <c r="EH10" t="n">
         <v>3.9955</v>
       </c>
-      <c r="EG10" t="n">
+      <c r="EI10" t="n">
         <v>0.0241</v>
       </c>
-      <c r="EH10" t="n">
+      <c r="EJ10" t="n">
         <v>0.4988</v>
       </c>
-      <c r="EI10" t="n">
+      <c r="EK10" t="n">
         <v>64.64</v>
       </c>
-      <c r="EJ10" t="inlineStr">
+      <c r="EL10" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="EK10" t="n">
+      <c r="EM10" t="n">
         <v>5</v>
       </c>
-      <c r="EL10" t="n">
+      <c r="EN10" t="n">
         <v>9</v>
       </c>
-      <c r="EM10" t="n">
+      <c r="EO10" t="n">
         <v>3.81</v>
       </c>
-      <c r="EN10" t="n">
+      <c r="EP10" t="n">
         <v>0.2042</v>
       </c>
-      <c r="EO10" t="n">
+      <c r="EQ10" t="n">
         <v>0.0214</v>
       </c>
-      <c r="EP10" t="n">
+      <c r="ER10" t="n">
         <v>35.05</v>
       </c>
-      <c r="EQ10" t="n">
+      <c r="ES10" t="n">
         <v>17.796</v>
       </c>
-      <c r="ER10" t="n">
+      <c r="ET10" t="n">
         <v>29.927</v>
       </c>
-      <c r="ES10" t="n">
+      <c r="EU10" t="n">
         <v>3.36</v>
       </c>
-      <c r="ET10" t="n">
+      <c r="EV10" t="n">
         <v>2.5071</v>
       </c>
-      <c r="EU10" t="n">
+      <c r="EW10" t="n">
         <v>2.7428</v>
       </c>
-      <c r="EV10" t="n">
+      <c r="EX10" t="n">
         <v>25.1</v>
       </c>
-      <c r="EW10" t="inlineStr">
+      <c r="EY10" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX10" t="n">
+      <c r="EZ10" t="n">
         <v>3</v>
       </c>
-      <c r="EY10" t="n">
+      <c r="FA10" t="n">
         <v>6</v>
       </c>
-      <c r="EZ10" t="n">
+      <c r="FB10" t="n">
         <v>42.68</v>
       </c>
-      <c r="FA10" t="n">
+      <c r="FC10" t="n">
         <v>79.25</v>
       </c>
-      <c r="FB10" t="n">
+      <c r="FD10" t="n">
         <v>55.65</v>
       </c>
-      <c r="FC10" t="n">
+      <c r="FE10" t="n">
         <v>68.315</v>
       </c>
-      <c r="FD10" t="n">
+      <c r="FF10" t="n">
         <v>32.525</v>
       </c>
-      <c r="FE10" t="n">
+      <c r="FG10" t="n">
         <v>15.9623</v>
       </c>
-      <c r="FF10" t="n">
+      <c r="FH10" t="n">
         <v>47.957</v>
       </c>
-      <c r="FG10" t="n">
+      <c r="FI10" t="n">
         <v>57.455</v>
       </c>
-      <c r="FH10" t="n">
+      <c r="FJ10" t="n">
         <v>51.92</v>
       </c>
-      <c r="FI10" t="inlineStr">
+      <c r="FK10" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ10" t="n">
+      <c r="FL10" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM10" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN10" t="n">
         <v>56.37</v>
       </c>
-      <c r="FK10" t="n">
+      <c r="FO10" t="n">
         <v>73.87</v>
       </c>
-      <c r="FL10" t="n">
+      <c r="FP10" t="n">
         <v>31.72</v>
       </c>
-      <c r="FM10" t="n">
+      <c r="FQ10" t="n">
         <v>55.24</v>
       </c>
-      <c r="FN10" t="n">
+      <c r="FR10" t="n">
         <v>55.59</v>
       </c>
-      <c r="FO10" t="n">
+      <c r="FS10" t="n">
+        <v>93.77589999999999</v>
+      </c>
+      <c r="FT10" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU10" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW10" t="n">
+        <v>55.4155</v>
+      </c>
+      <c r="FX10" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY10" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ10" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA10" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB10" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC10" t="n">
         <v>0.02900378310214381</v>
       </c>
-      <c r="FP10" t="n">
+      <c r="GD10" t="n">
         <v>0.1872326423165514</v>
       </c>
-      <c r="FQ10" t="n">
+      <c r="GE10" t="n">
         <v>0.3473861720067453</v>
       </c>
-      <c r="FR10" t="n">
+      <c r="GF10" t="n">
         <v>0.02721088435374152</v>
       </c>
-      <c r="FS10" t="n">
-        <v>0</v>
-      </c>
-      <c r="FT10" t="n">
+      <c r="GG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GH10" t="n">
         <v>0.1211501310171017</v>
       </c>
-      <c r="FU10" t="n">
+      <c r="GI10" t="n">
         <v>0.08886589870613906</v>
       </c>
-      <c r="FV10" t="n">
+      <c r="GJ10" t="n">
         <v>8.886589870613907</v>
       </c>
-      <c r="FW10" t="n">
+      <c r="GK10" t="n">
         <v>0.08886589870613906</v>
       </c>
-      <c r="FX10" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY10" t="n">
+      <c r="GL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM10" t="n">
         <v>0.08886589870613906</v>
       </c>
-      <c r="FZ10" t="n">
+      <c r="GN10" t="n">
         <v>0.08886589870613906</v>
       </c>
-      <c r="GA10" t="inlineStr">
+      <c r="GO10" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB10" t="n">
+      <c r="GP10" t="n">
         <v>0.08886589870613906</v>
       </c>
-      <c r="GC10" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD10" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ10" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR10" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
     <row r="11">
@@ -6979,7 +7477,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -7156,10 +7654,10 @@
         <v>0.112</v>
       </c>
       <c r="BT11" t="n">
-        <v>792.03</v>
+        <v>792.04</v>
       </c>
       <c r="BU11" t="n">
-        <v>-24.24</v>
+        <v>-24.26</v>
       </c>
       <c r="BV11" t="n">
         <v>1.41</v>
@@ -7171,7 +7669,7 @@
         <v>2</v>
       </c>
       <c r="BY11" t="n">
-        <v>-92.13</v>
+        <v>-92.15000000000001</v>
       </c>
       <c r="BZ11" t="n">
         <v>8</v>
@@ -7248,10 +7746,10 @@
         <v>30.84886128364389</v>
       </c>
       <c r="CX11" t="n">
-        <v>82.40165631469979</v>
+        <v>82.50517598343686</v>
       </c>
       <c r="CY11" t="n">
-        <v>79.40000000000001</v>
+        <v>41</v>
       </c>
       <c r="CZ11" t="n">
         <v>16</v>
@@ -7311,206 +7809,252 @@
         <v>30.16</v>
       </c>
       <c r="DS11" t="n">
+        <v>2</v>
+      </c>
+      <c r="DT11" t="n">
+        <v>4</v>
+      </c>
+      <c r="DU11" t="n">
         <v>1</v>
       </c>
-      <c r="DT11" t="n">
+      <c r="DV11" t="n">
         <v>50</v>
       </c>
-      <c r="DU11" t="n">
+      <c r="DW11" t="n">
         <v>0.8096</v>
       </c>
-      <c r="DV11" t="n">
+      <c r="DX11" t="n">
         <v>82.40000000000001</v>
       </c>
-      <c r="DW11" t="n">
+      <c r="DY11" t="n">
         <v>34.5</v>
       </c>
-      <c r="DX11" t="n">
+      <c r="DZ11" t="n">
         <v>50.103</v>
       </c>
-      <c r="DY11" t="n">
+      <c r="EA11" t="n">
         <v>3</v>
       </c>
-      <c r="DZ11" t="n">
+      <c r="EB11" t="n">
         <v>6</v>
       </c>
-      <c r="EA11" t="n">
+      <c r="EC11" t="n">
         <v>60.77</v>
       </c>
-      <c r="EB11" t="n">
+      <c r="ED11" t="n">
         <v>77.15000000000001</v>
       </c>
-      <c r="EC11" t="n">
+      <c r="EE11" t="n">
         <v>0.8096</v>
       </c>
-      <c r="ED11" t="n">
+      <c r="EF11" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="EE11" t="n">
+      <c r="EG11" t="n">
         <v>0.1898</v>
       </c>
-      <c r="EF11" t="n">
+      <c r="EH11" t="n">
         <v>3.5011</v>
       </c>
-      <c r="EG11" t="n">
+      <c r="EI11" t="n">
         <v>0.0097</v>
       </c>
-      <c r="EH11" t="n">
+      <c r="EJ11" t="n">
         <v>0.389</v>
       </c>
-      <c r="EI11" t="n">
+      <c r="EK11" t="n">
         <v>46.2</v>
       </c>
-      <c r="EJ11" t="inlineStr">
+      <c r="EL11" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EK11" t="n">
+      <c r="EM11" t="n">
         <v>2</v>
       </c>
-      <c r="EL11" t="n">
+      <c r="EN11" t="n">
         <v>4</v>
       </c>
-      <c r="EM11" t="n">
+      <c r="EO11" t="n">
         <v>20.8</v>
       </c>
-      <c r="EN11" t="n">
+      <c r="EP11" t="n">
         <v>1.067</v>
       </c>
-      <c r="EO11" t="n">
+      <c r="EQ11" t="n">
         <v>0.0708</v>
       </c>
-      <c r="EP11" t="n">
+      <c r="ER11" t="n">
         <v>11.5942</v>
       </c>
-      <c r="EQ11" t="n">
+      <c r="ES11" t="n">
         <v>17.5799</v>
       </c>
-      <c r="ER11" t="n">
+      <c r="ET11" t="n">
         <v>32.143</v>
       </c>
-      <c r="ES11" t="n">
+      <c r="EU11" t="n">
         <v>5.106</v>
       </c>
-      <c r="ET11" t="n">
+      <c r="EV11" t="n">
         <v>1.9202</v>
       </c>
-      <c r="EU11" t="n">
+      <c r="EW11" t="n">
         <v>8.968999999999999</v>
       </c>
-      <c r="EV11" t="n">
+      <c r="EX11" t="n">
         <v>33.67</v>
       </c>
-      <c r="EW11" t="inlineStr">
+      <c r="EY11" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="EX11" t="n">
+      <c r="EZ11" t="n">
         <v>5</v>
       </c>
-      <c r="EY11" t="n">
+      <c r="FA11" t="n">
         <v>9</v>
       </c>
-      <c r="EZ11" t="n">
+      <c r="FB11" t="n">
         <v>40.85</v>
       </c>
-      <c r="FA11" t="n">
+      <c r="FC11" t="n">
         <v>99.98</v>
       </c>
-      <c r="FB11" t="n">
+      <c r="FD11" t="n">
         <v>52.28</v>
       </c>
-      <c r="FC11" t="n">
+      <c r="FE11" t="n">
         <v>44.66</v>
       </c>
-      <c r="FD11" t="n">
+      <c r="FF11" t="n">
         <v>33.895</v>
       </c>
-      <c r="FE11" t="n">
+      <c r="FG11" t="n">
         <v>7.7415</v>
       </c>
-      <c r="FF11" t="n">
+      <c r="FH11" t="n">
         <v>40.095</v>
       </c>
-      <c r="FG11" t="n">
+      <c r="FI11" t="n">
         <v>64.04000000000001</v>
       </c>
-      <c r="FH11" t="n">
+      <c r="FJ11" t="n">
         <v>49.69</v>
       </c>
-      <c r="FI11" t="inlineStr">
+      <c r="FK11" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="FJ11" t="n">
+      <c r="FL11" t="n">
+        <v>5</v>
+      </c>
+      <c r="FM11" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN11" t="n">
         <v>52.32</v>
       </c>
-      <c r="FK11" t="n">
+      <c r="FO11" t="n">
         <v>68.55</v>
       </c>
-      <c r="FL11" t="n">
+      <c r="FP11" t="n">
         <v>33.73</v>
       </c>
-      <c r="FM11" t="n">
+      <c r="FQ11" t="n">
         <v>58.3</v>
       </c>
-      <c r="FN11" t="n">
+      <c r="FR11" t="n">
         <v>53.86</v>
       </c>
-      <c r="FO11" t="n">
-        <v>0</v>
-      </c>
-      <c r="FP11" t="n">
+      <c r="FS11" t="n">
+        <v>91.7012</v>
+      </c>
+      <c r="FT11" t="n">
+        <v>5</v>
+      </c>
+      <c r="FU11" t="n">
+        <v>10</v>
+      </c>
+      <c r="FV11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="FW11" t="n">
+        <v>56.08</v>
+      </c>
+      <c r="FX11" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="FY11" t="b">
+        <v>1</v>
+      </c>
+      <c r="FZ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="GA11" t="b">
+        <v>1</v>
+      </c>
+      <c r="GB11" t="b">
+        <v>0</v>
+      </c>
+      <c r="GC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="GD11" t="n">
         <v>0.1312931885488648</v>
       </c>
-      <c r="FQ11" t="n">
+      <c r="GE11" t="n">
         <v>0.17519205546187</v>
       </c>
-      <c r="FR11" t="n">
-        <v>0</v>
-      </c>
-      <c r="FS11" t="n">
+      <c r="GF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="GG11" t="n">
         <v>0.1203007518796993</v>
       </c>
-      <c r="FT11" t="n">
+      <c r="GH11" t="n">
         <v>0.07769684007190987</v>
       </c>
-      <c r="FU11" t="n">
+      <c r="GI11" t="n">
         <v>0.08505262320195771</v>
       </c>
-      <c r="FV11" t="n">
+      <c r="GJ11" t="n">
         <v>8.50526232019577</v>
       </c>
-      <c r="FW11" t="n">
+      <c r="GK11" t="n">
         <v>0.08505262320195771</v>
       </c>
-      <c r="FX11" t="n">
-        <v>0</v>
-      </c>
-      <c r="FY11" t="n">
+      <c r="GL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="GM11" t="n">
         <v>0.08505262320195771</v>
       </c>
-      <c r="FZ11" t="n">
+      <c r="GN11" t="n">
         <v>0.08505262320195771</v>
       </c>
-      <c r="GA11" t="inlineStr">
+      <c r="GO11" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="GB11" t="n">
+      <c r="GP11" t="n">
         <v>0.08505262320195771</v>
       </c>
-      <c r="GC11" t="inlineStr">
-        <is>
-          <t>20260731_183252</t>
-        </is>
-      </c>
-      <c r="GD11" s="2" t="n">
-        <v>46234.77282865668</v>
+      <c r="GQ11" t="inlineStr">
+        <is>
+          <t>20260731_183848</t>
+        </is>
+      </c>
+      <c r="GR11" s="2" t="n">
+        <v>46234.7769546374</v>
       </c>
     </row>
   </sheetData>
@@ -7731,7 +8275,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -7838,7 +8382,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
@@ -7937,7 +8481,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
@@ -8036,7 +8580,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
@@ -8135,7 +8679,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>46234</v>
@@ -8242,7 +8786,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
@@ -8341,7 +8885,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
@@ -8440,7 +8984,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
@@ -8539,7 +9083,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -8638,7 +9182,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46234.77282407408</v>
+        <v>46234.77694444444</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>46234</v>
@@ -8810,7 +9354,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0134052185491485</v>
+        <v>0.01340521798895227</v>
       </c>
     </row>
     <row r="6">
@@ -8820,7 +9364,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.2128012473091021</v>
+        <v>0.2128012384162626</v>
       </c>
     </row>
     <row r="7">
@@ -8880,7 +9424,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.03005735472423519</v>
+        <v>0.03005735450929848</v>
       </c>
     </row>
     <row r="13">
@@ -8890,7 +9434,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.193080863460631</v>
+        <v>0.1930808634846145</v>
       </c>
     </row>
     <row r="14">
@@ -9189,7 +9733,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 18:32:52.439014+05:30</t>
+          <t>2026-07-31 18:38:48.932676+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-07-31 13:31 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1543.8</v>
+        <v>1543.78</v>
       </c>
       <c r="BU2" t="n">
         <v>-12.92</v>
@@ -2178,7 +2178,7 @@
         <v>89.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.79</v>
+        <v>42.74</v>
       </c>
       <c r="DS2" t="n">
         <v>3</v>
@@ -2311,10 +2311,10 @@
         <v>76.52800000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.39</v>
+        <v>41.365</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.92</v>
+        <v>73.93000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>74.66</v>
+        <v>74.73</v>
       </c>
       <c r="FO2" t="n">
         <v>72.64</v>
       </c>
       <c r="FP2" t="n">
-        <v>70.40000000000001</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>64.13</v>
+        <v>64.23999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.45999999999999</v>
+        <v>89.52</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.931</v>
+        <v>71.9555</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260731_185713</t>
+          <t>20260731_190130</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46234.78974197542</v>
+        <v>46234.79271174463</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.78973379629</v>
+        <v>46234.79270833333</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46234</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02070578543047197</v>
+        <v>0.02070578698678604</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3286941536957599</v>
+        <v>0.3286941784014799</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911166025863079</v>
+        <v>0.02911166344829994</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331351944721772</v>
+        <v>0.04331352199242269</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 18:57:13.740928+05:30</t>
+          <t>2026-07-31 19:01:30.323085+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-03 06:39 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.06</v>
+        <v>13.08</v>
       </c>
       <c r="R2" t="n">
-        <v>50.46</v>
+        <v>50.27</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1785</v>
+        <v>1821</v>
       </c>
       <c r="V2" t="n">
-        <v>1826.6</v>
+        <v>1838.3</v>
       </c>
       <c r="W2" t="n">
-        <v>1785</v>
+        <v>1789.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1816.2</v>
+        <v>1825</v>
       </c>
       <c r="Y2" t="n">
-        <v>1816.2</v>
+        <v>1825</v>
       </c>
       <c r="Z2" t="n">
-        <v>2502212</v>
+        <v>1081268</v>
       </c>
       <c r="AA2" t="n">
-        <v>2263459</v>
+        <v>2220806</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.11</v>
+        <v>0.49</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.96</v>
+        <v>0.48</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.21</v>
+        <v>0.26</v>
       </c>
       <c r="AE2" t="n">
-        <v>41.6</v>
+        <v>49.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.29</v>
+        <v>2.7</v>
       </c>
       <c r="AG2" t="n">
-        <v>44.91</v>
+        <v>45.22</v>
       </c>
       <c r="AH2" t="n">
-        <v>44.91</v>
+        <v>45.22</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.47</v>
+        <v>2.48</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,71 +1926,71 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>13.4</v>
+        <v>12.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>21.57</v>
+        <v>21.4</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.62</v>
+        <v>56.74</v>
       </c>
       <c r="AO2" t="n">
-        <v>81.83</v>
+        <v>82.27</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.72</v>
+        <v>17.07</v>
       </c>
       <c r="AQ2" t="n">
-        <v>56.17</v>
+        <v>55.13</v>
       </c>
       <c r="AR2" t="n">
-        <v>1816.2</v>
+        <v>1825</v>
       </c>
       <c r="AS2" t="n">
-        <v>1995.85</v>
+        <v>2005.88</v>
       </c>
       <c r="AT2" t="n">
-        <v>1726.37</v>
+        <v>1734.56</v>
       </c>
       <c r="AU2" t="n">
-        <v>1816.199951171875</v>
+        <v>1825</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.890000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="AY2" t="n">
-        <v>179.65</v>
+        <v>180.88</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="BA2" t="n">
-        <v>89.83</v>
+        <v>90.44</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>33.4</v>
+        <v>33.3</v>
       </c>
       <c r="BE2" t="n">
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.4</v>
+        <v>48.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="BN2" t="n">
-        <v>51</v>
+        <v>51.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.41</v>
+        <v>2.42</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.9</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.35</v>
@@ -2026,19 +2026,19 @@
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1543.78</v>
+        <v>1551.31</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.92</v>
+        <v>-13</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.2</v>
+        <v>48.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>56.5</v>
+        <v>57</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.90000000000001</v>
+        <v>73</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>99.31</v>
+        <v>89.83</v>
       </c>
       <c r="CO2" t="n">
-        <v>47.66</v>
+        <v>47.02</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.891500000000001</v>
+        <v>9.911199999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7064</v>
+        <v>0.6834</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3536</v>
+        <v>0.3421</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0989</v>
+        <v>0.09909999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2916</v>
+        <v>1.2962</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.004</v>
+        <v>3.996</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.946</v>
+        <v>4.9556</v>
       </c>
       <c r="DJ2" t="n">
-        <v>39.99</v>
+        <v>42.39</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.946</v>
+        <v>4.9556</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.004</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.004</v>
+        <v>3.996</v>
       </c>
       <c r="DO2" t="n">
         <v>1.9977</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8089</v>
+        <v>0.8056</v>
       </c>
       <c r="DQ2" t="n">
-        <v>89.83</v>
+        <v>90.44</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.74</v>
+        <v>41.55</v>
       </c>
       <c r="DS2" t="n">
         <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>7.5789</v>
+        <v>6.8831</v>
       </c>
       <c r="DX2" t="n">
-        <v>45.425</v>
+        <v>44.32500000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>55.5</v>
+        <v>24.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>98.038</v>
+        <v>93.014</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>26.69</v>
+        <v>7.34</v>
       </c>
       <c r="EE2" t="n">
-        <v>7.5789</v>
+        <v>6.8831</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.11</v>
+        <v>0.49</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.4448</v>
+        <v>2.2328</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0047</v>
+        <v>3.9965</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.3193</v>
+        <v>0.2921</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6731</v>
+        <v>0.6706</v>
       </c>
       <c r="EK2" t="n">
-        <v>76.08</v>
+        <v>66.3</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,75 +2246,75 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>80.38</v>
+        <v>30.14</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.4976</v>
+        <v>3.9423</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.145</v>
+        <v>0.0641</v>
       </c>
       <c r="ER2" t="n">
-        <v>8.9099</v>
+        <v>20.2245</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.5245</v>
+        <v>12.181</v>
       </c>
       <c r="ET2" t="n">
-        <v>63.953</v>
+        <v>48.652</v>
       </c>
       <c r="EU2" t="n">
-        <v>20.7792</v>
+        <v>8.3643</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.1706</v>
+        <v>1.6644</v>
       </c>
       <c r="EW2" t="n">
-        <v>79.8254</v>
+        <v>27.0748</v>
       </c>
       <c r="EX2" t="n">
-        <v>60.55</v>
+        <v>38.28</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.25</v>
+        <v>69.34</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.62</v>
+        <v>32.65</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.61</v>
+        <v>73.56999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>87.69499999999999</v>
+        <v>78.065</v>
       </c>
       <c r="FF2" t="n">
-        <v>54.105</v>
+        <v>42.65</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.6196</v>
+        <v>25.8132</v>
       </c>
       <c r="FH2" t="n">
-        <v>76.52800000000001</v>
+        <v>69.27500000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.365</v>
+        <v>41.97</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.93000000000001</v>
+        <v>72.79000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>74.73</v>
+        <v>72.41</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.64</v>
+        <v>73.05</v>
       </c>
       <c r="FP2" t="n">
-        <v>70.51000000000001</v>
+        <v>54.32</v>
       </c>
       <c r="FQ2" t="n">
-        <v>64.23999999999999</v>
+        <v>67.62</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.52</v>
+        <v>85.84</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.9555</v>
+        <v>70.069</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260731_193445</t>
+          <t>20260803_120930</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46234.81580332461</v>
+        <v>46237.50660158208</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.81579861111</v>
+        <v>46237.50659722222</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46248</v>
+        <v>46251.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.06</v>
+        <v>13.08</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,55 +2681,55 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1816.2</v>
+        <v>1825</v>
       </c>
       <c r="L2" t="n">
-        <v>1785</v>
+        <v>1821</v>
       </c>
       <c r="M2" t="n">
-        <v>1826.6</v>
+        <v>1838.3</v>
       </c>
       <c r="N2" t="n">
-        <v>1785</v>
+        <v>1789.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1816.2</v>
+        <v>1825</v>
       </c>
       <c r="P2" t="n">
-        <v>2502212</v>
+        <v>1081268</v>
       </c>
       <c r="Q2" t="n">
-        <v>1816.2</v>
+        <v>1825</v>
       </c>
       <c r="R2" t="n">
-        <v>1995.85</v>
+        <v>2005.88</v>
       </c>
       <c r="S2" t="n">
-        <v>1726.37</v>
+        <v>1734.56</v>
       </c>
       <c r="T2" t="n">
-        <v>9.891531769628887</v>
+        <v>9.911232876712335</v>
       </c>
       <c r="U2" t="n">
-        <v>179.6499999999999</v>
+        <v>180.8800000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.94604118489154</v>
+        <v>4.955616438356167</v>
       </c>
       <c r="W2" t="n">
-        <v>89.83000000000015</v>
+        <v>90.44000000000005</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999888678615157</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="Z2" t="n">
         <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="AB2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.891531769628887</v>
+        <v>9.911232876712335</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.94604118489154</v>
+        <v>4.955616438356167</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02070578685160832</v>
+        <v>0.02069027638228421</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3286941762556001</v>
+        <v>0.3284479551883032</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911166025863079</v>
+        <v>0.02909876709663517</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0433135169498943</v>
+        <v>0.04289544314416929</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.7</v>
+        <v>38.72</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31 19:34:45.441416+05:30</t>
+          <t>2026-08-03 12:09:30.414419+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.891531769628887, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999888678615157}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.911232876712335, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-03 13:19 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.08</v>
+        <v>12.93</v>
       </c>
       <c r="R2" t="n">
-        <v>50.27</v>
+        <v>50.31</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1789.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1825</v>
+        <v>1811.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>1825</v>
+        <v>1811.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>1081268</v>
+        <v>1918082</v>
       </c>
       <c r="AA2" t="n">
-        <v>2220806</v>
+        <v>2262646</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.49</v>
+        <v>0.85</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.48</v>
+        <v>-0.26</v>
       </c>
       <c r="AD2" t="n">
         <v>0.26</v>
@@ -1908,7 +1908,7 @@
         <v>49.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.7</v>
+        <v>2.72</v>
       </c>
       <c r="AG2" t="n">
         <v>45.22</v>
@@ -1917,7 +1917,7 @@
         <v>45.22</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.48</v>
+        <v>2.5</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>12.9</v>
+        <v>12.11</v>
       </c>
       <c r="AM2" t="n">
-        <v>21.4</v>
+        <v>20.52</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.74</v>
+        <v>55.58</v>
       </c>
       <c r="AO2" t="n">
-        <v>82.27</v>
+        <v>80.72</v>
       </c>
       <c r="AP2" t="n">
-        <v>17.07</v>
+        <v>16.2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>55.13</v>
+        <v>53.97</v>
       </c>
       <c r="AR2" t="n">
-        <v>1825</v>
+        <v>1811.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>2005.88</v>
+        <v>1992.28</v>
       </c>
       <c r="AT2" t="n">
-        <v>1734.56</v>
+        <v>1720.96</v>
       </c>
       <c r="AU2" t="n">
-        <v>1825</v>
+        <v>1811.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>14.5</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.91</v>
+        <v>9.99</v>
       </c>
       <c r="AY2" t="n">
         <v>180.88</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="BA2" t="n">
         <v>90.44</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,55 +1987,55 @@
         <v>48.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
         <v>642</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.1</v>
+        <v>50.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.42</v>
+        <v>2.4</v>
       </c>
       <c r="BP2" t="n">
         <v>8.890000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.35</v>
+        <v>-4.34</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.268</v>
+        <v>0.266</v>
       </c>
       <c r="BT2" t="n">
-        <v>1551.31</v>
+        <v>1538.97</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13</v>
+        <v>-13.14</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.4</v>
+        <v>48</v>
       </c>
       <c r="CE2" t="n">
-        <v>57</v>
+        <v>56.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>73</v>
+        <v>72.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>89.83</v>
+        <v>89.31</v>
       </c>
       <c r="CO2" t="n">
-        <v>47.02</v>
+        <v>43.69</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.911199999999999</v>
+        <v>9.9856</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6834</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3421</v>
+        <v>0.3441</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.0999</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2962</v>
+        <v>1.2917</v>
       </c>
       <c r="DH2" t="n">
         <v>3.996</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9556</v>
+        <v>4.9928</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.39</v>
+        <v>43.14</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9556</v>
+        <v>4.9928</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.996</v>
       </c>
       <c r="DN2" t="n">
         <v>3.996</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9977</v>
+        <v>2.0023</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8056</v>
+        <v>0.8008</v>
       </c>
       <c r="DQ2" t="n">
         <v>90.44</v>
       </c>
       <c r="DR2" t="n">
-        <v>41.55</v>
+        <v>63.36</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>6.8831</v>
+        <v>6.48</v>
       </c>
       <c r="DX2" t="n">
-        <v>44.32500000000002</v>
+        <v>48.2</v>
       </c>
       <c r="DY2" t="n">
-        <v>24.5</v>
+        <v>42.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>93.014</v>
+        <v>93.15000000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>7.34</v>
+        <v>26.13</v>
       </c>
       <c r="EE2" t="n">
-        <v>6.8831</v>
+        <v>6.48</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.49</v>
+        <v>0.85</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.2328</v>
+        <v>2.0947</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9965</v>
+        <v>3.9942</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2921</v>
+        <v>0.2708</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6706</v>
+        <v>0.6667999999999999</v>
       </c>
       <c r="EK2" t="n">
-        <v>66.3</v>
+        <v>68.89</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>30.14</v>
+        <v>31.5</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.9423</v>
+        <v>4.0729</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0641</v>
+        <v>0.1099</v>
       </c>
       <c r="ER2" t="n">
-        <v>20.2245</v>
+        <v>11.7529</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.181</v>
+        <v>12.3257</v>
       </c>
       <c r="ET2" t="n">
-        <v>48.652</v>
+        <v>47.524</v>
       </c>
       <c r="EU2" t="n">
-        <v>8.3643</v>
+        <v>13.77</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6644</v>
+        <v>1.3514</v>
       </c>
       <c r="EW2" t="n">
-        <v>27.0748</v>
+        <v>28.1326</v>
       </c>
       <c r="EX2" t="n">
-        <v>38.28</v>
+        <v>34.65</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.34</v>
+        <v>68.66</v>
       </c>
       <c r="FC2" t="n">
-        <v>32.65</v>
+        <v>33.39</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.56999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.065</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>42.65</v>
+        <v>39.17</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.8132</v>
+        <v>25.5171</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.27500000000001</v>
+        <v>68.053</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.97</v>
+        <v>53.25</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.79000000000001</v>
+        <v>73.3</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>72.41</v>
+        <v>77.45</v>
       </c>
       <c r="FO2" t="n">
-        <v>73.05</v>
+        <v>72.88</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.32</v>
+        <v>60.68</v>
       </c>
       <c r="FQ2" t="n">
-        <v>67.62</v>
+        <v>76.14</v>
       </c>
       <c r="FR2" t="n">
-        <v>85.84</v>
+        <v>88.45999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.069</v>
+        <v>74.86499999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260803_120930</t>
+          <t>20260803_184902</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46237.50660158208</v>
+        <v>46237.78405151079</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46237.50659722222</v>
+        <v>46237.78405092593</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46237</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.08</v>
+        <v>12.93</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1825</v>
+        <v>1811.4</v>
       </c>
       <c r="L2" t="n">
         <v>1821</v>
@@ -2693,34 +2693,34 @@
         <v>1789.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1825</v>
+        <v>1811.4</v>
       </c>
       <c r="P2" t="n">
-        <v>1081268</v>
+        <v>1918082</v>
       </c>
       <c r="Q2" t="n">
-        <v>1825</v>
+        <v>1811.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2005.88</v>
+        <v>1992.28</v>
       </c>
       <c r="S2" t="n">
-        <v>1734.56</v>
+        <v>1720.96</v>
       </c>
       <c r="T2" t="n">
-        <v>9.911232876712335</v>
+        <v>9.985646461300645</v>
       </c>
       <c r="U2" t="n">
-        <v>180.8800000000001</v>
+        <v>180.8799999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.955616438356167</v>
+        <v>4.992823230650329</v>
       </c>
       <c r="W2" t="n">
         <v>90.44000000000005</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>1.999999999999998</v>
       </c>
       <c r="Y2" t="n">
         <v>14.5</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.911232876712335</v>
+        <v>9.985646461300645</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.955616438356167</v>
+        <v>4.992823230650329</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02069027638228421</v>
+        <v>0.02069621048027015</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3284479551883032</v>
+        <v>0.3285421560734608</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909876709663517</v>
+        <v>0.02911166025863079</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289544314416929</v>
+        <v>0.04331352796684131</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-03 12:09:30.414419+05:30</t>
+          <t>2026-08-03 18:49:02.091345+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.911232876712335, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.985646461300645, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999976}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-04 06:06 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.93</v>
+        <v>13.08</v>
       </c>
       <c r="R2" t="n">
-        <v>50.31</v>
+        <v>50.22</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1821</v>
+        <v>1811</v>
       </c>
       <c r="V2" t="n">
-        <v>1838.3</v>
+        <v>1832.5</v>
       </c>
       <c r="W2" t="n">
-        <v>1789.1</v>
+        <v>1806.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1811.4</v>
+        <v>1826.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>1811.4</v>
+        <v>1826.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>1918082</v>
+        <v>660536</v>
       </c>
       <c r="AA2" t="n">
-        <v>2262646</v>
+        <v>2199769</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.26</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.26</v>
+        <v>-0.29</v>
       </c>
       <c r="AE2" t="n">
-        <v>49.2</v>
+        <v>26.4</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.72</v>
+        <v>1.45</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.22</v>
+        <v>43.59</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.22</v>
+        <v>43.59</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.5</v>
+        <v>2.39</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>12.11</v>
+        <v>12.99</v>
       </c>
       <c r="AM2" t="n">
-        <v>20.52</v>
+        <v>21.49</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.58</v>
+        <v>56.86</v>
       </c>
       <c r="AO2" t="n">
-        <v>80.72</v>
+        <v>82.34</v>
       </c>
       <c r="AP2" t="n">
-        <v>16.2</v>
+        <v>17.16</v>
       </c>
       <c r="AQ2" t="n">
-        <v>53.97</v>
+        <v>55.25</v>
       </c>
       <c r="AR2" t="n">
-        <v>1811.4</v>
+        <v>1826.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>1992.28</v>
+        <v>2000.76</v>
       </c>
       <c r="AT2" t="n">
-        <v>1720.96</v>
+        <v>1739.22</v>
       </c>
       <c r="AU2" t="n">
-        <v>1811.400024414062</v>
+        <v>1826.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>14.5</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.99</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>180.88</v>
+        <v>174.36</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.99</v>
+        <v>4.77</v>
       </c>
       <c r="BA2" t="n">
-        <v>90.44</v>
+        <v>87.18000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1987,52 +1987,52 @@
         <v>48.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
         <v>642</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.9</v>
+        <v>51.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.4</v>
+        <v>2.42</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.890000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.34</v>
+        <v>-4.35</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.266</v>
+        <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1538.97</v>
+        <v>1553.04</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.14</v>
+        <v>-12.93</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="BW2" t="n">
         <v>2.05</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48</v>
+        <v>48.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>56.5</v>
+        <v>57</v>
       </c>
       <c r="CF2" t="n">
         <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.7</v>
+        <v>73</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>89.31</v>
+        <v>85.79000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.69</v>
+        <v>25.46</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.9856</v>
+        <v>9.5466</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.6586</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3441</v>
+        <v>0.329</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0999</v>
+        <v>0.0955</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.002</v>
+        <v>2.0021</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2917</v>
+        <v>1.2491</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.996</v>
+        <v>3.9958</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9928</v>
+        <v>4.7733</v>
       </c>
       <c r="DJ2" t="n">
-        <v>43.14</v>
+        <v>35.87</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9928</v>
+        <v>4.7733</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.996</v>
+        <v>1.9958</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.996</v>
+        <v>3.9958</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0023</v>
+        <v>2.0018</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8008</v>
+        <v>0.8377</v>
       </c>
       <c r="DQ2" t="n">
-        <v>90.44</v>
+        <v>87.18000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>63.36</v>
+        <v>62.22</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>6.48</v>
+        <v>7.1799</v>
       </c>
       <c r="DX2" t="n">
-        <v>48.2</v>
+        <v>44.14999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>42.5</v>
+        <v>15</v>
       </c>
       <c r="DZ2" t="n">
-        <v>93.15000000000001</v>
+        <v>90.84399999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>26.13</v>
+        <v>20.5</v>
       </c>
       <c r="EE2" t="n">
-        <v>6.48</v>
+        <v>7.1799</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.0947</v>
+        <v>2.2445</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9942</v>
+        <v>3.9944</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2708</v>
+        <v>0.2936</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6667999999999999</v>
+        <v>0.6923</v>
       </c>
       <c r="EK2" t="n">
-        <v>68.89</v>
+        <v>67.67</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>31.5</v>
+        <v>8.44</v>
       </c>
       <c r="EP2" t="n">
-        <v>4.0729</v>
+        <v>1.104</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1099</v>
+        <v>0.0392</v>
       </c>
       <c r="ER2" t="n">
-        <v>11.7529</v>
+        <v>31.8333</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.3257</v>
+        <v>10.5811</v>
       </c>
       <c r="ET2" t="n">
-        <v>47.524</v>
+        <v>33.518</v>
       </c>
       <c r="EU2" t="n">
-        <v>13.77</v>
+        <v>5.148</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3514</v>
+        <v>1.8385</v>
       </c>
       <c r="EW2" t="n">
-        <v>28.1326</v>
+        <v>7.2407</v>
       </c>
       <c r="EX2" t="n">
-        <v>34.65</v>
+        <v>28.12</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="FB2" t="n">
-        <v>68.66</v>
+        <v>69.34</v>
       </c>
       <c r="FC2" t="n">
-        <v>33.39</v>
+        <v>26.37</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.09999999999999</v>
+        <v>73.94</v>
       </c>
       <c r="FE2" t="n">
-        <v>79.09999999999999</v>
+        <v>76.73</v>
       </c>
       <c r="FF2" t="n">
-        <v>39.17</v>
+        <v>26.79</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.5171</v>
+        <v>25.3068</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.053</v>
+        <v>66.03100000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>53.25</v>
+        <v>49.045</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.3</v>
+        <v>68.34</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>77.45</v>
+        <v>75.51000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.88</v>
+        <v>67.23</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.68</v>
+        <v>55.69</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.14</v>
+        <v>77.28</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.45999999999999</v>
+        <v>87.55</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.86499999999999</v>
+        <v>72.15649999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260803_184902</t>
+          <t>20260804_113641</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46237.78405151079</v>
+        <v>46238.48381008189</v>
       </c>
     </row>
   </sheetData>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46237.78405092593</v>
+        <v>46238.48380787037</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46251.5</v>
+        <v>46252.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.93</v>
+        <v>13.08</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1811.4</v>
+        <v>1826.4</v>
       </c>
       <c r="L2" t="n">
-        <v>1821</v>
+        <v>1811</v>
       </c>
       <c r="M2" t="n">
-        <v>1838.3</v>
+        <v>1832.5</v>
       </c>
       <c r="N2" t="n">
-        <v>1789.1</v>
+        <v>1806.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1811.4</v>
+        <v>1826.4</v>
       </c>
       <c r="P2" t="n">
-        <v>1918082</v>
+        <v>660536</v>
       </c>
       <c r="Q2" t="n">
-        <v>1811.4</v>
+        <v>1826.4</v>
       </c>
       <c r="R2" t="n">
-        <v>1992.28</v>
+        <v>2000.76</v>
       </c>
       <c r="S2" t="n">
-        <v>1720.96</v>
+        <v>1739.22</v>
       </c>
       <c r="T2" t="n">
-        <v>9.985646461300645</v>
+        <v>9.546649145860703</v>
       </c>
       <c r="U2" t="n">
-        <v>180.8799999999999</v>
+        <v>174.3599999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.992823230650329</v>
+        <v>4.773324572930358</v>
       </c>
       <c r="W2" t="n">
-        <v>90.44000000000005</v>
+        <v>87.18000000000006</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999998</v>
+        <v>1.999999999999997</v>
       </c>
       <c r="Y2" t="n">
         <v>14.5</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.985646461300645</v>
+        <v>9.546649145860703</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.992823230650329</v>
+        <v>4.773324572930358</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02069621048027015</v>
+        <v>0.02069554048260456</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3285421560734608</v>
+        <v>0.3285315201902479</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911166025863079</v>
+        <v>0.02911165706896164</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331352796684131</v>
+        <v>0.04331350863244116</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645465</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-03 18:49:02.091345+05:30</t>
+          <t>2026-08-04 11:36:41.229079+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.985646461300645, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999976}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.546649145860703, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999973}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-04 12:16 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.08</v>
+        <v>13.26</v>
       </c>
       <c r="R2" t="n">
-        <v>50.22</v>
+        <v>50.56</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1811</v>
       </c>
       <c r="V2" t="n">
-        <v>1832.5</v>
+        <v>1850</v>
       </c>
       <c r="W2" t="n">
         <v>1806.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1826.4</v>
+        <v>1850</v>
       </c>
       <c r="Y2" t="n">
-        <v>1826.4</v>
+        <v>1850</v>
       </c>
       <c r="Z2" t="n">
-        <v>660536</v>
+        <v>1404337</v>
       </c>
       <c r="AA2" t="n">
-        <v>2199769</v>
+        <v>2216454</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.3</v>
+        <v>0.63</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.5600000000000001</v>
+        <v>2.13</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.29</v>
+        <v>-0.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>26.4</v>
+        <v>43.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.45</v>
+        <v>2.37</v>
       </c>
       <c r="AG2" t="n">
-        <v>43.59</v>
+        <v>45.12</v>
       </c>
       <c r="AH2" t="n">
-        <v>43.59</v>
+        <v>45.12</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.39</v>
+        <v>2.44</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>12.99</v>
+        <v>13.19</v>
       </c>
       <c r="AM2" t="n">
-        <v>21.49</v>
+        <v>22.31</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.86</v>
+        <v>58.23</v>
       </c>
       <c r="AO2" t="n">
-        <v>82.34</v>
+        <v>82.73999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>17.16</v>
+        <v>16.12</v>
       </c>
       <c r="AQ2" t="n">
-        <v>55.25</v>
+        <v>53.49</v>
       </c>
       <c r="AR2" t="n">
-        <v>1826.4</v>
+        <v>1850</v>
       </c>
       <c r="AS2" t="n">
-        <v>2000.76</v>
+        <v>2030.5</v>
       </c>
       <c r="AT2" t="n">
-        <v>1739.22</v>
+        <v>1759.75</v>
       </c>
       <c r="AU2" t="n">
-        <v>1826.400024414062</v>
+        <v>1850</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.550000000000001</v>
+        <v>9.76</v>
       </c>
       <c r="AY2" t="n">
-        <v>174.36</v>
+        <v>180.5</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.77</v>
+        <v>4.88</v>
       </c>
       <c r="BA2" t="n">
-        <v>87.18000000000001</v>
+        <v>90.25</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,13 +1984,13 @@
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.3</v>
+        <v>48.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.1</v>
+        <v>51.2</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.42</v>
+        <v>2.45</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.9</v>
+        <v>8.94</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.35</v>
@@ -2023,19 +2023,19 @@
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.268</v>
+        <v>0.271</v>
       </c>
       <c r="BT2" t="n">
-        <v>1553.04</v>
+        <v>1575.3</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.93</v>
+        <v>-12.71</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.4</v>
+        <v>49</v>
       </c>
       <c r="CE2" t="n">
-        <v>57</v>
+        <v>57.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>73</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>85.79000000000001</v>
+        <v>87.89</v>
       </c>
       <c r="CO2" t="n">
-        <v>25.46</v>
+        <v>30.32</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.5466</v>
+        <v>9.7568</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6586</v>
+        <v>0.6506999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.329</v>
+        <v>0.3253</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0955</v>
+        <v>0.09760000000000001</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2491</v>
+        <v>1.2942</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9958</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7733</v>
+        <v>4.8784</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.87</v>
+        <v>39.14</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7733</v>
+        <v>4.8784</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9958</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9958</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0018</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8377</v>
+        <v>0.8197</v>
       </c>
       <c r="DQ2" t="n">
-        <v>87.18000000000001</v>
+        <v>90.25</v>
       </c>
       <c r="DR2" t="n">
-        <v>62.22</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>7.1799</v>
+        <v>6.6066</v>
       </c>
       <c r="DX2" t="n">
-        <v>44.14999999999999</v>
+        <v>43.15000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>15</v>
+        <v>31.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.84399999999999</v>
+        <v>91.283</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>20.5</v>
+        <v>20.92</v>
       </c>
       <c r="EE2" t="n">
-        <v>7.1799</v>
+        <v>6.6066</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.3</v>
+        <v>0.63</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.2445</v>
+        <v>2.1375</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9944</v>
+        <v>3.9987</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2936</v>
+        <v>0.2834</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6923</v>
+        <v>0.6801</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.67</v>
+        <v>67.5</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>8.44</v>
+        <v>12.83</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.104</v>
+        <v>1.7013</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0392</v>
+        <v>0.0835</v>
       </c>
       <c r="ER2" t="n">
-        <v>31.8333</v>
+        <v>15.4921</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5811</v>
+        <v>11.3779</v>
       </c>
       <c r="ET2" t="n">
-        <v>33.518</v>
+        <v>37.025</v>
       </c>
       <c r="EU2" t="n">
-        <v>5.148</v>
+        <v>10.1556</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8385</v>
+        <v>1.4969</v>
       </c>
       <c r="EW2" t="n">
-        <v>7.2407</v>
+        <v>11.2763</v>
       </c>
       <c r="EX2" t="n">
-        <v>28.12</v>
+        <v>37.29</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.34</v>
+        <v>70.16</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.37</v>
+        <v>29.29</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.94</v>
+        <v>74.38</v>
       </c>
       <c r="FE2" t="n">
-        <v>76.73</v>
+        <v>77.69499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>26.79</v>
+        <v>33.805</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.3068</v>
+        <v>25.5494</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.03100000000001</v>
+        <v>68.905</v>
       </c>
       <c r="FI2" t="n">
-        <v>49.045</v>
+        <v>53.52</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.34</v>
+        <v>69.11</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>75.51000000000001</v>
+        <v>75.19</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.23</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>55.69</v>
+        <v>61.03</v>
       </c>
       <c r="FQ2" t="n">
-        <v>77.28</v>
+        <v>75.62</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.55</v>
+        <v>87.48999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.15649999999999</v>
+        <v>73.623</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260804_113641</t>
+          <t>20260804_174645</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46238.48381008189</v>
+        <v>46238.74080298615</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46238.48380787037</v>
+        <v>46238.74079861111</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46238</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46252.5</v>
+        <v>46253</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.08</v>
+        <v>13.26</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,55 +2681,55 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1826.4</v>
+        <v>1850</v>
       </c>
       <c r="L2" t="n">
         <v>1811</v>
       </c>
       <c r="M2" t="n">
-        <v>1832.5</v>
+        <v>1850</v>
       </c>
       <c r="N2" t="n">
         <v>1806.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1826.4</v>
+        <v>1850</v>
       </c>
       <c r="P2" t="n">
-        <v>660536</v>
+        <v>1404337</v>
       </c>
       <c r="Q2" t="n">
-        <v>1826.4</v>
+        <v>1850</v>
       </c>
       <c r="R2" t="n">
-        <v>2000.76</v>
+        <v>2030.5</v>
       </c>
       <c r="S2" t="n">
-        <v>1739.22</v>
+        <v>1759.75</v>
       </c>
       <c r="T2" t="n">
-        <v>9.546649145860703</v>
+        <v>9.756756756756758</v>
       </c>
       <c r="U2" t="n">
-        <v>174.3599999999999</v>
+        <v>180.5</v>
       </c>
       <c r="V2" t="n">
-        <v>4.773324572930358</v>
+        <v>4.878378378378379</v>
       </c>
       <c r="W2" t="n">
-        <v>87.18000000000006</v>
+        <v>90.25</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999997</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="Z2" t="n">
         <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.546649145860703</v>
+        <v>9.756756756756758</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.773324572930358</v>
+        <v>4.878378378378379</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02069554048260456</v>
+        <v>0.02069334839980541</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3285315201902479</v>
+        <v>0.328496721954609</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911165706896164</v>
+        <v>0.02909876709663517</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04331350863244116</v>
+        <v>0.04289543414149807</v>
       </c>
     </row>
     <row r="13">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-04 11:36:41.229079+05:30</t>
+          <t>2026-08-04 17:46:45.416248+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.546649145860703, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999973}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.756756756756758, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-05 06:03 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.26</v>
+        <v>13.13</v>
       </c>
       <c r="R2" t="n">
-        <v>50.56</v>
+        <v>50.42</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1811</v>
+        <v>1854</v>
       </c>
       <c r="V2" t="n">
-        <v>1850</v>
+        <v>1856.6</v>
       </c>
       <c r="W2" t="n">
-        <v>1806.1</v>
+        <v>1834.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1850</v>
+        <v>1840.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>1850</v>
+        <v>1840.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>1404337</v>
+        <v>1203955</v>
       </c>
       <c r="AA2" t="n">
-        <v>2216454</v>
+        <v>2180769</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.63</v>
+        <v>0.55</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.13</v>
+        <v>-0.51</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.02</v>
+        <v>0.22</v>
       </c>
       <c r="AE2" t="n">
-        <v>43.9</v>
+        <v>22.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.37</v>
+        <v>1.2</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.12</v>
+        <v>43.48</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.12</v>
+        <v>43.48</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.44</v>
+        <v>2.36</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,65 +1926,65 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>13.19</v>
+        <v>11.35</v>
       </c>
       <c r="AM2" t="n">
-        <v>22.31</v>
+        <v>20.95</v>
       </c>
       <c r="AN2" t="n">
-        <v>58.23</v>
+        <v>56.78</v>
       </c>
       <c r="AO2" t="n">
-        <v>82.73999999999999</v>
+        <v>80.53</v>
       </c>
       <c r="AP2" t="n">
-        <v>16.12</v>
+        <v>16.66</v>
       </c>
       <c r="AQ2" t="n">
-        <v>53.49</v>
+        <v>49.85</v>
       </c>
       <c r="AR2" t="n">
-        <v>1850</v>
+        <v>1840.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2030.5</v>
+        <v>2014.52</v>
       </c>
       <c r="AT2" t="n">
-        <v>1759.75</v>
+        <v>1753.64</v>
       </c>
       <c r="AU2" t="n">
-        <v>1850</v>
+        <v>1840.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.76</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>180.5</v>
+        <v>173.92</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.88</v>
+        <v>4.72</v>
       </c>
       <c r="BA2" t="n">
-        <v>90.25</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>33.3</v>
+        <v>33.2</v>
       </c>
       <c r="BE2" t="n">
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.2</v>
+        <v>48.1</v>
       </c>
       <c r="BG2" t="n">
         <v>119</v>
@@ -1993,49 +1993,49 @@
         <v>18.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.45</v>
+        <v>2.43</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.94</v>
+        <v>8.91</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.35</v>
+        <v>-4.34</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.271</v>
+        <v>0.269</v>
       </c>
       <c r="BT2" t="n">
-        <v>1575.3</v>
+        <v>1565.57</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.71</v>
+        <v>-13.01</v>
       </c>
       <c r="BV2" t="n">
         <v>2.15</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>49</v>
+        <v>48.6</v>
       </c>
       <c r="CE2" t="n">
         <v>57.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>73.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.89</v>
+        <v>81.62</v>
       </c>
       <c r="CO2" t="n">
-        <v>30.32</v>
+        <v>42.19</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.7568</v>
+        <v>9.4491</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6506999999999999</v>
+        <v>0.63</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3253</v>
+        <v>0.3147</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09760000000000001</v>
+        <v>0.0945</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0021</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2942</v>
+        <v>1.2408</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0042</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8784</v>
+        <v>4.7245</v>
       </c>
       <c r="DJ2" t="n">
-        <v>39.14</v>
+        <v>36.85</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8784</v>
+        <v>4.7245</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2166,19 +2166,19 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0042</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2.0019</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8197</v>
+        <v>0.8484</v>
       </c>
       <c r="DQ2" t="n">
-        <v>90.25</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>67.90000000000001</v>
+        <v>61.96</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>6.6066</v>
+        <v>7.0593</v>
       </c>
       <c r="DX2" t="n">
-        <v>43.15000000000001</v>
+        <v>48.675</v>
       </c>
       <c r="DY2" t="n">
-        <v>31.5</v>
+        <v>27.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>91.283</v>
+        <v>90.584</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>20.92</v>
+        <v>24.06</v>
       </c>
       <c r="EE2" t="n">
-        <v>6.6066</v>
+        <v>7.0593</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.63</v>
+        <v>0.55</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.1375</v>
+        <v>2.1875</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9987</v>
+        <v>4.0039</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2834</v>
+        <v>0.2872</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6801</v>
+        <v>0.7</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.5</v>
+        <v>64.51000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2249,72 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>12.83</v>
+        <v>5.84</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.7013</v>
+        <v>0.7668</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0835</v>
+        <v>0.0722</v>
       </c>
       <c r="ER2" t="n">
-        <v>15.4921</v>
+        <v>17.1818</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.3779</v>
+        <v>10.9673</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.025</v>
+        <v>39.499</v>
       </c>
       <c r="EU2" t="n">
-        <v>10.1556</v>
+        <v>9.163</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4969</v>
+        <v>1.5226</v>
       </c>
       <c r="EW2" t="n">
-        <v>11.2763</v>
+        <v>4.7666</v>
       </c>
       <c r="EX2" t="n">
-        <v>37.29</v>
+        <v>61.26</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>70.16</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.29</v>
+        <v>26.91</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.38</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>77.69499999999999</v>
+        <v>73.065</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.805</v>
+        <v>51.725</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.5494</v>
+        <v>24.2917</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.905</v>
+        <v>71.523</v>
       </c>
       <c r="FI2" t="n">
-        <v>53.52</v>
+        <v>49.405</v>
       </c>
       <c r="FJ2" t="n">
-        <v>69.11</v>
+        <v>74.66</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>75.19</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.26000000000001</v>
+        <v>69.77</v>
       </c>
       <c r="FP2" t="n">
-        <v>61.03</v>
+        <v>85.94</v>
       </c>
       <c r="FQ2" t="n">
-        <v>75.62</v>
+        <v>75.81999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.48999999999999</v>
+        <v>94.88</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>73.623</v>
+        <v>77.1935</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260804_174645</t>
+          <t>20260805_113323</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46238.74080298615</v>
+        <v>46239.48151830545</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46238.74079861111</v>
+        <v>46239.4815162037</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.26</v>
+        <v>13.13</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1850</v>
+        <v>1840.6</v>
       </c>
       <c r="L2" t="n">
-        <v>1811</v>
+        <v>1854</v>
       </c>
       <c r="M2" t="n">
-        <v>1850</v>
+        <v>1856.6</v>
       </c>
       <c r="N2" t="n">
-        <v>1806.1</v>
+        <v>1834.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1850</v>
+        <v>1840.6</v>
       </c>
       <c r="P2" t="n">
-        <v>1404337</v>
+        <v>1203955</v>
       </c>
       <c r="Q2" t="n">
-        <v>1850</v>
+        <v>1840.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2030.5</v>
+        <v>2014.52</v>
       </c>
       <c r="S2" t="n">
-        <v>1759.75</v>
+        <v>1753.64</v>
       </c>
       <c r="T2" t="n">
-        <v>9.756756756756758</v>
+        <v>9.449092687167232</v>
       </c>
       <c r="U2" t="n">
-        <v>180.5</v>
+        <v>173.9200000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.878378378378379</v>
+        <v>4.724546343583604</v>
       </c>
       <c r="W2" t="n">
-        <v>90.25</v>
+        <v>86.95999999999981</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000000000000005</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.756756756756758</v>
+        <v>9.449092687167232</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.878378378378379</v>
+        <v>4.724546343583604</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02069334839980541</v>
+        <v>0.02067760840800907</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.328496721954609</v>
+        <v>0.3282468573310212</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909876709663517</v>
+        <v>0.02909870789015188</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543414149807</v>
+        <v>0.04289544896845562</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645465</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.72</v>
+        <v>38.74</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-04 17:46:45.416248+05:30</t>
+          <t>2026-08-05 11:33:23.217022+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.756756756756758, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.449092687167232, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000053}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-05 12:13 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.13</v>
+        <v>13.09</v>
       </c>
       <c r="R2" t="n">
-        <v>50.42</v>
+        <v>50.49</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1834.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1840.6</v>
+        <v>1835</v>
       </c>
       <c r="Y2" t="n">
-        <v>1840.6</v>
+        <v>1835</v>
       </c>
       <c r="Z2" t="n">
-        <v>1203955</v>
+        <v>2090240</v>
       </c>
       <c r="AA2" t="n">
-        <v>2180769</v>
+        <v>2225083</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.55</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.51</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="AD2" t="n">
         <v>0.22</v>
@@ -1917,7 +1917,7 @@
         <v>43.48</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>11.35</v>
+        <v>11.03</v>
       </c>
       <c r="AM2" t="n">
-        <v>20.95</v>
+        <v>20.59</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.78</v>
+        <v>56.3</v>
       </c>
       <c r="AO2" t="n">
-        <v>80.53</v>
+        <v>79.27</v>
       </c>
       <c r="AP2" t="n">
-        <v>16.66</v>
+        <v>16.3</v>
       </c>
       <c r="AQ2" t="n">
-        <v>49.85</v>
+        <v>49.39</v>
       </c>
       <c r="AR2" t="n">
-        <v>1840.6</v>
+        <v>1835</v>
       </c>
       <c r="AS2" t="n">
-        <v>2014.52</v>
+        <v>2008.92</v>
       </c>
       <c r="AT2" t="n">
-        <v>1753.64</v>
+        <v>1748.04</v>
       </c>
       <c r="AU2" t="n">
-        <v>1840.599975585938</v>
+        <v>1835</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.449999999999999</v>
+        <v>9.48</v>
       </c>
       <c r="AY2" t="n">
         <v>173.92</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.72</v>
+        <v>4.74</v>
       </c>
       <c r="BA2" t="n">
         <v>86.95999999999999</v>
@@ -2011,10 +2011,10 @@
         <v>51.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.43</v>
+        <v>2.42</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.91</v>
+        <v>8.9</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.34</v>
@@ -2023,16 +2023,16 @@
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.269</v>
+        <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1565.57</v>
+        <v>1559.96</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.01</v>
+        <v>-13.07</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
       <c r="BW2" t="n">
         <v>2.05</v>
@@ -2058,10 +2058,10 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.6</v>
+        <v>48.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>57.5</v>
+        <v>57</v>
       </c>
       <c r="CF2" t="n">
         <v>68.3</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>81.62</v>
+        <v>82.17</v>
       </c>
       <c r="CO2" t="n">
-        <v>42.19</v>
+        <v>40.52</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.4491</v>
+        <v>9.4779</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.63</v>
+        <v>0.632</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3147</v>
+        <v>0.316</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0945</v>
+        <v>0.0948</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2408</v>
+        <v>1.2409</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0042</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7245</v>
+        <v>4.739</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.85</v>
+        <v>36.33</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7245</v>
+        <v>4.739</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2166,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0042</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0019</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8484</v>
+        <v>0.8439</v>
       </c>
       <c r="DQ2" t="n">
         <v>86.95999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.96</v>
+        <v>65.98</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>7.0593</v>
+        <v>6.8776</v>
       </c>
       <c r="DX2" t="n">
-        <v>48.675</v>
+        <v>51.82500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>27.5</v>
+        <v>47</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.584</v>
+        <v>90.803</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>24.06</v>
+        <v>31.87</v>
       </c>
       <c r="EE2" t="n">
-        <v>7.0593</v>
+        <v>6.8776</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.55</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.1875</v>
+        <v>2.1337</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0039</v>
+        <v>3.9991</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2872</v>
+        <v>0.2793</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7</v>
+        <v>0.6967</v>
       </c>
       <c r="EK2" t="n">
-        <v>64.51000000000001</v>
+        <v>63.36</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>5.84</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.7668</v>
+        <v>1.0511</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0722</v>
+        <v>0.123</v>
       </c>
       <c r="ER2" t="n">
-        <v>17.1818</v>
+        <v>10.0851</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.9673</v>
+        <v>10.7804</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.499</v>
+        <v>39.434</v>
       </c>
       <c r="EU2" t="n">
-        <v>9.163</v>
+        <v>15.322</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5226</v>
+        <v>1.2216</v>
       </c>
       <c r="EW2" t="n">
-        <v>4.7666</v>
+        <v>6.5983</v>
       </c>
       <c r="EX2" t="n">
-        <v>61.26</v>
+        <v>60.59</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.56999999999999</v>
+        <v>69.39</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.91</v>
+        <v>27.03</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.09999999999999</v>
+        <v>73.86</v>
       </c>
       <c r="FE2" t="n">
-        <v>73.065</v>
+        <v>72.765</v>
       </c>
       <c r="FF2" t="n">
-        <v>51.725</v>
+        <v>50.555</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.2917</v>
+        <v>24.3828</v>
       </c>
       <c r="FH2" t="n">
-        <v>71.523</v>
+        <v>71.464</v>
       </c>
       <c r="FI2" t="n">
-        <v>49.405</v>
+        <v>51.155</v>
       </c>
       <c r="FJ2" t="n">
-        <v>74.66</v>
+        <v>73.97</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>82.34999999999999</v>
+        <v>82.34</v>
       </c>
       <c r="FO2" t="n">
-        <v>69.77</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>85.94</v>
+        <v>86.81999999999999</v>
       </c>
       <c r="FQ2" t="n">
-        <v>75.81999999999999</v>
+        <v>77.41</v>
       </c>
       <c r="FR2" t="n">
-        <v>94.88</v>
+        <v>95.88</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>77.1935</v>
+        <v>78.0805</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260805_113323</t>
+          <t>20260805_174344</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46239.48151830545</v>
+        <v>46239.73871286353</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46239.4815162037</v>
+        <v>46239.7387037037</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46239</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.13</v>
+        <v>13.09</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1840.6</v>
+        <v>1835</v>
       </c>
       <c r="L2" t="n">
         <v>1854</v>
@@ -2693,34 +2693,34 @@
         <v>1834.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1840.6</v>
+        <v>1835</v>
       </c>
       <c r="P2" t="n">
-        <v>1203955</v>
+        <v>2090240</v>
       </c>
       <c r="Q2" t="n">
-        <v>1840.6</v>
+        <v>1835</v>
       </c>
       <c r="R2" t="n">
-        <v>2014.52</v>
+        <v>2008.92</v>
       </c>
       <c r="S2" t="n">
-        <v>1753.64</v>
+        <v>1748.04</v>
       </c>
       <c r="T2" t="n">
-        <v>9.449092687167232</v>
+        <v>9.477929155313355</v>
       </c>
       <c r="U2" t="n">
         <v>173.9200000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.724546343583604</v>
+        <v>4.738964577656677</v>
       </c>
       <c r="W2" t="n">
-        <v>86.95999999999981</v>
+        <v>86.96000000000004</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000005</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.449092687167232</v>
+        <v>9.477929155313355</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.724546343583604</v>
+        <v>4.738964577656677</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02067760840800907</v>
+        <v>0.0206767969681825</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3282468573310212</v>
+        <v>0.3282339761231112</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909870789015188</v>
+        <v>0.02909864868366858</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289544896845562</v>
+        <v>0.04289544137935808</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347617</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-05 11:33:23.217022+05:30</t>
+          <t>2026-08-05 17:43:44.828156+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.449092687167232, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000053}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.477929155313355, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-06 06:07 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.09</v>
+        <v>13.06</v>
       </c>
       <c r="R2" t="n">
-        <v>50.49</v>
+        <v>50.45</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1854</v>
+        <v>1843</v>
       </c>
       <c r="V2" t="n">
-        <v>1856.6</v>
+        <v>1854.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1834.5</v>
+        <v>1837</v>
       </c>
       <c r="X2" t="n">
-        <v>1835</v>
+        <v>1843.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>1835</v>
+        <v>1843.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>2090240</v>
+        <v>1222690</v>
       </c>
       <c r="AA2" t="n">
-        <v>2225083</v>
+        <v>2184504</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.8100000000000001</v>
+        <v>0.47</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="AE2" t="n">
-        <v>22.1</v>
+        <v>17.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.2</v>
+        <v>0.97</v>
       </c>
       <c r="AG2" t="n">
-        <v>43.48</v>
+        <v>41.8</v>
       </c>
       <c r="AH2" t="n">
-        <v>43.48</v>
+        <v>41.8</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.37</v>
+        <v>2.27</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>11.03</v>
+        <v>10.43</v>
       </c>
       <c r="AM2" t="n">
-        <v>20.59</v>
+        <v>20.43</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.3</v>
+        <v>56.41</v>
       </c>
       <c r="AO2" t="n">
-        <v>79.27</v>
+        <v>79.79000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>16.3</v>
+        <v>17.55</v>
       </c>
       <c r="AQ2" t="n">
-        <v>49.39</v>
+        <v>45.53</v>
       </c>
       <c r="AR2" t="n">
-        <v>1835</v>
+        <v>1843.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2008.92</v>
+        <v>2010.78</v>
       </c>
       <c r="AT2" t="n">
-        <v>1748.04</v>
+        <v>1760.01</v>
       </c>
       <c r="AU2" t="n">
-        <v>1835</v>
+        <v>1843.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.48</v>
+        <v>9.07</v>
       </c>
       <c r="AY2" t="n">
-        <v>173.92</v>
+        <v>167.18</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.74</v>
+        <v>4.53</v>
       </c>
       <c r="BA2" t="n">
-        <v>86.95999999999999</v>
+        <v>83.59</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,10 +1987,10 @@
         <v>48.1</v>
       </c>
       <c r="BG2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="BI2" t="n">
         <v>1</v>
@@ -2005,37 +2005,37 @@
         <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.42</v>
+        <v>2.43</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.9</v>
+        <v>8.92</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.34</v>
+        <v>-4.33</v>
       </c>
       <c r="BR2" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="BS2" t="n">
         <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1559.96</v>
+        <v>1568.34</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.07</v>
+        <v>-12.91</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.4</v>
+        <v>48.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>57</v>
+        <v>57.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>73</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.17</v>
+        <v>83.38</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.52</v>
+        <v>50</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.4779</v>
+        <v>9.068099999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.632</v>
+        <v>0.6047</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.316</v>
+        <v>0.302</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0948</v>
+        <v>0.0907</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0022</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2409</v>
+        <v>1.1845</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9956</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.739</v>
+        <v>4.5341</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.33</v>
+        <v>34.78</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.739</v>
+        <v>4.5341</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9956</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9956</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>2.0023</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8439</v>
+        <v>0.882</v>
       </c>
       <c r="DQ2" t="n">
-        <v>86.95999999999999</v>
+        <v>83.59</v>
       </c>
       <c r="DR2" t="n">
-        <v>65.98</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>6.8776</v>
+        <v>7.7313</v>
       </c>
       <c r="DX2" t="n">
-        <v>51.82500000000001</v>
+        <v>50.52499999999998</v>
       </c>
       <c r="DY2" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.803</v>
+        <v>91.499</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>31.87</v>
+        <v>31.54</v>
       </c>
       <c r="EE2" t="n">
-        <v>6.8776</v>
+        <v>7.7313</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.1337</v>
+        <v>2.292</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9991</v>
+        <v>3.9948</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2793</v>
+        <v>0.2993</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6967</v>
+        <v>0.7224</v>
       </c>
       <c r="EK2" t="n">
-        <v>63.36</v>
+        <v>62.34</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,41 +2246,41 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>8.029999999999999</v>
+        <v>14.99</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.0511</v>
+        <v>1.9577</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.123</v>
+        <v>0.0731</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.0851</v>
+        <v>16.1964</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.7804</v>
+        <v>10.6361</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.434</v>
+        <v>45.272</v>
       </c>
       <c r="EU2" t="n">
-        <v>15.322</v>
+        <v>9.827999999999999</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2216</v>
+        <v>1.4551</v>
       </c>
       <c r="EW2" t="n">
-        <v>6.5983</v>
+        <v>12.4987</v>
       </c>
       <c r="EX2" t="n">
-        <v>60.59</v>
+        <v>46.67</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.39</v>
+        <v>69.25</v>
       </c>
       <c r="FC2" t="n">
-        <v>27.03</v>
+        <v>24.38</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.86</v>
+        <v>74.72</v>
       </c>
       <c r="FE2" t="n">
-        <v>72.765</v>
+        <v>72.86</v>
       </c>
       <c r="FF2" t="n">
-        <v>50.555</v>
+        <v>48.335</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.3828</v>
+        <v>25.4985</v>
       </c>
       <c r="FH2" t="n">
-        <v>71.464</v>
+        <v>68.973</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.155</v>
+        <v>51.145</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.97</v>
+        <v>71.20999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>82.34</v>
+        <v>79</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.04000000000001</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>86.81999999999999</v>
+        <v>73.33</v>
       </c>
       <c r="FQ2" t="n">
-        <v>77.41</v>
+        <v>78.06</v>
       </c>
       <c r="FR2" t="n">
-        <v>95.88</v>
+        <v>92.81</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>78.0805</v>
+        <v>75.9905</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260805_174344</t>
+          <t>20260806_113714</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46239.73871286353</v>
+        <v>46240.48419326112</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46239.7387037037</v>
+        <v>46240.48418981482</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.09</v>
+        <v>13.06</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1835</v>
+        <v>1843.6</v>
       </c>
       <c r="L2" t="n">
-        <v>1854</v>
+        <v>1843</v>
       </c>
       <c r="M2" t="n">
-        <v>1856.6</v>
+        <v>1854.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1834.5</v>
+        <v>1837</v>
       </c>
       <c r="O2" t="n">
-        <v>1835</v>
+        <v>1843.6</v>
       </c>
       <c r="P2" t="n">
-        <v>2090240</v>
+        <v>1222690</v>
       </c>
       <c r="Q2" t="n">
-        <v>1835</v>
+        <v>1843.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2008.92</v>
+        <v>2010.78</v>
       </c>
       <c r="S2" t="n">
-        <v>1748.04</v>
+        <v>1760.01</v>
       </c>
       <c r="T2" t="n">
-        <v>9.477929155313355</v>
+        <v>9.068127576480803</v>
       </c>
       <c r="U2" t="n">
-        <v>173.9200000000001</v>
+        <v>167.1800000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.738964577656677</v>
+        <v>4.534063788240395</v>
       </c>
       <c r="W2" t="n">
-        <v>86.96000000000004</v>
+        <v>83.58999999999992</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000000000000003</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.477929155313355</v>
+        <v>9.068127576480803</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.738964577656677</v>
+        <v>4.534063788240395</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0206767969681825</v>
+        <v>0.02067274353944541</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3282339761231112</v>
+        <v>0.3281696299367384</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289544137935808</v>
+        <v>0.04289545712491855</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347617</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.74</v>
+        <v>38.75</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-05 17:43:44.828156+05:30</t>
+          <t>2026-08-06 11:37:14.332490+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.477929155313355, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.068127576480803, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-06 12:16 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.06</v>
+        <v>12.96</v>
       </c>
       <c r="R2" t="n">
-        <v>50.45</v>
+        <v>50.44</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>1854.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1837</v>
+        <v>1830</v>
       </c>
       <c r="X2" t="n">
-        <v>1843.6</v>
+        <v>1830</v>
       </c>
       <c r="Y2" t="n">
-        <v>1843.6</v>
+        <v>1830</v>
       </c>
       <c r="Z2" t="n">
-        <v>1222690</v>
+        <v>2037365</v>
       </c>
       <c r="AA2" t="n">
-        <v>2184504</v>
+        <v>2225238</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.92</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.47</v>
+        <v>-0.27</v>
       </c>
       <c r="AD2" t="n">
         <v>0.44</v>
       </c>
       <c r="AE2" t="n">
-        <v>17.9</v>
+        <v>24.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.97</v>
+        <v>1.36</v>
       </c>
       <c r="AG2" t="n">
-        <v>41.8</v>
+        <v>42.15</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.8</v>
+        <v>42.15</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.27</v>
+        <v>2.3</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>10.43</v>
+        <v>9.66</v>
       </c>
       <c r="AM2" t="n">
-        <v>20.43</v>
+        <v>19.56</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.41</v>
+        <v>55.26</v>
       </c>
       <c r="AO2" t="n">
-        <v>79.79000000000001</v>
+        <v>78.09</v>
       </c>
       <c r="AP2" t="n">
-        <v>17.55</v>
+        <v>16.69</v>
       </c>
       <c r="AQ2" t="n">
-        <v>45.53</v>
+        <v>44.46</v>
       </c>
       <c r="AR2" t="n">
-        <v>1843.6</v>
+        <v>1830</v>
       </c>
       <c r="AS2" t="n">
-        <v>2010.78</v>
+        <v>1998.61</v>
       </c>
       <c r="AT2" t="n">
-        <v>1760.01</v>
+        <v>1745.69</v>
       </c>
       <c r="AU2" t="n">
-        <v>1843.599975585938</v>
+        <v>1830</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.07</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>167.18</v>
+        <v>168.61</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.53</v>
+        <v>4.61</v>
       </c>
       <c r="BA2" t="n">
-        <v>83.59</v>
+        <v>84.31</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,22 +1987,22 @@
         <v>48.1</v>
       </c>
       <c r="BG2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.6</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BM2" t="n">
         <v>645</v>
@@ -2011,10 +2011,10 @@
         <v>51</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.43</v>
+        <v>2.41</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.92</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.33</v>
@@ -2023,22 +2023,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.268</v>
+        <v>0.266</v>
       </c>
       <c r="BT2" t="n">
-        <v>1568.34</v>
+        <v>1554.09</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.91</v>
+        <v>-13.06</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,13 +2058,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.6</v>
+        <v>48.2</v>
       </c>
       <c r="CE2" t="n">
-        <v>57.5</v>
+        <v>57</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
         <v>72.90000000000001</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.38</v>
+        <v>83.87</v>
       </c>
       <c r="CO2" t="n">
-        <v>50</v>
+        <v>42.45</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.068099999999999</v>
+        <v>9.213699999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6047</v>
+        <v>0.614</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.302</v>
+        <v>0.3073</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0907</v>
+        <v>0.0921</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0022</v>
+        <v>1.9978</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1845</v>
+        <v>1.1936</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9956</v>
+        <v>4.0043</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.5341</v>
+        <v>4.6071</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.78</v>
+        <v>34.81</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.5341</v>
+        <v>4.6071</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9956</v>
+        <v>2.0043</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9956</v>
+        <v>4.0043</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0023</v>
+        <v>1.998</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.882</v>
+        <v>0.8686</v>
       </c>
       <c r="DQ2" t="n">
-        <v>83.59</v>
+        <v>84.31</v>
       </c>
       <c r="DR2" t="n">
-        <v>67.51000000000001</v>
+        <v>57.67</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>7.7313</v>
+        <v>7.2565</v>
       </c>
       <c r="DX2" t="n">
-        <v>50.52499999999998</v>
+        <v>54.77499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="DZ2" t="n">
-        <v>91.499</v>
+        <v>91.402</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>31.54</v>
+        <v>37.6</v>
       </c>
       <c r="EE2" t="n">
-        <v>7.7313</v>
+        <v>7.2565</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.92</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.292</v>
+        <v>2.163</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9948</v>
+        <v>4.006</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2993</v>
+        <v>0.2803</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7224</v>
+        <v>0.7141</v>
       </c>
       <c r="EK2" t="n">
-        <v>62.34</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>14.99</v>
+        <v>14.02</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.9577</v>
+        <v>1.817</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0731</v>
+        <v>0.1192</v>
       </c>
       <c r="ER2" t="n">
-        <v>16.1964</v>
+        <v>10.0109</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.6361</v>
+        <v>10.5485</v>
       </c>
       <c r="ET2" t="n">
-        <v>45.272</v>
+        <v>41.826</v>
       </c>
       <c r="EU2" t="n">
-        <v>9.827999999999999</v>
+        <v>15.3548</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4551</v>
+        <v>1.1979</v>
       </c>
       <c r="EW2" t="n">
-        <v>12.4987</v>
+        <v>11.7586</v>
       </c>
       <c r="EX2" t="n">
-        <v>46.67</v>
+        <v>37.58</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.25</v>
+        <v>68.8</v>
       </c>
       <c r="FC2" t="n">
-        <v>24.38</v>
+        <v>24.68</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.72</v>
+        <v>73.53</v>
       </c>
       <c r="FE2" t="n">
-        <v>72.86</v>
+        <v>76.91500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>48.335</v>
+        <v>40.015</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.4985</v>
+        <v>25.4152</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.973</v>
+        <v>67.077</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.145</v>
+        <v>46.24</v>
       </c>
       <c r="FJ2" t="n">
-        <v>71.20999999999999</v>
+        <v>68.81</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>79</v>
+        <v>69.14</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.20999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="FP2" t="n">
-        <v>73.33</v>
+        <v>54.85</v>
       </c>
       <c r="FQ2" t="n">
-        <v>78.06</v>
+        <v>62.33</v>
       </c>
       <c r="FR2" t="n">
-        <v>92.81</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.9905</v>
+        <v>66.764</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260806_113714</t>
+          <t>20260806_174615</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46240.48419326112</v>
+        <v>46240.74045367252</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46240.48418981482</v>
+        <v>46240.74045138889</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46240</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.06</v>
+        <v>12.96</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1843.6</v>
+        <v>1830</v>
       </c>
       <c r="L2" t="n">
         <v>1843</v>
@@ -2690,37 +2690,37 @@
         <v>1854.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1837</v>
+        <v>1830</v>
       </c>
       <c r="O2" t="n">
-        <v>1843.6</v>
+        <v>1830</v>
       </c>
       <c r="P2" t="n">
-        <v>1222690</v>
+        <v>2037365</v>
       </c>
       <c r="Q2" t="n">
-        <v>1843.6</v>
+        <v>1830</v>
       </c>
       <c r="R2" t="n">
-        <v>2010.78</v>
+        <v>1998.61</v>
       </c>
       <c r="S2" t="n">
-        <v>1760.01</v>
+        <v>1745.69</v>
       </c>
       <c r="T2" t="n">
-        <v>9.068127576480803</v>
+        <v>9.213661202185786</v>
       </c>
       <c r="U2" t="n">
-        <v>167.1800000000001</v>
+        <v>168.6099999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.534063788240395</v>
+        <v>4.607103825136609</v>
       </c>
       <c r="W2" t="n">
-        <v>83.58999999999992</v>
+        <v>84.30999999999995</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000003</v>
+        <v>1.999881390107935</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.068127576480803</v>
+        <v>9.213661202185786</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.534063788240395</v>
+        <v>4.607103825136609</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02067274353944541</v>
+        <v>0.02066223797434001</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3281696299367384</v>
+        <v>0.3280028592608319</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909864868366858</v>
+        <v>0.02909858947718529</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289545712491855</v>
+        <v>0.04289542403727443</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.75</v>
+        <v>38.76</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-06 11:37:14.332490+05:30</t>
+          <t>2026-08-06 17:46:15.233221+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.068127576480803, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.213661202185786, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999881390107935}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-07 05:05 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.96</v>
+        <v>13.16</v>
       </c>
       <c r="R2" t="n">
-        <v>50.44</v>
+        <v>50.31</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1843</v>
+        <v>1838</v>
       </c>
       <c r="V2" t="n">
-        <v>1854.9</v>
+        <v>1848</v>
       </c>
       <c r="W2" t="n">
-        <v>1830</v>
+        <v>1833.2</v>
       </c>
       <c r="X2" t="n">
-        <v>1830</v>
+        <v>1844.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>1830</v>
+        <v>1844.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>2037365</v>
+        <v>536055</v>
       </c>
       <c r="AA2" t="n">
-        <v>2225238</v>
+        <v>2150172</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.92</v>
+        <v>0.25</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.27</v>
+        <v>0.54</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.44</v>
+        <v>0.16</v>
       </c>
       <c r="AE2" t="n">
-        <v>24.9</v>
+        <v>14.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.36</v>
+        <v>0.8</v>
       </c>
       <c r="AG2" t="n">
-        <v>42.15</v>
+        <v>41.43</v>
       </c>
       <c r="AH2" t="n">
-        <v>42.15</v>
+        <v>41.43</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.3</v>
+        <v>2.25</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>9.66</v>
+        <v>10.5</v>
       </c>
       <c r="AM2" t="n">
-        <v>19.56</v>
+        <v>20.51</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.26</v>
+        <v>56.52</v>
       </c>
       <c r="AO2" t="n">
-        <v>78.09</v>
+        <v>79.87</v>
       </c>
       <c r="AP2" t="n">
-        <v>16.69</v>
+        <v>17.64</v>
       </c>
       <c r="AQ2" t="n">
-        <v>44.46</v>
+        <v>45.63</v>
       </c>
       <c r="AR2" t="n">
-        <v>1830</v>
+        <v>1844.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>1998.61</v>
+        <v>2010.63</v>
       </c>
       <c r="AT2" t="n">
-        <v>1745.69</v>
+        <v>1762.04</v>
       </c>
       <c r="AU2" t="n">
-        <v>1830</v>
+        <v>1844.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.210000000000001</v>
+        <v>8.98</v>
       </c>
       <c r="AY2" t="n">
-        <v>168.61</v>
+        <v>165.73</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.61</v>
+        <v>4.49</v>
       </c>
       <c r="BA2" t="n">
-        <v>84.31</v>
+        <v>82.86</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1987,58 +1987,58 @@
         <v>48.1</v>
       </c>
       <c r="BG2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="BI2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
         <v>645</v>
       </c>
       <c r="BN2" t="n">
-        <v>51</v>
+        <v>51.2</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.41</v>
+        <v>2.43</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.880000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.33</v>
+        <v>-4.34</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.266</v>
+        <v>0.269</v>
       </c>
       <c r="BT2" t="n">
-        <v>1554.09</v>
+        <v>1569.96</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.06</v>
+        <v>-12.87</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
       <c r="BW2" t="n">
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.2</v>
+        <v>48.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>57</v>
+        <v>57.5</v>
       </c>
       <c r="CF2" t="n">
         <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.90000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.87</v>
+        <v>82.75</v>
       </c>
       <c r="CO2" t="n">
-        <v>42.45</v>
+        <v>45.07</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.213699999999999</v>
+        <v>8.9831</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.614</v>
+        <v>0.5987</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3073</v>
+        <v>0.2993</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0921</v>
+        <v>0.0898</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9978</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1936</v>
+        <v>1.1818</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0043</v>
+        <v>3.9911</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6071</v>
+        <v>4.4913</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.81</v>
+        <v>35.85</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6071</v>
+        <v>4.4913</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0043</v>
+        <v>1.9956</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0043</v>
+        <v>3.9911</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.998</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8686</v>
+        <v>0.8889</v>
       </c>
       <c r="DQ2" t="n">
-        <v>84.31</v>
+        <v>82.86</v>
       </c>
       <c r="DR2" t="n">
-        <v>57.67</v>
+        <v>62.76</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>7.2565</v>
+        <v>7.84</v>
       </c>
       <c r="DX2" t="n">
-        <v>54.77499999999999</v>
+        <v>50.32499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>46</v>
+        <v>12.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>91.402</v>
+        <v>91.068</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,69 +2214,69 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>37.6</v>
+        <v>19.81</v>
       </c>
       <c r="EE2" t="n">
-        <v>7.2565</v>
+        <v>7.84</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.92</v>
+        <v>0.25</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.163</v>
+        <v>2.3214</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.006</v>
+        <v>3.9925</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2803</v>
+        <v>0.3055</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7141</v>
+        <v>0.7272</v>
       </c>
       <c r="EK2" t="n">
-        <v>69.95999999999999</v>
+        <v>57.83</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>14.02</v>
+        <v>10.68</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.817</v>
+        <v>1.4055</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1192</v>
+        <v>0.0329</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.0109</v>
+        <v>35.92</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5485</v>
+        <v>11.0308</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.826</v>
+        <v>42.178</v>
       </c>
       <c r="EU2" t="n">
-        <v>15.3548</v>
+        <v>4.41</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.1979</v>
+        <v>1.8</v>
       </c>
       <c r="EW2" t="n">
-        <v>11.7586</v>
+        <v>8.8377</v>
       </c>
       <c r="EX2" t="n">
-        <v>37.58</v>
+        <v>34.86</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>68.8</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="FC2" t="n">
-        <v>24.68</v>
+        <v>25.71</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.53</v>
+        <v>73.23</v>
       </c>
       <c r="FE2" t="n">
-        <v>76.91500000000001</v>
+        <v>70.29000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>40.015</v>
+        <v>39.965</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.4152</v>
+        <v>25.4615</v>
       </c>
       <c r="FH2" t="n">
-        <v>67.077</v>
+        <v>66.70699999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>46.24</v>
+        <v>49.305</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.81</v>
+        <v>70.5</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.14</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.2</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.85</v>
+        <v>54.06</v>
       </c>
       <c r="FQ2" t="n">
-        <v>62.33</v>
+        <v>63.93</v>
       </c>
       <c r="FR2" t="n">
-        <v>78.26000000000001</v>
+        <v>74.58</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.764</v>
+        <v>66.1815</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260806_174615</t>
+          <t>20260807_103459</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46240.74045367252</v>
+        <v>46241.44096415323</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46240.74045138889</v>
+        <v>46241.44096064815</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.96</v>
+        <v>13.16</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1830</v>
+        <v>1844.9</v>
       </c>
       <c r="L2" t="n">
-        <v>1843</v>
+        <v>1838</v>
       </c>
       <c r="M2" t="n">
-        <v>1854.9</v>
+        <v>1848</v>
       </c>
       <c r="N2" t="n">
-        <v>1830</v>
+        <v>1833.2</v>
       </c>
       <c r="O2" t="n">
-        <v>1830</v>
+        <v>1844.9</v>
       </c>
       <c r="P2" t="n">
-        <v>2037365</v>
+        <v>536055</v>
       </c>
       <c r="Q2" t="n">
-        <v>1830</v>
+        <v>1844.9</v>
       </c>
       <c r="R2" t="n">
-        <v>1998.61</v>
+        <v>2010.63</v>
       </c>
       <c r="S2" t="n">
-        <v>1745.69</v>
+        <v>1762.04</v>
       </c>
       <c r="T2" t="n">
-        <v>9.213661202185786</v>
+        <v>8.983142717762481</v>
       </c>
       <c r="U2" t="n">
-        <v>168.6099999999999</v>
+        <v>165.73</v>
       </c>
       <c r="V2" t="n">
-        <v>4.607103825136609</v>
+        <v>4.49130034148193</v>
       </c>
       <c r="W2" t="n">
-        <v>84.30999999999995</v>
+        <v>82.86000000000013</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999881390107935</v>
+        <v>2.000120685493601</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.213661202185786</v>
+        <v>8.983142717762481</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.607103825136609</v>
+        <v>4.49130034148193</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02066223797434001</v>
+        <v>0.02066654055344173</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3280028592608319</v>
+        <v>0.3280711605866279</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909858947718529</v>
+        <v>0.02909864868366858</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289542403727443</v>
+        <v>0.04289543368252276</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.76</v>
+        <v>38.75</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-06 17:46:15.233221+05:30</t>
+          <t>2026-08-07 10:34:59.341896+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.213661202185786, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999881390107935}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.983142717762481, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000120685493601}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-07 11:05 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.16</v>
+        <v>13.09</v>
       </c>
       <c r="R2" t="n">
-        <v>50.31</v>
+        <v>50.52</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1838</v>
       </c>
       <c r="V2" t="n">
-        <v>1848</v>
+        <v>1856</v>
       </c>
       <c r="W2" t="n">
         <v>1833.2</v>
       </c>
       <c r="X2" t="n">
-        <v>1844.9</v>
+        <v>1844.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1844.9</v>
+        <v>1844.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>536055</v>
+        <v>1553047</v>
       </c>
       <c r="AA2" t="n">
-        <v>2150172</v>
+        <v>2200812</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.25</v>
+        <v>0.71</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.54</v>
+        <v>0.78</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.16</v>
+        <v>0.44</v>
       </c>
       <c r="AE2" t="n">
-        <v>14.8</v>
+        <v>22.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.8</v>
+        <v>1.24</v>
       </c>
       <c r="AG2" t="n">
-        <v>41.43</v>
+        <v>41</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.43</v>
+        <v>41</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.25</v>
+        <v>2.22</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,71 +1926,71 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>10.5</v>
+        <v>9.51</v>
       </c>
       <c r="AM2" t="n">
-        <v>20.51</v>
+        <v>19.74</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.52</v>
+        <v>55.86</v>
       </c>
       <c r="AO2" t="n">
-        <v>79.87</v>
+        <v>79.05</v>
       </c>
       <c r="AP2" t="n">
-        <v>17.64</v>
+        <v>15.18</v>
       </c>
       <c r="AQ2" t="n">
-        <v>45.63</v>
+        <v>45.45</v>
       </c>
       <c r="AR2" t="n">
-        <v>1844.9</v>
+        <v>1844.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>2010.63</v>
+        <v>2008.3</v>
       </c>
       <c r="AT2" t="n">
-        <v>1762.04</v>
+        <v>1762.3</v>
       </c>
       <c r="AU2" t="n">
-        <v>1844.900024414062</v>
+        <v>1844.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.98</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>165.73</v>
+        <v>164</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.49</v>
+        <v>4.45</v>
       </c>
       <c r="BA2" t="n">
-        <v>82.86</v>
+        <v>82</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="BE2" t="n">
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.1</v>
+        <v>48</v>
       </c>
       <c r="BG2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.6</v>
+        <v>18.7</v>
       </c>
       <c r="BI2" t="n">
         <v>1</v>
@@ -2005,10 +2005,10 @@
         <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
       </c>
       <c r="BO2" t="n">
         <v>2.43</v>
@@ -2017,28 +2017,28 @@
         <v>8.9</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.34</v>
+        <v>-4.33</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.269</v>
+        <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1569.96</v>
+        <v>1569.22</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.87</v>
+        <v>-12.88</v>
       </c>
       <c r="BV2" t="n">
         <v>2.15</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2064,10 +2064,10 @@
         <v>57.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>73.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.75</v>
+        <v>84.29000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>45.07</v>
+        <v>37.45</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.9831</v>
+        <v>8.892300000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5987</v>
+        <v>0.5927</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2993</v>
+        <v>0.2967</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0898</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.9978</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.1637</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>4.0045</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.4461</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>32.09</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.4461</v>
+      </c>
+      <c r="DL2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.1818</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>3.9911</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>4.4913</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>35.85</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>4.4913</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>2.0001</v>
-      </c>
       <c r="DM2" t="n">
-        <v>1.9956</v>
+        <v>2.0045</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9911</v>
+        <v>4.0045</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9976</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8889</v>
+        <v>0.8999</v>
       </c>
       <c r="DQ2" t="n">
-        <v>82.86</v>
+        <v>82</v>
       </c>
       <c r="DR2" t="n">
-        <v>62.76</v>
+        <v>58.29</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>7.84</v>
+        <v>6.8378</v>
       </c>
       <c r="DX2" t="n">
-        <v>50.32499999999999</v>
+        <v>52.37500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>12.5</v>
+        <v>35.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>91.068</v>
+        <v>91.40900000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,107 +2214,107 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>19.81</v>
+        <v>34.21</v>
       </c>
       <c r="EE2" t="n">
-        <v>7.84</v>
+        <v>6.8378</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.25</v>
+        <v>0.71</v>
       </c>
       <c r="EG2" t="n">
-        <v>2.3214</v>
+        <v>1.9871</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9925</v>
+        <v>4.0055</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.3055</v>
+        <v>0.2601</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7272</v>
+        <v>0.735</v>
       </c>
       <c r="EK2" t="n">
-        <v>57.83</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="EM2" t="n">
+        <v>5</v>
+      </c>
+      <c r="EN2" t="n">
+        <v>10</v>
+      </c>
+      <c r="EO2" t="n">
+        <v>14.09</v>
+      </c>
+      <c r="EP2" t="n">
+        <v>1.8444</v>
+      </c>
+      <c r="EQ2" t="n">
+        <v>0.0929</v>
+      </c>
+      <c r="ER2" t="n">
+        <v>12.5211</v>
+      </c>
+      <c r="ES2" t="n">
+        <v>9.9658</v>
+      </c>
+      <c r="ET2" t="n">
+        <v>40.057</v>
+      </c>
+      <c r="EU2" t="n">
+        <v>10.7778</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>1.2982</v>
+      </c>
+      <c r="EW2" t="n">
+        <v>11.8765</v>
+      </c>
+      <c r="EX2" t="n">
+        <v>40.15</v>
+      </c>
+      <c r="EY2" t="inlineStr">
+        <is>
           <t>Average</t>
-        </is>
-      </c>
-      <c r="EM2" t="n">
-        <v>4</v>
-      </c>
-      <c r="EN2" t="n">
-        <v>8</v>
-      </c>
-      <c r="EO2" t="n">
-        <v>10.68</v>
-      </c>
-      <c r="EP2" t="n">
-        <v>1.4055</v>
-      </c>
-      <c r="EQ2" t="n">
-        <v>0.0329</v>
-      </c>
-      <c r="ER2" t="n">
-        <v>35.92</v>
-      </c>
-      <c r="ES2" t="n">
-        <v>11.0308</v>
-      </c>
-      <c r="ET2" t="n">
-        <v>42.178</v>
-      </c>
-      <c r="EU2" t="n">
-        <v>4.41</v>
-      </c>
-      <c r="EV2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="EW2" t="n">
-        <v>8.8377</v>
-      </c>
-      <c r="EX2" t="n">
-        <v>34.86</v>
-      </c>
-      <c r="EY2" t="inlineStr">
-        <is>
-          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.81999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.71</v>
+        <v>22.28</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.23</v>
+        <v>73.75</v>
       </c>
       <c r="FE2" t="n">
-        <v>70.29000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>39.965</v>
+        <v>38.8</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.4615</v>
+        <v>26.177</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.70699999999999</v>
+        <v>68.06699999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>49.305</v>
+        <v>45.19</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.5</v>
+        <v>68.27</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.09999999999999</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.26000000000001</v>
+        <v>66.72</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.06</v>
+        <v>60.13</v>
       </c>
       <c r="FQ2" t="n">
-        <v>63.93</v>
+        <v>66.45999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.58</v>
+        <v>82.47</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.1815</v>
+        <v>68.446</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260807_103459</t>
+          <t>20260807_163539</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46241.44096415323</v>
+        <v>46241.69142448709</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46241.44096064815</v>
+        <v>46241.69142361111</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46241</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.16</v>
+        <v>13.09</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1844.9</v>
+        <v>1844.3</v>
       </c>
       <c r="L2" t="n">
         <v>1838</v>
       </c>
       <c r="M2" t="n">
-        <v>1848</v>
+        <v>1856</v>
       </c>
       <c r="N2" t="n">
         <v>1833.2</v>
       </c>
       <c r="O2" t="n">
-        <v>1844.9</v>
+        <v>1844.3</v>
       </c>
       <c r="P2" t="n">
-        <v>536055</v>
+        <v>1553047</v>
       </c>
       <c r="Q2" t="n">
-        <v>1844.9</v>
+        <v>1844.3</v>
       </c>
       <c r="R2" t="n">
-        <v>2010.63</v>
+        <v>2008.3</v>
       </c>
       <c r="S2" t="n">
-        <v>1762.04</v>
+        <v>1762.3</v>
       </c>
       <c r="T2" t="n">
-        <v>8.983142717762481</v>
+        <v>8.892262647074771</v>
       </c>
       <c r="U2" t="n">
-        <v>165.73</v>
+        <v>164</v>
       </c>
       <c r="V2" t="n">
-        <v>4.49130034148193</v>
+        <v>4.446131323537386</v>
       </c>
       <c r="W2" t="n">
-        <v>82.86000000000013</v>
+        <v>82</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000120685493601</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.983142717762481</v>
+        <v>8.892262647074771</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.49130034148193</v>
+        <v>4.446131323537386</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02066654055344173</v>
+        <v>0.02064766242726204</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3280711605866279</v>
+        <v>0.3277714796240858</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909864868366858</v>
+        <v>0.02909850771828228</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543368252276</v>
+        <v>0.04289543702777602</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.75</v>
+        <v>38.78</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-07 10:34:59.341896+05:30</t>
+          <t>2026-08-07 16:35:39.116787+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.983142717762481, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000120685493601}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.892262647074771, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-10 04:57 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.09</v>
+        <v>13.29</v>
       </c>
       <c r="R2" t="n">
-        <v>50.52</v>
+        <v>50.47</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1838</v>
+        <v>1845</v>
       </c>
       <c r="V2" t="n">
-        <v>1856</v>
+        <v>1870.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1833.2</v>
+        <v>1844.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1844.3</v>
+        <v>1861.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>1844.3</v>
+        <v>1861.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>1553047</v>
+        <v>596789</v>
       </c>
       <c r="AA2" t="n">
-        <v>2200812</v>
+        <v>2133729</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.71</v>
+        <v>0.28</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.78</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.44</v>
+        <v>0.04</v>
       </c>
       <c r="AE2" t="n">
-        <v>22.8</v>
+        <v>26.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.24</v>
+        <v>1.41</v>
       </c>
       <c r="AG2" t="n">
-        <v>41</v>
+        <v>39.96</v>
       </c>
       <c r="AH2" t="n">
-        <v>41</v>
+        <v>39.96</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.22</v>
+        <v>2.15</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>9.51</v>
+        <v>9.56</v>
       </c>
       <c r="AM2" t="n">
-        <v>19.74</v>
+        <v>20.13</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.86</v>
+        <v>56.71</v>
       </c>
       <c r="AO2" t="n">
-        <v>79.05</v>
+        <v>80.18000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>15.18</v>
+        <v>8.66</v>
       </c>
       <c r="AQ2" t="n">
-        <v>45.45</v>
+        <v>45.39</v>
       </c>
       <c r="AR2" t="n">
-        <v>1844.3</v>
+        <v>1861.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>2008.3</v>
+        <v>2021.55</v>
       </c>
       <c r="AT2" t="n">
-        <v>1762.3</v>
+        <v>1781.77</v>
       </c>
       <c r="AU2" t="n">
-        <v>1844.300048828125</v>
+        <v>1861.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.890000000000001</v>
+        <v>8.59</v>
       </c>
       <c r="AY2" t="n">
-        <v>164</v>
+        <v>159.85</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.45</v>
+        <v>4.29</v>
       </c>
       <c r="BA2" t="n">
-        <v>82</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,61 +1984,61 @@
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>48</v>
+        <v>47.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.7</v>
+        <v>19</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.1</v>
+        <v>51.5</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.43</v>
+        <v>2.46</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.9</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.33</v>
+        <v>-4.35</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.268</v>
+        <v>0.27</v>
       </c>
       <c r="BT2" t="n">
-        <v>1569.22</v>
+        <v>1588.59</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.88</v>
+        <v>-12.73</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.15</v>
+        <v>2.16</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.6</v>
+        <v>49.2</v>
       </c>
       <c r="CE2" t="n">
-        <v>57.5</v>
+        <v>58</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>73</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,19 +2088,19 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>84.29000000000001</v>
+        <v>80.31</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.45</v>
+        <v>45.96</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
@@ -2109,22 +2109,22 @@
         <v>100</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>76.19047619047619</v>
       </c>
       <c r="CX2" t="n">
-        <v>63.63636363636363</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CY2" t="n">
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.892300000000001</v>
+        <v>8.5862</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5927</v>
+        <v>0.5727</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2967</v>
+        <v>0.286</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0859</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9978</v>
+        <v>2.0023</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1637</v>
+        <v>1.1416</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0045</v>
+        <v>3.9953</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.4461</v>
+        <v>4.2934</v>
       </c>
       <c r="DJ2" t="n">
-        <v>32.09</v>
+        <v>33.07</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.4461</v>
+        <v>4.2934</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0045</v>
+        <v>1.9953</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0045</v>
+        <v>3.9953</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9976</v>
+        <v>2.0024</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8999</v>
+        <v>0.9313</v>
       </c>
       <c r="DQ2" t="n">
-        <v>82</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>58.29</v>
+        <v>61.43</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,90 +2193,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>6.8378</v>
+        <v>4.0279</v>
       </c>
       <c r="DX2" t="n">
-        <v>52.37500000000001</v>
+        <v>49.54999999999998</v>
       </c>
       <c r="DY2" t="n">
-        <v>35.5</v>
+        <v>14</v>
       </c>
       <c r="DZ2" t="n">
-        <v>91.40900000000001</v>
+        <v>84.452</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>100</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>34.21</v>
+        <v>30.54</v>
       </c>
       <c r="EE2" t="n">
-        <v>6.8378</v>
+        <v>4.0279</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.71</v>
+        <v>0.28</v>
       </c>
       <c r="EG2" t="n">
-        <v>1.9871</v>
+        <v>1.1509</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0055</v>
+        <v>3.9936</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.2601</v>
+        <v>0.153</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.735</v>
+        <v>0.7549</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.79000000000001</v>
+        <v>53.46</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>14.09</v>
+        <v>28.82</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.8444</v>
+        <v>3.8302</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0929</v>
+        <v>0.0372</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.5211</v>
+        <v>30.6786</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.9658</v>
+        <v>10.4984</v>
       </c>
       <c r="ET2" t="n">
-        <v>40.057</v>
+        <v>48.075</v>
       </c>
       <c r="EU2" t="n">
-        <v>10.7778</v>
+        <v>2.4248</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2982</v>
+        <v>1.6797</v>
       </c>
       <c r="EW2" t="n">
-        <v>11.8765</v>
+        <v>23.1453</v>
       </c>
       <c r="EX2" t="n">
-        <v>40.15</v>
+        <v>55.8</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.5</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="FC2" t="n">
-        <v>22.28</v>
+        <v>22.75</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.75</v>
+        <v>72.62</v>
       </c>
       <c r="FE2" t="n">
-        <v>77.54000000000001</v>
+        <v>66.88500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>38.8</v>
+        <v>50.88</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.177</v>
+        <v>25.4952</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.06699999999999</v>
+        <v>70.328</v>
       </c>
       <c r="FI2" t="n">
-        <v>45.19</v>
+        <v>47.25</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.27</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>72.23999999999999</v>
+        <v>76.12</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.72</v>
+        <v>55.02</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.13</v>
+        <v>84.04000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.45999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.47</v>
+        <v>86.23</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>95.2381</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.446</v>
+        <v>70.87</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260807_163539</t>
+          <t>20260810_102733</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46241.69142448709</v>
+        <v>46244.43580983184</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46241.69142361111</v>
+        <v>46244.43579861111</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.09</v>
+        <v>13.29</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1844.3</v>
+        <v>1861.7</v>
       </c>
       <c r="L2" t="n">
-        <v>1838</v>
+        <v>1845</v>
       </c>
       <c r="M2" t="n">
-        <v>1856</v>
+        <v>1870.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1833.2</v>
+        <v>1844.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1844.3</v>
+        <v>1861.7</v>
       </c>
       <c r="P2" t="n">
-        <v>1553047</v>
+        <v>596789</v>
       </c>
       <c r="Q2" t="n">
-        <v>1844.3</v>
+        <v>1861.7</v>
       </c>
       <c r="R2" t="n">
-        <v>2008.3</v>
+        <v>2021.55</v>
       </c>
       <c r="S2" t="n">
-        <v>1762.3</v>
+        <v>1781.77</v>
       </c>
       <c r="T2" t="n">
-        <v>8.892262647074771</v>
+        <v>8.586238384272434</v>
       </c>
       <c r="U2" t="n">
-        <v>164</v>
+        <v>159.8499999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.446131323537386</v>
+        <v>4.293387763871733</v>
       </c>
       <c r="W2" t="n">
-        <v>82</v>
+        <v>79.93000000000006</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>1.99987489052921</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.892262647074771</v>
+        <v>8.586238384272434</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.446131323537386</v>
+        <v>4.293387763871733</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02064766242726204</v>
+        <v>0.02063382349793515</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3277714796240858</v>
+        <v>0.3275517934316238</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909850771828228</v>
+        <v>0.0290984710642187</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543702777602</v>
+        <v>0.04289545299741193</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.78</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-07 16:35:39.116787+05:30</t>
+          <t>2026-08-10 10:27:33.993576+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.892262647074771, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.586238384272434, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998748905292103}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-10 11:19 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.29</v>
+        <v>13.14</v>
       </c>
       <c r="R2" t="n">
-        <v>50.47</v>
+        <v>50.55</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>1870.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1844.5</v>
+        <v>1832.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1861.7</v>
+        <v>1854</v>
       </c>
       <c r="Y2" t="n">
-        <v>1861.7</v>
+        <v>1854</v>
       </c>
       <c r="Z2" t="n">
-        <v>596789</v>
+        <v>1386095</v>
       </c>
       <c r="AA2" t="n">
-        <v>2133729</v>
+        <v>2173194</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.28</v>
+        <v>0.64</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.53</v>
       </c>
       <c r="AD2" t="n">
         <v>0.04</v>
       </c>
       <c r="AE2" t="n">
-        <v>26.3</v>
+        <v>38</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.41</v>
+        <v>2.05</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.96</v>
+        <v>40.78</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.96</v>
+        <v>40.78</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.15</v>
+        <v>2.2</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>9.56</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="AM2" t="n">
-        <v>20.13</v>
+        <v>19.65</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.71</v>
+        <v>56.07</v>
       </c>
       <c r="AO2" t="n">
-        <v>80.18000000000001</v>
+        <v>79.7</v>
       </c>
       <c r="AP2" t="n">
-        <v>8.66</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="AQ2" t="n">
-        <v>45.39</v>
+        <v>44.79</v>
       </c>
       <c r="AR2" t="n">
-        <v>1861.7</v>
+        <v>1854</v>
       </c>
       <c r="AS2" t="n">
-        <v>2021.55</v>
+        <v>2017.14</v>
       </c>
       <c r="AT2" t="n">
-        <v>1781.77</v>
+        <v>1772.43</v>
       </c>
       <c r="AU2" t="n">
-        <v>1861.699951171875</v>
+        <v>1854</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.59</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>159.85</v>
+        <v>163.14</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.29</v>
+        <v>4.4</v>
       </c>
       <c r="BA2" t="n">
-        <v>79.93000000000001</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -1987,49 +1987,49 @@
         <v>47.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
         <v>647</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.5</v>
+        <v>51.3</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.46</v>
+        <v>2.44</v>
       </c>
       <c r="BP2" t="n">
         <v>8.869999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.35</v>
+        <v>-4.34</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.27</v>
+        <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1588.59</v>
+        <v>1579.96</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.73</v>
+        <v>-12.81</v>
       </c>
       <c r="BV2" t="n">
         <v>2.16</v>
@@ -2038,7 +2038,7 @@
         <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>49.2</v>
+        <v>48.8</v>
       </c>
       <c r="CE2" t="n">
         <v>58</v>
@@ -2067,7 +2067,7 @@
         <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>73.59999999999999</v>
+        <v>73.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,19 +2088,19 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>80.31</v>
+        <v>73.14</v>
       </c>
       <c r="CO2" t="n">
-        <v>45.96</v>
+        <v>34.3</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
@@ -2109,22 +2109,22 @@
         <v>100</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>76.19047619047619</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>66.66666666666666</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.5862</v>
+        <v>8.7994</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5727</v>
+        <v>0.5867</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.286</v>
+        <v>0.2933</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0859</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0023</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1416</v>
+        <v>1.1563</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9953</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2934</v>
+        <v>4.3997</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.07</v>
+        <v>33.09</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2934</v>
+        <v>4.3997</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9953</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9953</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0024</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9313</v>
+        <v>0.9091</v>
       </c>
       <c r="DQ2" t="n">
-        <v>79.93000000000001</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.43</v>
+        <v>63.47</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>4.0279</v>
+        <v>3.7318</v>
       </c>
       <c r="DX2" t="n">
-        <v>49.54999999999998</v>
+        <v>50.74999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.452</v>
+        <v>77.503</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>71.90000000000001</v>
+        <v>58.65</v>
       </c>
       <c r="ED2" t="n">
-        <v>30.54</v>
+        <v>35.59</v>
       </c>
       <c r="EE2" t="n">
-        <v>4.0279</v>
+        <v>3.7318</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.28</v>
+        <v>0.64</v>
       </c>
       <c r="EG2" t="n">
-        <v>1.1509</v>
+        <v>1.0788</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9936</v>
+        <v>3.9997</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.153</v>
+        <v>0.1418</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7549</v>
+        <v>0.7407</v>
       </c>
       <c r="EK2" t="n">
-        <v>53.46</v>
+        <v>52.41</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>28.82</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.8302</v>
+        <v>1.201</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0372</v>
+        <v>0.08409999999999999</v>
       </c>
       <c r="ER2" t="n">
-        <v>30.6786</v>
+        <v>13.75</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.4984</v>
+        <v>10.3406</v>
       </c>
       <c r="ET2" t="n">
-        <v>48.075</v>
+        <v>37.381</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.4248</v>
+        <v>5.2544</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6797</v>
+        <v>1.3415</v>
       </c>
       <c r="EW2" t="n">
-        <v>23.1453</v>
+        <v>6.685</v>
       </c>
       <c r="EX2" t="n">
-        <v>55.8</v>
+        <v>51.75</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,34 +2287,34 @@
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>70.15000000000001</v>
+        <v>69.73</v>
       </c>
       <c r="FC2" t="n">
-        <v>22.75</v>
+        <v>23.28</v>
       </c>
       <c r="FD2" t="n">
         <v>72.62</v>
       </c>
       <c r="FE2" t="n">
-        <v>66.88500000000001</v>
+        <v>62.775</v>
       </c>
       <c r="FF2" t="n">
-        <v>50.88</v>
+        <v>43.025</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.4952</v>
+        <v>22.8562</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.328</v>
+        <v>67.157</v>
       </c>
       <c r="FI2" t="n">
-        <v>47.25</v>
+        <v>48.28</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.90000000000001</v>
+        <v>66.69</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.12</v>
+        <v>70.81</v>
       </c>
       <c r="FO2" t="n">
-        <v>55.02</v>
+        <v>55.35</v>
       </c>
       <c r="FP2" t="n">
-        <v>84.04000000000001</v>
+        <v>70.59</v>
       </c>
       <c r="FQ2" t="n">
-        <v>78.72</v>
+        <v>71.61</v>
       </c>
       <c r="FR2" t="n">
-        <v>86.23</v>
+        <v>81.38</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.2381</v>
+        <v>86.36360000000001</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.87</v>
+        <v>68.512</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260810_102733</t>
+          <t>20260810_164949</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46244.43580983184</v>
+        <v>46244.70126294962</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46244.43579861111</v>
+        <v>46244.70126157408</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46244</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.29</v>
+        <v>13.14</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1861.7</v>
+        <v>1854</v>
       </c>
       <c r="L2" t="n">
         <v>1845</v>
@@ -2690,37 +2690,37 @@
         <v>1870.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1844.5</v>
+        <v>1832.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1861.7</v>
+        <v>1854</v>
       </c>
       <c r="P2" t="n">
-        <v>596789</v>
+        <v>1386095</v>
       </c>
       <c r="Q2" t="n">
-        <v>1861.7</v>
+        <v>1854</v>
       </c>
       <c r="R2" t="n">
-        <v>2021.55</v>
+        <v>2017.14</v>
       </c>
       <c r="S2" t="n">
-        <v>1781.77</v>
+        <v>1772.43</v>
       </c>
       <c r="T2" t="n">
-        <v>8.586238384272434</v>
+        <v>8.799352750809067</v>
       </c>
       <c r="U2" t="n">
-        <v>159.8499999999999</v>
+        <v>163.1400000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.293387763871733</v>
+        <v>4.399676375404527</v>
       </c>
       <c r="W2" t="n">
-        <v>79.93000000000006</v>
+        <v>81.56999999999994</v>
       </c>
       <c r="X2" t="n">
-        <v>1.99987489052921</v>
+        <v>2.000000000000003</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.586238384272434</v>
+        <v>8.799352750809067</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.293387763871733</v>
+        <v>4.399676375404527</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02063382349793515</v>
+        <v>0.02063739751213444</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3275517934316238</v>
+        <v>0.3276085291481449</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290984710642187</v>
+        <v>0.02909850771828228</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289545299741193</v>
+        <v>0.04289544765902224</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.8</v>
+        <v>38.79</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10 10:27:33.993576+05:30</t>
+          <t>2026-08-10 16:49:49.158789+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.586238384272434, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998748905292103}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.799352750809067, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-11 04:42 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.14</v>
+        <v>12.89</v>
       </c>
       <c r="R2" t="n">
-        <v>50.55</v>
+        <v>50.21</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1845</v>
+        <v>1851</v>
       </c>
       <c r="V2" t="n">
-        <v>1870.8</v>
+        <v>1851.1</v>
       </c>
       <c r="W2" t="n">
-        <v>1832.8</v>
+        <v>1834.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="Y2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="Z2" t="n">
-        <v>1386095</v>
+        <v>383731</v>
       </c>
       <c r="AA2" t="n">
-        <v>2173194</v>
+        <v>2127957</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.64</v>
+        <v>0.18</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.53</v>
+        <v>-0.65</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.04</v>
+        <v>-0.16</v>
       </c>
       <c r="AE2" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.05</v>
+        <v>0.92</v>
       </c>
       <c r="AG2" t="n">
-        <v>40.78</v>
+        <v>39.29</v>
       </c>
       <c r="AH2" t="n">
-        <v>40.78</v>
+        <v>39.29</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.2</v>
+        <v>2.13</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>9.130000000000001</v>
+        <v>7.53</v>
       </c>
       <c r="AM2" t="n">
-        <v>19.65</v>
+        <v>18.17</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.07</v>
+        <v>54.47</v>
       </c>
       <c r="AO2" t="n">
-        <v>79.7</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>8.210000000000001</v>
+        <v>4.72</v>
       </c>
       <c r="AQ2" t="n">
-        <v>44.79</v>
+        <v>40.02</v>
       </c>
       <c r="AR2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="AS2" t="n">
-        <v>2017.14</v>
+        <v>1999.17</v>
       </c>
       <c r="AT2" t="n">
-        <v>1772.43</v>
+        <v>1763.41</v>
       </c>
       <c r="AU2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>163.14</v>
+        <v>157.17</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.4</v>
+        <v>4.27</v>
       </c>
       <c r="BA2" t="n">
-        <v>81.56999999999999</v>
+        <v>78.59</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>33.1</v>
+        <v>33</v>
       </c>
       <c r="BE2" t="n">
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>47.9</v>
+        <v>47.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.9</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.3</v>
+        <v>50.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.44</v>
+        <v>2.42</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.869999999999999</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.34</v>
+        <v>-4.3</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.268</v>
+        <v>0.265</v>
       </c>
       <c r="BT2" t="n">
-        <v>1579.96</v>
+        <v>1565.59</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.81</v>
+        <v>-12.96</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.16</v>
+        <v>2.14</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.8</v>
+        <v>48.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>73.3</v>
+        <v>72.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>73.14</v>
+        <v>70.38</v>
       </c>
       <c r="CO2" t="n">
-        <v>34.3</v>
+        <v>34.82</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.7994</v>
+        <v>8.5326</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5867</v>
+        <v>0.5687</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2933</v>
+        <v>0.2847</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.0853</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.9977</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1563</v>
+        <v>1.0995</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0047</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.3997</v>
+        <v>4.2666</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.09</v>
+        <v>31.98</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.3997</v>
+        <v>4.2666</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0047</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0047</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9975</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9091</v>
+        <v>0.9379</v>
       </c>
       <c r="DQ2" t="n">
-        <v>81.56999999999999</v>
+        <v>78.59</v>
       </c>
       <c r="DR2" t="n">
-        <v>63.47</v>
+        <v>42.85</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>3.7318</v>
+        <v>2.216</v>
       </c>
       <c r="DX2" t="n">
-        <v>50.74999999999999</v>
+        <v>58.64999999999998</v>
       </c>
       <c r="DY2" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="DZ2" t="n">
-        <v>77.503</v>
+        <v>71.036</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>58.65</v>
+        <v>36.04</v>
       </c>
       <c r="ED2" t="n">
-        <v>35.59</v>
+        <v>46.81</v>
       </c>
       <c r="EE2" t="n">
-        <v>3.7318</v>
+        <v>2.216</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.64</v>
+        <v>0.18</v>
       </c>
       <c r="EG2" t="n">
-        <v>1.0788</v>
+        <v>0.6084000000000001</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9997</v>
+        <v>4.0059</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1418</v>
+        <v>0.0784</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7407</v>
+        <v>0.7601</v>
       </c>
       <c r="EK2" t="n">
-        <v>52.41</v>
+        <v>50.79</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,78 +2243,78 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="EO2" t="n">
-        <v>9.140000000000001</v>
+        <v>23.24</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.201</v>
+        <v>2.9956</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.0232</v>
       </c>
       <c r="ER2" t="n">
-        <v>13.75</v>
+        <v>47.3889</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.3406</v>
+        <v>10.2173</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.381</v>
+        <v>41.48</v>
       </c>
       <c r="EU2" t="n">
-        <v>5.2544</v>
+        <v>0.8496</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3415</v>
+        <v>1.8051</v>
       </c>
       <c r="EW2" t="n">
-        <v>6.685</v>
+        <v>16.3563</v>
       </c>
       <c r="EX2" t="n">
-        <v>51.75</v>
+        <v>36.87</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.73</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="FC2" t="n">
-        <v>23.28</v>
+        <v>22.54</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.62</v>
+        <v>74.27</v>
       </c>
       <c r="FE2" t="n">
-        <v>62.775</v>
+        <v>60.585</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.025</v>
+        <v>35.845</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.8562</v>
+        <v>22.4856</v>
       </c>
       <c r="FH2" t="n">
-        <v>67.157</v>
+        <v>62.788</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.28</v>
+        <v>37.415</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.69</v>
+        <v>64.03</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,47 +2328,47 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.81</v>
+        <v>58.44</v>
       </c>
       <c r="FO2" t="n">
-        <v>55.35</v>
+        <v>53.28</v>
       </c>
       <c r="FP2" t="n">
-        <v>70.59</v>
+        <v>48.87</v>
       </c>
       <c r="FQ2" t="n">
-        <v>71.61</v>
+        <v>57.59</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.38</v>
+        <v>64.97</v>
       </c>
       <c r="FS2" t="n">
-        <v>86.36360000000001</v>
+        <v>72.7273</v>
       </c>
       <c r="FT2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.512</v>
+        <v>56.5155</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="FY2" t="b">
         <v>0</v>
       </c>
       <c r="FZ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GA2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260810_164949</t>
+          <t>20260811_101233</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46244.70126294962</v>
+        <v>46245.42539003941</v>
       </c>
     </row>
   </sheetData>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46244.70126157408</v>
+        <v>46245.42538194444</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.14</v>
+        <v>12.89</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="L2" t="n">
-        <v>1845</v>
+        <v>1851</v>
       </c>
       <c r="M2" t="n">
-        <v>1870.8</v>
+        <v>1851.1</v>
       </c>
       <c r="N2" t="n">
-        <v>1832.8</v>
+        <v>1834.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="P2" t="n">
-        <v>1386095</v>
+        <v>383731</v>
       </c>
       <c r="Q2" t="n">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="R2" t="n">
-        <v>2017.14</v>
+        <v>1999.17</v>
       </c>
       <c r="S2" t="n">
-        <v>1772.43</v>
+        <v>1763.41</v>
       </c>
       <c r="T2" t="n">
-        <v>8.799352750809067</v>
+        <v>8.532573289902285</v>
       </c>
       <c r="U2" t="n">
-        <v>163.1400000000001</v>
+        <v>157.1700000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.399676375404527</v>
+        <v>4.266558089033655</v>
       </c>
       <c r="W2" t="n">
-        <v>81.56999999999994</v>
+        <v>78.58999999999992</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000003</v>
+        <v>1.999872757348266</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.799352750809067</v>
+        <v>8.532573289902285</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.399676375404527</v>
+        <v>4.266558089033655</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02063739751213444</v>
+        <v>0.0206351389956304</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3276085291481449</v>
+        <v>0.3275726763101351</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909850771828228</v>
+        <v>0.0290984710642187</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289544765902224</v>
+        <v>0.04289543477169911</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10 16:49:49.158789+05:30</t>
+          <t>2026-08-11 10:12:33.735682+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.799352750809067, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.532573289902285, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998727573482662}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-11 11:03 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.89</v>
+        <v>13.19</v>
       </c>
       <c r="R2" t="n">
-        <v>50.21</v>
+        <v>50.59</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1851</v>
       </c>
       <c r="V2" t="n">
-        <v>1851.1</v>
+        <v>1859</v>
       </c>
       <c r="W2" t="n">
-        <v>1834.1</v>
+        <v>1833.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="Y2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="Z2" t="n">
-        <v>383731</v>
+        <v>1514031</v>
       </c>
       <c r="AA2" t="n">
-        <v>2127957</v>
+        <v>2184472</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.18</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.65</v>
+        <v>0.22</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.16</v>
       </c>
       <c r="AE2" t="n">
-        <v>17</v>
+        <v>25.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.92</v>
+        <v>1.39</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.29</v>
+        <v>39.72</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.29</v>
+        <v>39.72</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>7.53</v>
+        <v>8.42</v>
       </c>
       <c r="AM2" t="n">
-        <v>18.17</v>
+        <v>19.17</v>
       </c>
       <c r="AN2" t="n">
-        <v>54.47</v>
+        <v>55.8</v>
       </c>
       <c r="AO2" t="n">
-        <v>76.54000000000001</v>
+        <v>79.97</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.72</v>
+        <v>5.63</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.02</v>
+        <v>41.24</v>
       </c>
       <c r="AR2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="AS2" t="n">
-        <v>1999.17</v>
+        <v>2016.89</v>
       </c>
       <c r="AT2" t="n">
-        <v>1763.41</v>
+        <v>1778.56</v>
       </c>
       <c r="AU2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.529999999999999</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>157.17</v>
+        <v>158.89</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.27</v>
+        <v>4.28</v>
       </c>
       <c r="BA2" t="n">
-        <v>78.59</v>
+        <v>79.44</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.03</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,58 +1987,58 @@
         <v>47.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>19.1</v>
       </c>
       <c r="BI2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
         <v>648</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.9</v>
+        <v>51.5</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.42</v>
+        <v>2.45</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.890000000000001</v>
+        <v>8.83</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.3</v>
+        <v>-4.35</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.265</v>
+        <v>0.268</v>
       </c>
       <c r="BT2" t="n">
-        <v>1565.59</v>
+        <v>1584.6</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.96</v>
+        <v>-12.79</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.14</v>
+        <v>2.16</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.03</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.4</v>
+        <v>49</v>
       </c>
       <c r="CE2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>67.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>70.38</v>
+        <v>75.19</v>
       </c>
       <c r="CO2" t="n">
-        <v>34.82</v>
+        <v>34.95</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>63.63636363636363</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.5326</v>
+        <v>8.5517</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5687</v>
+        <v>0.57</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2847</v>
+        <v>0.2853</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0853</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="DF2" t="n">
         <v>1.9977</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0995</v>
+        <v>1.1277</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0047</v>
+        <v>3.9953</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2666</v>
+        <v>4.2756</v>
       </c>
       <c r="DJ2" t="n">
-        <v>31.98</v>
+        <v>30.54</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2666</v>
+        <v>4.2756</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0047</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0047</v>
+        <v>3.9953</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9975</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9379</v>
+        <v>0.9335</v>
       </c>
       <c r="DQ2" t="n">
-        <v>78.59</v>
+        <v>79.44</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.85</v>
+        <v>42.18</v>
       </c>
       <c r="DS2" t="n">
         <v>3</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.216</v>
+        <v>2.6308</v>
       </c>
       <c r="DX2" t="n">
-        <v>58.64999999999998</v>
+        <v>50.075</v>
       </c>
       <c r="DY2" t="n">
-        <v>9</v>
+        <v>34.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>71.036</v>
+        <v>75.175</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>36.04</v>
+        <v>43.98</v>
       </c>
       <c r="ED2" t="n">
-        <v>46.81</v>
+        <v>38.6</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.216</v>
+        <v>2.6308</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.18</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.6084000000000001</v>
+        <v>0.7426</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0059</v>
+        <v>3.9961</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0784</v>
+        <v>0.0979</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7601</v>
+        <v>0.7568</v>
       </c>
       <c r="EK2" t="n">
-        <v>50.79</v>
+        <v>47.09</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,40 +2243,40 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="EN2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>23.24</v>
+        <v>30.25</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.9956</v>
+        <v>3.99</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0232</v>
+        <v>0.091</v>
       </c>
       <c r="ER2" t="n">
-        <v>47.3889</v>
+        <v>12.3913</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.2173</v>
+        <v>9.726100000000001</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.48</v>
+        <v>44.043</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.8496</v>
+        <v>3.8847</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8051</v>
+        <v>1.2663</v>
       </c>
       <c r="EW2" t="n">
-        <v>16.3563</v>
+        <v>22.745</v>
       </c>
       <c r="EX2" t="n">
-        <v>36.87</v>
+        <v>32.57</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>7</v>
       </c>
       <c r="FB2" t="n">
-        <v>68.59999999999999</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="FC2" t="n">
-        <v>22.54</v>
+        <v>21.51</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.27</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>60.585</v>
+        <v>61.14</v>
       </c>
       <c r="FF2" t="n">
-        <v>35.845</v>
+        <v>33.76</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.4856</v>
+        <v>23.9459</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.788</v>
+        <v>64.051</v>
       </c>
       <c r="FI2" t="n">
-        <v>37.415</v>
+        <v>36.36</v>
       </c>
       <c r="FJ2" t="n">
-        <v>64.03</v>
+        <v>63.73</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>58.44</v>
+        <v>60.09</v>
       </c>
       <c r="FO2" t="n">
-        <v>53.28</v>
+        <v>51.61</v>
       </c>
       <c r="FP2" t="n">
-        <v>48.87</v>
+        <v>50.4</v>
       </c>
       <c r="FQ2" t="n">
-        <v>57.59</v>
+        <v>61.86</v>
       </c>
       <c r="FR2" t="n">
-        <v>64.97</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>72.7273</v>
+        <v>77.2727</v>
       </c>
       <c r="FT2" t="n">
         <v>4</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>56.5155</v>
+        <v>57.329</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260811_101233</t>
+          <t>20260811_163339</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46245.42539003941</v>
+        <v>46245.69004349141</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46245.42538194444</v>
+        <v>46245.69003472223</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46245</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.89</v>
+        <v>13.19</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="L2" t="n">
         <v>1851</v>
       </c>
       <c r="M2" t="n">
-        <v>1851.1</v>
+        <v>1859</v>
       </c>
       <c r="N2" t="n">
-        <v>1834.1</v>
+        <v>1833.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="P2" t="n">
-        <v>383731</v>
+        <v>1514031</v>
       </c>
       <c r="Q2" t="n">
-        <v>1842</v>
+        <v>1858</v>
       </c>
       <c r="R2" t="n">
-        <v>1999.17</v>
+        <v>2016.89</v>
       </c>
       <c r="S2" t="n">
-        <v>1763.41</v>
+        <v>1778.56</v>
       </c>
       <c r="T2" t="n">
-        <v>8.532573289902285</v>
+        <v>8.551668460710447</v>
       </c>
       <c r="U2" t="n">
-        <v>157.1700000000001</v>
+        <v>158.8900000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.266558089033655</v>
+        <v>4.275565123789024</v>
       </c>
       <c r="W2" t="n">
-        <v>78.58999999999992</v>
+        <v>79.44000000000005</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999872757348266</v>
+        <v>2.000125881168177</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.532573289902285</v>
+        <v>8.551668460710447</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.266558089033655</v>
+        <v>4.275565123789024</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0206351389956304</v>
+        <v>0.02062187992086927</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3275726763101351</v>
+        <v>0.3273621950235386</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290984710642187</v>
+        <v>0.02909844287369406</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543477169911</v>
+        <v>0.04289543695258682</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.79</v>
+        <v>38.81</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-11 10:12:33.735682+05:30</t>
+          <t>2026-08-11 16:33:39.796457+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.532573289902285, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998727573482662}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.551668460710447, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001258811681772}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-12 05:06 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.19</v>
+        <v>13.02</v>
       </c>
       <c r="R2" t="n">
-        <v>50.59</v>
+        <v>50.35</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1851</v>
+        <v>1856.3</v>
       </c>
       <c r="V2" t="n">
-        <v>1859</v>
+        <v>1862.3</v>
       </c>
       <c r="W2" t="n">
-        <v>1833.1</v>
+        <v>1847.2</v>
       </c>
       <c r="X2" t="n">
-        <v>1858</v>
+        <v>1853.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>1858</v>
+        <v>1853.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>1514031</v>
+        <v>316710</v>
       </c>
       <c r="AA2" t="n">
-        <v>2184472</v>
+        <v>2128794</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.22</v>
+        <v>-0.24</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.16</v>
+        <v>-0.09</v>
       </c>
       <c r="AE2" t="n">
-        <v>25.9</v>
+        <v>15.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.39</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.72</v>
+        <v>37.96</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.72</v>
+        <v>37.96</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.14</v>
+        <v>2.05</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>8.42</v>
+        <v>7.22</v>
       </c>
       <c r="AM2" t="n">
-        <v>19.17</v>
+        <v>18.2</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.8</v>
+        <v>54.83</v>
       </c>
       <c r="AO2" t="n">
-        <v>79.97</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>5.63</v>
+        <v>4.06</v>
       </c>
       <c r="AQ2" t="n">
-        <v>41.24</v>
+        <v>40.04</v>
       </c>
       <c r="AR2" t="n">
-        <v>1858</v>
+        <v>1853.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2016.89</v>
+        <v>2005.45</v>
       </c>
       <c r="AT2" t="n">
-        <v>1778.56</v>
+        <v>1777.67</v>
       </c>
       <c r="AU2" t="n">
-        <v>1858</v>
+        <v>1853.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.550000000000001</v>
+        <v>8.19</v>
       </c>
       <c r="AY2" t="n">
-        <v>158.89</v>
+        <v>151.85</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.28</v>
+        <v>4.1</v>
       </c>
       <c r="BA2" t="n">
-        <v>79.44</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.03</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,58 +1987,58 @@
         <v>47.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BM2" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.5</v>
+        <v>51.2</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.45</v>
+        <v>2.43</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.83</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.35</v>
+        <v>-4.31</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.268</v>
+        <v>0.266</v>
       </c>
       <c r="BT2" t="n">
-        <v>1584.6</v>
+        <v>1579.1</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.79</v>
+        <v>-12.86</v>
       </c>
       <c r="BV2" t="n">
         <v>2.16</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.03</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>49</v>
+        <v>48.6</v>
       </c>
       <c r="CE2" t="n">
         <v>58</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.7</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>73.59999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.19</v>
+        <v>68.86</v>
       </c>
       <c r="CO2" t="n">
-        <v>34.95</v>
+        <v>24.99</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>100</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.5517</v>
+        <v>8.1922</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.57</v>
+        <v>0.546</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2853</v>
+        <v>0.2733</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.0819</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9977</v>
+        <v>1.9976</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1277</v>
+        <v>1.0663</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9953</v>
+        <v>3.9951</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2756</v>
+        <v>4.0964</v>
       </c>
       <c r="DJ2" t="n">
-        <v>30.54</v>
+        <v>30.5</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2756</v>
+        <v>4.0964</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9953</v>
+        <v>3.9951</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>1.9978</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9335</v>
+        <v>0.9744</v>
       </c>
       <c r="DQ2" t="n">
-        <v>79.44</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.18</v>
+        <v>44.18</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.6308</v>
+        <v>1.9805</v>
       </c>
       <c r="DX2" t="n">
-        <v>50.075</v>
+        <v>53.22500000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>34.5</v>
+        <v>7.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>75.175</v>
+        <v>71.71899999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>43.98</v>
+        <v>40.79</v>
       </c>
       <c r="ED2" t="n">
-        <v>38.6</v>
+        <v>41.69</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.6308</v>
+        <v>1.9805</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.7426</v>
+        <v>0.5286</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9961</v>
+        <v>3.9962</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0979</v>
+        <v>0.0688</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7568</v>
+        <v>0.7836</v>
       </c>
       <c r="EK2" t="n">
-        <v>47.09</v>
+        <v>43.13</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>30.25</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.99</v>
+        <v>1.2421</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.091</v>
+        <v>0.0195</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.3913</v>
+        <v>54.6</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.726100000000001</v>
+        <v>10</v>
       </c>
       <c r="ET2" t="n">
-        <v>44.043</v>
+        <v>33.657</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.8847</v>
+        <v>0.609</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2663</v>
+        <v>1.7826</v>
       </c>
       <c r="EW2" t="n">
-        <v>22.745</v>
+        <v>6.5692</v>
       </c>
       <c r="EX2" t="n">
-        <v>32.57</v>
+        <v>23.28</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,41 +2284,41 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.95999999999999</v>
+        <v>69.33</v>
       </c>
       <c r="FC2" t="n">
-        <v>21.51</v>
+        <v>21.3</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.18000000000001</v>
+        <v>73.83</v>
       </c>
       <c r="FE2" t="n">
-        <v>61.14</v>
+        <v>55.995</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.76</v>
+        <v>24.135</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.9459</v>
+        <v>22.577</v>
       </c>
       <c r="FH2" t="n">
-        <v>64.051</v>
+        <v>59.979</v>
       </c>
       <c r="FI2" t="n">
-        <v>36.36</v>
+        <v>37.34</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.73</v>
+        <v>59.14</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="FL2" t="n">
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>60.09</v>
+        <v>54.68</v>
       </c>
       <c r="FO2" t="n">
-        <v>51.61</v>
+        <v>45.66</v>
       </c>
       <c r="FP2" t="n">
-        <v>50.4</v>
+        <v>43.52</v>
       </c>
       <c r="FQ2" t="n">
-        <v>61.86</v>
+        <v>60.12</v>
       </c>
       <c r="FR2" t="n">
-        <v>67.34999999999999</v>
+        <v>64.19</v>
       </c>
       <c r="FS2" t="n">
-        <v>77.2727</v>
+        <v>63.6364</v>
       </c>
       <c r="FT2" t="n">
         <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>57.329</v>
+        <v>55.125</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260811_163339</t>
+          <t>20260812_103637</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46245.69004349141</v>
+        <v>46246.44209809289</v>
       </c>
     </row>
   </sheetData>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46245.69003472223</v>
+        <v>46246.4420949074</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.19</v>
+        <v>13.02</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1858</v>
+        <v>1853.6</v>
       </c>
       <c r="L2" t="n">
-        <v>1851</v>
+        <v>1856.3</v>
       </c>
       <c r="M2" t="n">
-        <v>1859</v>
+        <v>1862.3</v>
       </c>
       <c r="N2" t="n">
-        <v>1833.1</v>
+        <v>1847.2</v>
       </c>
       <c r="O2" t="n">
-        <v>1858</v>
+        <v>1853.6</v>
       </c>
       <c r="P2" t="n">
-        <v>1514031</v>
+        <v>316710</v>
       </c>
       <c r="Q2" t="n">
-        <v>1858</v>
+        <v>1853.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2016.89</v>
+        <v>2005.45</v>
       </c>
       <c r="S2" t="n">
-        <v>1778.56</v>
+        <v>1777.67</v>
       </c>
       <c r="T2" t="n">
-        <v>8.551668460710447</v>
+        <v>8.192166594734578</v>
       </c>
       <c r="U2" t="n">
-        <v>158.8900000000001</v>
+        <v>151.8500000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.275565123789024</v>
+        <v>4.096353042727657</v>
       </c>
       <c r="W2" t="n">
-        <v>79.44000000000005</v>
+        <v>75.92999999999984</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000125881168177</v>
+        <v>1.999868299749776</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.551668460710447</v>
+        <v>8.192166594734578</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.275565123789024</v>
+        <v>4.096353042727657</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02062187992086927</v>
+        <v>0.02062276900301135</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3273621950235386</v>
+        <v>0.327376308764997</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909844287369406</v>
+        <v>0.0290984710642187</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543695258682</v>
+        <v>0.04289543623072582</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-11 16:33:39.796457+05:30</t>
+          <t>2026-08-12 10:36:37.313071+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.551668460710447, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001258811681772}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.192166594734578, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998682997497756}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-12 11:09 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>13.02</v>
+        <v>12.97</v>
       </c>
       <c r="R2" t="n">
-        <v>50.35</v>
+        <v>50.44</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>1862.3</v>
       </c>
       <c r="W2" t="n">
-        <v>1847.2</v>
+        <v>1835</v>
       </c>
       <c r="X2" t="n">
-        <v>1853.6</v>
+        <v>1850</v>
       </c>
       <c r="Y2" t="n">
-        <v>1853.6</v>
+        <v>1850</v>
       </c>
       <c r="Z2" t="n">
-        <v>316710</v>
+        <v>1088423</v>
       </c>
       <c r="AA2" t="n">
-        <v>2128794</v>
+        <v>2167380</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.24</v>
+        <v>-0.43</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.09</v>
       </c>
       <c r="AE2" t="n">
-        <v>15.1</v>
+        <v>27.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.48</v>
       </c>
       <c r="AG2" t="n">
-        <v>37.96</v>
+        <v>38.83</v>
       </c>
       <c r="AH2" t="n">
-        <v>37.96</v>
+        <v>38.83</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>7.22</v>
+        <v>7.03</v>
       </c>
       <c r="AM2" t="n">
-        <v>18.2</v>
+        <v>17.97</v>
       </c>
       <c r="AN2" t="n">
-        <v>54.83</v>
+        <v>54.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>78.70999999999999</v>
+        <v>77.7</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.06</v>
+        <v>3.86</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.04</v>
+        <v>39.77</v>
       </c>
       <c r="AR2" t="n">
-        <v>1853.6</v>
+        <v>1850</v>
       </c>
       <c r="AS2" t="n">
-        <v>2005.45</v>
+        <v>2005.34</v>
       </c>
       <c r="AT2" t="n">
-        <v>1777.67</v>
+        <v>1772.33</v>
       </c>
       <c r="AU2" t="n">
-        <v>1853.599975585938</v>
+        <v>1850</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.19</v>
+        <v>8.4</v>
       </c>
       <c r="AY2" t="n">
-        <v>151.85</v>
+        <v>155.34</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="BA2" t="n">
-        <v>75.93000000000001</v>
+        <v>77.67</v>
       </c>
       <c r="BB2" t="n">
         <v>2.06</v>
@@ -1987,22 +1987,22 @@
         <v>47.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="BI2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BM2" t="n">
         <v>649</v>
@@ -2014,7 +2014,7 @@
         <v>2.43</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.869999999999999</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.31</v>
@@ -2023,22 +2023,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.266</v>
+        <v>0.265</v>
       </c>
       <c r="BT2" t="n">
-        <v>1579.1</v>
+        <v>1574.65</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.86</v>
+        <v>-12.9</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.16</v>
+        <v>2.15</v>
       </c>
       <c r="BW2" t="n">
         <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2061,7 +2061,7 @@
         <v>48.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>58</v>
+        <v>57.5</v>
       </c>
       <c r="CF2" t="n">
         <v>68.7</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>68.86</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>24.99</v>
+        <v>26.48</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.1922</v>
+        <v>8.396800000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.546</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2733</v>
+        <v>0.28</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0819</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9976</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0663</v>
+        <v>1.0895</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9951</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.0964</v>
+        <v>4.1984</v>
       </c>
       <c r="DJ2" t="n">
-        <v>30.5</v>
+        <v>30.8</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.0964</v>
+        <v>4.1984</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9951</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9978</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9744</v>
+        <v>0.9524</v>
       </c>
       <c r="DQ2" t="n">
-        <v>75.93000000000001</v>
+        <v>77.67</v>
       </c>
       <c r="DR2" t="n">
-        <v>44.18</v>
+        <v>48.75</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.9805</v>
+        <v>1.8381</v>
       </c>
       <c r="DX2" t="n">
-        <v>53.22500000000002</v>
+        <v>55.74999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>7.5</v>
+        <v>25</v>
       </c>
       <c r="DZ2" t="n">
-        <v>71.71899999999999</v>
+        <v>70.121</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>40.79</v>
+        <v>36.92</v>
       </c>
       <c r="ED2" t="n">
-        <v>41.69</v>
+        <v>44.56</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.9805</v>
+        <v>1.8381</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5286</v>
+        <v>0.5006</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9962</v>
+        <v>3.9985</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0688</v>
+        <v>0.0649</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7836</v>
+        <v>0.7689</v>
       </c>
       <c r="EK2" t="n">
-        <v>43.13</v>
+        <v>43.37</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,40 +2243,40 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="EO2" t="n">
-        <v>9.539999999999999</v>
+        <v>7.43</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.2421</v>
+        <v>0.9637</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0195</v>
+        <v>0.0648</v>
       </c>
       <c r="ER2" t="n">
-        <v>54.6</v>
+        <v>16.8</v>
       </c>
       <c r="ES2" t="n">
-        <v>10</v>
+        <v>9.935499999999999</v>
       </c>
       <c r="ET2" t="n">
-        <v>33.657</v>
+        <v>33.509</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.609</v>
+        <v>1.93</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7826</v>
+        <v>1.4</v>
       </c>
       <c r="EW2" t="n">
-        <v>6.5692</v>
+        <v>5.0784</v>
       </c>
       <c r="EX2" t="n">
-        <v>23.28</v>
+        <v>25.85</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>5</v>
       </c>
       <c r="FB2" t="n">
-        <v>69.33</v>
+        <v>68.95999999999999</v>
       </c>
       <c r="FC2" t="n">
-        <v>21.3</v>
+        <v>20.64</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.83</v>
+        <v>73.75</v>
       </c>
       <c r="FE2" t="n">
-        <v>55.995</v>
+        <v>55.86</v>
       </c>
       <c r="FF2" t="n">
-        <v>24.135</v>
+        <v>26.165</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.577</v>
+        <v>22.0484</v>
       </c>
       <c r="FH2" t="n">
-        <v>59.979</v>
+        <v>60.155</v>
       </c>
       <c r="FI2" t="n">
-        <v>37.34</v>
+        <v>39.775</v>
       </c>
       <c r="FJ2" t="n">
-        <v>59.14</v>
+        <v>59.29</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>54.68</v>
+        <v>57.23</v>
       </c>
       <c r="FO2" t="n">
-        <v>45.66</v>
+        <v>45.65</v>
       </c>
       <c r="FP2" t="n">
-        <v>43.52</v>
+        <v>48.1</v>
       </c>
       <c r="FQ2" t="n">
-        <v>60.12</v>
+        <v>63.68</v>
       </c>
       <c r="FR2" t="n">
-        <v>64.19</v>
+        <v>68.81</v>
       </c>
       <c r="FS2" t="n">
-        <v>63.6364</v>
+        <v>72.7273</v>
       </c>
       <c r="FT2" t="n">
         <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>55.125</v>
+        <v>58.1955</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260812_103637</t>
+          <t>20260812_163946</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46246.44209809289</v>
+        <v>46246.6942906041</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46246.4420949074</v>
+        <v>46246.69428240741</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46246</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>13.02</v>
+        <v>12.97</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1853.6</v>
+        <v>1850</v>
       </c>
       <c r="L2" t="n">
         <v>1856.3</v>
@@ -2690,37 +2690,37 @@
         <v>1862.3</v>
       </c>
       <c r="N2" t="n">
-        <v>1847.2</v>
+        <v>1835</v>
       </c>
       <c r="O2" t="n">
-        <v>1853.6</v>
+        <v>1850</v>
       </c>
       <c r="P2" t="n">
-        <v>316710</v>
+        <v>1088423</v>
       </c>
       <c r="Q2" t="n">
-        <v>1853.6</v>
+        <v>1850</v>
       </c>
       <c r="R2" t="n">
-        <v>2005.45</v>
+        <v>2005.34</v>
       </c>
       <c r="S2" t="n">
-        <v>1777.67</v>
+        <v>1772.33</v>
       </c>
       <c r="T2" t="n">
-        <v>8.192166594734578</v>
+        <v>8.396756756756753</v>
       </c>
       <c r="U2" t="n">
-        <v>151.8500000000001</v>
+        <v>155.3399999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.096353042727657</v>
+        <v>4.198378378378383</v>
       </c>
       <c r="W2" t="n">
-        <v>75.92999999999984</v>
+        <v>77.67000000000007</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999868299749776</v>
+        <v>1.999999999999997</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.192166594734578</v>
+        <v>8.396756756756753</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.096353042727657</v>
+        <v>4.198378378378383</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02062276900301135</v>
+        <v>0.0206238008639876</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.327376308764997</v>
+        <v>0.3273926890501814</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290984710642187</v>
+        <v>0.02909850771828228</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543623072582</v>
+        <v>0.04289543702777602</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-12 10:36:37.313071+05:30</t>
+          <t>2026-08-12 16:39:46.740197+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.192166594734578, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998682997497756}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.396756756756753, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999971}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-13 05:10 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.97</v>
+        <v>12.65</v>
       </c>
       <c r="R2" t="n">
-        <v>50.44</v>
+        <v>50.06</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1856.3</v>
+        <v>1850</v>
       </c>
       <c r="V2" t="n">
-        <v>1862.3</v>
+        <v>1850.1</v>
       </c>
       <c r="W2" t="n">
-        <v>1835</v>
+        <v>1820.6</v>
       </c>
       <c r="X2" t="n">
-        <v>1850</v>
+        <v>1830.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1850</v>
+        <v>1830.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>1088423</v>
+        <v>505290</v>
       </c>
       <c r="AA2" t="n">
-        <v>2167380</v>
+        <v>2138223</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.5</v>
+        <v>0.24</v>
       </c>
       <c r="AC2" t="n">
+        <v>-1.49</v>
+      </c>
+      <c r="AD2" t="n">
         <v>-0.43</v>
       </c>
-      <c r="AD2" t="n">
-        <v>-0.09</v>
-      </c>
       <c r="AE2" t="n">
-        <v>27.3</v>
+        <v>29.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.48</v>
+        <v>1.61</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.83</v>
+        <v>39.56</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.83</v>
+        <v>39.56</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.1</v>
+        <v>2.16</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>7.03</v>
+        <v>5.95</v>
       </c>
       <c r="AM2" t="n">
-        <v>17.97</v>
+        <v>16.74</v>
       </c>
       <c r="AN2" t="n">
-        <v>54.53</v>
+        <v>52.89</v>
       </c>
       <c r="AO2" t="n">
-        <v>77.7</v>
+        <v>72.62</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.86</v>
+        <v>2.75</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.77</v>
+        <v>38.28</v>
       </c>
       <c r="AR2" t="n">
-        <v>1850</v>
+        <v>1830.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>2005.34</v>
+        <v>1988.52</v>
       </c>
       <c r="AT2" t="n">
-        <v>1772.33</v>
+        <v>1751.19</v>
       </c>
       <c r="AU2" t="n">
-        <v>1850</v>
+        <v>1830.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.4</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>155.34</v>
+        <v>158.22</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.2</v>
+        <v>4.32</v>
       </c>
       <c r="BA2" t="n">
-        <v>77.67</v>
+        <v>79.11</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,55 +1987,55 @@
         <v>47.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.8</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BM2" t="n">
         <v>649</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.2</v>
+        <v>50.7</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.43</v>
+        <v>2.39</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.859999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.31</v>
+        <v>-4.29</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.265</v>
+        <v>0.261</v>
       </c>
       <c r="BT2" t="n">
-        <v>1574.65</v>
+        <v>1550.2</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.9</v>
+        <v>-13.07</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.15</v>
+        <v>2.13</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.6</v>
+        <v>47.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>57.5</v>
+        <v>56.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>73.09999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>68.34999999999999</v>
+        <v>69.98</v>
       </c>
       <c r="CO2" t="n">
-        <v>26.48</v>
+        <v>43.78</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>90.90909090909091</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>63.63636363636363</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.396800000000001</v>
+        <v>8.644500000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.576</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.28</v>
+        <v>0.288</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.0864</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0895</v>
+        <v>1.093</v>
       </c>
       <c r="DH2" t="n">
         <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.1984</v>
+        <v>4.3222</v>
       </c>
       <c r="DJ2" t="n">
-        <v>30.8</v>
+        <v>38.61</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.1984</v>
+        <v>4.3222</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2172,13 +2172,13 @@
         <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9524</v>
+        <v>0.9258999999999999</v>
       </c>
       <c r="DQ2" t="n">
-        <v>77.67</v>
+        <v>79.11</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.75</v>
+        <v>44.52</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.8381</v>
+        <v>1.2731</v>
       </c>
       <c r="DX2" t="n">
-        <v>55.74999999999999</v>
+        <v>68.44999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="DZ2" t="n">
-        <v>70.121</v>
+        <v>68.857</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>36.92</v>
+        <v>32.17</v>
       </c>
       <c r="ED2" t="n">
-        <v>44.56</v>
+        <v>59.98</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.8381</v>
+        <v>1.2731</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.5</v>
+        <v>0.24</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5006</v>
+        <v>0.3479</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9985</v>
+        <v>4.0021</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0649</v>
+        <v>0.044</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7689</v>
+        <v>0.7523</v>
       </c>
       <c r="EK2" t="n">
-        <v>43.37</v>
+        <v>47.54</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>7.43</v>
+        <v>23.68</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.9637</v>
+        <v>2.9955</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0648</v>
+        <v>0.0304</v>
       </c>
       <c r="ER2" t="n">
-        <v>16.8</v>
+        <v>36</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.935499999999999</v>
+        <v>12.2184</v>
       </c>
       <c r="ET2" t="n">
-        <v>33.509</v>
+        <v>44.908</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.93</v>
+        <v>0.66</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4</v>
+        <v>1.7419</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.0784</v>
+        <v>16.5713</v>
       </c>
       <c r="EX2" t="n">
-        <v>25.85</v>
+        <v>38.5</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,41 +2284,41 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>68.95999999999999</v>
+        <v>67.64</v>
       </c>
       <c r="FC2" t="n">
-        <v>20.64</v>
+        <v>28.97</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.75</v>
+        <v>74.44</v>
       </c>
       <c r="FE2" t="n">
-        <v>55.86</v>
+        <v>58.76</v>
       </c>
       <c r="FF2" t="n">
-        <v>26.165</v>
+        <v>41.14</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.0484</v>
+        <v>22.1456</v>
       </c>
       <c r="FH2" t="n">
-        <v>60.155</v>
+        <v>62.514</v>
       </c>
       <c r="FI2" t="n">
-        <v>39.775</v>
+        <v>41.565</v>
       </c>
       <c r="FJ2" t="n">
-        <v>59.29</v>
+        <v>65.53</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="FL2" t="n">
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>57.23</v>
+        <v>64.11</v>
       </c>
       <c r="FO2" t="n">
-        <v>45.65</v>
+        <v>56.01</v>
       </c>
       <c r="FP2" t="n">
-        <v>48.1</v>
+        <v>54.73</v>
       </c>
       <c r="FQ2" t="n">
-        <v>63.68</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>68.81</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>72.7273</v>
+        <v>86.36360000000001</v>
       </c>
       <c r="FT2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,18 +2357,18 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>58.1955</v>
+        <v>64.90049999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="FY2" t="b">
         <v>0</v>
       </c>
       <c r="FZ2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GA2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260812_163946</t>
+          <t>20260813_104006</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46246.6942906041</v>
+        <v>46247.4445192844</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2465,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46246.69428240741</v>
+        <v>46247.44451388889</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.97</v>
+        <v>12.65</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
+        <v>1830.3</v>
+      </c>
+      <c r="L2" t="n">
         <v>1850</v>
       </c>
-      <c r="L2" t="n">
-        <v>1856.3</v>
-      </c>
       <c r="M2" t="n">
-        <v>1862.3</v>
+        <v>1850.1</v>
       </c>
       <c r="N2" t="n">
-        <v>1835</v>
+        <v>1820.6</v>
       </c>
       <c r="O2" t="n">
-        <v>1850</v>
+        <v>1830.3</v>
       </c>
       <c r="P2" t="n">
-        <v>1088423</v>
+        <v>505290</v>
       </c>
       <c r="Q2" t="n">
-        <v>1850</v>
+        <v>1830.3</v>
       </c>
       <c r="R2" t="n">
-        <v>2005.34</v>
+        <v>1988.52</v>
       </c>
       <c r="S2" t="n">
-        <v>1772.33</v>
+        <v>1751.19</v>
       </c>
       <c r="T2" t="n">
-        <v>8.396756756756753</v>
+        <v>8.644484510735946</v>
       </c>
       <c r="U2" t="n">
-        <v>155.3399999999999</v>
+        <v>158.22</v>
       </c>
       <c r="V2" t="n">
-        <v>4.198378378378383</v>
+        <v>4.322242255367967</v>
       </c>
       <c r="W2" t="n">
-        <v>77.67000000000007</v>
+        <v>79.1099999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999997</v>
+        <v>2.000000000000003</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.396756756756753</v>
+        <v>8.644484510735946</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.198378378378383</v>
+        <v>4.322242255367967</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0206238008639876</v>
+        <v>0.02063322985788376</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3273926890501814</v>
+        <v>0.327542369687958</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909850771828228</v>
+        <v>0.02909853027070199</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543702777602</v>
+        <v>0.04289544890610384</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.81</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-12 16:39:46.740197+05:30</t>
+          <t>2026-08-13 10:40:06.505291+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.396756756756753, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999971}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.644484510735946, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-13 11:10 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.65</v>
+        <v>12.94</v>
       </c>
       <c r="R2" t="n">
-        <v>50.06</v>
+        <v>50.48</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1850</v>
       </c>
       <c r="V2" t="n">
-        <v>1850.1</v>
+        <v>1851.7</v>
       </c>
       <c r="W2" t="n">
         <v>1820.6</v>
       </c>
       <c r="X2" t="n">
-        <v>1830.3</v>
+        <v>1851.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>1830.3</v>
+        <v>1851.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>505290</v>
+        <v>1345712</v>
       </c>
       <c r="AA2" t="n">
-        <v>2138223</v>
+        <v>2184587</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.24</v>
+        <v>0.62</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.49</v>
+        <v>0.09</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>29.5</v>
+        <v>31.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.61</v>
+        <v>1.68</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.56</v>
+        <v>38.28</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.56</v>
+        <v>38.28</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.16</v>
+        <v>2.07</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.95</v>
+        <v>6.22</v>
       </c>
       <c r="AM2" t="n">
-        <v>16.74</v>
+        <v>17.44</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.89</v>
+        <v>54.08</v>
       </c>
       <c r="AO2" t="n">
-        <v>72.62</v>
+        <v>77.84999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.75</v>
+        <v>3.95</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.28</v>
+        <v>39.51</v>
       </c>
       <c r="AR2" t="n">
-        <v>1830.3</v>
+        <v>1851.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>1988.52</v>
+        <v>2004.83</v>
       </c>
       <c r="AT2" t="n">
-        <v>1751.19</v>
+        <v>1775.14</v>
       </c>
       <c r="AU2" t="n">
-        <v>1830.300048828125</v>
+        <v>1851.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.640000000000001</v>
+        <v>8.27</v>
       </c>
       <c r="AY2" t="n">
-        <v>158.22</v>
+        <v>153.13</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.32</v>
+        <v>4.13</v>
       </c>
       <c r="BA2" t="n">
-        <v>79.11</v>
+        <v>76.56</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>33</v>
+        <v>32.9</v>
       </c>
       <c r="BE2" t="n">
         <v>310</v>
       </c>
       <c r="BF2" t="n">
-        <v>47.8</v>
+        <v>47.7</v>
       </c>
       <c r="BG2" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="BI2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="BM2" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.7</v>
+        <v>51.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.39</v>
+        <v>2.43</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.880000000000001</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.29</v>
+        <v>-4.3</v>
       </c>
       <c r="BR2" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.261</v>
+        <v>0.265</v>
       </c>
       <c r="BT2" t="n">
-        <v>1550.2</v>
+        <v>1576.67</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.07</v>
+        <v>-12.84</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.13</v>
+        <v>2.15</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>47.8</v>
+        <v>48.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>69.98</v>
+        <v>73.04000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.78</v>
+        <v>40.18</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.644500000000001</v>
+        <v>8.2697</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.576</v>
+        <v>0.5513</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.288</v>
+        <v>0.2753</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0864</v>
+        <v>0.0827</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0024</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.093</v>
+        <v>1.0701</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9952</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.3222</v>
+        <v>4.1346</v>
       </c>
       <c r="DJ2" t="n">
-        <v>38.61</v>
+        <v>34.32</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.3222</v>
+        <v>4.1346</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9952</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9952</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>2.0025</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9258999999999999</v>
+        <v>0.9674</v>
       </c>
       <c r="DQ2" t="n">
-        <v>79.11</v>
+        <v>76.56</v>
       </c>
       <c r="DR2" t="n">
-        <v>44.52</v>
+        <v>72.59</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2731</v>
+        <v>1.9082</v>
       </c>
       <c r="DX2" t="n">
-        <v>68.44999999999999</v>
+        <v>55.37500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="DZ2" t="n">
-        <v>68.857</v>
+        <v>70.45099999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>32.17</v>
+        <v>33.43</v>
       </c>
       <c r="ED2" t="n">
-        <v>59.98</v>
+        <v>38.99</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2731</v>
+        <v>1.9082</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.24</v>
+        <v>0.62</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3479</v>
+        <v>0.5111</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0021</v>
+        <v>3.995</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.044</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7523</v>
+        <v>0.7788</v>
       </c>
       <c r="EK2" t="n">
-        <v>47.54</v>
+        <v>42.41</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,44 +2243,44 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>23.68</v>
+        <v>27.94</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.9955</v>
+        <v>3.6154</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0304</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="ER2" t="n">
-        <v>36</v>
+        <v>13.3387</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.2184</v>
+        <v>11.1792</v>
       </c>
       <c r="ET2" t="n">
-        <v>44.908</v>
+        <v>45.145</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.66</v>
+        <v>2.449</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7419</v>
+        <v>1.2778</v>
       </c>
       <c r="EW2" t="n">
-        <v>16.5713</v>
+        <v>20.4074</v>
       </c>
       <c r="EX2" t="n">
-        <v>38.5</v>
+        <v>43.45</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2290,31 +2290,31 @@
         <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>67.64</v>
+        <v>68.97</v>
       </c>
       <c r="FC2" t="n">
-        <v>28.97</v>
+        <v>24.64</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.44</v>
+        <v>73.83</v>
       </c>
       <c r="FE2" t="n">
-        <v>58.76</v>
+        <v>57.725</v>
       </c>
       <c r="FF2" t="n">
-        <v>41.14</v>
+        <v>41.815</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.1456</v>
+        <v>23.7915</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.514</v>
+        <v>65.087</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.565</v>
+        <v>53.455</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.53</v>
+        <v>66.55</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,36 +2328,36 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>64.11</v>
+        <v>71.95</v>
       </c>
       <c r="FO2" t="n">
-        <v>56.01</v>
+        <v>51.13</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.73</v>
+        <v>72.72</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.40000000000001</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>78.65000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>86.36360000000001</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>64.90049999999999</v>
+        <v>73.3965</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260813_104006</t>
+          <t>20260813_164009</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46247.4445192844</v>
+        <v>46247.69455994905</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2465,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46247.44451388889</v>
+        <v>46247.69454861111</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46247</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.65</v>
+        <v>12.94</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1830.3</v>
+        <v>1851.7</v>
       </c>
       <c r="L2" t="n">
         <v>1850</v>
       </c>
       <c r="M2" t="n">
-        <v>1850.1</v>
+        <v>1851.7</v>
       </c>
       <c r="N2" t="n">
         <v>1820.6</v>
       </c>
       <c r="O2" t="n">
-        <v>1830.3</v>
+        <v>1851.7</v>
       </c>
       <c r="P2" t="n">
-        <v>505290</v>
+        <v>1345712</v>
       </c>
       <c r="Q2" t="n">
-        <v>1830.3</v>
+        <v>1851.7</v>
       </c>
       <c r="R2" t="n">
-        <v>1988.52</v>
+        <v>2004.83</v>
       </c>
       <c r="S2" t="n">
-        <v>1751.19</v>
+        <v>1775.14</v>
       </c>
       <c r="T2" t="n">
-        <v>8.644484510735946</v>
+        <v>8.269698115245443</v>
       </c>
       <c r="U2" t="n">
-        <v>158.22</v>
+        <v>153.1299999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.322242255367967</v>
+        <v>4.134579035480907</v>
       </c>
       <c r="W2" t="n">
-        <v>79.1099999999999</v>
+        <v>76.55999999999995</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000003</v>
+        <v>2.000130616509927</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.644484510735946</v>
+        <v>8.269698115245443</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.322242255367967</v>
+        <v>4.134579035480907</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02063322985788376</v>
+        <v>0.02059277388375667</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.327542369687958</v>
+        <v>0.3269001510084352</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909853027070199</v>
+        <v>0.02909835265125211</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289544890610384</v>
+        <v>0.04289543701493845</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.8</v>
+        <v>38.85</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13 10:40:06.505291+05:30</t>
+          <t>2026-08-13 16:40:10.018024+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.644484510735946, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.269698115245443, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001306165099266}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-14 05:06 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portfolio Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Holdings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Daily Monitor" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Risk Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Execution Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Performance" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Metadata" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Monitor" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="20" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.94</v>
+        <v>12.53</v>
       </c>
       <c r="R2" t="n">
-        <v>50.48</v>
+        <v>49.93</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1850</v>
+        <v>1849.9</v>
       </c>
       <c r="V2" t="n">
-        <v>1851.7</v>
+        <v>1853.2</v>
       </c>
       <c r="W2" t="n">
-        <v>1820.6</v>
+        <v>1827</v>
       </c>
       <c r="X2" t="n">
-        <v>1851.7</v>
+        <v>1828</v>
       </c>
       <c r="Y2" t="n">
-        <v>1851.7</v>
+        <v>1828</v>
       </c>
       <c r="Z2" t="n">
-        <v>1345712</v>
+        <v>397197</v>
       </c>
       <c r="AA2" t="n">
-        <v>2184587</v>
+        <v>2137162</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.62</v>
+        <v>0.19</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.09</v>
+        <v>-1.19</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="AE2" t="n">
-        <v>31.1</v>
+        <v>26.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.68</v>
+        <v>1.43</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.28</v>
+        <v>37.93</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.28</v>
+        <v>37.93</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>6.22</v>
+        <v>4.93</v>
       </c>
       <c r="AM2" t="n">
-        <v>17.44</v>
+        <v>15.98</v>
       </c>
       <c r="AN2" t="n">
-        <v>54.08</v>
+        <v>52.12</v>
       </c>
       <c r="AO2" t="n">
-        <v>77.84999999999999</v>
+        <v>71.67</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.95</v>
+        <v>2.62</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.51</v>
+        <v>37.72</v>
       </c>
       <c r="AR2" t="n">
-        <v>1851.7</v>
+        <v>1828</v>
       </c>
       <c r="AS2" t="n">
-        <v>2004.83</v>
+        <v>1979.73</v>
       </c>
       <c r="AT2" t="n">
-        <v>1775.14</v>
+        <v>1752.14</v>
       </c>
       <c r="AU2" t="n">
-        <v>1851.699951171875</v>
+        <v>1828</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.27</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>153.13</v>
+        <v>151.73</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.13</v>
+        <v>4.15</v>
       </c>
       <c r="BA2" t="n">
-        <v>76.56</v>
+        <v>75.86</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,55 +1987,55 @@
         <v>47.7</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.1</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3</v>
+        <v>1.1</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="BM2" t="n">
         <v>650</v>
       </c>
       <c r="BN2" t="n">
-        <v>51.1</v>
+        <v>50.6</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.43</v>
+        <v>2.38</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.869999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.3</v>
+        <v>-4.28</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.265</v>
+        <v>0.259</v>
       </c>
       <c r="BT2" t="n">
-        <v>1576.67</v>
+        <v>1545.58</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.84</v>
+        <v>-13.09</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.15</v>
+        <v>2.12</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
         <v>2.0001</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>48.6</v>
+        <v>47.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>57.5</v>
+        <v>56</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>73</v>
+        <v>72.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>73.04000000000001</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.18</v>
+        <v>39</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.2697</v>
+        <v>8.3003</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5513</v>
+        <v>0.5533</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2753</v>
+        <v>0.2767</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0827</v>
+        <v>0.083</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0024</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0701</v>
+        <v>1.04</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9952</v>
+        <v>3.9904</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.1346</v>
+        <v>4.1499</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.32</v>
+        <v>32.59</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.1346</v>
+        <v>4.1499</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2166,25 +2166,25 @@
         <v>1.9952</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9952</v>
+        <v>3.9904</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0025</v>
+        <v>1.9996</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9674</v>
+        <v>0.9615</v>
       </c>
       <c r="DQ2" t="n">
-        <v>76.56</v>
+        <v>75.86</v>
       </c>
       <c r="DR2" t="n">
-        <v>72.59</v>
+        <v>48.76</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.9082</v>
+        <v>1.2596</v>
       </c>
       <c r="DX2" t="n">
-        <v>55.37500000000001</v>
+        <v>70.82499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>31</v>
+        <v>9.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>70.45099999999999</v>
+        <v>66.245</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>33.43</v>
+        <v>29.78</v>
       </c>
       <c r="ED2" t="n">
-        <v>38.99</v>
+        <v>63.59</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.9082</v>
+        <v>1.2596</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.62</v>
+        <v>0.19</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5111</v>
+        <v>0.3283</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.995</v>
+        <v>3.9905</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.0411</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7788</v>
+        <v>0.7749</v>
       </c>
       <c r="EK2" t="n">
-        <v>42.41</v>
+        <v>40.13</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2249,72 @@
         <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>27.94</v>
+        <v>6.53</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.6154</v>
+        <v>0.8182</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.0238</v>
       </c>
       <c r="ER2" t="n">
-        <v>13.3387</v>
+        <v>43.6842</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.1792</v>
+        <v>10.5812</v>
       </c>
       <c r="ET2" t="n">
-        <v>45.145</v>
+        <v>37.686</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.449</v>
+        <v>0.4978</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2778</v>
+        <v>1.7479</v>
       </c>
       <c r="EW2" t="n">
-        <v>20.4074</v>
+        <v>4.2909</v>
       </c>
       <c r="EX2" t="n">
-        <v>43.45</v>
+        <v>25.68</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="FB2" t="n">
-        <v>68.97</v>
+        <v>67.09</v>
       </c>
       <c r="FC2" t="n">
-        <v>24.64</v>
+        <v>23.71</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.83</v>
+        <v>74.27</v>
       </c>
       <c r="FE2" t="n">
-        <v>57.725</v>
+        <v>52.92</v>
       </c>
       <c r="FF2" t="n">
-        <v>41.815</v>
+        <v>32.34</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.7915</v>
+        <v>21.3344</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.087</v>
+        <v>58.394</v>
       </c>
       <c r="FI2" t="n">
-        <v>53.455</v>
+        <v>40.675</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.55</v>
+        <v>63.88</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,50 +2328,50 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.95</v>
+        <v>59.29</v>
       </c>
       <c r="FO2" t="n">
-        <v>51.13</v>
+        <v>53.7</v>
       </c>
       <c r="FP2" t="n">
-        <v>72.72</v>
+        <v>44.74</v>
       </c>
       <c r="FQ2" t="n">
-        <v>79.59999999999999</v>
+        <v>61.53</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.09999999999999</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>72.7273</v>
       </c>
       <c r="FT2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>73.3965</v>
+        <v>57.6935</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260813_164009</t>
+          <t>20260814_103620</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46247.69455994905</v>
+        <v>46248.44190410954</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2465,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46247.69454861111</v>
+        <v>46248.44189814815</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.94</v>
+        <v>12.53</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1851.7</v>
+        <v>1828</v>
       </c>
       <c r="L2" t="n">
-        <v>1850</v>
+        <v>1849.9</v>
       </c>
       <c r="M2" t="n">
-        <v>1851.7</v>
+        <v>1853.2</v>
       </c>
       <c r="N2" t="n">
-        <v>1820.6</v>
+        <v>1827</v>
       </c>
       <c r="O2" t="n">
-        <v>1851.7</v>
+        <v>1828</v>
       </c>
       <c r="P2" t="n">
-        <v>1345712</v>
+        <v>397197</v>
       </c>
       <c r="Q2" t="n">
-        <v>1851.7</v>
+        <v>1828</v>
       </c>
       <c r="R2" t="n">
-        <v>2004.83</v>
+        <v>1979.73</v>
       </c>
       <c r="S2" t="n">
-        <v>1775.14</v>
+        <v>1752.14</v>
       </c>
       <c r="T2" t="n">
-        <v>8.269698115245443</v>
+        <v>8.300328227571118</v>
       </c>
       <c r="U2" t="n">
-        <v>153.1299999999999</v>
+        <v>151.73</v>
       </c>
       <c r="V2" t="n">
-        <v>4.134579035480907</v>
+        <v>4.149890590809623</v>
       </c>
       <c r="W2" t="n">
-        <v>76.55999999999995</v>
+        <v>75.8599999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000130616509927</v>
+        <v>2.00013182177696</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.269698115245443</v>
+        <v>8.300328227571118</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.134579035480907</v>
+        <v>4.149890590809623</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02059277388375667</v>
+        <v>0.02061591576048027</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3269001510084352</v>
+        <v>0.3272675169125271</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909835265125211</v>
+        <v>0.0290984710642187</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543701493845</v>
+        <v>0.04289543230181916</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.85</v>
+        <v>38.82</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13 16:40:10.018024+05:30</t>
+          <t>2026-08-14 10:36:20.541096+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.269698115245443, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001306165099266}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.300328227571118, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001318217769604}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-14 11:07 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1818,9 +1818,7 @@
       <c r="D2" s="1" t="n">
         <v>46248</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>46248</v>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
@@ -1849,31 +1847,27 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>WATCH</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.53</v>
+        <v>11.95</v>
       </c>
       <c r="R2" t="n">
-        <v>49.93</v>
+        <v>49.51</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
         <v>1849.9</v>
       </c>
@@ -1881,43 +1875,43 @@
         <v>1853.2</v>
       </c>
       <c r="W2" t="n">
-        <v>1827</v>
+        <v>1777.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1828</v>
+        <v>1787.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1828</v>
+        <v>1787.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>397197</v>
+        <v>1579823</v>
       </c>
       <c r="AA2" t="n">
-        <v>2137162</v>
+        <v>2196293</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.19</v>
+        <v>0.72</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.19</v>
+        <v>-3.39</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.01</v>
       </c>
       <c r="AE2" t="n">
-        <v>26.2</v>
+        <v>75.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.43</v>
+        <v>4.22</v>
       </c>
       <c r="AG2" t="n">
-        <v>37.93</v>
+        <v>41.45</v>
       </c>
       <c r="AH2" t="n">
-        <v>37.93</v>
+        <v>41.45</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.08</v>
+        <v>2.32</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.93</v>
+        <v>2.72</v>
       </c>
       <c r="AM2" t="n">
-        <v>15.98</v>
+        <v>13.45</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.12</v>
+        <v>48.76</v>
       </c>
       <c r="AO2" t="n">
-        <v>71.67</v>
+        <v>62.68</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.62</v>
+        <v>0.34</v>
       </c>
       <c r="AQ2" t="n">
-        <v>37.72</v>
+        <v>34.66</v>
       </c>
       <c r="AR2" t="n">
-        <v>1828</v>
+        <v>1787.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>1979.73</v>
+        <v>1953.11</v>
       </c>
       <c r="AT2" t="n">
-        <v>1752.14</v>
+        <v>1704.39</v>
       </c>
       <c r="AU2" t="n">
-        <v>1828</v>
+        <v>1787.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.300000000000001</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>151.73</v>
+        <v>165.81</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.15</v>
+        <v>4.64</v>
       </c>
       <c r="BA2" t="n">
-        <v>75.86</v>
+        <v>82.91</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -1981,64 +1975,64 @@
         <v>32.9</v>
       </c>
       <c r="BE2" t="n">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="BF2" t="n">
-        <v>47.7</v>
+        <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>17.7</v>
       </c>
       <c r="BI2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
         <v>650</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.6</v>
+        <v>50</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.38</v>
+        <v>2.29</v>
       </c>
       <c r="BP2" t="n">
         <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.28</v>
+        <v>-4.3</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="BT2" t="n">
-        <v>1545.58</v>
+        <v>1489.23</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.09</v>
+        <v>-13.52</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.12</v>
+        <v>2.07</v>
       </c>
       <c r="BW2" t="n">
         <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2052,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>47.6</v>
+        <v>45.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>56</v>
+        <v>53.5</v>
       </c>
       <c r="CF2" t="n">
         <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>65.70999999999999</v>
+        <v>64.39</v>
       </c>
       <c r="CO2" t="n">
-        <v>39</v>
+        <v>44.64</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2109,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.3003</v>
+        <v>9.277100000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2127,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5533</v>
+        <v>0.6187</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2767</v>
+        <v>0.3093</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.083</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.04</v>
+        <v>1.109</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9904</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.1499</v>
+        <v>4.6388</v>
       </c>
       <c r="DJ2" t="n">
-        <v>32.59</v>
+        <v>46.5</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.1499</v>
+        <v>4.6388</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9952</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9904</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9996</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9615</v>
+        <v>0.8621</v>
       </c>
       <c r="DQ2" t="n">
-        <v>75.86</v>
+        <v>82.91</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.76</v>
+        <v>53.16</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,90 +2187,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2596</v>
+        <v>0.1466</v>
       </c>
       <c r="DX2" t="n">
-        <v>70.82499999999999</v>
+        <v>93.3</v>
       </c>
       <c r="DY2" t="n">
-        <v>9.5</v>
+        <v>36</v>
       </c>
       <c r="DZ2" t="n">
-        <v>66.245</v>
+        <v>60.544</v>
       </c>
       <c r="EA2" t="n">
+        <v>3</v>
+      </c>
+      <c r="EB2" t="n">
+        <v>6</v>
+      </c>
+      <c r="EC2" t="n">
+        <v>15.89</v>
+      </c>
+      <c r="ED2" t="n">
+        <v>94.53</v>
+      </c>
+      <c r="EE2" t="n">
+        <v>0.1466</v>
+      </c>
+      <c r="EF2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="EG2" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="EH2" t="n">
+        <v>3.9988</v>
+      </c>
+      <c r="EI2" t="n">
+        <v>0.0049</v>
+      </c>
+      <c r="EJ2" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="EK2" t="n">
+        <v>45.02</v>
+      </c>
+      <c r="EL2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="EM2" t="n">
         <v>4</v>
       </c>
-      <c r="EB2" t="n">
-        <v>8</v>
-      </c>
-      <c r="EC2" t="n">
-        <v>29.78</v>
-      </c>
-      <c r="ED2" t="n">
-        <v>63.59</v>
-      </c>
-      <c r="EE2" t="n">
-        <v>1.2596</v>
-      </c>
-      <c r="EF2" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="EG2" t="n">
-        <v>0.3283</v>
-      </c>
-      <c r="EH2" t="n">
-        <v>3.9905</v>
-      </c>
-      <c r="EI2" t="n">
-        <v>0.0411</v>
-      </c>
-      <c r="EJ2" t="n">
-        <v>0.7749</v>
-      </c>
-      <c r="EK2" t="n">
-        <v>40.13</v>
-      </c>
-      <c r="EL2" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="EM2" t="n">
-        <v>3</v>
-      </c>
       <c r="EN2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="EO2" t="n">
-        <v>6.53</v>
+        <v>13.61</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.8182</v>
+        <v>1.6264</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0238</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="ER2" t="n">
-        <v>43.6842</v>
+        <v>12.8889</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5812</v>
+        <v>14.006</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.686</v>
+        <v>41.262</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.4978</v>
+        <v>0.2448</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7479</v>
+        <v>1.3488</v>
       </c>
       <c r="EW2" t="n">
-        <v>4.2909</v>
+        <v>8.763500000000001</v>
       </c>
       <c r="EX2" t="n">
-        <v>25.68</v>
+        <v>35.03</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2278,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="FB2" t="n">
-        <v>67.09</v>
+        <v>64.41</v>
       </c>
       <c r="FC2" t="n">
-        <v>23.71</v>
+        <v>36.88</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.27</v>
+        <v>74.44</v>
       </c>
       <c r="FE2" t="n">
-        <v>52.92</v>
+        <v>54.705</v>
       </c>
       <c r="FF2" t="n">
-        <v>32.34</v>
+        <v>39.835</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.3344</v>
+        <v>19.3946</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.394</v>
+        <v>58.528</v>
       </c>
       <c r="FI2" t="n">
-        <v>40.675</v>
+        <v>49.83</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.88</v>
+        <v>65.54000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2322,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>59.29</v>
+        <v>64.55</v>
       </c>
       <c r="FO2" t="n">
-        <v>53.7</v>
+        <v>57.91</v>
       </c>
       <c r="FP2" t="n">
-        <v>44.74</v>
+        <v>54.11</v>
       </c>
       <c r="FQ2" t="n">
-        <v>61.53</v>
+        <v>69.45</v>
       </c>
       <c r="FR2" t="n">
-        <v>65.43000000000001</v>
+        <v>74.27</v>
       </c>
       <c r="FS2" t="n">
-        <v>72.7273</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,21 +2351,21 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>57.6935</v>
+        <v>65.19199999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260814_103620</t>
+          <t>20260814_163739</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46248.44190410954</v>
+        <v>46248.69281383184</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2464,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46248.44189814815</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46248</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46263</v>
-      </c>
+        <v>46248.6928125</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2673,15 +2663,11 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.53</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+        <v>11.95</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1828</v>
+        <v>1787.3</v>
       </c>
       <c r="L2" t="n">
         <v>1849.9</v>
@@ -2690,37 +2676,37 @@
         <v>1853.2</v>
       </c>
       <c r="N2" t="n">
-        <v>1827</v>
+        <v>1777.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1828</v>
+        <v>1787.3</v>
       </c>
       <c r="P2" t="n">
-        <v>397197</v>
+        <v>1579823</v>
       </c>
       <c r="Q2" t="n">
-        <v>1828</v>
+        <v>1787.3</v>
       </c>
       <c r="R2" t="n">
-        <v>1979.73</v>
+        <v>1953.11</v>
       </c>
       <c r="S2" t="n">
-        <v>1752.14</v>
+        <v>1704.39</v>
       </c>
       <c r="T2" t="n">
-        <v>8.300328227571118</v>
+        <v>9.277121915738821</v>
       </c>
       <c r="U2" t="n">
-        <v>151.73</v>
+        <v>165.8099999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.149890590809623</v>
+        <v>4.63884070945</v>
       </c>
       <c r="W2" t="n">
-        <v>75.8599999999999</v>
+        <v>82.90999999999985</v>
       </c>
       <c r="X2" t="n">
-        <v>2.00013182177696</v>
+        <v>1.999879387287423</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.300328227571118</v>
+        <v>9.277121915738821</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.149890590809623</v>
+        <v>4.63884070945</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02061591576048027</v>
+        <v>0.02065669322015341</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3272675169125271</v>
+        <v>0.3279148390168796</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290984710642187</v>
+        <v>0.02929225881206887</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543230181916</v>
+        <v>0.04303642623939091</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.82</v>
+        <v>38.77</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-14 10:36:20.541096+05:30</t>
+          <t>2026-08-14 16:37:39.156059+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.300328227571118, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001318217769604}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.277121915738821, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999879387287423}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-17 04:05 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46248</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46251</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46251</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1852,66 +1854,70 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.95</v>
+        <v>11.83</v>
       </c>
       <c r="R2" t="n">
-        <v>49.51</v>
+        <v>49.17</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>1849.9</v>
+        <v>1770</v>
       </c>
       <c r="V2" t="n">
-        <v>1853.2</v>
+        <v>1824</v>
       </c>
       <c r="W2" t="n">
-        <v>1777.7</v>
+        <v>1769.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1787.3</v>
+        <v>1818.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>1787.3</v>
+        <v>1818.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>1579823</v>
+        <v>357471</v>
       </c>
       <c r="AA2" t="n">
-        <v>2196293</v>
+        <v>2169193</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.72</v>
+        <v>0.16</v>
       </c>
       <c r="AC2" t="n">
-        <v>-3.39</v>
+        <v>1.75</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.01</v>
+        <v>-0.97</v>
       </c>
       <c r="AE2" t="n">
-        <v>75.5</v>
+        <v>54.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.22</v>
+        <v>3</v>
       </c>
       <c r="AG2" t="n">
-        <v>41.45</v>
+        <v>41.92</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.45</v>
+        <v>41.92</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.32</v>
+        <v>2.3</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.72</v>
+        <v>2.79</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.45</v>
+        <v>14.25</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.76</v>
+        <v>50.26</v>
       </c>
       <c r="AO2" t="n">
-        <v>62.68</v>
+        <v>65.38</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.66</v>
+        <v>33.61</v>
       </c>
       <c r="AR2" t="n">
-        <v>1787.3</v>
+        <v>1818.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>1953.11</v>
+        <v>1986.16</v>
       </c>
       <c r="AT2" t="n">
-        <v>1704.39</v>
+        <v>1734.67</v>
       </c>
       <c r="AU2" t="n">
-        <v>1787.300048828125</v>
+        <v>1818.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.279999999999999</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>165.81</v>
+        <v>167.66</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.64</v>
+        <v>4.61</v>
       </c>
       <c r="BA2" t="n">
-        <v>82.91</v>
+        <v>83.83</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -1975,10 +1981,10 @@
         <v>32.9</v>
       </c>
       <c r="BE2" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.2</v>
+        <v>49.5</v>
       </c>
       <c r="BG2" t="n">
         <v>115</v>
@@ -1987,25 +1993,25 @@
         <v>17.7</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="BN2" t="n">
-        <v>50</v>
+        <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.29</v>
+        <v>2.28</v>
       </c>
       <c r="BP2" t="n">
         <v>8.880000000000001</v>
@@ -2017,22 +2023,22 @@
         <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.25</v>
+        <v>0.248</v>
       </c>
       <c r="BT2" t="n">
-        <v>1489.23</v>
+        <v>1482.98</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.52</v>
+        <v>-13.61</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BW2" t="n">
         <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2052,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.8</v>
+        <v>45.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>53.5</v>
+        <v>53</v>
       </c>
       <c r="CF2" t="n">
         <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.40000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2082,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>64.39</v>
+        <v>71.22</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.64</v>
+        <v>57.06</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2109,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>63.63636363636363</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.277100000000001</v>
+        <v>9.2197</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6187</v>
+        <v>0.6147</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3093</v>
+        <v>0.3073</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.0922</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.109</v>
+        <v>1.0907</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0087</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6388</v>
+        <v>4.6098</v>
       </c>
       <c r="DJ2" t="n">
-        <v>46.5</v>
+        <v>52.71</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6388</v>
+        <v>4.6098</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0043</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0087</v>
       </c>
       <c r="DO2" t="n">
         <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8621</v>
+        <v>0.8696</v>
       </c>
       <c r="DQ2" t="n">
-        <v>82.91</v>
+        <v>83.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>53.16</v>
+        <v>65.75</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.1466</v>
+        <v>0.1696</v>
       </c>
       <c r="DX2" t="n">
-        <v>93.3</v>
+        <v>86.55000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="DZ2" t="n">
-        <v>60.544</v>
+        <v>68.795</v>
       </c>
       <c r="EA2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>15.89</v>
+        <v>33.91</v>
       </c>
       <c r="ED2" t="n">
-        <v>94.53</v>
+        <v>86.48</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.1466</v>
+        <v>0.1696</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.72</v>
+        <v>0.16</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.0406</v>
+        <v>0.0461</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9988</v>
+        <v>4.0086</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0049</v>
+        <v>0.0055</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.709</v>
+        <v>0.7145</v>
       </c>
       <c r="EK2" t="n">
-        <v>45.02</v>
+        <v>54.64</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,75 +2246,75 @@
         <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>13.61</v>
+        <v>36.78</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.6264</v>
+        <v>4.3511</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0189</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.8889</v>
+        <v>57.625</v>
       </c>
       <c r="ES2" t="n">
-        <v>14.006</v>
+        <v>15.9727</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.262</v>
+        <v>53.013</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.2448</v>
+        <v>0.0624</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3488</v>
+        <v>1.9828</v>
       </c>
       <c r="EW2" t="n">
-        <v>8.763500000000001</v>
+        <v>26.1947</v>
       </c>
       <c r="EX2" t="n">
-        <v>35.03</v>
+        <v>66.06</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.41</v>
+        <v>63.85</v>
       </c>
       <c r="FC2" t="n">
-        <v>36.88</v>
+        <v>42.76</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.44</v>
+        <v>74.34999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>54.705</v>
+        <v>62.93</v>
       </c>
       <c r="FF2" t="n">
-        <v>39.835</v>
+        <v>61.56</v>
       </c>
       <c r="FG2" t="n">
-        <v>19.3946</v>
+        <v>21.5818</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.528</v>
+        <v>66.503</v>
       </c>
       <c r="FI2" t="n">
-        <v>49.83</v>
+        <v>59.23</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.54000000000001</v>
+        <v>70.36</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>64.55</v>
+        <v>76.06999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.91</v>
+        <v>63.74</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.11</v>
+        <v>83.13</v>
       </c>
       <c r="FQ2" t="n">
-        <v>69.45</v>
+        <v>76.16</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.27</v>
+        <v>88.16</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.19199999999999</v>
+        <v>75.92100000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260814_163739</t>
+          <t>20260817_093540</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46248.69281383184</v>
+        <v>46251.39977175275</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2458,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46248.6928125</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46251.39976851852</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46266</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2663,50 +2673,54 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.95</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>11.83</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
-        <v>1787.3</v>
+        <v>1818.5</v>
       </c>
       <c r="L2" t="n">
-        <v>1849.9</v>
+        <v>1770</v>
       </c>
       <c r="M2" t="n">
-        <v>1853.2</v>
+        <v>1824</v>
       </c>
       <c r="N2" t="n">
-        <v>1777.7</v>
+        <v>1769.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1787.3</v>
+        <v>1818.5</v>
       </c>
       <c r="P2" t="n">
-        <v>1579823</v>
+        <v>357471</v>
       </c>
       <c r="Q2" t="n">
-        <v>1787.3</v>
+        <v>1818.5</v>
       </c>
       <c r="R2" t="n">
-        <v>1953.11</v>
+        <v>1986.16</v>
       </c>
       <c r="S2" t="n">
-        <v>1704.39</v>
+        <v>1734.67</v>
       </c>
       <c r="T2" t="n">
-        <v>9.277121915738821</v>
+        <v>9.219686554852906</v>
       </c>
       <c r="U2" t="n">
-        <v>165.8099999999999</v>
+        <v>167.6600000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.63884070945</v>
+        <v>4.609843277426447</v>
       </c>
       <c r="W2" t="n">
-        <v>82.90999999999985</v>
+        <v>83.82999999999993</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999879387287423</v>
+        <v>2.000000000000003</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.277121915738821</v>
+        <v>9.219686554852906</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.63884070945</v>
+        <v>4.609843277426447</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02065669322015341</v>
+        <v>0.02063626132348255</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3279148390168796</v>
+        <v>0.3275904927124527</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02929225881206887</v>
+        <v>0.02926637820257836</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04303642623939091</v>
+        <v>0.04306250218942306</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.77</v>
+        <v>38.79</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-14 16:37:39.156059+05:30</t>
+          <t>2026-08-17 09:35:40.318609+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.277121915738821, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999879387287423}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.219686554852906, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-17 10:46 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>11.83</v>
       </c>
       <c r="R2" t="n">
-        <v>49.17</v>
+        <v>49.41</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1769.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1818.5</v>
+        <v>1809.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>1818.5</v>
+        <v>1809.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>357471</v>
+        <v>1631744</v>
       </c>
       <c r="AA2" t="n">
-        <v>2169193</v>
+        <v>2232907</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.16</v>
+        <v>0.73</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.75</v>
+        <v>1.25</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.97</v>
@@ -1908,7 +1908,7 @@
         <v>54.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>3</v>
+        <v>3.02</v>
       </c>
       <c r="AG2" t="n">
         <v>41.92</v>
@@ -1917,7 +1917,7 @@
         <v>41.92</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.3</v>
+        <v>2.32</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.79</v>
+        <v>2.32</v>
       </c>
       <c r="AM2" t="n">
-        <v>14.25</v>
+        <v>13.71</v>
       </c>
       <c r="AN2" t="n">
-        <v>50.26</v>
+        <v>49.54</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.38</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.39</v>
+        <v>-0.09</v>
       </c>
       <c r="AQ2" t="n">
-        <v>33.61</v>
+        <v>32.96</v>
       </c>
       <c r="AR2" t="n">
-        <v>1818.5</v>
+        <v>1809.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>1986.16</v>
+        <v>1977.36</v>
       </c>
       <c r="AT2" t="n">
-        <v>1734.67</v>
+        <v>1725.87</v>
       </c>
       <c r="AU2" t="n">
-        <v>1818.5</v>
+        <v>1809.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.220000000000001</v>
+        <v>9.26</v>
       </c>
       <c r="AY2" t="n">
         <v>167.66</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.61</v>
+        <v>4.63</v>
       </c>
       <c r="BA2" t="n">
         <v>83.83</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>71.22</v>
+        <v>70.91</v>
       </c>
       <c r="CO2" t="n">
-        <v>57.06</v>
+        <v>33.08</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.2197</v>
+        <v>9.2645</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6147</v>
+        <v>0.6173</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3073</v>
+        <v>0.3087</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0922</v>
+        <v>0.0926</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0907</v>
+        <v>1.0955</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0087</v>
+        <v>3.9914</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6098</v>
+        <v>4.6323</v>
       </c>
       <c r="DJ2" t="n">
-        <v>52.71</v>
+        <v>50.18</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6098</v>
+        <v>4.6323</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0043</v>
+        <v>1.9957</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0087</v>
+        <v>3.9914</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8696</v>
+        <v>0.8621</v>
       </c>
       <c r="DQ2" t="n">
         <v>83.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>65.75</v>
+        <v>65.28</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.1696</v>
+        <v>-0.0388</v>
       </c>
       <c r="DX2" t="n">
-        <v>86.55000000000001</v>
+        <v>88.99999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>8</v>
+        <v>36.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>68.795</v>
+        <v>66.83199999999999</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="EC2" t="n">
-        <v>33.91</v>
+        <v>31.8</v>
       </c>
       <c r="ED2" t="n">
-        <v>86.48</v>
+        <v>82.26000000000001</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.1696</v>
+        <v>-0.0388</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.16</v>
+        <v>0.73</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.0461</v>
+        <v>-0.0106</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0086</v>
+        <v>3.9933</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0055</v>
+        <v>-0.0013</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7145</v>
+        <v>0.7093</v>
       </c>
       <c r="EK2" t="n">
-        <v>54.64</v>
+        <v>45.02</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,44 +2243,44 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="EO2" t="n">
-        <v>36.78</v>
+        <v>27.42</v>
       </c>
       <c r="EP2" t="n">
-        <v>4.3511</v>
+        <v>3.2438</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0189</v>
+        <v>0.0864</v>
       </c>
       <c r="ER2" t="n">
-        <v>57.625</v>
+        <v>12.6849</v>
       </c>
       <c r="ES2" t="n">
-        <v>15.9727</v>
+        <v>15.1145</v>
       </c>
       <c r="ET2" t="n">
-        <v>53.013</v>
+        <v>40.613</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.0624</v>
+        <v>-0.06569999999999999</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.9828</v>
+        <v>1.341</v>
       </c>
       <c r="EW2" t="n">
-        <v>26.1947</v>
+        <v>19.4435</v>
       </c>
       <c r="EX2" t="n">
-        <v>66.06</v>
+        <v>54.85</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2293,28 +2293,28 @@
         <v>63.85</v>
       </c>
       <c r="FC2" t="n">
-        <v>42.76</v>
+        <v>40.6</v>
       </c>
       <c r="FD2" t="n">
         <v>74.34999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>62.93</v>
+        <v>57.965</v>
       </c>
       <c r="FF2" t="n">
-        <v>61.56</v>
+        <v>43.965</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.5818</v>
+        <v>21.3584</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.503</v>
+        <v>64.16800000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>59.23</v>
+        <v>57.73</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.36</v>
+        <v>65.45999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.06999999999999</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.74</v>
+        <v>57.88</v>
       </c>
       <c r="FP2" t="n">
-        <v>83.13</v>
+        <v>71.31</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.16</v>
+        <v>78.42</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.16</v>
+        <v>83.66</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.92100000000001</v>
+        <v>72.241</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260817_093540</t>
+          <t>20260817_161642</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46251.39977175275</v>
+        <v>46251.67826597691</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46251.39976851852</v>
+        <v>46251.67826388889</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46251</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1818.5</v>
+        <v>1809.7</v>
       </c>
       <c r="L2" t="n">
         <v>1770</v>
@@ -2693,34 +2693,34 @@
         <v>1769.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1818.5</v>
+        <v>1809.7</v>
       </c>
       <c r="P2" t="n">
-        <v>357471</v>
+        <v>1631744</v>
       </c>
       <c r="Q2" t="n">
-        <v>1818.5</v>
+        <v>1809.7</v>
       </c>
       <c r="R2" t="n">
-        <v>1986.16</v>
+        <v>1977.36</v>
       </c>
       <c r="S2" t="n">
-        <v>1734.67</v>
+        <v>1725.87</v>
       </c>
       <c r="T2" t="n">
-        <v>9.219686554852906</v>
+        <v>9.264518981046574</v>
       </c>
       <c r="U2" t="n">
-        <v>167.6600000000001</v>
+        <v>167.6599999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.609843277426447</v>
+        <v>4.6322594905233</v>
       </c>
       <c r="W2" t="n">
-        <v>83.82999999999993</v>
+        <v>83.83000000000015</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000003</v>
+        <v>1.999999999999995</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.219686554852906</v>
+        <v>9.264518981046574</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.609843277426447</v>
+        <v>4.6322594905233</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02063626132348255</v>
+        <v>0.02061619503255699</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3275904927124527</v>
+        <v>0.3272719502193057</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02926637820257836</v>
+        <v>0.02924052273587874</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306250218942306</v>
+        <v>0.04306248670371647</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.79</v>
+        <v>38.82</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-17 09:35:40.318609+05:30</t>
+          <t>2026-08-17 16:16:42.209603+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.219686554852906, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.264518981046574, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999947}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-18 04:00 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.83</v>
+        <v>11.81</v>
       </c>
       <c r="R2" t="n">
-        <v>49.41</v>
+        <v>49.08</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1770</v>
+        <v>1810</v>
       </c>
       <c r="V2" t="n">
-        <v>1824</v>
+        <v>1815</v>
       </c>
       <c r="W2" t="n">
-        <v>1769.4</v>
+        <v>1803.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1809.7</v>
+        <v>1809.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>1809.7</v>
+        <v>1809.1</v>
       </c>
       <c r="Z2" t="n">
-        <v>1631744</v>
+        <v>129370</v>
       </c>
       <c r="AA2" t="n">
-        <v>2232907</v>
+        <v>2145789</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.73</v>
+        <v>0.06</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.25</v>
+        <v>-0.03</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.97</v>
+        <v>0.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>54.6</v>
+        <v>11.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.02</v>
+        <v>0.64</v>
       </c>
       <c r="AG2" t="n">
-        <v>41.92</v>
+        <v>39.74</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.92</v>
+        <v>39.74</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.32</v>
+        <v>2.2</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.32</v>
+        <v>1.67</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.71</v>
+        <v>13.12</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.54</v>
+        <v>48.97</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.40000000000001</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>-0.09</v>
+        <v>-2.21</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.96</v>
+        <v>33.91</v>
       </c>
       <c r="AR2" t="n">
-        <v>1809.7</v>
+        <v>1809.1</v>
       </c>
       <c r="AS2" t="n">
-        <v>1977.36</v>
+        <v>1968.07</v>
       </c>
       <c r="AT2" t="n">
-        <v>1725.87</v>
+        <v>1729.61</v>
       </c>
       <c r="AU2" t="n">
-        <v>1809.699951171875</v>
+        <v>1809.099975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.26</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>167.66</v>
+        <v>158.97</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.63</v>
+        <v>4.39</v>
       </c>
       <c r="BA2" t="n">
-        <v>83.83</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -1978,46 +1978,46 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.9</v>
+        <v>32.8</v>
       </c>
       <c r="BE2" t="n">
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.5</v>
+        <v>49.4</v>
       </c>
       <c r="BG2" t="n">
         <v>115</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.9</v>
+        <v>49.8</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="BP2" t="n">
         <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.3</v>
+        <v>-4.29</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
@@ -2026,10 +2026,10 @@
         <v>0.248</v>
       </c>
       <c r="BT2" t="n">
-        <v>1482.98</v>
+        <v>1482.73</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.61</v>
+        <v>-13.63</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
@@ -2038,7 +2038,7 @@
         <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.6</v>
+        <v>45.4</v>
       </c>
       <c r="CE2" t="n">
         <v>53</v>
@@ -2067,7 +2067,7 @@
         <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>70.91</v>
+        <v>60.49</v>
       </c>
       <c r="CO2" t="n">
-        <v>33.08</v>
+        <v>39.91</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>90.90909090909091</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.2645</v>
+        <v>8.7872</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6173</v>
+        <v>0.586</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3087</v>
+        <v>0.2927</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0926</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0023</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0955</v>
+        <v>1.0381</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9914</v>
+        <v>3.9955</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6323</v>
+        <v>4.3939</v>
       </c>
       <c r="DJ2" t="n">
-        <v>50.18</v>
+        <v>48.94</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6323</v>
+        <v>4.3939</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9957</v>
+        <v>1.9955</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9914</v>
+        <v>3.9955</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>2.002</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8621</v>
+        <v>0.9101</v>
       </c>
       <c r="DQ2" t="n">
-        <v>83.83</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>65.28</v>
+        <v>68.53</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,128 +2193,128 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.0388</v>
+        <v>-1.0045</v>
       </c>
       <c r="DX2" t="n">
-        <v>88.99999999999999</v>
+        <v>89.34999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>36.5</v>
+        <v>3</v>
       </c>
       <c r="DZ2" t="n">
-        <v>66.83199999999999</v>
+        <v>60.87</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="EB2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="EC2" t="n">
-        <v>31.8</v>
+        <v>17.08</v>
       </c>
       <c r="ED2" t="n">
-        <v>82.26000000000001</v>
+        <v>87</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.0388</v>
+        <v>-1.0045</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.73</v>
+        <v>0.06</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.0106</v>
+        <v>-0.261</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9933</v>
+        <v>3.9942</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0013</v>
+        <v>-0.0308</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7093</v>
+        <v>0.741</v>
       </c>
       <c r="EK2" t="n">
-        <v>45.02</v>
+        <v>34.94</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EM2" t="n">
         <v>3</v>
       </c>
       <c r="EN2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="EO2" t="n">
-        <v>27.42</v>
+        <v>11.16</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.2438</v>
+        <v>1.318</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0864</v>
+        <v>0.0071</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.6849</v>
+        <v>146.5</v>
       </c>
       <c r="ES2" t="n">
-        <v>15.1145</v>
+        <v>15.2938</v>
       </c>
       <c r="ET2" t="n">
-        <v>40.613</v>
+        <v>38.437</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.06569999999999999</v>
+        <v>-0.1326</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.341</v>
+        <v>2.0755</v>
       </c>
       <c r="EW2" t="n">
-        <v>19.4435</v>
+        <v>6.7507</v>
       </c>
       <c r="EX2" t="n">
-        <v>54.85</v>
+        <v>34.51</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.85</v>
+        <v>63.75</v>
       </c>
       <c r="FC2" t="n">
-        <v>40.6</v>
+        <v>39.45</v>
       </c>
       <c r="FD2" t="n">
         <v>74.34999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>57.965</v>
+        <v>47.715</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.965</v>
+        <v>37.21</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.3584</v>
+        <v>18.9031</v>
       </c>
       <c r="FH2" t="n">
-        <v>64.16800000000001</v>
+        <v>56.924</v>
       </c>
       <c r="FI2" t="n">
-        <v>57.73</v>
+        <v>58.735</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.45999999999999</v>
+        <v>62.1</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,36 +2328,36 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>72.43000000000001</v>
+        <v>67.91</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.88</v>
+        <v>50.25</v>
       </c>
       <c r="FP2" t="n">
-        <v>71.31</v>
+        <v>64.42</v>
       </c>
       <c r="FQ2" t="n">
-        <v>78.42</v>
+        <v>81.23</v>
       </c>
       <c r="FR2" t="n">
-        <v>83.66</v>
+        <v>75.02</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>81.8182</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.241</v>
+        <v>67.5505</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260817_161642</t>
+          <t>20260818_093043</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46251.67826597691</v>
+        <v>46252.39633125019</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46251.67826388889</v>
+        <v>46252.39633101852</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.83</v>
+        <v>11.81</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1809.7</v>
+        <v>1809.1</v>
       </c>
       <c r="L2" t="n">
-        <v>1770</v>
+        <v>1810</v>
       </c>
       <c r="M2" t="n">
-        <v>1824</v>
+        <v>1815</v>
       </c>
       <c r="N2" t="n">
-        <v>1769.4</v>
+        <v>1803.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1809.7</v>
+        <v>1809.1</v>
       </c>
       <c r="P2" t="n">
-        <v>1631744</v>
+        <v>129370</v>
       </c>
       <c r="Q2" t="n">
-        <v>1809.7</v>
+        <v>1809.1</v>
       </c>
       <c r="R2" t="n">
-        <v>1977.36</v>
+        <v>1968.07</v>
       </c>
       <c r="S2" t="n">
-        <v>1725.87</v>
+        <v>1729.61</v>
       </c>
       <c r="T2" t="n">
-        <v>9.264518981046574</v>
+        <v>8.787242275164449</v>
       </c>
       <c r="U2" t="n">
-        <v>167.6599999999999</v>
+        <v>158.97</v>
       </c>
       <c r="V2" t="n">
-        <v>4.6322594905233</v>
+        <v>4.393897518102925</v>
       </c>
       <c r="W2" t="n">
-        <v>83.83000000000015</v>
+        <v>79.49000000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999995</v>
+        <v>1.999874198012329</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.264518981046574</v>
+        <v>8.787242275164449</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.6322594905233</v>
+        <v>4.393897518102925</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02061619503255699</v>
+        <v>0.02061287173036461</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3272719502193057</v>
+        <v>0.3272191944325104</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02924052273587874</v>
+        <v>0.0292405918785871</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306248670371647</v>
+        <v>0.0430625089637657</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-17 16:16:42.209603+05:30</t>
+          <t>2026-08-18 09:30:43.058321+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.264518981046574, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999947}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.787242275164449, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998741980123287}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-18 10:44 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.81</v>
+        <v>11.85</v>
       </c>
       <c r="R2" t="n">
-        <v>49.08</v>
+        <v>49.3</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1810</v>
       </c>
       <c r="V2" t="n">
-        <v>1815</v>
+        <v>1824.6</v>
       </c>
       <c r="W2" t="n">
-        <v>1803.5</v>
+        <v>1802.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1809.1</v>
+        <v>1814</v>
       </c>
       <c r="Y2" t="n">
-        <v>1809.1</v>
+        <v>1814</v>
       </c>
       <c r="Z2" t="n">
-        <v>129370</v>
+        <v>1291687</v>
       </c>
       <c r="AA2" t="n">
-        <v>2145789</v>
+        <v>2203905</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.06</v>
+        <v>0.59</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.03</v>
+        <v>0.24</v>
       </c>
       <c r="AD2" t="n">
         <v>0.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.5</v>
+        <v>22.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.64</v>
+        <v>1.24</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.74</v>
+        <v>40.53</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.74</v>
+        <v>40.53</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.2</v>
+        <v>2.23</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.67</v>
+        <v>1.93</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.12</v>
+        <v>13.42</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.97</v>
+        <v>49.38</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.26000000000001</v>
+        <v>64.92</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.21</v>
+        <v>-1.95</v>
       </c>
       <c r="AQ2" t="n">
-        <v>33.91</v>
+        <v>34.27</v>
       </c>
       <c r="AR2" t="n">
-        <v>1809.1</v>
+        <v>1814</v>
       </c>
       <c r="AS2" t="n">
-        <v>1968.07</v>
+        <v>1976.12</v>
       </c>
       <c r="AT2" t="n">
-        <v>1729.61</v>
+        <v>1732.94</v>
       </c>
       <c r="AU2" t="n">
-        <v>1809.099975585938</v>
+        <v>1814</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.789999999999999</v>
+        <v>8.94</v>
       </c>
       <c r="AY2" t="n">
-        <v>158.97</v>
+        <v>162.12</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.39</v>
+        <v>4.47</v>
       </c>
       <c r="BA2" t="n">
-        <v>79.48999999999999</v>
+        <v>81.06</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,37 +1987,37 @@
         <v>49.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
         <v>652</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.8</v>
+        <v>50</v>
       </c>
       <c r="BO2" t="n">
         <v>2.27</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.880000000000001</v>
+        <v>8.85</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.29</v>
+        <v>-4.3</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
@@ -2026,19 +2026,19 @@
         <v>0.248</v>
       </c>
       <c r="BT2" t="n">
-        <v>1482.73</v>
+        <v>1482.99</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.63</v>
+        <v>-13.6</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2064,10 +2064,10 @@
         <v>53</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.09999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>60.49</v>
+        <v>69.61</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.91</v>
+        <v>32.03</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>90.90909090909091</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.7872</v>
+        <v>8.937200000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.586</v>
+        <v>0.596</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2927</v>
+        <v>0.298</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0023</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0381</v>
+        <v>1.0594</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9955</v>
+        <v>4.009</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.3939</v>
+        <v>4.4686</v>
       </c>
       <c r="DJ2" t="n">
-        <v>48.94</v>
+        <v>44.51</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.3939</v>
+        <v>4.4686</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9955</v>
+        <v>2.0045</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9955</v>
+        <v>4.009</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.002</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9101</v>
+        <v>0.8969</v>
       </c>
       <c r="DQ2" t="n">
-        <v>79.48999999999999</v>
+        <v>81.06</v>
       </c>
       <c r="DR2" t="n">
-        <v>68.53</v>
+        <v>60.53</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-1.0045</v>
+        <v>-0.8744</v>
       </c>
       <c r="DX2" t="n">
-        <v>89.34999999999999</v>
+        <v>87.69999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>3</v>
+        <v>29.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>60.87</v>
+        <v>66.98</v>
       </c>
       <c r="EA2" t="n">
         <v>3</v>
@@ -2211,110 +2211,110 @@
         <v>6</v>
       </c>
       <c r="EC2" t="n">
-        <v>17.08</v>
+        <v>27.87</v>
       </c>
       <c r="ED2" t="n">
-        <v>87</v>
+        <v>85.63</v>
       </c>
       <c r="EE2" t="n">
-        <v>-1.0045</v>
+        <v>-0.8744</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.06</v>
+        <v>0.59</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.261</v>
+        <v>-0.2311</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9942</v>
+        <v>4.0077</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0308</v>
+        <v>-0.0274</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.741</v>
+        <v>0.7327</v>
       </c>
       <c r="EK2" t="n">
-        <v>34.94</v>
+        <v>52.29</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
+        <v>8</v>
+      </c>
+      <c r="EO2" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="EP2" t="n">
+        <v>3.9567</v>
+      </c>
+      <c r="EQ2" t="n">
+        <v>0.0699</v>
+      </c>
+      <c r="ER2" t="n">
+        <v>15.1525</v>
+      </c>
+      <c r="ES2" t="n">
+        <v>13.7802</v>
+      </c>
+      <c r="ET2" t="n">
+        <v>42.011</v>
+      </c>
+      <c r="EU2" t="n">
+        <v>-1.1505</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>1.4025</v>
+      </c>
+      <c r="EW2" t="n">
+        <v>23.2428</v>
+      </c>
+      <c r="EX2" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="EY2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="EZ2" t="n">
         <v>5</v>
       </c>
-      <c r="EO2" t="n">
-        <v>11.16</v>
-      </c>
-      <c r="EP2" t="n">
-        <v>1.318</v>
-      </c>
-      <c r="EQ2" t="n">
-        <v>0.0071</v>
-      </c>
-      <c r="ER2" t="n">
-        <v>146.5</v>
-      </c>
-      <c r="ES2" t="n">
-        <v>15.2938</v>
-      </c>
-      <c r="ET2" t="n">
-        <v>38.437</v>
-      </c>
-      <c r="EU2" t="n">
-        <v>-0.1326</v>
-      </c>
-      <c r="EV2" t="n">
-        <v>2.0755</v>
-      </c>
-      <c r="EW2" t="n">
-        <v>6.7507</v>
-      </c>
-      <c r="EX2" t="n">
-        <v>34.51</v>
-      </c>
-      <c r="EY2" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="EZ2" t="n">
-        <v>4</v>
-      </c>
       <c r="FA2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.75</v>
+        <v>63.94</v>
       </c>
       <c r="FC2" t="n">
-        <v>39.45</v>
+        <v>35.44</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.34999999999999</v>
+        <v>73.75</v>
       </c>
       <c r="FE2" t="n">
-        <v>47.715</v>
+        <v>60.95</v>
       </c>
       <c r="FF2" t="n">
-        <v>37.21</v>
+        <v>39.77</v>
       </c>
       <c r="FG2" t="n">
-        <v>18.9031</v>
+        <v>21.5511</v>
       </c>
       <c r="FH2" t="n">
-        <v>56.924</v>
+        <v>62.355</v>
       </c>
       <c r="FI2" t="n">
-        <v>58.735</v>
+        <v>52.52</v>
       </c>
       <c r="FJ2" t="n">
-        <v>62.1</v>
+        <v>63.95</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>67.91</v>
+        <v>67.81</v>
       </c>
       <c r="FO2" t="n">
-        <v>50.25</v>
+        <v>57.66</v>
       </c>
       <c r="FP2" t="n">
-        <v>64.42</v>
+        <v>62.8</v>
       </c>
       <c r="FQ2" t="n">
-        <v>81.23</v>
+        <v>69.97</v>
       </c>
       <c r="FR2" t="n">
-        <v>75.02</v>
+        <v>79.25</v>
       </c>
       <c r="FS2" t="n">
-        <v>81.8182</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.5505</v>
+        <v>68.17100000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260818_093043</t>
+          <t>20260818_161417</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46252.39633125019</v>
+        <v>46252.67658931954</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46252.39633101852</v>
+        <v>46252.67658564815</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46252</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.81</v>
+        <v>11.85</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1809.1</v>
+        <v>1814</v>
       </c>
       <c r="L2" t="n">
         <v>1810</v>
       </c>
       <c r="M2" t="n">
-        <v>1815</v>
+        <v>1824.6</v>
       </c>
       <c r="N2" t="n">
-        <v>1803.5</v>
+        <v>1802.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1809.1</v>
+        <v>1814</v>
       </c>
       <c r="P2" t="n">
-        <v>129370</v>
+        <v>1291687</v>
       </c>
       <c r="Q2" t="n">
-        <v>1809.1</v>
+        <v>1814</v>
       </c>
       <c r="R2" t="n">
-        <v>1968.07</v>
+        <v>1976.12</v>
       </c>
       <c r="S2" t="n">
-        <v>1729.61</v>
+        <v>1732.94</v>
       </c>
       <c r="T2" t="n">
-        <v>8.787242275164449</v>
+        <v>8.937155457552365</v>
       </c>
       <c r="U2" t="n">
-        <v>158.97</v>
+        <v>162.1199999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.393897518102925</v>
+        <v>4.468577728776182</v>
       </c>
       <c r="W2" t="n">
-        <v>79.49000000000001</v>
+        <v>81.05999999999995</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999874198012329</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.787242275164449</v>
+        <v>8.937155457552365</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.393897518102925</v>
+        <v>4.468577728776182</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02061287173036461</v>
+        <v>0.02058107225176457</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3272191944325104</v>
+        <v>0.3267143933593271</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0292405918785871</v>
+        <v>0.02909835265125211</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0430625089637657</v>
+        <v>0.04289543264576713</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.82</v>
+        <v>38.86</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-18 09:30:43.058321+05:30</t>
+          <t>2026-08-18 16:14:17.353298+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.787242275164449, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998741980123287}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.937155457552365, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-19 04:02 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.85</v>
+        <v>11.76</v>
       </c>
       <c r="R2" t="n">
-        <v>49.3</v>
+        <v>49.09</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1810</v>
+        <v>1814</v>
       </c>
       <c r="V2" t="n">
-        <v>1824.6</v>
+        <v>1818</v>
       </c>
       <c r="W2" t="n">
-        <v>1802.1</v>
+        <v>1802.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1814</v>
+        <v>1803</v>
       </c>
       <c r="Y2" t="n">
-        <v>1814</v>
+        <v>1803</v>
       </c>
       <c r="Z2" t="n">
-        <v>1291687</v>
+        <v>177707</v>
       </c>
       <c r="AA2" t="n">
-        <v>2203905</v>
+        <v>2153648</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.59</v>
+        <v>0.08</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.24</v>
+        <v>-0.61</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>22.5</v>
+        <v>15.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.24</v>
+        <v>0.86</v>
       </c>
       <c r="AG2" t="n">
-        <v>40.53</v>
+        <v>38.74</v>
       </c>
       <c r="AH2" t="n">
-        <v>40.53</v>
+        <v>38.74</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.23</v>
+        <v>2.15</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.93</v>
+        <v>0.67</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.42</v>
+        <v>12.15</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.38</v>
+        <v>47.95</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.92</v>
+        <v>62.38</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.95</v>
+        <v>-1.74</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.27</v>
+        <v>34.2</v>
       </c>
       <c r="AR2" t="n">
-        <v>1814</v>
+        <v>1803</v>
       </c>
       <c r="AS2" t="n">
-        <v>1976.12</v>
+        <v>1957.97</v>
       </c>
       <c r="AT2" t="n">
-        <v>1732.94</v>
+        <v>1725.52</v>
       </c>
       <c r="AU2" t="n">
-        <v>1814</v>
+        <v>1803</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.94</v>
+        <v>8.6</v>
       </c>
       <c r="AY2" t="n">
-        <v>162.12</v>
+        <v>154.97</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.47</v>
+        <v>4.3</v>
       </c>
       <c r="BA2" t="n">
-        <v>81.06</v>
+        <v>77.48</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,61 +1984,61 @@
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.4</v>
+        <v>49.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BM2" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="BN2" t="n">
-        <v>50</v>
+        <v>49.8</v>
       </c>
       <c r="BO2" t="n">
         <v>2.27</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.85</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.3</v>
+        <v>-4.28</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.248</v>
+        <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1482.99</v>
+        <v>1481.57</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.6</v>
+        <v>-13.75</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2064,10 +2064,10 @@
         <v>53</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>69.61</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>32.03</v>
+        <v>33.88</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>90.90909090909091</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.937200000000001</v>
+        <v>8.5951</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.596</v>
+        <v>0.5733</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.298</v>
+        <v>0.2867</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0594</v>
+        <v>1.0114</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.009</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.4686</v>
+        <v>4.2973</v>
       </c>
       <c r="DJ2" t="n">
-        <v>44.51</v>
+        <v>37.02</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.4686</v>
+        <v>4.2973</v>
       </c>
       <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2.0045</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.009</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8969</v>
+        <v>0.9302</v>
       </c>
       <c r="DQ2" t="n">
-        <v>81.06</v>
+        <v>77.48</v>
       </c>
       <c r="DR2" t="n">
-        <v>60.53</v>
+        <v>49.94</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.8744</v>
+        <v>-0.8093</v>
       </c>
       <c r="DX2" t="n">
-        <v>87.69999999999999</v>
+        <v>94.05</v>
       </c>
       <c r="DY2" t="n">
-        <v>29.5</v>
+        <v>4</v>
       </c>
       <c r="DZ2" t="n">
-        <v>66.98</v>
+        <v>67.108</v>
       </c>
       <c r="EA2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="EC2" t="n">
-        <v>27.87</v>
+        <v>34.17</v>
       </c>
       <c r="ED2" t="n">
-        <v>85.63</v>
+        <v>98.11</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.8744</v>
+        <v>-0.8093</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.59</v>
+        <v>0.08</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2311</v>
+        <v>-0.2046</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0077</v>
+        <v>3.9977</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0274</v>
+        <v>-0.0241</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7327</v>
+        <v>0.7543</v>
       </c>
       <c r="EK2" t="n">
-        <v>52.29</v>
+        <v>47.64</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2249,72 @@
         <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>33.39</v>
+        <v>6.09</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.9567</v>
+        <v>0.7161999999999999</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0699</v>
+        <v>0.0094</v>
       </c>
       <c r="ER2" t="n">
-        <v>15.1525</v>
+        <v>107.5</v>
       </c>
       <c r="ES2" t="n">
-        <v>13.7802</v>
+        <v>11.7524</v>
       </c>
       <c r="ET2" t="n">
-        <v>42.011</v>
+        <v>34.435</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.1505</v>
+        <v>-0.1392</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4025</v>
+        <v>1.9907</v>
       </c>
       <c r="EW2" t="n">
-        <v>23.2428</v>
+        <v>3.8982</v>
       </c>
       <c r="EX2" t="n">
-        <v>47.51</v>
+        <v>25.32</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.94</v>
+        <v>63.52</v>
       </c>
       <c r="FC2" t="n">
-        <v>35.44</v>
+        <v>29.45</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.75</v>
+        <v>74.34999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>60.95</v>
+        <v>55.825</v>
       </c>
       <c r="FF2" t="n">
-        <v>39.77</v>
+        <v>29.6</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.5511</v>
+        <v>20.3206</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.355</v>
+        <v>56.027</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.52</v>
+        <v>43.48</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.95</v>
+        <v>62.99</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>67.81</v>
+        <v>63.77</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.66</v>
+        <v>55.89</v>
       </c>
       <c r="FP2" t="n">
-        <v>62.8</v>
+        <v>46.98</v>
       </c>
       <c r="FQ2" t="n">
-        <v>69.97</v>
+        <v>68.48</v>
       </c>
       <c r="FR2" t="n">
-        <v>79.25</v>
+        <v>76.43000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.17100000000001</v>
+        <v>63.857</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260818_161417</t>
+          <t>20260819_093220</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46252.67658931954</v>
+        <v>46253.39746125175</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46252.67658564815</v>
+        <v>46253.39745370371</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.85</v>
+        <v>11.76</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
+        <v>1803</v>
+      </c>
+      <c r="L2" t="n">
         <v>1814</v>
       </c>
-      <c r="L2" t="n">
-        <v>1810</v>
-      </c>
       <c r="M2" t="n">
-        <v>1824.6</v>
+        <v>1818</v>
       </c>
       <c r="N2" t="n">
-        <v>1802.1</v>
+        <v>1802.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1814</v>
+        <v>1803</v>
       </c>
       <c r="P2" t="n">
-        <v>1291687</v>
+        <v>177707</v>
       </c>
       <c r="Q2" t="n">
-        <v>1814</v>
+        <v>1803</v>
       </c>
       <c r="R2" t="n">
-        <v>1976.12</v>
+        <v>1957.97</v>
       </c>
       <c r="S2" t="n">
-        <v>1732.94</v>
+        <v>1725.52</v>
       </c>
       <c r="T2" t="n">
-        <v>8.937155457552365</v>
+        <v>8.595119245701611</v>
       </c>
       <c r="U2" t="n">
-        <v>162.1199999999999</v>
+        <v>154.97</v>
       </c>
       <c r="V2" t="n">
-        <v>4.468577728776182</v>
+        <v>4.297282307265669</v>
       </c>
       <c r="W2" t="n">
-        <v>81.05999999999995</v>
+        <v>77.48000000000002</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000129065565307</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.937155457552365</v>
+        <v>8.595119245701611</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.468577728776182</v>
+        <v>4.297282307265669</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058107225176457</v>
+        <v>0.02058379841394827</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3267143933593271</v>
+        <v>0.3267576698423573</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543264576713</v>
+        <v>0.04289543414149807</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645465</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-18 16:14:17.353298+05:30</t>
+          <t>2026-08-19 09:32:20.676171+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.937155457552365, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.59511924570161, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001290655653072}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-19 10:43 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1864,7 +1864,7 @@
         <v>11.76</v>
       </c>
       <c r="R2" t="n">
-        <v>49.09</v>
+        <v>49.33</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>1818</v>
       </c>
       <c r="W2" t="n">
-        <v>1802.5</v>
+        <v>1789.9</v>
       </c>
       <c r="X2" t="n">
-        <v>1803</v>
+        <v>1801.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>1803</v>
+        <v>1801.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>177707</v>
+        <v>1426121</v>
       </c>
       <c r="AA2" t="n">
-        <v>2153648</v>
+        <v>2216069</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.08</v>
+        <v>0.64</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.61</v>
+        <v>-0.67</v>
       </c>
       <c r="AD2" t="n">
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>15.5</v>
+        <v>28.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.86</v>
+        <v>1.56</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.74</v>
+        <v>39.64</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.74</v>
+        <v>39.64</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.15</v>
+        <v>2.2</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.67</v>
+        <v>0.61</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.15</v>
+        <v>12.07</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.95</v>
+        <v>47.85</v>
       </c>
       <c r="AO2" t="n">
-        <v>62.38</v>
+        <v>62.12</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.74</v>
+        <v>-1.81</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.2</v>
+        <v>34.11</v>
       </c>
       <c r="AR2" t="n">
-        <v>1803</v>
+        <v>1801.8</v>
       </c>
       <c r="AS2" t="n">
-        <v>1957.97</v>
+        <v>1960.37</v>
       </c>
       <c r="AT2" t="n">
-        <v>1725.52</v>
+        <v>1722.52</v>
       </c>
       <c r="AU2" t="n">
-        <v>1803</v>
+        <v>1801.800048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>154.97</v>
+        <v>158.57</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="BA2" t="n">
-        <v>77.48</v>
+        <v>79.28</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -2026,10 +2026,10 @@
         <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1481.57</v>
+        <v>1481.46</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.75</v>
+        <v>-13.76</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>64.01000000000001</v>
+        <v>64.58</v>
       </c>
       <c r="CO2" t="n">
-        <v>33.88</v>
+        <v>32.02</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>63.63636363636363</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.5951</v>
+        <v>8.800599999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5733</v>
+        <v>0.5867</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2867</v>
+        <v>0.2933</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0114</v>
+        <v>1.0349</v>
       </c>
       <c r="DH2" t="n">
         <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2973</v>
+        <v>4.4</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.02</v>
+        <v>36.38</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2973</v>
+        <v>4.4</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2169,16 +2169,16 @@
         <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9302</v>
+        <v>0.9091</v>
       </c>
       <c r="DQ2" t="n">
-        <v>77.48</v>
+        <v>79.28</v>
       </c>
       <c r="DR2" t="n">
-        <v>49.94</v>
+        <v>64.95</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.8093</v>
+        <v>-0.8227</v>
       </c>
       <c r="DX2" t="n">
-        <v>94.05</v>
+        <v>94.7</v>
       </c>
       <c r="DY2" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="DZ2" t="n">
-        <v>67.108</v>
+        <v>67.283</v>
       </c>
       <c r="EA2" t="n">
         <v>4</v>
@@ -2211,31 +2211,31 @@
         <v>7</v>
       </c>
       <c r="EC2" t="n">
-        <v>34.17</v>
+        <v>32.91</v>
       </c>
       <c r="ED2" t="n">
-        <v>98.11</v>
+        <v>98.62</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.8093</v>
+        <v>-0.8227</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.08</v>
+        <v>0.64</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2046</v>
+        <v>-0.2129</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9977</v>
+        <v>4.0003</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0241</v>
+        <v>-0.025</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7543</v>
+        <v>0.7408</v>
       </c>
       <c r="EK2" t="n">
-        <v>47.64</v>
+        <v>50.99</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>6.09</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.7161999999999999</v>
+        <v>0.9455</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0094</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="ER2" t="n">
-        <v>107.5</v>
+        <v>13.75</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.7524</v>
+        <v>11.3688</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.435</v>
+        <v>34.276</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.1392</v>
+        <v>-1.1584</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.9907</v>
+        <v>1.3415</v>
       </c>
       <c r="EW2" t="n">
-        <v>3.8982</v>
+        <v>5.1922</v>
       </c>
       <c r="EX2" t="n">
-        <v>25.32</v>
+        <v>35.45</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
         <v>63.52</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.45</v>
+        <v>28.85</v>
       </c>
       <c r="FD2" t="n">
         <v>74.34999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>55.825</v>
+        <v>57.785</v>
       </c>
       <c r="FF2" t="n">
-        <v>29.6</v>
+        <v>33.735</v>
       </c>
       <c r="FG2" t="n">
-        <v>20.3206</v>
+        <v>20.1812</v>
       </c>
       <c r="FH2" t="n">
-        <v>56.027</v>
+        <v>58.224</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.48</v>
+        <v>50.665</v>
       </c>
       <c r="FJ2" t="n">
-        <v>62.99</v>
+        <v>63.19</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>63.77</v>
+        <v>69.93000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>55.89</v>
+        <v>54.67</v>
       </c>
       <c r="FP2" t="n">
-        <v>46.98</v>
+        <v>61.53</v>
       </c>
       <c r="FQ2" t="n">
-        <v>68.48</v>
+        <v>76.16</v>
       </c>
       <c r="FR2" t="n">
-        <v>76.43000000000001</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>63.857</v>
+        <v>66.4675</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260819_093220</t>
+          <t>20260819_161352</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46253.39746125175</v>
+        <v>46253.67629744824</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46253.39745370371</v>
+        <v>46253.6762962963</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46253</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1803</v>
+        <v>1801.8</v>
       </c>
       <c r="L2" t="n">
         <v>1814</v>
@@ -2690,37 +2690,37 @@
         <v>1818</v>
       </c>
       <c r="N2" t="n">
-        <v>1802.5</v>
+        <v>1789.9</v>
       </c>
       <c r="O2" t="n">
-        <v>1803</v>
+        <v>1801.8</v>
       </c>
       <c r="P2" t="n">
-        <v>177707</v>
+        <v>1426121</v>
       </c>
       <c r="Q2" t="n">
-        <v>1803</v>
+        <v>1801.8</v>
       </c>
       <c r="R2" t="n">
-        <v>1957.97</v>
+        <v>1960.37</v>
       </c>
       <c r="S2" t="n">
-        <v>1725.52</v>
+        <v>1722.52</v>
       </c>
       <c r="T2" t="n">
-        <v>8.595119245701611</v>
+        <v>8.800643800643797</v>
       </c>
       <c r="U2" t="n">
-        <v>154.97</v>
+        <v>158.5699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.297282307265669</v>
+        <v>4.400044400044399</v>
       </c>
       <c r="W2" t="n">
-        <v>77.48000000000002</v>
+        <v>79.27999999999997</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000129065565307</v>
+        <v>2.000126135216953</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.595119245701611</v>
+        <v>8.800643800643797</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.297282307265669</v>
+        <v>4.400044400044399</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058379841394827</v>
+        <v>0.02060405199033586</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3267576698423573</v>
+        <v>0.3270791854000446</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909835265125211</v>
+        <v>0.02924066102128654</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04289543414149807</v>
+        <v>0.04306250876103246</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645465</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.86</v>
+        <v>38.83</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-19 09:32:20.676171+05:30</t>
+          <t>2026-08-19 16:13:52.140153+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.59511924570161, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001290655653072}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.800643800643797, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001261352169526}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-20 04:02 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.76</v>
+        <v>11.9</v>
       </c>
       <c r="R2" t="n">
-        <v>49.33</v>
+        <v>49.09</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1814</v>
+        <v>1819</v>
       </c>
       <c r="V2" t="n">
-        <v>1818</v>
+        <v>1831.1</v>
       </c>
       <c r="W2" t="n">
-        <v>1789.9</v>
+        <v>1813.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1801.8</v>
+        <v>1826.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1801.8</v>
+        <v>1826.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1426121</v>
+        <v>246388</v>
       </c>
       <c r="AA2" t="n">
-        <v>2216069</v>
+        <v>2173488</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.64</v>
+        <v>0.11</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.67</v>
+        <v>1.35</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="AE2" t="n">
-        <v>28.1</v>
+        <v>17.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.56</v>
+        <v>0.95</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.64</v>
+        <v>38.9</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.64</v>
+        <v>38.9</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.2</v>
+        <v>2.13</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.61</v>
+        <v>1.24</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.07</v>
+        <v>12.98</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.85</v>
+        <v>49.33</v>
       </c>
       <c r="AO2" t="n">
-        <v>62.12</v>
+        <v>65.34</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.81</v>
+        <v>-0.21</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.11</v>
+        <v>34.65</v>
       </c>
       <c r="AR2" t="n">
-        <v>1801.8</v>
+        <v>1826.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>1960.37</v>
+        <v>1981.81</v>
       </c>
       <c r="AT2" t="n">
-        <v>1722.52</v>
+        <v>1748.39</v>
       </c>
       <c r="AU2" t="n">
-        <v>1801.800048828125</v>
+        <v>1826.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.52</v>
       </c>
       <c r="AY2" t="n">
-        <v>158.57</v>
+        <v>155.61</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.4</v>
+        <v>4.26</v>
       </c>
       <c r="BA2" t="n">
-        <v>79.28</v>
+        <v>77.81</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="BE2" t="n">
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="BI2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.8</v>
+        <v>50.2</v>
       </c>
       <c r="BO2" t="n">
         <v>2.27</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.880000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.28</v>
+        <v>-4.3</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.247</v>
+        <v>0.248</v>
       </c>
       <c r="BT2" t="n">
-        <v>1481.46</v>
+        <v>1484.08</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.76</v>
+        <v>-13.52</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2064,10 +2064,10 @@
         <v>53</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>64.58</v>
+        <v>78.05</v>
       </c>
       <c r="CO2" t="n">
-        <v>32.02</v>
+        <v>46.03</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.800599999999999</v>
+        <v>8.521000000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,34 +2133,34 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5867</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2933</v>
+        <v>0.284</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.0852</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0349</v>
+        <v>1.0139</v>
       </c>
       <c r="DH2" t="n">
         <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.4</v>
+        <v>4.2608</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.38</v>
+        <v>36.8</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.4</v>
+        <v>4.2608</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
@@ -2169,22 +2169,22 @@
         <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9091</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="DQ2" t="n">
-        <v>79.28</v>
+        <v>77.81</v>
       </c>
       <c r="DR2" t="n">
-        <v>64.95</v>
+        <v>48.62</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.8227</v>
+        <v>-0.09859999999999999</v>
       </c>
       <c r="DX2" t="n">
-        <v>94.7</v>
+        <v>86.64999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>32</v>
+        <v>5.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>67.283</v>
+        <v>74.556</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>32.91</v>
+        <v>38.37</v>
       </c>
       <c r="ED2" t="n">
-        <v>98.62</v>
+        <v>83.88</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.8227</v>
+        <v>-0.09859999999999999</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.64</v>
+        <v>0.11</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2129</v>
+        <v>-0.025</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0003</v>
+        <v>4.0005</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.025</v>
+        <v>-0.003</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7408</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="EK2" t="n">
-        <v>50.99</v>
+        <v>56.19</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,78 +2243,78 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>8.039999999999999</v>
+        <v>54.09</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.9455</v>
+        <v>6.4367</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0131</v>
       </c>
       <c r="ER2" t="n">
-        <v>13.75</v>
+        <v>77.4545</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.3688</v>
+        <v>11.7572</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.276</v>
+        <v>53.89</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.1584</v>
+        <v>-0.0231</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3415</v>
+        <v>1.9189</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.1922</v>
+        <v>42.2172</v>
       </c>
       <c r="EX2" t="n">
-        <v>35.45</v>
+        <v>48.96</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.52</v>
+        <v>64.17</v>
       </c>
       <c r="FC2" t="n">
-        <v>28.85</v>
+        <v>29.27</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.34999999999999</v>
+        <v>73.31</v>
       </c>
       <c r="FE2" t="n">
-        <v>57.785</v>
+        <v>67.12</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.735</v>
+        <v>47.495</v>
       </c>
       <c r="FG2" t="n">
-        <v>20.1812</v>
+        <v>24.9361</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.224</v>
+        <v>65.292</v>
       </c>
       <c r="FI2" t="n">
-        <v>50.665</v>
+        <v>42.71</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.19</v>
+        <v>68.22</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.93000000000001</v>
+        <v>73.52</v>
       </c>
       <c r="FO2" t="n">
-        <v>54.67</v>
+        <v>60.9</v>
       </c>
       <c r="FP2" t="n">
-        <v>61.53</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.16</v>
+        <v>72.89</v>
       </c>
       <c r="FR2" t="n">
-        <v>77.26000000000001</v>
+        <v>83.88</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.4675</v>
+        <v>68.39700000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260819_161352</t>
+          <t>20260820_093202</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46253.67629744824</v>
+        <v>46254.39725031897</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46253.6762962963</v>
+        <v>46254.39724537037</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.76</v>
+        <v>11.9</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1801.8</v>
+        <v>1826.2</v>
       </c>
       <c r="L2" t="n">
-        <v>1814</v>
+        <v>1819</v>
       </c>
       <c r="M2" t="n">
-        <v>1818</v>
+        <v>1831.1</v>
       </c>
       <c r="N2" t="n">
-        <v>1789.9</v>
+        <v>1813.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1801.8</v>
+        <v>1826.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1426121</v>
+        <v>246388</v>
       </c>
       <c r="Q2" t="n">
-        <v>1801.8</v>
+        <v>1826.2</v>
       </c>
       <c r="R2" t="n">
-        <v>1960.37</v>
+        <v>1981.81</v>
       </c>
       <c r="S2" t="n">
-        <v>1722.52</v>
+        <v>1748.39</v>
       </c>
       <c r="T2" t="n">
-        <v>8.800643800643797</v>
+        <v>8.520972511225491</v>
       </c>
       <c r="U2" t="n">
-        <v>158.5699999999999</v>
+        <v>155.6099999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.400044400044399</v>
+        <v>4.260760048187491</v>
       </c>
       <c r="W2" t="n">
-        <v>79.27999999999997</v>
+        <v>77.80999999999995</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000126135216953</v>
+        <v>1.999871481814677</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.800643800643797</v>
+        <v>8.520972511225491</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.400044400044399</v>
+        <v>4.260760048187491</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02060405199033586</v>
+        <v>0.02058981998804869</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3270791854000446</v>
+        <v>0.3268532593677824</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02924066102128654</v>
+        <v>0.02921480555459584</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306250876103246</v>
+        <v>0.04306249763441346</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.83</v>
+        <v>38.85</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-19 16:13:52.140153+05:30</t>
+          <t>2026-08-20 09:32:02.466317+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.800643800643797, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001261352169526}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.52097251122549, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999871481814677}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-20 10:45 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>11.9</v>
       </c>
       <c r="R2" t="n">
-        <v>49.09</v>
+        <v>49.29</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1819</v>
       </c>
       <c r="V2" t="n">
-        <v>1831.1</v>
+        <v>1832</v>
       </c>
       <c r="W2" t="n">
         <v>1813.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1826.2</v>
+        <v>1825</v>
       </c>
       <c r="Y2" t="n">
-        <v>1826.2</v>
+        <v>1825</v>
       </c>
       <c r="Z2" t="n">
-        <v>246388</v>
+        <v>1314558</v>
       </c>
       <c r="AA2" t="n">
-        <v>2173488</v>
+        <v>2226896</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.11</v>
+        <v>0.59</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.35</v>
+        <v>1.29</v>
       </c>
       <c r="AD2" t="n">
         <v>0.95</v>
       </c>
       <c r="AE2" t="n">
-        <v>17.3</v>
+        <v>18.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.9</v>
+        <v>38.97</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.9</v>
+        <v>38.97</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.24</v>
+        <v>1.18</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.98</v>
+        <v>12.91</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.33</v>
+        <v>49.24</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.34</v>
+        <v>65.19</v>
       </c>
       <c r="AP2" t="n">
-        <v>-0.21</v>
+        <v>-0.27</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.65</v>
+        <v>34.56</v>
       </c>
       <c r="AR2" t="n">
-        <v>1826.2</v>
+        <v>1825</v>
       </c>
       <c r="AS2" t="n">
-        <v>1981.81</v>
+        <v>1980.87</v>
       </c>
       <c r="AT2" t="n">
-        <v>1748.39</v>
+        <v>1747.07</v>
       </c>
       <c r="AU2" t="n">
-        <v>1826.199951171875</v>
+        <v>1825</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.52</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>155.61</v>
+        <v>155.87</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.26</v>
+        <v>4.27</v>
       </c>
       <c r="BA2" t="n">
-        <v>77.81</v>
+        <v>77.93000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2026,10 +2026,10 @@
         <v>0.248</v>
       </c>
       <c r="BT2" t="n">
-        <v>1484.08</v>
+        <v>1483.9</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.52</v>
+        <v>-13.53</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
@@ -2038,7 +2038,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>78.05</v>
+        <v>74.48</v>
       </c>
       <c r="CO2" t="n">
-        <v>46.03</v>
+        <v>40.72</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.521000000000001</v>
+        <v>8.540800000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.5693</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.284</v>
+        <v>0.2847</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0852</v>
+        <v>0.0854</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0139</v>
+        <v>1.0163</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9907</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2608</v>
+        <v>4.2701</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.8</v>
+        <v>34.9</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2608</v>
+        <v>4.2701</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9953</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9907</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9996</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9346</v>
       </c>
       <c r="DQ2" t="n">
-        <v>77.81</v>
+        <v>77.93000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.62</v>
+        <v>66.23</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,128 +2193,128 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.09859999999999999</v>
+        <v>-0.1262</v>
       </c>
       <c r="DX2" t="n">
-        <v>86.64999999999999</v>
+        <v>87.02500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>5.5</v>
+        <v>29.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>74.556</v>
+        <v>71.884</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>38.37</v>
+        <v>41.93</v>
       </c>
       <c r="ED2" t="n">
-        <v>83.88</v>
+        <v>93.62</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.09859999999999999</v>
+        <v>-0.1262</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.11</v>
+        <v>0.59</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.025</v>
+        <v>-0.0321</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0005</v>
+        <v>3.991</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.003</v>
+        <v>-0.0038</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7606000000000001</v>
+        <v>0.7573</v>
       </c>
       <c r="EK2" t="n">
-        <v>56.19</v>
+        <v>62.83</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>54.09</v>
+        <v>20.31</v>
       </c>
       <c r="EP2" t="n">
-        <v>6.4367</v>
+        <v>2.4169</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0131</v>
+        <v>0.0702</v>
       </c>
       <c r="ER2" t="n">
-        <v>77.4545</v>
+        <v>14.4746</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.7572</v>
+        <v>11.1146</v>
       </c>
       <c r="ET2" t="n">
-        <v>53.89</v>
+        <v>41.632</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.0231</v>
+        <v>-0.1593</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.9189</v>
+        <v>1.3459</v>
       </c>
       <c r="EW2" t="n">
-        <v>42.2172</v>
+        <v>15.1269</v>
       </c>
       <c r="EX2" t="n">
-        <v>48.96</v>
+        <v>34.11</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
         <v>64.17</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.27</v>
+        <v>27.15</v>
       </c>
       <c r="FD2" t="n">
         <v>73.31</v>
       </c>
       <c r="FE2" t="n">
-        <v>67.12</v>
+        <v>68.655</v>
       </c>
       <c r="FF2" t="n">
-        <v>47.495</v>
+        <v>37.415</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.9361</v>
+        <v>23.7197</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.292</v>
+        <v>61.251</v>
       </c>
       <c r="FI2" t="n">
-        <v>42.71</v>
+        <v>50.565</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.22</v>
+        <v>65.33</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,36 +2328,36 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.52</v>
+        <v>68.11</v>
       </c>
       <c r="FO2" t="n">
-        <v>60.9</v>
+        <v>58.19</v>
       </c>
       <c r="FP2" t="n">
-        <v>70.79000000000001</v>
+        <v>55.68</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.89</v>
+        <v>70.28</v>
       </c>
       <c r="FR2" t="n">
-        <v>83.88</v>
+        <v>77.59</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>86.36360000000001</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.39700000000001</v>
+        <v>67.0305</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260820_093202</t>
+          <t>20260820_161510</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46254.39725031897</v>
+        <v>46254.67720021964</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46254.39724537037</v>
+        <v>46254.67719907407</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46254</v>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1826.2</v>
+        <v>1825</v>
       </c>
       <c r="L2" t="n">
         <v>1819</v>
       </c>
       <c r="M2" t="n">
-        <v>1831.1</v>
+        <v>1832</v>
       </c>
       <c r="N2" t="n">
         <v>1813.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1826.2</v>
+        <v>1825</v>
       </c>
       <c r="P2" t="n">
-        <v>246388</v>
+        <v>1314558</v>
       </c>
       <c r="Q2" t="n">
-        <v>1826.2</v>
+        <v>1825</v>
       </c>
       <c r="R2" t="n">
-        <v>1981.81</v>
+        <v>1980.87</v>
       </c>
       <c r="S2" t="n">
-        <v>1748.39</v>
+        <v>1747.07</v>
       </c>
       <c r="T2" t="n">
-        <v>8.520972511225491</v>
+        <v>8.540821917808213</v>
       </c>
       <c r="U2" t="n">
-        <v>155.6099999999999</v>
+        <v>155.8699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.260760048187491</v>
+        <v>4.270136986301373</v>
       </c>
       <c r="W2" t="n">
-        <v>77.80999999999995</v>
+        <v>77.93000000000006</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999871481814677</v>
+        <v>2.000128320287434</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.520972511225491</v>
+        <v>8.540821917808213</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.260760048187491</v>
+        <v>4.270136986301373</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058981998804869</v>
+        <v>0.02057709670485883</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3268532593677824</v>
+        <v>0.3266512835086987</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02921480555459584</v>
+        <v>0.02920191314170374</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249763441346</v>
+        <v>0.04306250689360566</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.85</v>
+        <v>38.87</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-20 09:32:02.466317+05:30</t>
+          <t>2026-08-20 16:15:10.126830+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.52097251122549, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999871481814677}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.540821917808213, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001283202874345}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-21 04:04 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.9</v>
+        <v>11.83</v>
       </c>
       <c r="R2" t="n">
-        <v>49.29</v>
+        <v>49.04</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1819</v>
+        <v>1825</v>
       </c>
       <c r="V2" t="n">
-        <v>1832</v>
+        <v>1836.4</v>
       </c>
       <c r="W2" t="n">
-        <v>1813.8</v>
+        <v>1816.3</v>
       </c>
       <c r="X2" t="n">
-        <v>1825</v>
+        <v>1823.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>1825</v>
+        <v>1823.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>1314558</v>
+        <v>223857</v>
       </c>
       <c r="AA2" t="n">
-        <v>2226896</v>
+        <v>2105744</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.59</v>
+        <v>0.11</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.29</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>18.2</v>
+        <v>20.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.97</v>
+        <v>37.62</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.97</v>
+        <v>37.62</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.14</v>
+        <v>2.06</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.18</v>
+        <v>0.49</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.91</v>
+        <v>12.24</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.24</v>
+        <v>48.63</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.19</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>-0.27</v>
+        <v>-1.11</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.56</v>
+        <v>32.75</v>
       </c>
       <c r="AR2" t="n">
-        <v>1825</v>
+        <v>1823.8</v>
       </c>
       <c r="AS2" t="n">
-        <v>1980.87</v>
+        <v>1974.28</v>
       </c>
       <c r="AT2" t="n">
-        <v>1747.07</v>
+        <v>1748.56</v>
       </c>
       <c r="AU2" t="n">
-        <v>1825</v>
+        <v>1823.800048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.539999999999999</v>
+        <v>8.25</v>
       </c>
       <c r="AY2" t="n">
-        <v>155.87</v>
+        <v>150.48</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.27</v>
+        <v>4.13</v>
       </c>
       <c r="BA2" t="n">
-        <v>77.93000000000001</v>
+        <v>75.23999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1993,43 +1993,43 @@
         <v>18</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.27</v>
+        <v>2.26</v>
       </c>
       <c r="BP2" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.3</v>
+        <v>-4.29</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.248</v>
+        <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1483.9</v>
+        <v>1483.47</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.53</v>
+        <v>-13.57</v>
       </c>
       <c r="BV2" t="n">
         <v>2.06</v>
@@ -2038,7 +2038,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.4</v>
+        <v>45.2</v>
       </c>
       <c r="CE2" t="n">
         <v>53</v>
@@ -2067,7 +2067,7 @@
         <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>74.48</v>
+        <v>74.61</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.72</v>
+        <v>45.49</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.540800000000001</v>
+        <v>8.2509</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5693</v>
+        <v>0.55</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2847</v>
+        <v>0.2753</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0854</v>
+        <v>0.0825</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.9976</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>4.0049</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.1255</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>33.28</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.1255</v>
+      </c>
+      <c r="DL2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.0163</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>3.9907</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>4.2701</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>4.2701</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>2.0001</v>
-      </c>
       <c r="DM2" t="n">
-        <v>1.9953</v>
+        <v>2.0049</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9907</v>
+        <v>4.0049</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9996</v>
+        <v>1.9978</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9346</v>
+        <v>0.9697</v>
       </c>
       <c r="DQ2" t="n">
-        <v>77.93000000000001</v>
+        <v>75.23999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>66.23</v>
+        <v>53.87</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,90 +2193,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.1262</v>
+        <v>-0.5387999999999999</v>
       </c>
       <c r="DX2" t="n">
-        <v>87.02500000000001</v>
+        <v>87.74999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>29.5</v>
+        <v>5.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>71.884</v>
+        <v>69.27800000000001</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>41.93</v>
+        <v>35.12</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.62</v>
+        <v>87.28</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.1262</v>
+        <v>-0.5387999999999999</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.59</v>
+        <v>0.11</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.0321</v>
+        <v>-0.1313</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.991</v>
+        <v>4.0053</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0038</v>
+        <v>-0.0155</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7573</v>
+        <v>0.7808</v>
       </c>
       <c r="EK2" t="n">
-        <v>62.83</v>
+        <v>59.46</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>20.31</v>
+        <v>21.7</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.4169</v>
+        <v>2.5671</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0702</v>
+        <v>0.013</v>
       </c>
       <c r="ER2" t="n">
-        <v>14.4746</v>
+        <v>75</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.1146</v>
+        <v>10.8758</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.632</v>
+        <v>43.861</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.1593</v>
+        <v>-0.1221</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3459</v>
+        <v>1.8559</v>
       </c>
       <c r="EW2" t="n">
-        <v>15.1269</v>
+        <v>16.1904</v>
       </c>
       <c r="EX2" t="n">
-        <v>34.11</v>
+        <v>39.95</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.17</v>
+        <v>63.85</v>
       </c>
       <c r="FC2" t="n">
-        <v>27.15</v>
+        <v>26.36</v>
       </c>
       <c r="FD2" t="n">
         <v>73.31</v>
       </c>
       <c r="FE2" t="n">
-        <v>68.655</v>
+        <v>67.035</v>
       </c>
       <c r="FF2" t="n">
-        <v>37.415</v>
+        <v>42.72</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.7197</v>
+        <v>24.3824</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.251</v>
+        <v>62.298</v>
       </c>
       <c r="FI2" t="n">
-        <v>50.565</v>
+        <v>43.575</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.33</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>68.11</v>
+        <v>69.16</v>
       </c>
       <c r="FO2" t="n">
-        <v>58.19</v>
+        <v>58.12</v>
       </c>
       <c r="FP2" t="n">
-        <v>55.68</v>
+        <v>60.3</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.28</v>
+        <v>69.88</v>
       </c>
       <c r="FR2" t="n">
-        <v>77.59</v>
+        <v>78.16</v>
       </c>
       <c r="FS2" t="n">
-        <v>86.36360000000001</v>
+        <v>77.2727</v>
       </c>
       <c r="FT2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.0305</v>
+        <v>65.2385</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="FZ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GA2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260820_161510</t>
+          <t>20260821_093417</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46254.67720021964</v>
+        <v>46255.39881624525</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46254.67719907407</v>
+        <v>46255.39880787037</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.9</v>
+        <v>11.83</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
+        <v>1823.8</v>
+      </c>
+      <c r="L2" t="n">
         <v>1825</v>
       </c>
-      <c r="L2" t="n">
-        <v>1819</v>
-      </c>
       <c r="M2" t="n">
-        <v>1832</v>
+        <v>1836.4</v>
       </c>
       <c r="N2" t="n">
-        <v>1813.8</v>
+        <v>1816.3</v>
       </c>
       <c r="O2" t="n">
-        <v>1825</v>
+        <v>1823.8</v>
       </c>
       <c r="P2" t="n">
-        <v>1314558</v>
+        <v>223857</v>
       </c>
       <c r="Q2" t="n">
-        <v>1825</v>
+        <v>1823.8</v>
       </c>
       <c r="R2" t="n">
-        <v>1980.87</v>
+        <v>1974.28</v>
       </c>
       <c r="S2" t="n">
-        <v>1747.07</v>
+        <v>1748.56</v>
       </c>
       <c r="T2" t="n">
-        <v>8.540821917808213</v>
+        <v>8.25090470446321</v>
       </c>
       <c r="U2" t="n">
-        <v>155.8699999999999</v>
+        <v>150.48</v>
       </c>
       <c r="V2" t="n">
-        <v>4.270136986301373</v>
+        <v>4.125452352231605</v>
       </c>
       <c r="W2" t="n">
-        <v>77.93000000000006</v>
+        <v>75.24000000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000128320287434</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.540821917808213</v>
+        <v>8.25090470446321</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.270136986301373</v>
+        <v>4.125452352231605</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057709670485883</v>
+        <v>0.02057359729981881</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266512835086987</v>
+        <v>0.3265957321758633</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306250689360566</v>
+        <v>0.04306250088489286</v>
       </c>
     </row>
     <row r="13">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-20 16:15:10.126830+05:30</t>
+          <t>2026-08-21 09:34:17.765608+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.540821917808213, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001283202874345}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.25090470446321, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-21 10:44 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.83</v>
+        <v>11.71</v>
       </c>
       <c r="R2" t="n">
-        <v>49.04</v>
+        <v>49.25</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>1836.4</v>
       </c>
       <c r="W2" t="n">
-        <v>1816.3</v>
+        <v>1790.3</v>
       </c>
       <c r="X2" t="n">
-        <v>1823.8</v>
+        <v>1802</v>
       </c>
       <c r="Y2" t="n">
-        <v>1823.8</v>
+        <v>1802</v>
       </c>
       <c r="Z2" t="n">
-        <v>223857</v>
+        <v>1401832</v>
       </c>
       <c r="AA2" t="n">
-        <v>2105744</v>
+        <v>2164643</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.11</v>
+        <v>0.65</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-1.26</v>
       </c>
       <c r="AD2" t="n">
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>20.1</v>
+        <v>46.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.1</v>
+        <v>2.56</v>
       </c>
       <c r="AG2" t="n">
-        <v>37.62</v>
+        <v>39.48</v>
       </c>
       <c r="AH2" t="n">
-        <v>37.62</v>
+        <v>39.48</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.06</v>
+        <v>2.19</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.49</v>
+        <v>-0.65</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.24</v>
+        <v>10.92</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.63</v>
+        <v>46.86</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.90000000000001</v>
+        <v>60</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.11</v>
+        <v>-2.29</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.75</v>
+        <v>31.16</v>
       </c>
       <c r="AR2" t="n">
-        <v>1823.8</v>
+        <v>1802</v>
       </c>
       <c r="AS2" t="n">
-        <v>1974.28</v>
+        <v>1959.91</v>
       </c>
       <c r="AT2" t="n">
-        <v>1748.56</v>
+        <v>1723.05</v>
       </c>
       <c r="AU2" t="n">
-        <v>1823.800048828125</v>
+        <v>1802</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.25</v>
+        <v>8.76</v>
       </c>
       <c r="AY2" t="n">
-        <v>150.48</v>
+        <v>157.91</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.13</v>
+        <v>4.38</v>
       </c>
       <c r="BA2" t="n">
-        <v>75.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.08</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,37 +1987,37 @@
         <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="BH2" t="n">
-        <v>18</v>
+        <v>17.6</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BM2" t="n">
         <v>655</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.1</v>
+        <v>49.6</v>
       </c>
       <c r="BO2" t="n">
         <v>2.26</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.29</v>
+        <v>-4.26</v>
       </c>
       <c r="BR2" t="n">
         <v>9.199999999999999</v>
@@ -2026,19 +2026,19 @@
         <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1483.47</v>
+        <v>1478.88</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.57</v>
+        <v>-13.81</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.08</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2061,13 +2061,13 @@
         <v>45.2</v>
       </c>
       <c r="CE2" t="n">
-        <v>53</v>
+        <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>69.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>74.61</v>
+        <v>71.51000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>45.49</v>
+        <v>35.81</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.2509</v>
+        <v>8.763</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.55</v>
+        <v>0.584</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2753</v>
+        <v>0.292</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0825</v>
+        <v>0.0876</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9976</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>0.976</v>
+        <v>1.0258</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0049</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.1255</v>
+        <v>4.3812</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.28</v>
+        <v>39.35</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.1255</v>
+        <v>4.3812</v>
       </c>
       <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2.0049</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0049</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9978</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9697</v>
+        <v>0.9132</v>
       </c>
       <c r="DQ2" t="n">
-        <v>75.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="DR2" t="n">
-        <v>53.87</v>
+        <v>57.93</v>
       </c>
       <c r="DS2" t="n">
         <v>4</v>
@@ -2193,128 +2193,128 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.5387999999999999</v>
+        <v>-1.0457</v>
       </c>
       <c r="DX2" t="n">
-        <v>87.74999999999999</v>
+        <v>100</v>
       </c>
       <c r="DY2" t="n">
-        <v>5.5</v>
+        <v>32.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>69.27800000000001</v>
+        <v>67.64100000000001</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="EC2" t="n">
-        <v>35.12</v>
+        <v>41.85</v>
       </c>
       <c r="ED2" t="n">
-        <v>87.28</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.5387999999999999</v>
+        <v>-1.0457</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.11</v>
+        <v>0.65</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.1313</v>
+        <v>-0.2682</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0053</v>
+        <v>4.0014</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0155</v>
+        <v>-0.0314</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7808</v>
+        <v>0.7438</v>
       </c>
       <c r="EK2" t="n">
-        <v>59.46</v>
+        <v>61.75</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="EM2" t="n">
+        <v>4</v>
+      </c>
+      <c r="EN2" t="n">
+        <v>8</v>
+      </c>
+      <c r="EO2" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="EP2" t="n">
+        <v>1.1804</v>
+      </c>
+      <c r="EQ2" t="n">
+        <v>0.0761</v>
+      </c>
+      <c r="ER2" t="n">
+        <v>13.4769</v>
+      </c>
+      <c r="ES2" t="n">
+        <v>12.3354</v>
+      </c>
+      <c r="ET2" t="n">
+        <v>36.332</v>
+      </c>
+      <c r="EU2" t="n">
+        <v>-1.4885</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>1.3273</v>
+      </c>
+      <c r="EW2" t="n">
+        <v>7.2082</v>
+      </c>
+      <c r="EX2" t="n">
+        <v>44.79</v>
+      </c>
+      <c r="EY2" t="inlineStr">
+        <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="EM2" t="n">
-        <v>5</v>
-      </c>
-      <c r="EN2" t="n">
-        <v>9</v>
-      </c>
-      <c r="EO2" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="EP2" t="n">
-        <v>2.5671</v>
-      </c>
-      <c r="EQ2" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="ER2" t="n">
-        <v>75</v>
-      </c>
-      <c r="ES2" t="n">
-        <v>10.8758</v>
-      </c>
-      <c r="ET2" t="n">
-        <v>43.861</v>
-      </c>
-      <c r="EU2" t="n">
-        <v>-0.1221</v>
-      </c>
-      <c r="EV2" t="n">
-        <v>1.8559</v>
-      </c>
-      <c r="EW2" t="n">
-        <v>16.1904</v>
-      </c>
-      <c r="EX2" t="n">
-        <v>39.95</v>
-      </c>
-      <c r="EY2" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.85</v>
+        <v>63.28</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.36</v>
+        <v>30.63</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.31</v>
+        <v>74.88</v>
       </c>
       <c r="FE2" t="n">
-        <v>67.035</v>
+        <v>66.63</v>
       </c>
       <c r="FF2" t="n">
-        <v>42.72</v>
+        <v>40.3</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.3824</v>
+        <v>22.4169</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.298</v>
+        <v>62.051</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.575</v>
+        <v>48.64</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.43000000000001</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,36 +2328,36 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.16</v>
+        <v>70.5</v>
       </c>
       <c r="FO2" t="n">
-        <v>58.12</v>
+        <v>59.84</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.3</v>
+        <v>60.8</v>
       </c>
       <c r="FQ2" t="n">
-        <v>69.88</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>78.16</v>
+        <v>80.64</v>
       </c>
       <c r="FS2" t="n">
-        <v>77.2727</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.2385</v>
+        <v>67.97</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260821_093417</t>
+          <t>20260821_161442</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46255.39881624525</v>
+        <v>46255.67687956813</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46255.39880787037</v>
+        <v>46255.676875</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46255</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.83</v>
+        <v>11.71</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1823.8</v>
+        <v>1802</v>
       </c>
       <c r="L2" t="n">
         <v>1825</v>
@@ -2690,37 +2690,37 @@
         <v>1836.4</v>
       </c>
       <c r="N2" t="n">
-        <v>1816.3</v>
+        <v>1790.3</v>
       </c>
       <c r="O2" t="n">
-        <v>1823.8</v>
+        <v>1802</v>
       </c>
       <c r="P2" t="n">
-        <v>223857</v>
+        <v>1401832</v>
       </c>
       <c r="Q2" t="n">
-        <v>1823.8</v>
+        <v>1802</v>
       </c>
       <c r="R2" t="n">
-        <v>1974.28</v>
+        <v>1959.91</v>
       </c>
       <c r="S2" t="n">
-        <v>1748.56</v>
+        <v>1723.05</v>
       </c>
       <c r="T2" t="n">
-        <v>8.25090470446321</v>
+        <v>8.763041065482803</v>
       </c>
       <c r="U2" t="n">
-        <v>150.48</v>
+        <v>157.9100000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.125452352231605</v>
+        <v>4.381243063263043</v>
       </c>
       <c r="W2" t="n">
-        <v>75.24000000000001</v>
+        <v>78.95000000000005</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000126662444585</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.25090470446321</v>
+        <v>8.763041065482803</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.125452352231605</v>
+        <v>4.381243063263043</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057359729981881</v>
+        <v>0.02056531203343287</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3265957321758633</v>
+        <v>0.3264642076494446</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02920191314170374</v>
+        <v>0.02917612606860895</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306250088489286</v>
+        <v>0.04306250308306914</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.87</v>
+        <v>38.88</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-21 09:34:17.765608+05:30</t>
+          <t>2026-08-21 16:14:42.433150+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.25090470446321, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.763041065482803, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001266624445853}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-24 04:08 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.71</v>
+        <v>11.69</v>
       </c>
       <c r="R2" t="n">
-        <v>49.25</v>
+        <v>49.02</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1825</v>
+        <v>1800</v>
       </c>
       <c r="V2" t="n">
-        <v>1836.4</v>
+        <v>1810.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1790.3</v>
+        <v>1795.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1802</v>
+        <v>1803.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1802</v>
+        <v>1803.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>1401832</v>
+        <v>257328</v>
       </c>
       <c r="AA2" t="n">
-        <v>2164643</v>
+        <v>1778029</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.65</v>
+        <v>0.14</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.26</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>-0.11</v>
       </c>
       <c r="AE2" t="n">
-        <v>46.1</v>
+        <v>15.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.56</v>
+        <v>0.85</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.48</v>
+        <v>37.75</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.48</v>
+        <v>37.75</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.19</v>
+        <v>2.09</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,71 +1926,71 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.65</v>
+        <v>-0.82</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.92</v>
+        <v>10.44</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.86</v>
+        <v>46.48</v>
       </c>
       <c r="AO2" t="n">
-        <v>60</v>
+        <v>60.19</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.29</v>
+        <v>-2.73</v>
       </c>
       <c r="AQ2" t="n">
-        <v>31.16</v>
+        <v>30.51</v>
       </c>
       <c r="AR2" t="n">
-        <v>1802</v>
+        <v>1803.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>1959.91</v>
+        <v>1954.3</v>
       </c>
       <c r="AT2" t="n">
-        <v>1723.05</v>
+        <v>1727.8</v>
       </c>
       <c r="AU2" t="n">
-        <v>1802</v>
+        <v>1803.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.76</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>157.91</v>
+        <v>151</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.38</v>
+        <v>4.19</v>
       </c>
       <c r="BA2" t="n">
-        <v>78.95</v>
+        <v>75.5</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="BE2" t="n">
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.2</v>
+        <v>49.1</v>
       </c>
       <c r="BG2" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.6</v>
+        <v>17.7</v>
       </c>
       <c r="BI2" t="n">
         <v>4</v>
@@ -2005,40 +2005,40 @@
         <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
       <c r="BP2" t="n">
         <v>8.880000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.26</v>
+        <v>-4.25</v>
       </c>
       <c r="BR2" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="BS2" t="n">
         <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1478.88</v>
+        <v>1479.14</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.81</v>
+        <v>-13.64</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.2</v>
+        <v>45</v>
       </c>
       <c r="CE2" t="n">
         <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>69.3</v>
+        <v>69.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.90000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>71.51000000000001</v>
+        <v>70.77</v>
       </c>
       <c r="CO2" t="n">
-        <v>35.81</v>
+        <v>46.49</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.763</v>
+        <v>8.3735</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.584</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.292</v>
+        <v>0.2793</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0876</v>
+        <v>0.0837</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.9976</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>0.9785</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>4.0048</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.1868</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>36.08</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.1868</v>
+      </c>
+      <c r="DL2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.0258</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>4</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>4.3812</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>39.35</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>4.3812</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>2.0001</v>
-      </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0048</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0048</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9132</v>
+        <v>0.9558</v>
       </c>
       <c r="DQ2" t="n">
-        <v>78.95</v>
+        <v>75.5</v>
       </c>
       <c r="DR2" t="n">
-        <v>57.93</v>
+        <v>65.3</v>
       </c>
       <c r="DS2" t="n">
         <v>4</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-1.0457</v>
+        <v>-1.3062</v>
       </c>
       <c r="DX2" t="n">
-        <v>100</v>
+        <v>99.52500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>32.5</v>
+        <v>7</v>
       </c>
       <c r="DZ2" t="n">
-        <v>67.64100000000001</v>
+        <v>74.04300000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>4</v>
@@ -2211,31 +2211,31 @@
         <v>7</v>
       </c>
       <c r="EC2" t="n">
-        <v>41.85</v>
+        <v>55.16</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-1.0457</v>
+        <v>-1.3062</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.65</v>
+        <v>0.14</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2682</v>
+        <v>-0.3191</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0014</v>
+        <v>4.0065</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0314</v>
+        <v>-0.0373</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7438</v>
+        <v>0.772</v>
       </c>
       <c r="EK2" t="n">
-        <v>61.75</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>10.08</v>
+        <v>23.33</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.1804</v>
+        <v>2.7273</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0761</v>
+        <v>0.0164</v>
       </c>
       <c r="ER2" t="n">
-        <v>13.4769</v>
+        <v>59.7857</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.3354</v>
+        <v>11.6764</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.332</v>
+        <v>44.552</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.4885</v>
+        <v>-0.3822</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3273</v>
+        <v>1.8333</v>
       </c>
       <c r="EW2" t="n">
-        <v>7.2082</v>
+        <v>16.5106</v>
       </c>
       <c r="EX2" t="n">
-        <v>44.79</v>
+        <v>46.97</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.28</v>
+        <v>63.19</v>
       </c>
       <c r="FC2" t="n">
-        <v>30.63</v>
+        <v>28.03</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.88</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>66.63</v>
+        <v>67.39</v>
       </c>
       <c r="FF2" t="n">
-        <v>40.3</v>
+        <v>46.73</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.4169</v>
+        <v>22.9029</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.051</v>
+        <v>62.22</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.64</v>
+        <v>50.69</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.29000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.5</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>59.84</v>
+        <v>58.13</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.8</v>
+        <v>67.95999999999999</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.54000000000001</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>80.64</v>
+        <v>74.87</v>
       </c>
       <c r="FS2" t="n">
         <v>90.9091</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.97</v>
+        <v>65.94199999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260821_161442</t>
+          <t>20260824_093855</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46255.67687956813</v>
+        <v>46258.40203115254</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46255.676875</v>
+        <v>46258.40202546296</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.71</v>
+        <v>11.69</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1802</v>
+        <v>1803.3</v>
       </c>
       <c r="L2" t="n">
-        <v>1825</v>
+        <v>1800</v>
       </c>
       <c r="M2" t="n">
-        <v>1836.4</v>
+        <v>1810.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1790.3</v>
+        <v>1795.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1802</v>
+        <v>1803.3</v>
       </c>
       <c r="P2" t="n">
-        <v>1401832</v>
+        <v>257328</v>
       </c>
       <c r="Q2" t="n">
-        <v>1802</v>
+        <v>1803.3</v>
       </c>
       <c r="R2" t="n">
-        <v>1959.91</v>
+        <v>1954.3</v>
       </c>
       <c r="S2" t="n">
-        <v>1723.05</v>
+        <v>1727.8</v>
       </c>
       <c r="T2" t="n">
-        <v>8.763041065482803</v>
+        <v>8.373537403648866</v>
       </c>
       <c r="U2" t="n">
-        <v>157.9100000000001</v>
+        <v>151</v>
       </c>
       <c r="V2" t="n">
-        <v>4.381243063263043</v>
+        <v>4.186768701824433</v>
       </c>
       <c r="W2" t="n">
-        <v>78.95000000000005</v>
+        <v>75.5</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000126662444585</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.763041065482803</v>
+        <v>8.373537403648866</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.381243063263043</v>
+        <v>4.186768701824433</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02056531203343287</v>
+        <v>0.02055019133575736</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3264642076494446</v>
+        <v>0.3262241740152493</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02917612606860895</v>
+        <v>0.02916321742645627</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306250308306914</v>
+        <v>0.04306249500830515</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.88</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-21 16:14:42.433150+05:30</t>
+          <t>2026-08-24 09:38:55.529104+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.763041065482803, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001266624445853}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.373537403648866, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-24 10:50 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1818,9 +1818,7 @@
       <c r="D2" s="1" t="n">
         <v>46258</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>46258</v>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
@@ -1854,26 +1852,22 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.69</v>
+        <v>11.64</v>
       </c>
       <c r="R2" t="n">
-        <v>49.02</v>
+        <v>49.6</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
         <v>1800</v>
       </c>
@@ -1881,43 +1875,43 @@
         <v>1810.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1795.5</v>
+        <v>1790</v>
       </c>
       <c r="X2" t="n">
-        <v>1803.3</v>
+        <v>1801</v>
       </c>
       <c r="Y2" t="n">
-        <v>1803.3</v>
+        <v>1801</v>
       </c>
       <c r="Z2" t="n">
-        <v>257328</v>
+        <v>2894133</v>
       </c>
       <c r="AA2" t="n">
-        <v>1778029</v>
+        <v>1909869</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.14</v>
+        <v>1.52</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.06</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.11</v>
       </c>
       <c r="AE2" t="n">
-        <v>15.3</v>
+        <v>20.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.85</v>
+        <v>1.15</v>
       </c>
       <c r="AG2" t="n">
-        <v>37.75</v>
+        <v>38.14</v>
       </c>
       <c r="AH2" t="n">
-        <v>37.75</v>
+        <v>38.14</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.09</v>
+        <v>2.12</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.82</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.44</v>
+        <v>10.3</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.48</v>
+        <v>46.29</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.19</v>
+        <v>59.77</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.73</v>
+        <v>-2.86</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.51</v>
+        <v>30.35</v>
       </c>
       <c r="AR2" t="n">
-        <v>1803.3</v>
+        <v>1801</v>
       </c>
       <c r="AS2" t="n">
-        <v>1954.3</v>
+        <v>1953.57</v>
       </c>
       <c r="AT2" t="n">
-        <v>1727.8</v>
+        <v>1724.72</v>
       </c>
       <c r="AU2" t="n">
-        <v>1803.300048828125</v>
+        <v>1801</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.369999999999999</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>151</v>
+        <v>152.57</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.19</v>
+        <v>4.24</v>
       </c>
       <c r="BA2" t="n">
-        <v>75.5</v>
+        <v>76.28</v>
       </c>
       <c r="BB2" t="n">
         <v>2.09</v>
@@ -2023,13 +2017,13 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.247</v>
+        <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.14</v>
+        <v>1478.5</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.64</v>
+        <v>-13.67</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2038,7 +2032,7 @@
         <v>2.09</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2088,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>70.77</v>
+        <v>78.47</v>
       </c>
       <c r="CO2" t="n">
-        <v>46.49</v>
+        <v>51.84</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2115,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.3735</v>
+        <v>8.471399999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.5647</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2793</v>
+        <v>0.2827</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0837</v>
+        <v>0.0847</v>
       </c>
       <c r="DF2" t="n">
         <v>1.9976</v>
       </c>
       <c r="DG2" t="n">
-        <v>0.9785</v>
+        <v>0.9859</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0048</v>
+        <v>3.9953</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.1868</v>
+        <v>4.2354</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.08</v>
+        <v>36.14</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.1868</v>
+        <v>4.2354</v>
       </c>
       <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2.0048</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0048</v>
+        <v>3.9953</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>1.9975</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9558</v>
+        <v>0.9423</v>
       </c>
       <c r="DQ2" t="n">
-        <v>75.5</v>
+        <v>76.28</v>
       </c>
       <c r="DR2" t="n">
-        <v>65.3</v>
+        <v>45.3</v>
       </c>
       <c r="DS2" t="n">
         <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-1.3062</v>
+        <v>-1.3491</v>
       </c>
       <c r="DX2" t="n">
-        <v>99.52500000000001</v>
+        <v>99.42500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>7</v>
+        <v>76</v>
       </c>
       <c r="DZ2" t="n">
-        <v>74.04300000000001</v>
+        <v>77.23099999999999</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>55.16</v>
+        <v>56.29</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-1.3062</v>
+        <v>-1.3491</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.14</v>
+        <v>1.52</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.3191</v>
+        <v>-0.3329</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0065</v>
+        <v>3.9959</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0373</v>
+        <v>-0.0387</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.772</v>
+        <v>0.7625999999999999</v>
       </c>
       <c r="EK2" t="n">
-        <v>64.01000000000001</v>
+        <v>67.87</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2243,34 @@
         <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>23.33</v>
+        <v>57.82</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.7273</v>
+        <v>6.7302</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0164</v>
+        <v>0.1769</v>
       </c>
       <c r="ER2" t="n">
-        <v>59.7857</v>
+        <v>5.5724</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.6764</v>
+        <v>11.5833</v>
       </c>
       <c r="ET2" t="n">
-        <v>44.552</v>
+        <v>56.97</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.3822</v>
+        <v>-4.3472</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8333</v>
+        <v>0.8413</v>
       </c>
       <c r="EW2" t="n">
-        <v>16.5106</v>
+        <v>45.3714</v>
       </c>
       <c r="EX2" t="n">
-        <v>46.97</v>
+        <v>58.96</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.19</v>
+        <v>62.96</v>
       </c>
       <c r="FC2" t="n">
-        <v>28.03</v>
+        <v>27.91</v>
       </c>
       <c r="FD2" t="n">
         <v>75.40000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>67.39</v>
+        <v>73.17</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.73</v>
+        <v>55.4</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.9029</v>
+        <v>25.1506</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.22</v>
+        <v>66.813</v>
       </c>
       <c r="FI2" t="n">
-        <v>50.69</v>
+        <v>40.72</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.5</v>
+        <v>69.79000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.23999999999999</v>
+        <v>71.18000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>58.13</v>
+        <v>61.37</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.95999999999999</v>
+        <v>72</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.18000000000001</v>
+        <v>66.86</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.87</v>
+        <v>79.3</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.94199999999999</v>
+        <v>65.824</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260824_093855</t>
+          <t>20260824_162035</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46258.40203115254</v>
+        <v>46258.68096153643</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2465,8 +2459,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46258.40202546296</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46258</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46273</v>
-      </c>
+        <v>46258.68096064815</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2673,15 +2663,11 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.69</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+        <v>11.64</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1803.3</v>
+        <v>1801</v>
       </c>
       <c r="L2" t="n">
         <v>1800</v>
@@ -2690,37 +2676,37 @@
         <v>1810.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1795.5</v>
+        <v>1790</v>
       </c>
       <c r="O2" t="n">
-        <v>1803.3</v>
+        <v>1801</v>
       </c>
       <c r="P2" t="n">
-        <v>257328</v>
+        <v>2894133</v>
       </c>
       <c r="Q2" t="n">
-        <v>1803.3</v>
+        <v>1801</v>
       </c>
       <c r="R2" t="n">
-        <v>1954.3</v>
+        <v>1953.57</v>
       </c>
       <c r="S2" t="n">
-        <v>1727.8</v>
+        <v>1724.72</v>
       </c>
       <c r="T2" t="n">
-        <v>8.373537403648866</v>
+        <v>8.471404775124928</v>
       </c>
       <c r="U2" t="n">
-        <v>151</v>
+        <v>152.5699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.186768701824433</v>
+        <v>4.235424764019988</v>
       </c>
       <c r="W2" t="n">
-        <v>75.5</v>
+        <v>76.27999999999997</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000131095962244</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.373537403648866</v>
+        <v>8.471404775124928</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.186768701824433</v>
+        <v>4.235424764019988</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02055019133575736</v>
+        <v>0.02055041729361061</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3262241740152493</v>
+        <v>0.3262277609849683</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249500830515</v>
+        <v>0.04306249936603321</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-24 09:38:55.529104+05:30</t>
+          <t>2026-08-24 16:20:35.114940+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.373537403648866, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.471404775124928, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000131095962244}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-25 04:03 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46259</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1852,63 +1854,67 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
         <v>11.64</v>
       </c>
       <c r="R2" t="n">
-        <v>49.6</v>
+        <v>49.02</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>1800</v>
+        <v>1808</v>
       </c>
       <c r="V2" t="n">
-        <v>1810.8</v>
+        <v>1818.2</v>
       </c>
       <c r="W2" t="n">
-        <v>1790</v>
+        <v>1796.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="Y2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="Z2" t="n">
-        <v>2894133</v>
+        <v>256879</v>
       </c>
       <c r="AA2" t="n">
-        <v>1909869</v>
+        <v>1778006</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.52</v>
+        <v>0.14</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.06</v>
+        <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.11</v>
+        <v>0.33</v>
       </c>
       <c r="AE2" t="n">
-        <v>20.8</v>
+        <v>21.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.15</v>
+        <v>1.2</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.14</v>
+        <v>38.21</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.14</v>
+        <v>38.21</v>
       </c>
       <c r="AI2" t="n">
         <v>2.12</v>
@@ -1920,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.89</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.3</v>
+        <v>10.36</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.29</v>
+        <v>46.37</v>
       </c>
       <c r="AO2" t="n">
-        <v>59.77</v>
+        <v>60</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.86</v>
+        <v>-2.8</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.35</v>
+        <v>30.42</v>
       </c>
       <c r="AR2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="AS2" t="n">
-        <v>1953.57</v>
+        <v>1954.83</v>
       </c>
       <c r="AT2" t="n">
-        <v>1724.72</v>
+        <v>1725.59</v>
       </c>
       <c r="AU2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.470000000000001</v>
+        <v>8.48</v>
       </c>
       <c r="AY2" t="n">
-        <v>152.57</v>
+        <v>152.83</v>
       </c>
       <c r="AZ2" t="n">
         <v>4.24</v>
       </c>
       <c r="BA2" t="n">
-        <v>76.28</v>
+        <v>76.41</v>
       </c>
       <c r="BB2" t="n">
         <v>2.09</v>
@@ -1981,22 +1987,22 @@
         <v>49.1</v>
       </c>
       <c r="BG2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BM2" t="n">
         <v>656</v>
@@ -2020,10 +2026,10 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1478.5</v>
+        <v>1478.36</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.67</v>
+        <v>-13.7</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2082,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>78.47</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>51.84</v>
+        <v>40.33</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2121,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.471399999999999</v>
+        <v>8.4811</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5647</v>
+        <v>0.5653</v>
       </c>
       <c r="DD2" t="n">
         <v>0.2827</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0847</v>
+        <v>0.0848</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9976</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>0.9859</v>
+        <v>0.9871</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9953</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2354</v>
+        <v>4.2403</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.14</v>
+        <v>37.48</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2354</v>
+        <v>4.2403</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2160,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9953</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9975</v>
+        <v>1.9996</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9423</v>
+        <v>0.9434</v>
       </c>
       <c r="DQ2" t="n">
-        <v>76.28</v>
+        <v>76.41</v>
       </c>
       <c r="DR2" t="n">
-        <v>45.3</v>
+        <v>45.7</v>
       </c>
       <c r="DS2" t="n">
         <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-1.3491</v>
+        <v>-1.3208</v>
       </c>
       <c r="DX2" t="n">
-        <v>99.42500000000001</v>
+        <v>100</v>
       </c>
       <c r="DY2" t="n">
-        <v>76</v>
+        <v>7</v>
       </c>
       <c r="DZ2" t="n">
-        <v>77.23099999999999</v>
+        <v>71.992</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="EC2" t="n">
-        <v>56.29</v>
+        <v>51.03</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-1.3491</v>
+        <v>-1.3208</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.52</v>
+        <v>0.14</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.3329</v>
+        <v>-0.3259</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9959</v>
+        <v>4.0005</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0387</v>
+        <v>-0.0379</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7625999999999999</v>
+        <v>0.7635</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.87</v>
+        <v>62.82</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,72 +2249,72 @@
         <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>57.82</v>
+        <v>20.97</v>
       </c>
       <c r="EP2" t="n">
-        <v>6.7302</v>
+        <v>2.4409</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1769</v>
+        <v>0.0163</v>
       </c>
       <c r="ER2" t="n">
-        <v>5.5724</v>
+        <v>60.5714</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.5833</v>
+        <v>12.0128</v>
       </c>
       <c r="ET2" t="n">
-        <v>56.97</v>
+        <v>41.311</v>
       </c>
       <c r="EU2" t="n">
-        <v>-4.3472</v>
+        <v>-0.392</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.8413</v>
+        <v>1.8596</v>
       </c>
       <c r="EW2" t="n">
-        <v>45.3714</v>
+        <v>14.3854</v>
       </c>
       <c r="EX2" t="n">
-        <v>58.96</v>
+        <v>31.07</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
         <v>62.96</v>
       </c>
       <c r="FC2" t="n">
-        <v>27.91</v>
+        <v>29.59</v>
       </c>
       <c r="FD2" t="n">
         <v>75.40000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>73.17</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>55.4</v>
+        <v>35.7</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.1506</v>
+        <v>21.9872</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.813</v>
+        <v>58.274</v>
       </c>
       <c r="FI2" t="n">
-        <v>40.72</v>
+        <v>41.59</v>
       </c>
       <c r="FJ2" t="n">
-        <v>69.79000000000001</v>
+        <v>64.81</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.18000000000001</v>
+        <v>63.82</v>
       </c>
       <c r="FO2" t="n">
-        <v>61.37</v>
+        <v>57.44</v>
       </c>
       <c r="FP2" t="n">
-        <v>72</v>
+        <v>49.89</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.86</v>
+        <v>65.84999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>79.3</v>
+        <v>70.72</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.824</v>
+        <v>60.799</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260824_162035</t>
+          <t>20260825_093317</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46258.68096153643</v>
+        <v>46259.3981150408</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2460,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46258.68096064815</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46259.39811342592</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46274</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2665,48 +2675,52 @@
       <c r="I2" t="n">
         <v>11.64</v>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="L2" t="n">
-        <v>1800</v>
+        <v>1808</v>
       </c>
       <c r="M2" t="n">
-        <v>1810.8</v>
+        <v>1818.2</v>
       </c>
       <c r="N2" t="n">
-        <v>1790</v>
+        <v>1796.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="P2" t="n">
-        <v>2894133</v>
+        <v>256879</v>
       </c>
       <c r="Q2" t="n">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="R2" t="n">
-        <v>1953.57</v>
+        <v>1954.83</v>
       </c>
       <c r="S2" t="n">
-        <v>1724.72</v>
+        <v>1725.59</v>
       </c>
       <c r="T2" t="n">
-        <v>8.471404775124928</v>
+        <v>8.481132075471693</v>
       </c>
       <c r="U2" t="n">
-        <v>152.5699999999999</v>
+        <v>152.8299999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.235424764019988</v>
+        <v>4.240288568257497</v>
       </c>
       <c r="W2" t="n">
-        <v>76.27999999999997</v>
+        <v>76.41000000000008</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000131095962244</v>
+        <v>2.000130872922389</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.471404775124928</v>
+        <v>8.481132075471693</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.235424764019988</v>
+        <v>4.240288568257497</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02055041729361061</v>
+        <v>0.02055030313440252</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3262277609849683</v>
+        <v>0.3262259487637214</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02916321742645627</v>
+        <v>0.02916321695826756</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249936603321</v>
+        <v>0.04306249530059571</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-24 16:20:35.114940+05:30</t>
+          <t>2026-08-25 09:33:17.167190+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.471404775124928, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000131095962244}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.481132075471693, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001308729223894}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-26 04:05 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="H2" t="n">
         <v>8.6</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.64</v>
+        <v>11.95</v>
       </c>
       <c r="R2" t="n">
-        <v>49.02</v>
+        <v>49.2</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,46 +1875,46 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1808</v>
+        <v>1871.1</v>
       </c>
       <c r="V2" t="n">
-        <v>1818.2</v>
+        <v>1883</v>
       </c>
       <c r="W2" t="n">
-        <v>1796.5</v>
+        <v>1857.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="Y2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="Z2" t="n">
-        <v>256879</v>
+        <v>404320</v>
       </c>
       <c r="AA2" t="n">
-        <v>1778006</v>
+        <v>1737202</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.33</v>
+        <v>0.26</v>
       </c>
       <c r="AE2" t="n">
-        <v>21.7</v>
+        <v>25.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.2</v>
+        <v>1.37</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.21</v>
+        <v>39.55</v>
       </c>
       <c r="AH2" t="n">
-        <v>38.21</v>
+        <v>39.55</v>
       </c>
       <c r="AI2" t="n">
         <v>2.12</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.89</v>
+        <v>2.3</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.36</v>
+        <v>13.16</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.37</v>
+        <v>50.82</v>
       </c>
       <c r="AO2" t="n">
-        <v>60</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.8</v>
+        <v>1.08</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.42</v>
+        <v>37.3</v>
       </c>
       <c r="AR2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="AS2" t="n">
-        <v>1954.83</v>
+        <v>2028.21</v>
       </c>
       <c r="AT2" t="n">
-        <v>1725.59</v>
+        <v>1790.9</v>
       </c>
       <c r="AU2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.48</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>152.83</v>
+        <v>158.21</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.24</v>
+        <v>4.23</v>
       </c>
       <c r="BA2" t="n">
-        <v>76.41</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.09</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,58 +1984,58 @@
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.1</v>
+        <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="BH2" t="n">
-        <v>17.5</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.5</v>
+        <v>50.2</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.880000000000001</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.25</v>
+        <v>-4.29</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.246</v>
+        <v>0.249</v>
       </c>
       <c r="BT2" t="n">
-        <v>1478.36</v>
+        <v>1494.36</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.7</v>
+        <v>-13.34</v>
       </c>
       <c r="BV2" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="BW2" t="n">
         <v>2.05</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>2.09</v>
       </c>
       <c r="BX2" t="n">
         <v>2.0001</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45</v>
+        <v>45.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>52.5</v>
+        <v>53.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>69.7</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.7</v>
+        <v>71.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>68.59999999999999</v>
+        <v>91.88</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.33</v>
+        <v>57.53</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.4811</v>
+        <v>8.4604</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5653</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2827</v>
+        <v>0.282</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0848</v>
+        <v>0.08459999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>0.9871</v>
+        <v>1.011</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9906</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2403</v>
+        <v>4.2299</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.48</v>
+        <v>38.29</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2403</v>
+        <v>4.2299</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
+        <v>1.9953</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>3.9906</v>
+      </c>
+      <c r="DO2" t="n">
         <v>2</v>
-      </c>
-      <c r="DN2" t="n">
-        <v>4</v>
-      </c>
-      <c r="DO2" t="n">
-        <v>1.9996</v>
       </c>
       <c r="DP2" t="n">
         <v>0.9434</v>
       </c>
       <c r="DQ2" t="n">
-        <v>76.41</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>45.7</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-1.3208</v>
+        <v>0.5094</v>
       </c>
       <c r="DX2" t="n">
-        <v>100</v>
+        <v>78.72499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>7</v>
+        <v>11.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>71.992</v>
+        <v>83.94199999999999</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>51.03</v>
+        <v>68.97</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>73.16</v>
       </c>
       <c r="EE2" t="n">
-        <v>-1.3208</v>
+        <v>0.5094</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.3259</v>
+        <v>0.1291</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0005</v>
+        <v>3.9908</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0379</v>
+        <v>0.0154</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7635</v>
+        <v>0.7631</v>
       </c>
       <c r="EK2" t="n">
-        <v>62.82</v>
+        <v>71.73</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,78 +2243,78 @@
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>20.97</v>
+        <v>65.27</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.4409</v>
+        <v>7.7998</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0163</v>
+        <v>0.0275</v>
       </c>
       <c r="ER2" t="n">
-        <v>60.5714</v>
+        <v>36.7826</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.0128</v>
+        <v>12.2724</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.311</v>
+        <v>61.916</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.392</v>
+        <v>0.2484</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8596</v>
+        <v>1.7236</v>
       </c>
       <c r="EW2" t="n">
-        <v>14.3854</v>
+        <v>59.9701</v>
       </c>
       <c r="EX2" t="n">
-        <v>31.07</v>
+        <v>64.13</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.96</v>
+        <v>64.41</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.59</v>
+        <v>30.54</v>
       </c>
       <c r="FD2" t="n">
-        <v>75.40000000000001</v>
+        <v>73.45999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>65.70999999999999</v>
+        <v>81.80500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>35.7</v>
+        <v>60.83</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.9872</v>
+        <v>29.4487</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.274</v>
+        <v>72.595</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.59</v>
+        <v>51.235</v>
       </c>
       <c r="FJ2" t="n">
-        <v>64.81</v>
+        <v>73.41</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>63.82</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.44</v>
+        <v>67.83</v>
       </c>
       <c r="FP2" t="n">
-        <v>49.89</v>
+        <v>81.79000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>65.84999999999999</v>
+        <v>72.91</v>
       </c>
       <c r="FR2" t="n">
-        <v>70.72</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>60.799</v>
+        <v>73.71250000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260825_093317</t>
+          <t>20260826_093554</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46259.3981150408</v>
+        <v>46260.39993505009</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46259.39811342592</v>
+        <v>46260.39993055556</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.64</v>
+        <v>11.95</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="L2" t="n">
-        <v>1808</v>
+        <v>1871.1</v>
       </c>
       <c r="M2" t="n">
-        <v>1818.2</v>
+        <v>1883</v>
       </c>
       <c r="N2" t="n">
-        <v>1796.5</v>
+        <v>1857.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="P2" t="n">
-        <v>256879</v>
+        <v>404320</v>
       </c>
       <c r="Q2" t="n">
-        <v>1802</v>
+        <v>1870</v>
       </c>
       <c r="R2" t="n">
-        <v>1954.83</v>
+        <v>2028.21</v>
       </c>
       <c r="S2" t="n">
-        <v>1725.59</v>
+        <v>1790.9</v>
       </c>
       <c r="T2" t="n">
-        <v>8.481132075471693</v>
+        <v>8.460427807486633</v>
       </c>
       <c r="U2" t="n">
-        <v>152.8299999999999</v>
+        <v>158.21</v>
       </c>
       <c r="V2" t="n">
-        <v>4.240288568257497</v>
+        <v>4.229946524064166</v>
       </c>
       <c r="W2" t="n">
-        <v>76.41000000000008</v>
+        <v>79.09999999999991</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000130872922389</v>
+        <v>2.000126422250319</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.481132075471693</v>
+        <v>8.460427807486633</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.240288568257497</v>
+        <v>4.229946524064166</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02055030313440252</v>
+        <v>0.02053522270817191</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3262259487637214</v>
+        <v>0.3259865544188951</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02916321695826756</v>
+        <v>0.02915033974461768</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249530059571</v>
+        <v>0.04306250302071769</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.9</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-25 09:33:17.167190+05:30</t>
+          <t>2026-08-26 09:35:54.421639+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.481132075471693, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001308729223894}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.460427807486633, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000126422250319}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-26 10:50 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.95</v>
+        <v>12</v>
       </c>
       <c r="R2" t="n">
-        <v>49.2</v>
+        <v>49.88</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>1871.1</v>
       </c>
       <c r="V2" t="n">
-        <v>1883</v>
+        <v>1898.3</v>
       </c>
       <c r="W2" t="n">
         <v>1857.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="Y2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="Z2" t="n">
-        <v>404320</v>
+        <v>3333619</v>
       </c>
       <c r="AA2" t="n">
-        <v>1737202</v>
+        <v>1883667</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.23</v>
+        <v>1.77</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.2</v>
+        <v>1.11</v>
       </c>
       <c r="AD2" t="n">
         <v>0.26</v>
       </c>
       <c r="AE2" t="n">
-        <v>25.6</v>
+        <v>40.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.37</v>
+        <v>2.17</v>
       </c>
       <c r="AG2" t="n">
-        <v>39.55</v>
+        <v>40.64</v>
       </c>
       <c r="AH2" t="n">
-        <v>39.55</v>
+        <v>40.64</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.12</v>
+        <v>2.15</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.3</v>
+        <v>3.18</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.16</v>
+        <v>14.16</v>
       </c>
       <c r="AN2" t="n">
-        <v>50.82</v>
+        <v>52.18</v>
       </c>
       <c r="AO2" t="n">
-        <v>68.51000000000001</v>
+        <v>70.22</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.08</v>
+        <v>2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>37.3</v>
+        <v>38.55</v>
       </c>
       <c r="AR2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="AS2" t="n">
-        <v>2028.21</v>
+        <v>2049.58</v>
       </c>
       <c r="AT2" t="n">
-        <v>1790.9</v>
+        <v>1805.71</v>
       </c>
       <c r="AU2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.460000000000001</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>158.21</v>
+        <v>162.58</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.23</v>
+        <v>4.31</v>
       </c>
       <c r="BA2" t="n">
-        <v>79.09999999999999</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,37 +1987,37 @@
         <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
         <v>657</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.2</v>
+        <v>50.4</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.779999999999999</v>
+        <v>8.76</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.29</v>
+        <v>-4.3</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
@@ -2026,19 +2026,19 @@
         <v>0.249</v>
       </c>
       <c r="BT2" t="n">
-        <v>1494.36</v>
+        <v>1498.89</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.34</v>
+        <v>-13.18</v>
       </c>
       <c r="BV2" t="n">
         <v>2.07</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.4</v>
+        <v>45.6</v>
       </c>
       <c r="CE2" t="n">
         <v>53.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.7</v>
+        <v>72</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>91.88</v>
+        <v>88.14</v>
       </c>
       <c r="CO2" t="n">
-        <v>57.53</v>
+        <v>50.25</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.4604</v>
+        <v>8.6158</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.5747</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.282</v>
+        <v>0.2873</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08459999999999999</v>
+        <v>0.0862</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.011</v>
+        <v>1.0344</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9906</v>
+        <v>4.0093</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2299</v>
+        <v>4.3079</v>
       </c>
       <c r="DJ2" t="n">
-        <v>38.29</v>
+        <v>37.9</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2299</v>
+        <v>4.3079</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9953</v>
+        <v>2.0047</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9906</v>
+        <v>4.0093</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9434</v>
+        <v>0.9302</v>
       </c>
       <c r="DQ2" t="n">
-        <v>79.09999999999999</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>64.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.5094</v>
+        <v>0.9302</v>
       </c>
       <c r="DX2" t="n">
-        <v>78.72499999999999</v>
+        <v>74.45</v>
       </c>
       <c r="DY2" t="n">
-        <v>11.5</v>
+        <v>88.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>83.94199999999999</v>
+        <v>84.40900000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>68.97</v>
+        <v>61.29</v>
       </c>
       <c r="ED2" t="n">
-        <v>73.16</v>
+        <v>64.98</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.5094</v>
+        <v>0.9302</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.23</v>
+        <v>1.77</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.1291</v>
+        <v>0.24</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9908</v>
+        <v>4.0073</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0154</v>
+        <v>0.0288</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7631</v>
+        <v>0.7547</v>
       </c>
       <c r="EK2" t="n">
-        <v>71.73</v>
+        <v>67.95</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>65.27</v>
+        <v>85.58</v>
       </c>
       <c r="EP2" t="n">
-        <v>7.7998</v>
+        <v>10.2696</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0275</v>
+        <v>0.2124</v>
       </c>
       <c r="ER2" t="n">
-        <v>36.7826</v>
+        <v>4.8701</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.2724</v>
+        <v>12.0317</v>
       </c>
       <c r="ET2" t="n">
-        <v>61.916</v>
+        <v>65.166</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.2484</v>
+        <v>3.54</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7236</v>
+        <v>0.7762</v>
       </c>
       <c r="EW2" t="n">
-        <v>59.9701</v>
+        <v>75.4302</v>
       </c>
       <c r="EX2" t="n">
-        <v>64.13</v>
+        <v>69.86</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.41</v>
+        <v>64.64</v>
       </c>
       <c r="FC2" t="n">
-        <v>30.54</v>
+        <v>29.77</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.45999999999999</v>
+        <v>73.5</v>
       </c>
       <c r="FE2" t="n">
-        <v>81.80500000000001</v>
+        <v>78.045</v>
       </c>
       <c r="FF2" t="n">
-        <v>60.83</v>
+        <v>60.055</v>
       </c>
       <c r="FG2" t="n">
-        <v>29.4487</v>
+        <v>27.981</v>
       </c>
       <c r="FH2" t="n">
-        <v>72.595</v>
+        <v>72.73399999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.235</v>
+        <v>54.045</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.41</v>
+        <v>72.23</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>78.59999999999999</v>
+        <v>79.02</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.83</v>
+        <v>64.54000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>81.79000000000001</v>
+        <v>85.95</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.91</v>
+        <v>74.43000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.31999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>73.71250000000001</v>
+        <v>74.8095</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260826_093554</t>
+          <t>20260826_162014</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46260.39993505009</v>
+        <v>46260.68072455253</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46260.39993055556</v>
+        <v>46260.68071759259</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46260</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.95</v>
+        <v>12</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="L2" t="n">
         <v>1871.1</v>
       </c>
       <c r="M2" t="n">
-        <v>1883</v>
+        <v>1898.3</v>
       </c>
       <c r="N2" t="n">
         <v>1857.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="P2" t="n">
-        <v>404320</v>
+        <v>3333619</v>
       </c>
       <c r="Q2" t="n">
-        <v>1870</v>
+        <v>1887</v>
       </c>
       <c r="R2" t="n">
-        <v>2028.21</v>
+        <v>2049.58</v>
       </c>
       <c r="S2" t="n">
-        <v>1790.9</v>
+        <v>1805.71</v>
       </c>
       <c r="T2" t="n">
-        <v>8.460427807486633</v>
+        <v>8.615792262851082</v>
       </c>
       <c r="U2" t="n">
-        <v>158.21</v>
+        <v>162.5799999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.229946524064166</v>
+        <v>4.307896131425541</v>
       </c>
       <c r="W2" t="n">
-        <v>79.09999999999991</v>
+        <v>81.28999999999996</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000126422250319</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.460427807486633</v>
+        <v>8.615792262851082</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.229946524064166</v>
+        <v>4.307896131425541</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02053522270817191</v>
+        <v>0.02056333973142376</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3259865544188951</v>
+        <v>0.326432898325686</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02915033974461768</v>
+        <v>0.02913744658262206</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306250302071769</v>
+        <v>0.04306249265824794</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.92</v>
+        <v>38.89</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-26 09:35:54.421639+05:30</t>
+          <t>2026-08-26 16:20:14.639570+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.460427807486633, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000126422250319}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.615792262851082, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-27 14:17 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,19 +1816,19 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="H2" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12</v>
+        <v>12.12</v>
       </c>
       <c r="R2" t="n">
-        <v>49.88</v>
+        <v>50.11</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,46 +1875,46 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1871.1</v>
+        <v>1891.3</v>
       </c>
       <c r="V2" t="n">
-        <v>1898.3</v>
+        <v>1930</v>
       </c>
       <c r="W2" t="n">
-        <v>1857.4</v>
+        <v>1878.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1887</v>
+        <v>1929.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>1887</v>
+        <v>1929.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>3333619</v>
+        <v>4248944</v>
       </c>
       <c r="AA2" t="n">
-        <v>1883667</v>
+        <v>1976032</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.77</v>
+        <v>2.15</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.11</v>
+        <v>2.25</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="AE2" t="n">
-        <v>40.9</v>
+        <v>51.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.17</v>
+        <v>2.67</v>
       </c>
       <c r="AG2" t="n">
-        <v>40.64</v>
+        <v>41.43</v>
       </c>
       <c r="AH2" t="n">
-        <v>40.64</v>
+        <v>41.43</v>
       </c>
       <c r="AI2" t="n">
         <v>2.15</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.18</v>
+        <v>5.08</v>
       </c>
       <c r="AM2" t="n">
-        <v>14.16</v>
+        <v>15.94</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.18</v>
+        <v>55.01</v>
       </c>
       <c r="AO2" t="n">
-        <v>70.22</v>
+        <v>74.01000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>2</v>
+        <v>4.2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.55</v>
+        <v>38.97</v>
       </c>
       <c r="AR2" t="n">
-        <v>1887</v>
+        <v>1929.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>2049.58</v>
+        <v>2095.11</v>
       </c>
       <c r="AT2" t="n">
-        <v>1805.71</v>
+        <v>1846.55</v>
       </c>
       <c r="AU2" t="n">
-        <v>1887</v>
+        <v>1929.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.619999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="AY2" t="n">
-        <v>162.58</v>
+        <v>165.71</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.31</v>
+        <v>4.29</v>
       </c>
       <c r="BA2" t="n">
-        <v>81.29000000000001</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -1978,19 +1978,19 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="BE2" t="n">
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49</v>
+        <v>48.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.28</v>
+        <v>2.3</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.76</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.3</v>
@@ -2023,22 +2023,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.249</v>
+        <v>0.251</v>
       </c>
       <c r="BT2" t="n">
-        <v>1498.89</v>
+        <v>1511.52</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.18</v>
+        <v>-12.89</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="BW2" t="n">
         <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2054,20 +2054,20 @@
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.6y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.7y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.6</v>
+        <v>46</v>
       </c>
       <c r="CE2" t="n">
-        <v>53.5</v>
+        <v>54</v>
       </c>
       <c r="CF2" t="n">
         <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>88.14</v>
+        <v>92.11</v>
       </c>
       <c r="CO2" t="n">
-        <v>50.25</v>
+        <v>54.53</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>80.95238095238095</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.6158</v>
+        <v>8.588699999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5747</v>
+        <v>0.5727</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2873</v>
+        <v>0.286</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0862</v>
+        <v>0.0859</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0023</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0344</v>
+        <v>1.0411</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0093</v>
+        <v>3.9953</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.3079</v>
+        <v>4.2941</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.9</v>
+        <v>34.91</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.3079</v>
+        <v>4.2941</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0047</v>
+        <v>1.9953</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0093</v>
+        <v>3.9953</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2.0024</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9302</v>
+        <v>0.9313</v>
       </c>
       <c r="DQ2" t="n">
-        <v>81.29000000000001</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>70.19</v>
+        <v>60.48</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9302</v>
+        <v>1.9535</v>
       </c>
       <c r="DX2" t="n">
-        <v>74.45</v>
+        <v>64.97499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>88.5</v>
+        <v>107.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.40900000000001</v>
+        <v>88.755</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>61.29</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>64.98</v>
+        <v>56.28</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9302</v>
+        <v>1.9535</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.77</v>
+        <v>2.15</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.24</v>
+        <v>0.509</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0073</v>
+        <v>3.9947</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0288</v>
+        <v>0.0617</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7547</v>
+        <v>0.7551</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.95</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>85.58</v>
+        <v>85.77</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.2696</v>
+        <v>10.3953</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.2124</v>
+        <v>0.2606</v>
       </c>
       <c r="ER2" t="n">
-        <v>4.8701</v>
+        <v>3.9953</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.0317</v>
+        <v>11.0825</v>
       </c>
       <c r="ET2" t="n">
-        <v>65.166</v>
+        <v>67.01600000000001</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.54</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.7762</v>
+        <v>0.6825</v>
       </c>
       <c r="EW2" t="n">
-        <v>75.4302</v>
+        <v>79.0027</v>
       </c>
       <c r="EX2" t="n">
-        <v>69.86</v>
+        <v>72.8</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.64</v>
+        <v>64.91</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.77</v>
+        <v>26.88</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.5</v>
+        <v>74.56999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.045</v>
+        <v>81.3</v>
       </c>
       <c r="FF2" t="n">
-        <v>60.055</v>
+        <v>63.665</v>
       </c>
       <c r="FG2" t="n">
-        <v>27.981</v>
+        <v>29.2413</v>
       </c>
       <c r="FH2" t="n">
-        <v>72.73399999999999</v>
+        <v>74.648</v>
       </c>
       <c r="FI2" t="n">
-        <v>54.045</v>
+        <v>47.695</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.23</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>79.02</v>
+        <v>81.75</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.54000000000001</v>
+        <v>68.34</v>
       </c>
       <c r="FP2" t="n">
-        <v>85.95</v>
+        <v>88.03</v>
       </c>
       <c r="FQ2" t="n">
         <v>74.43000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.3</v>
+        <v>90.75</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.8095</v>
+        <v>74.6815</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260826_162014</t>
+          <t>20260827_194717</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46260.68072455253</v>
+        <v>46261.82451270094</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46260.68071759259</v>
+        <v>46261.82450231481</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12</v>
+        <v>12.12</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1887</v>
+        <v>1929.4</v>
       </c>
       <c r="L2" t="n">
-        <v>1871.1</v>
+        <v>1891.3</v>
       </c>
       <c r="M2" t="n">
-        <v>1898.3</v>
+        <v>1930</v>
       </c>
       <c r="N2" t="n">
-        <v>1857.4</v>
+        <v>1878.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1887</v>
+        <v>1929.4</v>
       </c>
       <c r="P2" t="n">
-        <v>3333619</v>
+        <v>4248944</v>
       </c>
       <c r="Q2" t="n">
-        <v>1887</v>
+        <v>1929.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2049.58</v>
+        <v>2095.11</v>
       </c>
       <c r="S2" t="n">
-        <v>1805.71</v>
+        <v>1846.55</v>
       </c>
       <c r="T2" t="n">
-        <v>8.615792262851082</v>
+        <v>8.588680418783042</v>
       </c>
       <c r="U2" t="n">
-        <v>162.5799999999999</v>
+        <v>165.71</v>
       </c>
       <c r="V2" t="n">
-        <v>4.307896131425541</v>
+        <v>4.294081061469894</v>
       </c>
       <c r="W2" t="n">
-        <v>81.28999999999996</v>
+        <v>82.85000000000014</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000120700060347</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.615792262851082</v>
+        <v>8.588680418783042</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.307896131425541</v>
+        <v>4.294081061469894</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02056333973142376</v>
+        <v>0.02056230248623889</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.326432898325686</v>
+        <v>0.3264164325688394</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02913744658262206</v>
+        <v>0.02912454704128812</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249265824794</v>
+        <v>0.04306249094286813</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-26 16:20:14.639570+05:30</t>
+          <t>2026-08-27 19:47:17.935857+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.615792262851082, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.588680418783042, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001207000603474}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-27 20:23 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,19 +1816,19 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="H2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.12</v>
+        <v>12</v>
       </c>
       <c r="R2" t="n">
-        <v>50.11</v>
+        <v>49.88</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,46 +1875,46 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1891.3</v>
+        <v>1871.1</v>
       </c>
       <c r="V2" t="n">
-        <v>1930</v>
+        <v>1898.3</v>
       </c>
       <c r="W2" t="n">
-        <v>1878.4</v>
+        <v>1857.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1929.4</v>
+        <v>1887</v>
       </c>
       <c r="Y2" t="n">
-        <v>1929.4</v>
+        <v>1887</v>
       </c>
       <c r="Z2" t="n">
-        <v>4248944</v>
+        <v>3334188</v>
       </c>
       <c r="AA2" t="n">
-        <v>1976032</v>
+        <v>1883695</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.15</v>
+        <v>1.77</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.25</v>
+        <v>1.11</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.23</v>
+        <v>0.26</v>
       </c>
       <c r="AE2" t="n">
-        <v>51.6</v>
+        <v>40.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.67</v>
+        <v>2.17</v>
       </c>
       <c r="AG2" t="n">
-        <v>41.43</v>
+        <v>40.64</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.43</v>
+        <v>40.64</v>
       </c>
       <c r="AI2" t="n">
         <v>2.15</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.08</v>
+        <v>3.18</v>
       </c>
       <c r="AM2" t="n">
-        <v>15.94</v>
+        <v>14.16</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.01</v>
+        <v>52.18</v>
       </c>
       <c r="AO2" t="n">
-        <v>74.01000000000001</v>
+        <v>70.22</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.2</v>
+        <v>2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.97</v>
+        <v>38.55</v>
       </c>
       <c r="AR2" t="n">
-        <v>1929.4</v>
+        <v>1887</v>
       </c>
       <c r="AS2" t="n">
-        <v>2095.11</v>
+        <v>2049.58</v>
       </c>
       <c r="AT2" t="n">
-        <v>1846.55</v>
+        <v>1805.71</v>
       </c>
       <c r="AU2" t="n">
-        <v>1929.400024414062</v>
+        <v>1887</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.59</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>165.71</v>
+        <v>162.58</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.29</v>
+        <v>4.31</v>
       </c>
       <c r="BA2" t="n">
-        <v>82.84999999999999</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -1978,19 +1978,19 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.5</v>
+        <v>32.6</v>
       </c>
       <c r="BE2" t="n">
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.9</v>
+        <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.3</v>
+        <v>2.28</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.779999999999999</v>
+        <v>8.76</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.3</v>
@@ -2023,22 +2023,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.251</v>
+        <v>0.249</v>
       </c>
       <c r="BT2" t="n">
-        <v>1511.52</v>
+        <v>1498.89</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.89</v>
+        <v>-13.18</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="BW2" t="n">
         <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2054,20 +2054,20 @@
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.7y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.6y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>46</v>
+        <v>45.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>54</v>
+        <v>53.5</v>
       </c>
       <c r="CF2" t="n">
         <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.09999999999999</v>
+        <v>72</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>92.11</v>
+        <v>88.14</v>
       </c>
       <c r="CO2" t="n">
-        <v>54.53</v>
+        <v>50.23</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>90.47619047619048</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>90.47619047619048</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>80.95238095238095</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.588699999999999</v>
+        <v>8.6158</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5727</v>
+        <v>0.5747</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.286</v>
+        <v>0.2873</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0859</v>
+        <v>0.0862</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0023</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0411</v>
+        <v>1.0344</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9953</v>
+        <v>4.0093</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2941</v>
+        <v>4.3079</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.91</v>
+        <v>37.9</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2941</v>
+        <v>4.3079</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9953</v>
+        <v>2.0047</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9953</v>
+        <v>4.0093</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0024</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9313</v>
+        <v>0.9302</v>
       </c>
       <c r="DQ2" t="n">
-        <v>82.84999999999999</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>60.48</v>
+        <v>70.19</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.9535</v>
+        <v>0.9302</v>
       </c>
       <c r="DX2" t="n">
-        <v>64.97499999999999</v>
+        <v>74.45</v>
       </c>
       <c r="DY2" t="n">
-        <v>107.5</v>
+        <v>88.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.755</v>
+        <v>84.40900000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>67.26000000000001</v>
+        <v>61.29</v>
       </c>
       <c r="ED2" t="n">
-        <v>56.28</v>
+        <v>64.98</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.9535</v>
+        <v>0.9302</v>
       </c>
       <c r="EF2" t="n">
-        <v>2.15</v>
+        <v>1.77</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.509</v>
+        <v>0.24</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9947</v>
+        <v>4.0073</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0617</v>
+        <v>0.0288</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7551</v>
+        <v>0.7547</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.48999999999999</v>
+        <v>67.95</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>85.77</v>
+        <v>85.58</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.3953</v>
+        <v>10.2696</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.2606</v>
+        <v>0.2124</v>
       </c>
       <c r="ER2" t="n">
-        <v>3.9953</v>
+        <v>4.8701</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.0825</v>
+        <v>12.0317</v>
       </c>
       <c r="ET2" t="n">
-        <v>67.01600000000001</v>
+        <v>65.158</v>
       </c>
       <c r="EU2" t="n">
-        <v>9.029999999999999</v>
+        <v>3.54</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.6825</v>
+        <v>0.7762</v>
       </c>
       <c r="EW2" t="n">
-        <v>79.0027</v>
+        <v>75.4302</v>
       </c>
       <c r="EX2" t="n">
-        <v>72.8</v>
+        <v>69.86</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.91</v>
+        <v>64.64</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.88</v>
+        <v>29.77</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.56999999999999</v>
+        <v>73.5</v>
       </c>
       <c r="FE2" t="n">
-        <v>81.3</v>
+        <v>78.045</v>
       </c>
       <c r="FF2" t="n">
-        <v>63.665</v>
+        <v>60.045</v>
       </c>
       <c r="FG2" t="n">
-        <v>29.2413</v>
+        <v>27.981</v>
       </c>
       <c r="FH2" t="n">
-        <v>74.648</v>
+        <v>72.73399999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>47.695</v>
+        <v>54.045</v>
       </c>
       <c r="FJ2" t="n">
-        <v>74.98999999999999</v>
+        <v>72.23</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.75</v>
+        <v>79.02</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.34</v>
+        <v>64.54000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>88.03</v>
+        <v>85.95</v>
       </c>
       <c r="FQ2" t="n">
         <v>74.43000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>90.75</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.6815</v>
+        <v>74.7795</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260827_194717</t>
+          <t>20260828_015344</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46261.82451270094</v>
+        <v>46262.07898149439</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46261.82450231481</v>
+        <v>46262.07898148148</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.12</v>
+        <v>12</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1929.4</v>
+        <v>1887</v>
       </c>
       <c r="L2" t="n">
-        <v>1891.3</v>
+        <v>1871.1</v>
       </c>
       <c r="M2" t="n">
-        <v>1930</v>
+        <v>1898.3</v>
       </c>
       <c r="N2" t="n">
-        <v>1878.4</v>
+        <v>1857.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1929.4</v>
+        <v>1887</v>
       </c>
       <c r="P2" t="n">
-        <v>4248944</v>
+        <v>3334188</v>
       </c>
       <c r="Q2" t="n">
-        <v>1929.4</v>
+        <v>1887</v>
       </c>
       <c r="R2" t="n">
-        <v>2095.11</v>
+        <v>2049.58</v>
       </c>
       <c r="S2" t="n">
-        <v>1846.55</v>
+        <v>1805.71</v>
       </c>
       <c r="T2" t="n">
-        <v>8.588680418783042</v>
+        <v>8.615792262851082</v>
       </c>
       <c r="U2" t="n">
-        <v>165.71</v>
+        <v>162.5799999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.294081061469894</v>
+        <v>4.307896131425541</v>
       </c>
       <c r="W2" t="n">
-        <v>82.85000000000014</v>
+        <v>81.28999999999996</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000120700060347</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.588680418783042</v>
+        <v>8.615792262851082</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.294081061469894</v>
+        <v>4.307896131425541</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02056230248623889</v>
+        <v>0.02056333970456911</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3264164325688394</v>
+        <v>0.3264328978993817</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02912454704128812</v>
+        <v>0.0291374370136146</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249094286813</v>
+        <v>0.04306249456427596</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:47:17.935857+05:30</t>
+          <t>2026-08-28 01:53:44.043931+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.588680418783042, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001207000603474}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.615792262851082, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-28 15:27 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,19 +1816,19 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H2" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12</v>
+        <v>12.12</v>
       </c>
       <c r="R2" t="n">
-        <v>49.88</v>
+        <v>49.74</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1871.1</v>
+        <v>1929.7</v>
       </c>
       <c r="V2" t="n">
-        <v>1898.3</v>
+        <v>1938.5</v>
       </c>
       <c r="W2" t="n">
-        <v>1857.4</v>
+        <v>1910.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>3334188</v>
+        <v>2230824</v>
       </c>
       <c r="AA2" t="n">
-        <v>1883695</v>
+        <v>1962491</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.77</v>
+        <v>1.14</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.11</v>
+        <v>0.47</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.26</v>
+        <v>0.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>40.9</v>
+        <v>28.4</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.17</v>
+        <v>1.47</v>
       </c>
       <c r="AG2" t="n">
-        <v>40.64</v>
+        <v>40.5</v>
       </c>
       <c r="AH2" t="n">
-        <v>40.64</v>
+        <v>40.5</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.15</v>
+        <v>2.09</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.18</v>
+        <v>5.22</v>
       </c>
       <c r="AM2" t="n">
-        <v>14.16</v>
+        <v>15.76</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.18</v>
+        <v>55.15</v>
       </c>
       <c r="AO2" t="n">
-        <v>70.22</v>
+        <v>74.76000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>2</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.55</v>
+        <v>40.21</v>
       </c>
       <c r="AR2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2049.58</v>
+        <v>2100.49</v>
       </c>
       <c r="AT2" t="n">
-        <v>1805.71</v>
+        <v>1857.51</v>
       </c>
       <c r="AU2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.619999999999999</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>162.58</v>
+        <v>161.99</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.31</v>
+        <v>4.18</v>
       </c>
       <c r="BA2" t="n">
-        <v>81.29000000000001</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -1978,19 +1978,19 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="BE2" t="n">
         <v>322</v>
       </c>
       <c r="BF2" t="n">
-        <v>49</v>
+        <v>48.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.7</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,13 +2005,13 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.28</v>
+        <v>2.3</v>
       </c>
       <c r="BP2" t="n">
         <v>8.76</v>
@@ -2023,22 +2023,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.249</v>
+        <v>0.251</v>
       </c>
       <c r="BT2" t="n">
-        <v>1498.89</v>
+        <v>1514.5</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.18</v>
+        <v>-12.98</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="BW2" t="n">
         <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2054,20 +2054,20 @@
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.6y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.7y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>45.6</v>
+        <v>46</v>
       </c>
       <c r="CE2" t="n">
-        <v>53.5</v>
+        <v>54</v>
       </c>
       <c r="CF2" t="n">
         <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>88.14</v>
+        <v>87.31</v>
       </c>
       <c r="CO2" t="n">
-        <v>50.23</v>
+        <v>44.71</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.6158</v>
+        <v>8.3565</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5747</v>
+        <v>0.5573</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2873</v>
+        <v>0.2787</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0862</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0344</v>
+        <v>1.0132</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0093</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.3079</v>
+        <v>4.178</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.9</v>
+        <v>31.84</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.3079</v>
+        <v>4.178</v>
       </c>
       <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2.0047</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0093</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9996</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9302</v>
+        <v>0.9569</v>
       </c>
       <c r="DQ2" t="n">
-        <v>81.29000000000001</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>70.19</v>
+        <v>45.34</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9302</v>
+        <v>4.0478</v>
       </c>
       <c r="DX2" t="n">
-        <v>74.45</v>
+        <v>63.09999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>88.5</v>
+        <v>57</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.40900000000001</v>
+        <v>87.50700000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>61.29</v>
+        <v>73.18000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>64.98</v>
+        <v>42.14</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9302</v>
+        <v>4.0478</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.77</v>
+        <v>1.14</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.24</v>
+        <v>1.0254</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0073</v>
+        <v>3.9983</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0288</v>
+        <v>0.1243</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7547</v>
+        <v>0.7719</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.95</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>85.58</v>
+        <v>55.53</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.2696</v>
+        <v>6.7302</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.2124</v>
+        <v>0.1382</v>
       </c>
       <c r="ER2" t="n">
-        <v>4.8701</v>
+        <v>7.3333</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.0317</v>
+        <v>10.3042</v>
       </c>
       <c r="ET2" t="n">
-        <v>65.158</v>
+        <v>54.103</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.54</v>
+        <v>9.644399999999999</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.7762</v>
+        <v>0.9766</v>
       </c>
       <c r="EW2" t="n">
-        <v>75.4302</v>
+        <v>48.4832</v>
       </c>
       <c r="EX2" t="n">
-        <v>69.86</v>
+        <v>64.5</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.64</v>
+        <v>65.2</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.77</v>
+        <v>24.15</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.5</v>
+        <v>73.05</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.045</v>
+        <v>77.91</v>
       </c>
       <c r="FF2" t="n">
-        <v>60.045</v>
+        <v>54.605</v>
       </c>
       <c r="FG2" t="n">
-        <v>27.981</v>
+        <v>28.2557</v>
       </c>
       <c r="FH2" t="n">
-        <v>72.73399999999999</v>
+        <v>71.693</v>
       </c>
       <c r="FI2" t="n">
-        <v>54.045</v>
+        <v>38.59</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.23</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>79.02</v>
+        <v>75.20999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.54000000000001</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>85.95</v>
+        <v>78.28</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.43000000000001</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.23999999999999</v>
+        <v>88.29000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.7795</v>
+        <v>69.874</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260828_015344</t>
+          <t>20260828_205717</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46262.07898149439</v>
+        <v>46262.87312362779</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46262.07898148148</v>
+        <v>46262.87311342593</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46275</v>
+        <v>46277</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12</v>
+        <v>12.12</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="L2" t="n">
-        <v>1871.1</v>
+        <v>1929.7</v>
       </c>
       <c r="M2" t="n">
-        <v>1898.3</v>
+        <v>1938.5</v>
       </c>
       <c r="N2" t="n">
-        <v>1857.4</v>
+        <v>1910.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="P2" t="n">
-        <v>3334188</v>
+        <v>2230824</v>
       </c>
       <c r="Q2" t="n">
-        <v>1887</v>
+        <v>1938.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2049.58</v>
+        <v>2100.49</v>
       </c>
       <c r="S2" t="n">
-        <v>1805.71</v>
+        <v>1857.51</v>
       </c>
       <c r="T2" t="n">
-        <v>8.615792262851082</v>
+        <v>8.356461181325756</v>
       </c>
       <c r="U2" t="n">
-        <v>162.5799999999999</v>
+        <v>161.9899999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>4.307896131425541</v>
+        <v>4.177972659272633</v>
       </c>
       <c r="W2" t="n">
-        <v>81.28999999999996</v>
+        <v>80.99000000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000123472033581</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
-        <v>13.33333333333333</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.615792262851082</v>
+        <v>8.356461181325756</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.307896131425541</v>
+        <v>4.177972659272633</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02056333970456911</v>
+        <v>0.02054731058357317</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3264328978993817</v>
+        <v>0.3261784434920403</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0291374370136146</v>
+        <v>0.02911165716259938</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249456427596</v>
+        <v>0.04306249537827869</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.89</v>
+        <v>38.91</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-28 01:53:44.043931+05:30</t>
+          <t>2026-08-28 20:57:17.909337+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.615792262851082, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.356461181325756, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001234720335814}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-28 21:11 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1864,7 +1864,7 @@
         <v>12.12</v>
       </c>
       <c r="R2" t="n">
-        <v>49.74</v>
+        <v>50.11</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1929.7</v>
+        <v>1891.3</v>
       </c>
       <c r="V2" t="n">
-        <v>1938.5</v>
+        <v>1930</v>
       </c>
       <c r="W2" t="n">
-        <v>1910.1</v>
+        <v>1878.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1938.5</v>
+        <v>1929.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>1938.5</v>
+        <v>1929.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>2230824</v>
+        <v>4249869</v>
       </c>
       <c r="AA2" t="n">
-        <v>1962491</v>
+        <v>1976079</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.14</v>
+        <v>2.15</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.47</v>
+        <v>2.25</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.02</v>
+        <v>0.23</v>
       </c>
       <c r="AE2" t="n">
-        <v>28.4</v>
+        <v>51.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.47</v>
+        <v>2.67</v>
       </c>
       <c r="AG2" t="n">
-        <v>40.5</v>
+        <v>41.43</v>
       </c>
       <c r="AH2" t="n">
-        <v>40.5</v>
+        <v>41.43</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.09</v>
+        <v>2.15</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.22</v>
+        <v>5.08</v>
       </c>
       <c r="AM2" t="n">
-        <v>15.76</v>
+        <v>15.94</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.15</v>
+        <v>55.01</v>
       </c>
       <c r="AO2" t="n">
-        <v>74.76000000000001</v>
+        <v>74.01000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>8.460000000000001</v>
+        <v>4.2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.21</v>
+        <v>38.97</v>
       </c>
       <c r="AR2" t="n">
-        <v>1938.5</v>
+        <v>1929.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>2100.49</v>
+        <v>2095.11</v>
       </c>
       <c r="AT2" t="n">
-        <v>1857.51</v>
+        <v>1846.55</v>
       </c>
       <c r="AU2" t="n">
-        <v>1938.5</v>
+        <v>1929.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.359999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="AY2" t="n">
-        <v>161.99</v>
+        <v>165.71</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.18</v>
+        <v>4.29</v>
       </c>
       <c r="BA2" t="n">
-        <v>80.98999999999999</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -1987,10 +1987,10 @@
         <v>48.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.7</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,7 +2005,7 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="BN2" t="n">
         <v>50.5</v>
@@ -2014,7 +2014,7 @@
         <v>2.3</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.76</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.3</v>
@@ -2026,10 +2026,10 @@
         <v>0.251</v>
       </c>
       <c r="BT2" t="n">
-        <v>1514.5</v>
+        <v>1511.51</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.98</v>
+        <v>-12.89</v>
       </c>
       <c r="BV2" t="n">
         <v>2.08</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.31</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.71</v>
+        <v>54.44</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.3565</v>
+        <v>8.588699999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5573</v>
+        <v>0.5727</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.2787</v>
+        <v>0.286</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.08359999999999999</v>
+        <v>0.0859</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0023</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0132</v>
+        <v>1.0411</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9953</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.178</v>
+        <v>4.2941</v>
       </c>
       <c r="DJ2" t="n">
-        <v>31.84</v>
+        <v>34.87</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.178</v>
+        <v>4.2941</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9953</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9953</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9996</v>
+        <v>2.0024</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9569</v>
+        <v>0.9313</v>
       </c>
       <c r="DQ2" t="n">
-        <v>80.98999999999999</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>45.34</v>
+        <v>60.01</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>4.0478</v>
+        <v>1.9535</v>
       </c>
       <c r="DX2" t="n">
-        <v>63.09999999999999</v>
+        <v>64.97499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>57</v>
+        <v>107.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.50700000000001</v>
+        <v>88.389</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>73.18000000000001</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>42.14</v>
+        <v>56.23</v>
       </c>
       <c r="EE2" t="n">
-        <v>4.0478</v>
+        <v>1.9535</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.14</v>
+        <v>2.15</v>
       </c>
       <c r="EG2" t="n">
-        <v>1.0254</v>
+        <v>0.509</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9983</v>
+        <v>3.9947</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1243</v>
+        <v>0.0617</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7719</v>
+        <v>0.7551</v>
       </c>
       <c r="EK2" t="n">
-        <v>68.51000000000001</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>55.53</v>
+        <v>85.92</v>
       </c>
       <c r="EP2" t="n">
-        <v>6.7302</v>
+        <v>10.4135</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1382</v>
+        <v>0.2606</v>
       </c>
       <c r="ER2" t="n">
-        <v>7.3333</v>
+        <v>3.9953</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.3042</v>
+        <v>11.0698</v>
       </c>
       <c r="ET2" t="n">
-        <v>54.103</v>
+        <v>67.11199999999999</v>
       </c>
       <c r="EU2" t="n">
-        <v>9.644399999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.9766</v>
+        <v>0.6825</v>
       </c>
       <c r="EW2" t="n">
-        <v>48.4832</v>
+        <v>78.70269999999999</v>
       </c>
       <c r="EX2" t="n">
-        <v>64.5</v>
+        <v>72.78</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2293,28 +2293,28 @@
         <v>65.2</v>
       </c>
       <c r="FC2" t="n">
-        <v>24.15</v>
+        <v>26.82</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.05</v>
+        <v>73.02</v>
       </c>
       <c r="FE2" t="n">
-        <v>77.91</v>
+        <v>80.53</v>
       </c>
       <c r="FF2" t="n">
-        <v>54.605</v>
+        <v>63.61</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.2557</v>
+        <v>29.0794</v>
       </c>
       <c r="FH2" t="n">
-        <v>71.693</v>
+        <v>74.636</v>
       </c>
       <c r="FI2" t="n">
-        <v>38.59</v>
+        <v>47.44</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.76000000000001</v>
+        <v>74.13</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>75.20999999999999</v>
+        <v>80.34999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.98999999999999</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>78.28</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.01000000000001</v>
+        <v>74.17</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.29000000000001</v>
+        <v>90.31</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.874</v>
+        <v>74.21299999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260828_205717</t>
+          <t>20260829_024116</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46262.87312362779</v>
+        <v>46263.11199287001</v>
       </c>
     </row>
   </sheetData>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46262.87311342593</v>
+        <v>46263.11199074074</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1938.5</v>
+        <v>1929.4</v>
       </c>
       <c r="L2" t="n">
-        <v>1929.7</v>
+        <v>1891.3</v>
       </c>
       <c r="M2" t="n">
-        <v>1938.5</v>
+        <v>1930</v>
       </c>
       <c r="N2" t="n">
-        <v>1910.1</v>
+        <v>1878.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1938.5</v>
+        <v>1929.4</v>
       </c>
       <c r="P2" t="n">
-        <v>2230824</v>
+        <v>4249869</v>
       </c>
       <c r="Q2" t="n">
-        <v>1938.5</v>
+        <v>1929.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2100.49</v>
+        <v>2095.11</v>
       </c>
       <c r="S2" t="n">
-        <v>1857.51</v>
+        <v>1846.55</v>
       </c>
       <c r="T2" t="n">
-        <v>8.356461181325756</v>
+        <v>8.588680418783042</v>
       </c>
       <c r="U2" t="n">
-        <v>161.9899999999998</v>
+        <v>165.71</v>
       </c>
       <c r="V2" t="n">
-        <v>4.177972659272633</v>
+        <v>4.294081061469894</v>
       </c>
       <c r="W2" t="n">
-        <v>80.99000000000001</v>
+        <v>82.85000000000014</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000123472033581</v>
+        <v>2.000120700060347</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.356461181325756</v>
+        <v>8.588680418783042</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.177972659272633</v>
+        <v>4.294081061469894</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02054731058357317</v>
+        <v>0.02056230533056749</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3261784434920403</v>
+        <v>0.3264164777211562</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02911165716259938</v>
+        <v>0.02912455360790231</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249537827869</v>
+        <v>0.04306249899704509</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.91</v>
+        <v>38.89</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-28 20:57:17.909337+05:30</t>
+          <t>2026-08-29 02:41:16.222243+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.356461181325756, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001234720335814}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.588680418783042, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001207000603474}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-31 09:50 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.12</v>
+        <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>50.11</v>
+        <v>49.71</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1891.3</v>
+        <v>1945</v>
       </c>
       <c r="V2" t="n">
-        <v>1930</v>
+        <v>1949</v>
       </c>
       <c r="W2" t="n">
-        <v>1878.4</v>
+        <v>1847.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1929.4</v>
+        <v>1862.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>1929.4</v>
+        <v>1862.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>4249869</v>
+        <v>7154018</v>
       </c>
       <c r="AA2" t="n">
-        <v>1976079</v>
+        <v>2224255</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.15</v>
+        <v>3.22</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.25</v>
+        <v>-3.91</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.23</v>
+        <v>0.34</v>
       </c>
       <c r="AE2" t="n">
-        <v>51.6</v>
+        <v>101.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.67</v>
+        <v>5.43</v>
       </c>
       <c r="AG2" t="n">
-        <v>41.43</v>
+        <v>44.83</v>
       </c>
       <c r="AH2" t="n">
-        <v>41.43</v>
+        <v>44.83</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.15</v>
+        <v>2.41</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,71 +1926,71 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.08</v>
+        <v>0.97</v>
       </c>
       <c r="AM2" t="n">
-        <v>15.94</v>
+        <v>10.67</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.01</v>
+        <v>48.58</v>
       </c>
       <c r="AO2" t="n">
-        <v>74.01000000000001</v>
+        <v>59.52</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.2</v>
+        <v>2.93</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.97</v>
+        <v>33.6</v>
       </c>
       <c r="AR2" t="n">
-        <v>1929.4</v>
+        <v>1862.8</v>
       </c>
       <c r="AS2" t="n">
-        <v>2095.11</v>
+        <v>2042.13</v>
       </c>
       <c r="AT2" t="n">
-        <v>1846.55</v>
+        <v>1773.13</v>
       </c>
       <c r="AU2" t="n">
-        <v>1929.400024414062</v>
+        <v>1862.800048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>8.59</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>165.71</v>
+        <v>179.33</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.29</v>
+        <v>4.81</v>
       </c>
       <c r="BA2" t="n">
-        <v>82.84999999999999</v>
+        <v>89.67</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.5</v>
+        <v>32.4</v>
       </c>
       <c r="BE2" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.9</v>
+        <v>49.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>18.2</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,40 +2005,40 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.5</v>
+        <v>50</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.3</v>
+        <v>2.24</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.779999999999999</v>
+        <v>8.77</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.3</v>
+        <v>-4.28</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.251</v>
+        <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1511.51</v>
+        <v>1480.71</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.89</v>
+        <v>-13.83</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.08</v>
+        <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>46</v>
+        <v>44.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>54</v>
+        <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.09999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>91.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="CO2" t="n">
-        <v>54.44</v>
+        <v>59.69</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,7 +2115,7 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>8.588699999999999</v>
+        <v>9.626899999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.5727</v>
+        <v>0.642</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.286</v>
+        <v>0.3207</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0859</v>
+        <v>0.0963</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0023</v>
+        <v>2.0021</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0411</v>
+        <v>1.1335</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9953</v>
+        <v>3.9959</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.2941</v>
+        <v>4.8137</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.87</v>
+        <v>37.73</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.2941</v>
+        <v>4.8137</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9953</v>
+        <v>1.9959</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9953</v>
+        <v>3.9959</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0024</v>
+        <v>2.0019</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.9313</v>
+        <v>0.8307</v>
       </c>
       <c r="DQ2" t="n">
-        <v>82.84999999999999</v>
+        <v>89.67</v>
       </c>
       <c r="DR2" t="n">
-        <v>60.01</v>
+        <v>55.37</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.9535</v>
+        <v>1.2158</v>
       </c>
       <c r="DX2" t="n">
-        <v>64.97499999999999</v>
+        <v>98.80000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>107.5</v>
+        <v>161</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.389</v>
+        <v>80.99299999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>65.98999999999999</v>
+        <v>65.12</v>
       </c>
       <c r="ED2" t="n">
-        <v>56.23</v>
+        <v>99.39</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.9535</v>
+        <v>1.2158</v>
       </c>
       <c r="EF2" t="n">
-        <v>2.15</v>
+        <v>3.22</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.509</v>
+        <v>0.3449</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9947</v>
+        <v>3.9946</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0617</v>
+        <v>0.0406</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7551</v>
+        <v>0.6875</v>
       </c>
       <c r="EK2" t="n">
-        <v>69.45999999999999</v>
+        <v>77.28</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>85.92</v>
+        <v>70.37</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.4135</v>
+        <v>8.282500000000001</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.2606</v>
+        <v>0.379</v>
       </c>
       <c r="ER2" t="n">
-        <v>3.9953</v>
+        <v>2.9907</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.0698</v>
+        <v>11.0645</v>
       </c>
       <c r="ET2" t="n">
-        <v>67.11199999999999</v>
+        <v>64.05500000000001</v>
       </c>
       <c r="EU2" t="n">
-        <v>9.029999999999999</v>
+        <v>9.4346</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.6825</v>
+        <v>0.5711000000000001</v>
       </c>
       <c r="EW2" t="n">
-        <v>78.70269999999999</v>
+        <v>64.52930000000001</v>
       </c>
       <c r="EX2" t="n">
-        <v>72.78</v>
+        <v>74.23</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>65.2</v>
+        <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.82</v>
+        <v>29.94</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.02</v>
+        <v>73.36</v>
       </c>
       <c r="FE2" t="n">
-        <v>80.53</v>
+        <v>84.48999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>63.61</v>
+        <v>66.95999999999999</v>
       </c>
       <c r="FG2" t="n">
-        <v>29.0794</v>
+        <v>26.8915</v>
       </c>
       <c r="FH2" t="n">
-        <v>74.636</v>
+        <v>74.136</v>
       </c>
       <c r="FI2" t="n">
-        <v>47.44</v>
+        <v>46.55</v>
       </c>
       <c r="FJ2" t="n">
-        <v>74.13</v>
+        <v>74.98</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>80.34999999999999</v>
+        <v>80.45</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.20999999999999</v>
+        <v>71.78</v>
       </c>
       <c r="FP2" t="n">
-        <v>87.79000000000001</v>
+        <v>83.39</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.17</v>
+        <v>70.77</v>
       </c>
       <c r="FR2" t="n">
-        <v>90.31</v>
+        <v>94.62</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.21299999999999</v>
+        <v>76.271</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260829_024116</t>
+          <t>20260831_152045</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46263.11199287001</v>
+        <v>46265.6394103549</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46263.11199074074</v>
+        <v>46265.63940972222</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>12.12</v>
+        <v>11.77</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1929.4</v>
+        <v>1862.8</v>
       </c>
       <c r="L2" t="n">
-        <v>1891.3</v>
+        <v>1945</v>
       </c>
       <c r="M2" t="n">
-        <v>1930</v>
+        <v>1949</v>
       </c>
       <c r="N2" t="n">
-        <v>1878.4</v>
+        <v>1847.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1929.4</v>
+        <v>1862.8</v>
       </c>
       <c r="P2" t="n">
-        <v>4249869</v>
+        <v>7154018</v>
       </c>
       <c r="Q2" t="n">
-        <v>1929.4</v>
+        <v>1862.8</v>
       </c>
       <c r="R2" t="n">
-        <v>2095.11</v>
+        <v>2042.13</v>
       </c>
       <c r="S2" t="n">
-        <v>1846.55</v>
+        <v>1773.13</v>
       </c>
       <c r="T2" t="n">
-        <v>8.588680418783042</v>
+        <v>9.62690573330471</v>
       </c>
       <c r="U2" t="n">
-        <v>165.71</v>
+        <v>179.3300000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>4.294081061469894</v>
+        <v>4.81372127979385</v>
       </c>
       <c r="W2" t="n">
-        <v>82.85000000000014</v>
+        <v>89.66999999999985</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000120700060347</v>
+        <v>1.999888479982162</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
-        <v>13.33333333333333</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>8.588680418783042</v>
+        <v>9.62690573330471</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.294081061469894</v>
+        <v>4.81372127979385</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02056230533056749</v>
+        <v>0.02059425290637167</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3264164777211562</v>
+        <v>0.3269236297645716</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02912455360790231</v>
+        <v>0.02935663033654778</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04306249899704509</v>
+        <v>0.04294788444710936</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347613</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.89</v>
+        <v>38.85</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 02:41:16.222243+05:30</t>
+          <t>2026-08-31 15:20:45.092939+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 8.588680418783042, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001207000603474}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.62690573330471, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999888479982162}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-08-31 17:36 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1818,9 +1818,7 @@
       <c r="D2" s="1" t="n">
         <v>46265</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>46265</v>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
@@ -1854,11 +1852,11 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
         <v>11.77</v>
@@ -1869,11 +1867,7 @@
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
         <v>1945</v>
       </c>
@@ -1884,22 +1878,22 @@
         <v>1847.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1862.8</v>
+        <v>1915</v>
       </c>
       <c r="Y2" t="n">
-        <v>1862.8</v>
+        <v>1915</v>
       </c>
       <c r="Z2" t="n">
-        <v>7154018</v>
+        <v>30521088</v>
       </c>
       <c r="AA2" t="n">
-        <v>2224255</v>
+        <v>3392609</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.22</v>
+        <v>9</v>
       </c>
       <c r="AC2" t="n">
-        <v>-3.91</v>
+        <v>-1.21</v>
       </c>
       <c r="AD2" t="n">
         <v>0.34</v>
@@ -1908,7 +1902,7 @@
         <v>101.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.43</v>
+        <v>5.28</v>
       </c>
       <c r="AG2" t="n">
         <v>44.83</v>
@@ -1917,7 +1911,7 @@
         <v>44.83</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.41</v>
+        <v>2.34</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1920,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.97</v>
+        <v>3.65</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.67</v>
+        <v>13.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.58</v>
+        <v>52.71</v>
       </c>
       <c r="AO2" t="n">
-        <v>59.52</v>
+        <v>69.25</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.93</v>
+        <v>5.82</v>
       </c>
       <c r="AQ2" t="n">
-        <v>33.6</v>
+        <v>37.34</v>
       </c>
       <c r="AR2" t="n">
-        <v>1862.8</v>
+        <v>1915</v>
       </c>
       <c r="AS2" t="n">
-        <v>2042.13</v>
+        <v>2094.33</v>
       </c>
       <c r="AT2" t="n">
-        <v>1773.13</v>
+        <v>1825.33</v>
       </c>
       <c r="AU2" t="n">
-        <v>1862.800048828125</v>
+        <v>1915</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.630000000000001</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="AY2" t="n">
         <v>179.33</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.81</v>
+        <v>4.68</v>
       </c>
       <c r="BA2" t="n">
         <v>89.67</v>
@@ -2026,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.71</v>
+        <v>1480.7</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2088,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>91.7</v>
+        <v>97.94</v>
       </c>
       <c r="CO2" t="n">
-        <v>59.69</v>
+        <v>71.02</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.626899999999999</v>
+        <v>9.3645</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.642</v>
+        <v>0.624</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3207</v>
+        <v>0.312</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0963</v>
+        <v>0.0936</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1335</v>
+        <v>1.1017</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9959</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8137</v>
+        <v>4.6825</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.73</v>
+        <v>31.93</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8137</v>
+        <v>4.6825</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9959</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9959</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0019</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8307</v>
+        <v>0.8547</v>
       </c>
       <c r="DQ2" t="n">
         <v>89.67</v>
       </c>
       <c r="DR2" t="n">
-        <v>55.37</v>
+        <v>55.92</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2158</v>
+        <v>2.4872</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.80000000000001</v>
+        <v>76.875</v>
       </c>
       <c r="DY2" t="n">
-        <v>161</v>
+        <v>450</v>
       </c>
       <c r="DZ2" t="n">
-        <v>80.99299999999999</v>
+        <v>93.15600000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>65.12</v>
+        <v>78.5</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.39</v>
+        <v>71.05</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2158</v>
+        <v>2.4872</v>
       </c>
       <c r="EF2" t="n">
-        <v>3.22</v>
+        <v>9</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3449</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9946</v>
+        <v>4.0019</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0406</v>
+        <v>0.0806</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6875</v>
+        <v>0.7046</v>
       </c>
       <c r="EK2" t="n">
-        <v>77.28</v>
+        <v>79.65000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>70.37</v>
+        <v>100</v>
       </c>
       <c r="EP2" t="n">
-        <v>8.282500000000001</v>
+        <v>11.77</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.379</v>
+        <v>1.0593</v>
       </c>
       <c r="ER2" t="n">
-        <v>2.9907</v>
+        <v>1.04</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.0645</v>
+        <v>9.559900000000001</v>
       </c>
       <c r="ET2" t="n">
-        <v>64.05500000000001</v>
+        <v>77.476</v>
       </c>
       <c r="EU2" t="n">
-        <v>9.4346</v>
+        <v>52.38</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.5711000000000001</v>
+        <v>0.234</v>
       </c>
       <c r="EW2" t="n">
-        <v>64.52930000000001</v>
+        <v>97.94</v>
       </c>
       <c r="EX2" t="n">
-        <v>74.23</v>
+        <v>78.25</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2293,28 +2287,28 @@
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.94</v>
+        <v>25.87</v>
       </c>
       <c r="FD2" t="n">
         <v>73.36</v>
       </c>
       <c r="FE2" t="n">
-        <v>84.48999999999999</v>
+        <v>88.795</v>
       </c>
       <c r="FF2" t="n">
-        <v>66.95999999999999</v>
+        <v>74.63500000000001</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.8915</v>
+        <v>29.3234</v>
       </c>
       <c r="FH2" t="n">
-        <v>74.136</v>
+        <v>76.812</v>
       </c>
       <c r="FI2" t="n">
-        <v>46.55</v>
+        <v>43.925</v>
       </c>
       <c r="FJ2" t="n">
-        <v>74.98</v>
+        <v>75.05</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2331,16 +2325,16 @@
         <v>80.45</v>
       </c>
       <c r="FO2" t="n">
-        <v>71.78</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>83.39</v>
+        <v>86.55</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.77</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>94.62</v>
+        <v>94.92</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>76.271</v>
+        <v>75.64749999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260831_152045</t>
+          <t>20260831_230632</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46265.6394103549</v>
+        <v>46265.96288115138</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2464,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46265.63940972222</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46265</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46280</v>
-      </c>
+        <v>46265.96287037037</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2675,13 +2665,9 @@
       <c r="I2" t="n">
         <v>11.77</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1862.8</v>
+        <v>1915</v>
       </c>
       <c r="L2" t="n">
         <v>1945</v>
@@ -2693,34 +2679,34 @@
         <v>1847.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1862.8</v>
+        <v>1915</v>
       </c>
       <c r="P2" t="n">
-        <v>7154018</v>
+        <v>30521088</v>
       </c>
       <c r="Q2" t="n">
-        <v>1862.8</v>
+        <v>1915</v>
       </c>
       <c r="R2" t="n">
-        <v>2042.13</v>
+        <v>2094.33</v>
       </c>
       <c r="S2" t="n">
-        <v>1773.13</v>
+        <v>1825.33</v>
       </c>
       <c r="T2" t="n">
-        <v>9.62690573330471</v>
+        <v>9.364490861618794</v>
       </c>
       <c r="U2" t="n">
-        <v>179.3300000000002</v>
+        <v>179.3299999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.81372127979385</v>
+        <v>4.682506527415147</v>
       </c>
       <c r="W2" t="n">
-        <v>89.66999999999985</v>
+        <v>89.67000000000007</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999888479982162</v>
+        <v>1.999888479982154</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.62690573330471</v>
+        <v>9.364490861618794</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.81372127979385</v>
+        <v>4.682506527415147</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02059425290637167</v>
+        <v>0.02053998819686106</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3269236297645716</v>
+        <v>0.3260622042065783</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02935663033654778</v>
+        <v>0.02909876709663517</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04294788444710936</v>
+        <v>0.04266353895739713</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347613</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.85</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:20:45.092939+05:30</t>
+          <t>2026-08-31 23:06:32.960120+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.62690573330471, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999888479982162}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.364490861618794, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998884799821544}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-01 08:43 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.71</v>
+        <v>49.18</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1945</v>
+        <v>1888.9</v>
       </c>
       <c r="V2" t="n">
-        <v>1949</v>
+        <v>1895</v>
       </c>
       <c r="W2" t="n">
-        <v>1847.8</v>
+        <v>1837.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1915</v>
+        <v>1847.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1915</v>
+        <v>1847.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>30521088</v>
+        <v>2596221</v>
       </c>
       <c r="AA2" t="n">
-        <v>3392609</v>
+        <v>3475873</v>
       </c>
       <c r="AB2" t="n">
-        <v>9</v>
+        <v>0.75</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.21</v>
+        <v>-3.54</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.34</v>
+        <v>-1.36</v>
       </c>
       <c r="AE2" t="n">
-        <v>101.2</v>
+        <v>57.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.28</v>
+        <v>3.12</v>
       </c>
       <c r="AG2" t="n">
-        <v>44.83</v>
+        <v>47.17</v>
       </c>
       <c r="AH2" t="n">
-        <v>44.83</v>
+        <v>47.17</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.34</v>
+        <v>2.55</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.65</v>
+        <v>-0</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.7</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.71</v>
+        <v>46.81</v>
       </c>
       <c r="AO2" t="n">
-        <v>69.25</v>
+        <v>56.38</v>
       </c>
       <c r="AP2" t="n">
-        <v>5.82</v>
+        <v>1.84</v>
       </c>
       <c r="AQ2" t="n">
-        <v>37.34</v>
+        <v>29.44</v>
       </c>
       <c r="AR2" t="n">
-        <v>1915</v>
+        <v>1847.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>2094.33</v>
+        <v>2035.99</v>
       </c>
       <c r="AT2" t="n">
-        <v>1825.33</v>
+        <v>1752.95</v>
       </c>
       <c r="AU2" t="n">
-        <v>1915</v>
+        <v>1847.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.359999999999999</v>
+        <v>10.21</v>
       </c>
       <c r="AY2" t="n">
-        <v>179.33</v>
+        <v>188.69</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.68</v>
+        <v>5.11</v>
       </c>
       <c r="BA2" t="n">
-        <v>89.67</v>
+        <v>94.34999999999999</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.7</v>
+        <v>1480.71</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>97.94</v>
+        <v>80.34</v>
       </c>
       <c r="CO2" t="n">
-        <v>71.02</v>
+        <v>52.94</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2115,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.3645</v>
+        <v>10.2144</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.624</v>
+        <v>0.6807</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.312</v>
+        <v>0.3407</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0936</v>
+        <v>0.1021</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1017</v>
+        <v>1.2017</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0039</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6825</v>
+        <v>5.1075</v>
       </c>
       <c r="DJ2" t="n">
-        <v>31.93</v>
+        <v>40.79</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6825</v>
+        <v>5.1075</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0039</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0039</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8547</v>
+        <v>0.7835</v>
       </c>
       <c r="DQ2" t="n">
-        <v>89.67</v>
+        <v>94.34999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>55.92</v>
+        <v>52.8</v>
       </c>
       <c r="DS2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DT2" t="n">
         <v>5</v>
-      </c>
-      <c r="DT2" t="n">
-        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.4872</v>
+        <v>0.7216</v>
       </c>
       <c r="DX2" t="n">
-        <v>76.875</v>
+        <v>90.95</v>
       </c>
       <c r="DY2" t="n">
-        <v>450</v>
+        <v>37.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>93.15600000000001</v>
+        <v>77.72799999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>78.5</v>
+        <v>61.96</v>
       </c>
       <c r="ED2" t="n">
-        <v>71.05</v>
+        <v>90.95</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.4872</v>
+        <v>0.7216</v>
       </c>
       <c r="EF2" t="n">
-        <v>9</v>
+        <v>0.75</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.2166</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0019</v>
+        <v>4.0056</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0806</v>
+        <v>0.0255</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7046</v>
+        <v>0.6556</v>
       </c>
       <c r="EK2" t="n">
-        <v>79.65000000000001</v>
+        <v>69.97</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,72 +2243,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>100</v>
+        <v>31.52</v>
       </c>
       <c r="EP2" t="n">
-        <v>11.77</v>
+        <v>3.7099</v>
       </c>
       <c r="EQ2" t="n">
-        <v>1.0593</v>
+        <v>0.0883</v>
       </c>
       <c r="ER2" t="n">
-        <v>1.04</v>
+        <v>13.6133</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.559900000000001</v>
+        <v>11.4901</v>
       </c>
       <c r="ET2" t="n">
-        <v>77.476</v>
+        <v>49.7</v>
       </c>
       <c r="EU2" t="n">
-        <v>52.38</v>
+        <v>1.38</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.234</v>
+        <v>1.4571</v>
       </c>
       <c r="EW2" t="n">
-        <v>97.94</v>
+        <v>25.3232</v>
       </c>
       <c r="EX2" t="n">
-        <v>78.25</v>
+        <v>50.95</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.87</v>
+        <v>34.19</v>
       </c>
       <c r="FD2" t="n">
         <v>73.36</v>
       </c>
       <c r="FE2" t="n">
-        <v>88.795</v>
+        <v>75.155</v>
       </c>
       <c r="FF2" t="n">
-        <v>74.63500000000001</v>
+        <v>51.945</v>
       </c>
       <c r="FG2" t="n">
-        <v>29.3234</v>
+        <v>22.631</v>
       </c>
       <c r="FH2" t="n">
-        <v>76.812</v>
+        <v>66.072</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.925</v>
+        <v>46.795</v>
       </c>
       <c r="FJ2" t="n">
-        <v>75.05</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,36 +2322,36 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>80.45</v>
+        <v>73.52</v>
       </c>
       <c r="FO2" t="n">
-        <v>69.18000000000001</v>
+        <v>66.97</v>
       </c>
       <c r="FP2" t="n">
-        <v>86.55</v>
+        <v>65.58</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.68000000000001</v>
+        <v>70.34</v>
       </c>
       <c r="FR2" t="n">
-        <v>94.92</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>86.36360000000001</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.64749999999999</v>
+        <v>66.23050000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2359,13 +2359,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260831_230632</t>
+          <t>20260901_141319</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46265.96288115138</v>
+        <v>46266.59259137681</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46265.96287037037</v>
+        <v>46266.59258101852</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1915</v>
+        <v>1847.3</v>
       </c>
       <c r="L2" t="n">
-        <v>1945</v>
+        <v>1888.9</v>
       </c>
       <c r="M2" t="n">
-        <v>1949</v>
+        <v>1895</v>
       </c>
       <c r="N2" t="n">
-        <v>1847.8</v>
+        <v>1837.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1915</v>
+        <v>1847.3</v>
       </c>
       <c r="P2" t="n">
-        <v>30521088</v>
+        <v>2596221</v>
       </c>
       <c r="Q2" t="n">
-        <v>1915</v>
+        <v>1847.3</v>
       </c>
       <c r="R2" t="n">
-        <v>2094.33</v>
+        <v>2035.99</v>
       </c>
       <c r="S2" t="n">
-        <v>1825.33</v>
+        <v>1752.95</v>
       </c>
       <c r="T2" t="n">
-        <v>9.364490861618794</v>
+        <v>10.21436691387431</v>
       </c>
       <c r="U2" t="n">
-        <v>179.3299999999999</v>
+        <v>188.6900000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.682506527415147</v>
+        <v>5.107454122232443</v>
       </c>
       <c r="W2" t="n">
-        <v>89.67000000000007</v>
+        <v>94.34999999999991</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999888479982154</v>
+        <v>1.99989401165872</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.364490861618794</v>
+        <v>10.21436691387431</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.682506527415147</v>
+        <v>5.107454122232443</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02053998819686106</v>
+        <v>0.02058374518246228</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3260622042065783</v>
+        <v>0.3267568248187142</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909876709663517</v>
+        <v>0.02935663033654778</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353895739713</v>
+        <v>0.04284220885495441</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.92</v>
+        <v>38.86</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-31 23:06:32.960120+05:30</t>
+          <t>2026-09-01 14:13:19.930524+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.364490861618794, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998884799821544}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.214366913874306, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.99989401165872}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-01 14:50 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.18</v>
+        <v>49.29</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,22 +1878,22 @@
         <v>1837.4</v>
       </c>
       <c r="X2" t="n">
-        <v>1847.3</v>
+        <v>1861.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>1847.3</v>
+        <v>1861.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>2596221</v>
+        <v>3529595</v>
       </c>
       <c r="AA2" t="n">
-        <v>3475873</v>
+        <v>3522542</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="AC2" t="n">
-        <v>-3.54</v>
+        <v>-2.79</v>
       </c>
       <c r="AD2" t="n">
         <v>-1.36</v>
@@ -1902,7 +1902,7 @@
         <v>57.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.12</v>
+        <v>3.09</v>
       </c>
       <c r="AG2" t="n">
         <v>47.17</v>
@@ -1911,7 +1911,7 @@
         <v>47.17</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.55</v>
+        <v>2.53</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,47 +1920,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0</v>
+        <v>0.73</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.210000000000001</v>
+        <v>10.04</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.81</v>
+        <v>47.94</v>
       </c>
       <c r="AO2" t="n">
-        <v>56.38</v>
+        <v>58.68</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.84</v>
+        <v>2.62</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.44</v>
+        <v>30.44</v>
       </c>
       <c r="AR2" t="n">
-        <v>1847.3</v>
+        <v>1861.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2035.99</v>
+        <v>2050.29</v>
       </c>
       <c r="AT2" t="n">
-        <v>1752.95</v>
+        <v>1767.25</v>
       </c>
       <c r="AU2" t="n">
-        <v>1847.300048828125</v>
+        <v>1861.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.21</v>
+        <v>10.14</v>
       </c>
       <c r="AY2" t="n">
         <v>188.69</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.11</v>
+        <v>5.07</v>
       </c>
       <c r="BA2" t="n">
         <v>94.34999999999999</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>80.34</v>
+        <v>83.53</v>
       </c>
       <c r="CO2" t="n">
-        <v>52.94</v>
+        <v>43.21</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2115,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2144</v>
+        <v>10.1359</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6807</v>
+        <v>0.676</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3407</v>
+        <v>0.338</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1021</v>
+        <v>0.1014</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2017</v>
+        <v>1.1935</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0039</v>
+        <v>4.0079</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1075</v>
+        <v>5.0682</v>
       </c>
       <c r="DJ2" t="n">
-        <v>40.79</v>
+        <v>40.12</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1075</v>
+        <v>5.0682</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0039</v>
+        <v>2.004</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0039</v>
+        <v>4.0079</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7835</v>
+        <v>0.7905</v>
       </c>
       <c r="DQ2" t="n">
         <v>94.34999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>52.8</v>
+        <v>50.16</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.7216</v>
+        <v>1.0356</v>
       </c>
       <c r="DX2" t="n">
-        <v>90.95</v>
+        <v>96.7</v>
       </c>
       <c r="DY2" t="n">
-        <v>37.5</v>
+        <v>50</v>
       </c>
       <c r="DZ2" t="n">
-        <v>77.72799999999999</v>
+        <v>78.758</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>61.96</v>
+        <v>63.94</v>
       </c>
       <c r="ED2" t="n">
-        <v>90.95</v>
+        <v>99.87</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.7216</v>
+        <v>1.0356</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2166</v>
+        <v>0.3084</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0056</v>
+        <v>4.0063</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0255</v>
+        <v>0.0363</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6556</v>
+        <v>0.66</v>
       </c>
       <c r="EK2" t="n">
-        <v>69.97</v>
+        <v>73.83</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>31.52</v>
+        <v>30.52</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.7099</v>
+        <v>3.5922</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0883</v>
+        <v>0.1177</v>
       </c>
       <c r="ER2" t="n">
-        <v>13.6133</v>
+        <v>10.14</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.4901</v>
+        <v>11.3654</v>
       </c>
       <c r="ET2" t="n">
-        <v>49.7</v>
+        <v>45.508</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.38</v>
+        <v>2.62</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4571</v>
+        <v>1.265</v>
       </c>
       <c r="EW2" t="n">
-        <v>25.3232</v>
+        <v>25.4934</v>
       </c>
       <c r="EX2" t="n">
-        <v>50.95</v>
+        <v>50.57</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>34.19</v>
+        <v>33.65</v>
       </c>
       <c r="FD2" t="n">
         <v>73.36</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.155</v>
+        <v>78.68000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>51.945</v>
+        <v>46.89</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.631</v>
+        <v>23.6629</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.072</v>
+        <v>66.953</v>
       </c>
       <c r="FI2" t="n">
-        <v>46.795</v>
+        <v>45.14</v>
       </c>
       <c r="FJ2" t="n">
-        <v>69.26000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,36 +2322,36 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.52</v>
+        <v>73.06</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.97</v>
+        <v>68.64</v>
       </c>
       <c r="FP2" t="n">
-        <v>65.58</v>
+        <v>62.42</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.34</v>
+        <v>67.92</v>
       </c>
       <c r="FR2" t="n">
-        <v>76.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="FS2" t="n">
-        <v>86.36360000000001</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.23050000000001</v>
+        <v>69.842</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2359,13 +2359,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260901_141319</t>
+          <t>20260901_202055</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46266.59259137681</v>
+        <v>46266.84785936177</v>
       </c>
     </row>
   </sheetData>
@@ -2458,7 +2458,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46266.59258101852</v>
+        <v>46266.8478587963</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1847.3</v>
+        <v>1861.6</v>
       </c>
       <c r="L2" t="n">
         <v>1888.9</v>
@@ -2679,28 +2679,28 @@
         <v>1837.4</v>
       </c>
       <c r="O2" t="n">
-        <v>1847.3</v>
+        <v>1861.6</v>
       </c>
       <c r="P2" t="n">
-        <v>2596221</v>
+        <v>3529595</v>
       </c>
       <c r="Q2" t="n">
-        <v>1847.3</v>
+        <v>1861.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2035.99</v>
+        <v>2050.29</v>
       </c>
       <c r="S2" t="n">
-        <v>1752.95</v>
+        <v>1767.25</v>
       </c>
       <c r="T2" t="n">
-        <v>10.21436691387431</v>
+        <v>10.1359045981951</v>
       </c>
       <c r="U2" t="n">
         <v>188.6900000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.107454122232443</v>
+        <v>5.068220885259986</v>
       </c>
       <c r="W2" t="n">
         <v>94.34999999999991</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.21436691387431</v>
+        <v>10.1359045981951</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.107454122232443</v>
+        <v>5.068220885259986</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058374518246228</v>
+        <v>0.0205581071696241</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3267568248187142</v>
+        <v>0.3263498339822359</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02935663033654778</v>
+        <v>0.02909870789015188</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04284220885495441</v>
+        <v>0.04266353076209672</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.86</v>
+        <v>38.89</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-01 14:13:19.930524+05:30</t>
+          <t>2026-09-01 20:20:55.083720+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.214366913874306, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.99989401165872}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.135904598195104, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.99989401165872}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-02 07:58 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.29</v>
+        <v>49.07</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1888.9</v>
+        <v>1853.2</v>
       </c>
       <c r="V2" t="n">
-        <v>1895</v>
+        <v>1864.4</v>
       </c>
       <c r="W2" t="n">
-        <v>1837.4</v>
+        <v>1811.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1861.6</v>
+        <v>1837.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>1861.6</v>
+        <v>1837.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>3529595</v>
+        <v>1672130</v>
       </c>
       <c r="AA2" t="n">
-        <v>3522542</v>
+        <v>3501638</v>
       </c>
       <c r="AB2" t="n">
-        <v>1</v>
+        <v>0.48</v>
       </c>
       <c r="AC2" t="n">
-        <v>-2.79</v>
+        <v>-1.28</v>
       </c>
       <c r="AD2" t="n">
-        <v>-1.36</v>
+        <v>-0.45</v>
       </c>
       <c r="AE2" t="n">
-        <v>57.6</v>
+        <v>52.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.09</v>
+        <v>2.87</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.17</v>
+        <v>47.57</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.17</v>
+        <v>47.57</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.53</v>
+        <v>2.59</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.73</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.04</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.94</v>
+        <v>45.58</v>
       </c>
       <c r="AO2" t="n">
-        <v>58.68</v>
+        <v>54.67</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.62</v>
+        <v>2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.44</v>
+        <v>27.03</v>
       </c>
       <c r="AR2" t="n">
-        <v>1861.6</v>
+        <v>1837.8</v>
       </c>
       <c r="AS2" t="n">
-        <v>2050.29</v>
+        <v>2028.07</v>
       </c>
       <c r="AT2" t="n">
-        <v>1767.25</v>
+        <v>1742.66</v>
       </c>
       <c r="AU2" t="n">
-        <v>1861.599975585938</v>
+        <v>1837.800048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.14</v>
+        <v>10.35</v>
       </c>
       <c r="AY2" t="n">
-        <v>188.69</v>
+        <v>190.27</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.07</v>
+        <v>5.18</v>
       </c>
       <c r="BA2" t="n">
-        <v>94.34999999999999</v>
+        <v>95.14</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.71</v>
+        <v>1480.7</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.53</v>
+        <v>75.41</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.21</v>
+        <v>46.94</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2115,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.1359</v>
+        <v>10.3531</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.676</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.338</v>
+        <v>0.3453</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1014</v>
+        <v>0.1035</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.9981</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1935</v>
+        <v>1.2182</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0079</v>
+        <v>3.9961</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0682</v>
+        <v>5.1768</v>
       </c>
       <c r="DJ2" t="n">
-        <v>40.12</v>
+        <v>41.52</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0682</v>
+        <v>5.1768</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.004</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0079</v>
+        <v>3.9961</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9983</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7905</v>
+        <v>0.7715</v>
       </c>
       <c r="DQ2" t="n">
-        <v>94.34999999999999</v>
+        <v>95.14</v>
       </c>
       <c r="DR2" t="n">
-        <v>50.16</v>
+        <v>48.37</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.0356</v>
+        <v>0.7722</v>
       </c>
       <c r="DX2" t="n">
-        <v>96.7</v>
+        <v>86.67500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="DZ2" t="n">
-        <v>78.758</v>
+        <v>73.755</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>63.94</v>
+        <v>59.42</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.87</v>
+        <v>87.23</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.0356</v>
+        <v>0.7722</v>
       </c>
       <c r="EF2" t="n">
-        <v>1</v>
+        <v>0.48</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3084</v>
+        <v>0.2354</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0063</v>
+        <v>3.9973</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0363</v>
+        <v>0.0277</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.66</v>
+        <v>0.6468</v>
       </c>
       <c r="EK2" t="n">
-        <v>73.83</v>
+        <v>66.48</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>30.52</v>
+        <v>15.21</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.5922</v>
+        <v>1.7902</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1177</v>
+        <v>0.0565</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.14</v>
+        <v>21.5625</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.3654</v>
+        <v>11.5655</v>
       </c>
       <c r="ET2" t="n">
-        <v>45.508</v>
+        <v>42.407</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.62</v>
+        <v>0.96</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.265</v>
+        <v>1.75</v>
       </c>
       <c r="EW2" t="n">
-        <v>25.4934</v>
+        <v>11.4699</v>
       </c>
       <c r="EX2" t="n">
-        <v>50.57</v>
+        <v>43.26</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>33.65</v>
+        <v>34.97</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.36</v>
+        <v>73.25</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.68000000000001</v>
+        <v>70.94499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.89</v>
+        <v>45.1</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.6629</v>
+        <v>21.0056</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.953</v>
+        <v>63.055</v>
       </c>
       <c r="FI2" t="n">
-        <v>45.14</v>
+        <v>44.945</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.09999999999999</v>
+        <v>65.69</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.06</v>
+        <v>67.08</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.64</v>
+        <v>62.92</v>
       </c>
       <c r="FP2" t="n">
-        <v>62.42</v>
+        <v>54.88</v>
       </c>
       <c r="FQ2" t="n">
-        <v>67.92</v>
+        <v>65.78</v>
       </c>
       <c r="FR2" t="n">
-        <v>84.56</v>
+        <v>80.31</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.842</v>
+        <v>66.7765</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260901_202055</t>
+          <t>20260902_132815</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46266.84785936177</v>
+        <v>46267.56128774607</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46266.8478587963</v>
+        <v>46267.56128472222</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1861.6</v>
+        <v>1837.8</v>
       </c>
       <c r="L2" t="n">
-        <v>1888.9</v>
+        <v>1853.2</v>
       </c>
       <c r="M2" t="n">
-        <v>1895</v>
+        <v>1864.4</v>
       </c>
       <c r="N2" t="n">
-        <v>1837.4</v>
+        <v>1811.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1861.6</v>
+        <v>1837.8</v>
       </c>
       <c r="P2" t="n">
-        <v>3529595</v>
+        <v>1672130</v>
       </c>
       <c r="Q2" t="n">
-        <v>1861.6</v>
+        <v>1837.8</v>
       </c>
       <c r="R2" t="n">
-        <v>2050.29</v>
+        <v>2028.07</v>
       </c>
       <c r="S2" t="n">
-        <v>1767.25</v>
+        <v>1742.66</v>
       </c>
       <c r="T2" t="n">
-        <v>10.1359045981951</v>
+        <v>10.35313962346284</v>
       </c>
       <c r="U2" t="n">
-        <v>188.6900000000001</v>
+        <v>190.27</v>
       </c>
       <c r="V2" t="n">
-        <v>5.068220885259986</v>
+        <v>5.176841876156267</v>
       </c>
       <c r="W2" t="n">
-        <v>94.34999999999991</v>
+        <v>95.13999999999987</v>
       </c>
       <c r="X2" t="n">
-        <v>1.99989401165872</v>
+        <v>1.999894891738493</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.1359045981951</v>
+        <v>10.35313962346284</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.068220885259986</v>
+        <v>5.176841876156267</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0205581071696241</v>
+        <v>0.02053337518957066</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3263498339822359</v>
+        <v>0.3259572259703263</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909870789015188</v>
+        <v>0.02909870225204695</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353076209672</v>
+        <v>0.04266354089421848</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.89</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-01 20:20:55.083720+05:30</t>
+          <t>2026-09-02 13:28:15.300184+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.135904598195104, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.99989401165872}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.353139623462836, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999894891738493}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-02 14:26 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.07</v>
+        <v>49.14</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,22 +1878,22 @@
         <v>1811.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1837.8</v>
+        <v>1864</v>
       </c>
       <c r="Y2" t="n">
-        <v>1837.8</v>
+        <v>1864</v>
       </c>
       <c r="Z2" t="n">
-        <v>1672130</v>
+        <v>2265297</v>
       </c>
       <c r="AA2" t="n">
-        <v>3501638</v>
+        <v>3531296</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.48</v>
+        <v>0.64</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.28</v>
+        <v>0.13</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.45</v>
@@ -1902,7 +1902,7 @@
         <v>52.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.87</v>
+        <v>2.83</v>
       </c>
       <c r="AG2" t="n">
         <v>47.57</v>
@@ -1911,7 +1911,7 @@
         <v>47.57</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.59</v>
+        <v>2.55</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,47 +1920,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.140000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.58</v>
+        <v>47.64</v>
       </c>
       <c r="AO2" t="n">
-        <v>54.67</v>
+        <v>58.98</v>
       </c>
       <c r="AP2" t="n">
-        <v>2</v>
+        <v>3.45</v>
       </c>
       <c r="AQ2" t="n">
-        <v>27.03</v>
+        <v>28.84</v>
       </c>
       <c r="AR2" t="n">
-        <v>1837.8</v>
+        <v>1864</v>
       </c>
       <c r="AS2" t="n">
-        <v>2028.07</v>
+        <v>2054.27</v>
       </c>
       <c r="AT2" t="n">
-        <v>1742.66</v>
+        <v>1768.86</v>
       </c>
       <c r="AU2" t="n">
-        <v>1837.800048828125</v>
+        <v>1864</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.35</v>
+        <v>10.21</v>
       </c>
       <c r="AY2" t="n">
         <v>190.27</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.18</v>
+        <v>5.1</v>
       </c>
       <c r="BA2" t="n">
         <v>95.14</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.7</v>
+        <v>1480.71</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.41</v>
+        <v>76.89</v>
       </c>
       <c r="CO2" t="n">
-        <v>46.94</v>
+        <v>42.71</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.3531</v>
+        <v>10.2076</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2127,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6807</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3453</v>
+        <v>0.34</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1035</v>
+        <v>0.1021</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9981</v>
+        <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2182</v>
+        <v>1.2017</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9961</v>
+        <v>4.0039</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1768</v>
+        <v>5.1041</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41.52</v>
+        <v>39.65</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1768</v>
+        <v>5.1041</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
@@ -2160,25 +2160,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9961</v>
+        <v>4.0039</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9983</v>
+        <v>2.0021</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7715</v>
+        <v>0.7851</v>
       </c>
       <c r="DQ2" t="n">
         <v>95.14</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.37</v>
+        <v>57</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.7722</v>
+        <v>1.3529</v>
       </c>
       <c r="DX2" t="n">
-        <v>86.67500000000001</v>
+        <v>97.44999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="DZ2" t="n">
-        <v>73.755</v>
+        <v>76.548</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>59.42</v>
+        <v>64.77</v>
       </c>
       <c r="ED2" t="n">
-        <v>87.23</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.7722</v>
+        <v>1.3529</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.48</v>
+        <v>0.64</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2354</v>
+        <v>0.4061</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9973</v>
+        <v>4.003</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0277</v>
+        <v>0.0478</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6468</v>
+        <v>0.6562</v>
       </c>
       <c r="EK2" t="n">
-        <v>66.48</v>
+        <v>71.94</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>15.21</v>
+        <v>10.15</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.7902</v>
+        <v>1.1947</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0565</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="ER2" t="n">
-        <v>21.5625</v>
+        <v>15.9531</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.5655</v>
+        <v>11.169</v>
       </c>
       <c r="ET2" t="n">
-        <v>42.407</v>
+        <v>39.197</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.96</v>
+        <v>2.208</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.75</v>
+        <v>1.5549</v>
       </c>
       <c r="EW2" t="n">
-        <v>11.4699</v>
+        <v>7.8043</v>
       </c>
       <c r="EX2" t="n">
-        <v>43.26</v>
+        <v>41.58</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>34.97</v>
+        <v>33.14</v>
       </c>
       <c r="FD2" t="n">
         <v>73.25</v>
       </c>
       <c r="FE2" t="n">
-        <v>70.94499999999999</v>
+        <v>74.41500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>45.1</v>
+        <v>42.145</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.0056</v>
+        <v>21.6592</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.055</v>
+        <v>63.163</v>
       </c>
       <c r="FI2" t="n">
-        <v>44.945</v>
+        <v>48.325</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.69</v>
+        <v>66.83</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>67.08</v>
+        <v>76.89</v>
       </c>
       <c r="FO2" t="n">
-        <v>62.92</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.88</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="FQ2" t="n">
-        <v>65.78</v>
+        <v>78.17</v>
       </c>
       <c r="FR2" t="n">
-        <v>80.31</v>
+        <v>87.91</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.7765</v>
+        <v>71.8185</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260902_132815</t>
+          <t>20260902_195637</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46267.56128774607</v>
+        <v>46267.83099379978</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46267.56128472222</v>
+        <v>46267.8309837963</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1837.8</v>
+        <v>1864</v>
       </c>
       <c r="L2" t="n">
         <v>1853.2</v>
@@ -2679,34 +2679,34 @@
         <v>1811.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1837.8</v>
+        <v>1864</v>
       </c>
       <c r="P2" t="n">
-        <v>1672130</v>
+        <v>2265297</v>
       </c>
       <c r="Q2" t="n">
-        <v>1837.8</v>
+        <v>1864</v>
       </c>
       <c r="R2" t="n">
-        <v>2028.07</v>
+        <v>2054.27</v>
       </c>
       <c r="S2" t="n">
-        <v>1742.66</v>
+        <v>1768.86</v>
       </c>
       <c r="T2" t="n">
-        <v>10.35313962346284</v>
+        <v>10.20761802575107</v>
       </c>
       <c r="U2" t="n">
         <v>190.27</v>
       </c>
       <c r="V2" t="n">
-        <v>5.176841876156267</v>
+        <v>5.10407725321889</v>
       </c>
       <c r="W2" t="n">
-        <v>95.13999999999987</v>
+        <v>95.1400000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999894891738493</v>
+        <v>1.999894891738488</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.35313962346284</v>
+        <v>10.20761802575107</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.176841876156267</v>
+        <v>5.10407725321889</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02053337518957066</v>
+        <v>0.02054308955169515</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3259572259703263</v>
+        <v>0.3261114366882885</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909870225204695</v>
+        <v>0.02909864868366858</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266354089421848</v>
+        <v>0.04266354861729901</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.92</v>
+        <v>38.91</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-02 13:28:15.300184+05:30</t>
+          <t>2026-09-02 19:56:37.901490+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.353139623462836, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999894891738493}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.207618025751072, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998948917384884}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-03 08:07 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.14</v>
+        <v>48.97</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1853.2</v>
+        <v>1864.9</v>
       </c>
       <c r="V2" t="n">
-        <v>1864.4</v>
+        <v>1876.6</v>
       </c>
       <c r="W2" t="n">
-        <v>1811.7</v>
+        <v>1852.6</v>
       </c>
       <c r="X2" t="n">
-        <v>1864</v>
+        <v>1873.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>1864</v>
+        <v>1873.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>2265297</v>
+        <v>870122</v>
       </c>
       <c r="AA2" t="n">
-        <v>3531296</v>
+        <v>3461537</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.64</v>
+        <v>0.25</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.13</v>
+        <v>0.65</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.45</v>
+        <v>0.18</v>
       </c>
       <c r="AE2" t="n">
-        <v>52.7</v>
+        <v>24</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.83</v>
+        <v>1.28</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.57</v>
+        <v>45.52</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.57</v>
+        <v>45.52</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.55</v>
+        <v>2.43</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.78</v>
+        <v>1.28</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.65</v>
+        <v>10.2</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.64</v>
+        <v>48.4</v>
       </c>
       <c r="AO2" t="n">
-        <v>58.98</v>
+        <v>60.16</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.45</v>
+        <v>3.99</v>
       </c>
       <c r="AQ2" t="n">
-        <v>28.84</v>
+        <v>29.51</v>
       </c>
       <c r="AR2" t="n">
-        <v>1864</v>
+        <v>1873.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>2054.27</v>
+        <v>2055.77</v>
       </c>
       <c r="AT2" t="n">
-        <v>1768.86</v>
+        <v>1782.66</v>
       </c>
       <c r="AU2" t="n">
-        <v>1864</v>
+        <v>1873.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.21</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>190.27</v>
+        <v>182.07</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.1</v>
+        <v>4.86</v>
       </c>
       <c r="BA2" t="n">
-        <v>95.14</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>76.89</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>42.71</v>
+        <v>36.32</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2100,7 +2100,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>90.90909090909091</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2115,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2076</v>
+        <v>9.7171</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2127,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6807</v>
+        <v>0.648</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.34</v>
+        <v>0.324</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1021</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.002</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2017</v>
+        <v>1.144</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0039</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1041</v>
+        <v>4.8588</v>
       </c>
       <c r="DJ2" t="n">
-        <v>39.65</v>
+        <v>34.47</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1041</v>
+        <v>4.8588</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
@@ -2160,25 +2160,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0039</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0021</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7851</v>
+        <v>0.823</v>
       </c>
       <c r="DQ2" t="n">
-        <v>95.14</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>57</v>
+        <v>48.23</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.3529</v>
+        <v>1.642</v>
       </c>
       <c r="DX2" t="n">
-        <v>97.44999999999999</v>
+        <v>99.60000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>32</v>
+        <v>12.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>76.548</v>
+        <v>76.892</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>64.77</v>
+        <v>72.53</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.3529</v>
+        <v>1.642</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.64</v>
+        <v>0.25</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4061</v>
+        <v>0.4696</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.003</v>
+        <v>3.9988</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0478</v>
+        <v>0.0553</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6562</v>
+        <v>0.6824</v>
       </c>
       <c r="EK2" t="n">
-        <v>71.94</v>
+        <v>72.95999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,72 +2243,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>10.15</v>
+        <v>0.61</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.1947</v>
+        <v>0.0718</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0294</v>
       </c>
       <c r="ER2" t="n">
-        <v>15.9531</v>
+        <v>38.88</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.169</v>
+        <v>10.0496</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.197</v>
+        <v>33.779</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.208</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5549</v>
+        <v>1.944</v>
       </c>
       <c r="EW2" t="n">
-        <v>7.8043</v>
+        <v>0.4422</v>
       </c>
       <c r="EX2" t="n">
-        <v>41.58</v>
+        <v>26.71</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="FB2" t="n">
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>33.14</v>
+        <v>28.5</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.25</v>
+        <v>73.39</v>
       </c>
       <c r="FE2" t="n">
-        <v>74.41500000000001</v>
+        <v>72.72499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>42.145</v>
+        <v>31.515</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.6592</v>
+        <v>21.1341</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.163</v>
+        <v>58.869</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.325</v>
+        <v>41.35</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.83</v>
+        <v>63.49</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.89</v>
+        <v>66.34</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.98999999999999</v>
+        <v>61.52</v>
       </c>
       <c r="FP2" t="n">
-        <v>66.56999999999999</v>
+        <v>46.31</v>
       </c>
       <c r="FQ2" t="n">
-        <v>78.17</v>
+        <v>66.03</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.91</v>
+        <v>80.19</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.8185</v>
+        <v>65.19799999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260902_195637</t>
+          <t>20260903_133729</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46267.83099379978</v>
+        <v>46268.56770765664</v>
       </c>
     </row>
   </sheetData>
@@ -2458,8 +2458,8 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46267.8309837963</v>
+        <v>46268.56769675926</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1864</v>
+        <v>1873.7</v>
       </c>
       <c r="L2" t="n">
-        <v>1853.2</v>
+        <v>1864.9</v>
       </c>
       <c r="M2" t="n">
-        <v>1864.4</v>
+        <v>1876.6</v>
       </c>
       <c r="N2" t="n">
-        <v>1811.7</v>
+        <v>1852.6</v>
       </c>
       <c r="O2" t="n">
-        <v>1864</v>
+        <v>1873.7</v>
       </c>
       <c r="P2" t="n">
-        <v>2265297</v>
+        <v>870122</v>
       </c>
       <c r="Q2" t="n">
-        <v>1864</v>
+        <v>1873.7</v>
       </c>
       <c r="R2" t="n">
-        <v>2054.27</v>
+        <v>2055.77</v>
       </c>
       <c r="S2" t="n">
-        <v>1768.86</v>
+        <v>1782.66</v>
       </c>
       <c r="T2" t="n">
-        <v>10.20761802575107</v>
+        <v>9.717137215135823</v>
       </c>
       <c r="U2" t="n">
-        <v>190.27</v>
+        <v>182.0699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.10407725321889</v>
+        <v>4.858835459251746</v>
       </c>
       <c r="W2" t="n">
-        <v>95.1400000000001</v>
+        <v>91.03999999999996</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999894891738488</v>
+        <v>1.999890158172232</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.20761802575107</v>
+        <v>9.717137215135823</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.10407725321889</v>
+        <v>4.858835459251746</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02054308955169515</v>
+        <v>0.02054358141902422</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3261114366882885</v>
+        <v>0.326119244840073</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266354861729901</v>
+        <v>0.04266354656211883</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-02 19:56:37.901490+05:30</t>
+          <t>2026-09-03 13:37:29.965680+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.207618025751072, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998948917384884}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.717137215135823, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998901581722321}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-03 14:30 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.97</v>
+        <v>49.05</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,25 +1878,25 @@
         <v>1852.6</v>
       </c>
       <c r="X2" t="n">
-        <v>1873.7</v>
+        <v>1868.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>1873.7</v>
+        <v>1868.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>870122</v>
+        <v>1506252</v>
       </c>
       <c r="AA2" t="n">
-        <v>3461537</v>
+        <v>3504754</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.25</v>
+        <v>0.43</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.65</v>
+        <v>0.24</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="AE2" t="n">
         <v>24</v>
@@ -1905,13 +1905,13 @@
         <v>1.28</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.52</v>
+        <v>45.88</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.52</v>
+        <v>45.88</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.43</v>
+        <v>2.46</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.28</v>
+        <v>0.92</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.2</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.4</v>
+        <v>47.49</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.16</v>
+        <v>59.58</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.99</v>
+        <v>2.38</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.51</v>
+        <v>33.02</v>
       </c>
       <c r="AR2" t="n">
-        <v>1873.7</v>
+        <v>1868.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2055.77</v>
+        <v>2052.04</v>
       </c>
       <c r="AT2" t="n">
-        <v>1782.66</v>
+        <v>1776.73</v>
       </c>
       <c r="AU2" t="n">
-        <v>1873.699951171875</v>
+        <v>1868.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.720000000000001</v>
+        <v>9.82</v>
       </c>
       <c r="AY2" t="n">
-        <v>182.07</v>
+        <v>183.54</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.86</v>
+        <v>4.91</v>
       </c>
       <c r="BA2" t="n">
-        <v>91.04000000000001</v>
+        <v>91.77</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>72.48999999999999</v>
+        <v>69.88</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.32</v>
+        <v>39.49</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2100,7 +2100,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>90.90909090909091</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.7171</v>
+        <v>9.822900000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,52 +2127,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.648</v>
+        <v>0.6546999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.324</v>
+        <v>0.3273</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.0982</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.144</v>
+        <v>1.1558</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9919</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8588</v>
+        <v>4.9114</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.47</v>
+        <v>35.46</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8588</v>
+        <v>4.9114</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9959</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9919</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.823</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="DQ2" t="n">
-        <v>91.04000000000001</v>
+        <v>91.77</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.23</v>
+        <v>48.88</v>
       </c>
       <c r="DS2" t="n">
         <v>4</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.642</v>
+        <v>0.9675</v>
       </c>
       <c r="DX2" t="n">
-        <v>99.60000000000001</v>
+        <v>98.94999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>12.5</v>
+        <v>21.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>76.892</v>
+        <v>72.744</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>72.53</v>
+        <v>59.22</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>99.62</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.642</v>
+        <v>0.9675</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.25</v>
+        <v>0.43</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4696</v>
+        <v>0.2801</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9988</v>
+        <v>3.993</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0553</v>
+        <v>0.033</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6824</v>
+        <v>0.6756</v>
       </c>
       <c r="EK2" t="n">
-        <v>72.95999999999999</v>
+        <v>66.63</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>0.61</v>
+        <v>1.68</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.0718</v>
+        <v>0.1977</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0294</v>
+        <v>0.0506</v>
       </c>
       <c r="ER2" t="n">
-        <v>38.88</v>
+        <v>22.8372</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.0496</v>
+        <v>10.2486</v>
       </c>
       <c r="ET2" t="n">
-        <v>33.779</v>
+        <v>35.368</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.9975000000000001</v>
+        <v>1.0234</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.944</v>
+        <v>1.7203</v>
       </c>
       <c r="EW2" t="n">
-        <v>0.4422</v>
+        <v>1.174</v>
       </c>
       <c r="EX2" t="n">
-        <v>26.71</v>
+        <v>29.96</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>28.5</v>
+        <v>29.49</v>
       </c>
       <c r="FD2" t="n">
         <v>73.39</v>
       </c>
       <c r="FE2" t="n">
-        <v>72.72499999999999</v>
+        <v>68.255</v>
       </c>
       <c r="FF2" t="n">
-        <v>31.515</v>
+        <v>34.725</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.1341</v>
+        <v>20.1965</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.869</v>
+        <v>58.736</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.35</v>
+        <v>42.17</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.49</v>
+        <v>63.29</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>66.34</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>61.52</v>
+        <v>59.86</v>
       </c>
       <c r="FP2" t="n">
-        <v>46.31</v>
+        <v>50.44</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.03</v>
+        <v>67.70999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>80.19</v>
+        <v>81.73</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.19799999999999</v>
+        <v>66.17400000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260903_133729</t>
+          <t>20260903_200051</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46268.56770765664</v>
+        <v>46268.83392919807</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46268.56769675926</v>
+        <v>46268.83392361111</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1873.7</v>
+        <v>1868.5</v>
       </c>
       <c r="L2" t="n">
         <v>1864.9</v>
@@ -2679,34 +2679,34 @@
         <v>1852.6</v>
       </c>
       <c r="O2" t="n">
-        <v>1873.7</v>
+        <v>1868.5</v>
       </c>
       <c r="P2" t="n">
-        <v>870122</v>
+        <v>1506252</v>
       </c>
       <c r="Q2" t="n">
-        <v>1873.7</v>
+        <v>1868.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2055.77</v>
+        <v>2052.04</v>
       </c>
       <c r="S2" t="n">
-        <v>1782.66</v>
+        <v>1776.73</v>
       </c>
       <c r="T2" t="n">
-        <v>9.717137215135823</v>
+        <v>9.822852555525822</v>
       </c>
       <c r="U2" t="n">
-        <v>182.0699999999999</v>
+        <v>183.54</v>
       </c>
       <c r="V2" t="n">
-        <v>4.858835459251746</v>
+        <v>4.911426277762911</v>
       </c>
       <c r="W2" t="n">
-        <v>91.03999999999996</v>
+        <v>91.76999999999998</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999890158172232</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.717137215135823</v>
+        <v>9.822852555525822</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.858835459251746</v>
+        <v>4.911426277762911</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02054358141902422</v>
+        <v>0.02052804421462072</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.326119244840073</v>
+        <v>0.325872599366548</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909864868366858</v>
+        <v>0.02909858947718529</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266354656211883</v>
+        <v>0.04266353057055038</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.91</v>
+        <v>38.93</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-03 13:37:29.965680+05:30</t>
+          <t>2026-09-03 20:00:51.523849+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.717137215135823, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998901581722321}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.822852555525822, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-04 08:02 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.05</v>
+        <v>48.94</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1864.9</v>
+        <v>1855</v>
       </c>
       <c r="V2" t="n">
-        <v>1876.6</v>
+        <v>1871.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1852.6</v>
+        <v>1841</v>
       </c>
       <c r="X2" t="n">
-        <v>1868.5</v>
+        <v>1843.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>1868.5</v>
+        <v>1843.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1506252</v>
+        <v>634328</v>
       </c>
       <c r="AA2" t="n">
-        <v>3504754</v>
+        <v>3458823</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.43</v>
+        <v>0.18</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.24</v>
+        <v>-1.32</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.05</v>
+        <v>-0.72</v>
       </c>
       <c r="AE2" t="n">
-        <v>24</v>
+        <v>30.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.28</v>
+        <v>1.67</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.88</v>
+        <v>44.81</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.88</v>
+        <v>44.81</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.46</v>
+        <v>2.43</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.92</v>
+        <v>-0.41</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.369999999999999</v>
+        <v>7.44</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.49</v>
+        <v>45.06</v>
       </c>
       <c r="AO2" t="n">
-        <v>59.58</v>
+        <v>54.87</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.38</v>
+        <v>2.33</v>
       </c>
       <c r="AQ2" t="n">
-        <v>33.02</v>
+        <v>29.45</v>
       </c>
       <c r="AR2" t="n">
-        <v>1868.5</v>
+        <v>1843.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2052.04</v>
+        <v>2023.13</v>
       </c>
       <c r="AT2" t="n">
-        <v>1776.73</v>
+        <v>1754.29</v>
       </c>
       <c r="AU2" t="n">
-        <v>1868.5</v>
+        <v>1843.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.82</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>183.54</v>
+        <v>179.23</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.91</v>
+        <v>4.86</v>
       </c>
       <c r="BA2" t="n">
-        <v>91.77</v>
+        <v>89.61</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.71</v>
+        <v>1480.7</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>69.88</v>
+        <v>67.63</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.49</v>
+        <v>28</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.822900000000001</v>
+        <v>9.7202</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6546999999999999</v>
+        <v>0.648</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3273</v>
+        <v>0.324</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0982</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1558</v>
+        <v>1.144</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9919</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9114</v>
+        <v>4.8598</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.46</v>
+        <v>36.11</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9114</v>
+        <v>4.8598</v>
       </c>
       <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>1.9959</v>
-      </c>
       <c r="DN2" t="n">
-        <v>3.9919</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.823</v>
       </c>
       <c r="DQ2" t="n">
-        <v>91.77</v>
+        <v>89.61</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.88</v>
+        <v>66.78</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,90 +2187,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9675</v>
+        <v>0.9588</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.94999999999999</v>
+        <v>87.175</v>
       </c>
       <c r="DY2" t="n">
-        <v>21.5</v>
+        <v>9</v>
       </c>
       <c r="DZ2" t="n">
-        <v>72.744</v>
+        <v>67.404</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>59.22</v>
+        <v>53.26</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.62</v>
+        <v>86.02</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9675</v>
+        <v>0.9588</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.43</v>
+        <v>0.18</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2801</v>
+        <v>0.2742</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.993</v>
+        <v>4.0001</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.033</v>
+        <v>0.0323</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6756</v>
+        <v>0.6826</v>
       </c>
       <c r="EK2" t="n">
-        <v>66.63</v>
+        <v>56.76</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>1.68</v>
+        <v>0</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.1977</v>
+        <v>0</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0506</v>
+        <v>0.0212</v>
       </c>
       <c r="ER2" t="n">
-        <v>22.8372</v>
+        <v>54</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.2486</v>
+        <v>10.5277</v>
       </c>
       <c r="ET2" t="n">
-        <v>35.368</v>
+        <v>30.142</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.0234</v>
+        <v>0.4194</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7203</v>
+        <v>2.0593</v>
       </c>
       <c r="EW2" t="n">
-        <v>1.174</v>
+        <v>0</v>
       </c>
       <c r="EX2" t="n">
-        <v>29.96</v>
+        <v>22.46</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2278,37 +2278,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="FA2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.56</v>
+        <v>63.14</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.49</v>
+        <v>29.6</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.39</v>
+        <v>75.43000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>68.255</v>
+        <v>62.195</v>
       </c>
       <c r="FF2" t="n">
-        <v>34.725</v>
+        <v>25.23</v>
       </c>
       <c r="FG2" t="n">
-        <v>20.1965</v>
+        <v>19.7172</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.736</v>
+        <v>56.351</v>
       </c>
       <c r="FI2" t="n">
-        <v>42.17</v>
+        <v>51.445</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.29</v>
+        <v>61.36</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>66.81999999999999</v>
+        <v>68.64</v>
       </c>
       <c r="FO2" t="n">
-        <v>59.86</v>
+        <v>57.64</v>
       </c>
       <c r="FP2" t="n">
-        <v>50.44</v>
+        <v>51.34</v>
       </c>
       <c r="FQ2" t="n">
-        <v>67.70999999999999</v>
+        <v>73.70999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.73</v>
+        <v>76.26000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>95.2381</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.17400000000001</v>
+        <v>65.8355</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260903_200051</t>
+          <t>20260904_133217</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46268.83392919807</v>
+        <v>46269.56409637652</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46268.83392361111</v>
+        <v>46269.56408564815</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1868.5</v>
+        <v>1843.9</v>
       </c>
       <c r="L2" t="n">
-        <v>1864.9</v>
+        <v>1855</v>
       </c>
       <c r="M2" t="n">
-        <v>1876.6</v>
+        <v>1871.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1852.6</v>
+        <v>1841</v>
       </c>
       <c r="O2" t="n">
-        <v>1868.5</v>
+        <v>1843.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1506252</v>
+        <v>634328</v>
       </c>
       <c r="Q2" t="n">
-        <v>1868.5</v>
+        <v>1843.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2052.04</v>
+        <v>2023.13</v>
       </c>
       <c r="S2" t="n">
-        <v>1776.73</v>
+        <v>1754.29</v>
       </c>
       <c r="T2" t="n">
-        <v>9.822852555525822</v>
+        <v>9.72015835999783</v>
       </c>
       <c r="U2" t="n">
-        <v>183.54</v>
+        <v>179.23</v>
       </c>
       <c r="V2" t="n">
-        <v>4.911426277762911</v>
+        <v>4.859808015619075</v>
       </c>
       <c r="W2" t="n">
-        <v>91.76999999999998</v>
+        <v>89.61000000000013</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.00011159468809</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.822852555525822</v>
+        <v>9.72015835999783</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.911426277762911</v>
+        <v>4.859808015619075</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02052804421462072</v>
+        <v>0.02053686013661902</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.325872599366548</v>
+        <v>0.3260125477896594</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909858947718529</v>
+        <v>0.02909857256287051</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353057055038</v>
+        <v>0.04266354522577397</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.93</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-03 20:00:51.523849+05:30</t>
+          <t>2026-09-04 13:32:17.954310+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.822852555525822, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.72015835999783, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001115946880903}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-04 14:19 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.94</v>
+        <v>48.99</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,43 +1875,43 @@
         <v>1871.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1841</v>
+        <v>1835.2</v>
       </c>
       <c r="X2" t="n">
-        <v>1843.9</v>
+        <v>1840</v>
       </c>
       <c r="Y2" t="n">
-        <v>1843.9</v>
+        <v>1840</v>
       </c>
       <c r="Z2" t="n">
-        <v>634328</v>
+        <v>1074891</v>
       </c>
       <c r="AA2" t="n">
-        <v>3458823</v>
+        <v>3480851</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.18</v>
+        <v>0.31</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.32</v>
+        <v>-1.53</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.72</v>
       </c>
       <c r="AE2" t="n">
-        <v>30.8</v>
+        <v>36.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.67</v>
+        <v>1.99</v>
       </c>
       <c r="AG2" t="n">
-        <v>44.81</v>
+        <v>45.22</v>
       </c>
       <c r="AH2" t="n">
-        <v>44.81</v>
+        <v>45.22</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.43</v>
+        <v>2.46</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.41</v>
+        <v>-0.61</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.44</v>
+        <v>7.21</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.06</v>
+        <v>44.75</v>
       </c>
       <c r="AO2" t="n">
-        <v>54.87</v>
+        <v>54.19</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.33</v>
+        <v>2.11</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.45</v>
+        <v>29.18</v>
       </c>
       <c r="AR2" t="n">
-        <v>1843.9</v>
+        <v>1840</v>
       </c>
       <c r="AS2" t="n">
-        <v>2023.13</v>
+        <v>2020.89</v>
       </c>
       <c r="AT2" t="n">
-        <v>1754.29</v>
+        <v>1749.56</v>
       </c>
       <c r="AU2" t="n">
-        <v>1843.900024414062</v>
+        <v>1840</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.720000000000001</v>
+        <v>9.83</v>
       </c>
       <c r="AY2" t="n">
-        <v>179.23</v>
+        <v>180.89</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.86</v>
+        <v>4.92</v>
       </c>
       <c r="BA2" t="n">
-        <v>89.61</v>
+        <v>90.44</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2082,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>67.63</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>28</v>
+        <v>30.6</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>90.47619047619048</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>90.47619047619048</v>
+        <v>90.90909090909091</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>90.47619047619048</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>71.42857142857143</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.7202</v>
+        <v>9.831</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2127,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.648</v>
+        <v>0.6553</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.324</v>
+        <v>0.328</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.0983</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.144</v>
+        <v>1.157</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9959</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8598</v>
+        <v>4.9152</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.11</v>
+        <v>37.15</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8598</v>
+        <v>4.9152</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2160,25 +2160,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9959</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.823</v>
+        <v>0.8122</v>
       </c>
       <c r="DQ2" t="n">
-        <v>89.61</v>
+        <v>90.44</v>
       </c>
       <c r="DR2" t="n">
-        <v>66.78</v>
+        <v>39.68</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9588</v>
+        <v>0.8577</v>
       </c>
       <c r="DX2" t="n">
-        <v>87.175</v>
+        <v>85.47499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>9</v>
+        <v>15.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>67.404</v>
+        <v>66.8</v>
       </c>
       <c r="EA2" t="n">
         <v>4</v>
@@ -2205,31 +2205,31 @@
         <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>53.26</v>
+        <v>51.88</v>
       </c>
       <c r="ED2" t="n">
-        <v>86.02</v>
+        <v>82.88</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9588</v>
+        <v>0.8577</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.18</v>
+        <v>0.31</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2742</v>
+        <v>0.2483</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0001</v>
+        <v>3.9963</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0323</v>
+        <v>0.0292</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6826</v>
+        <v>0.6751</v>
       </c>
       <c r="EK2" t="n">
-        <v>56.76</v>
+        <v>56.21</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="EP2" t="n">
-        <v>0</v>
+        <v>0.0259</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0212</v>
+        <v>0.0365</v>
       </c>
       <c r="ER2" t="n">
-        <v>54</v>
+        <v>31.7097</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5277</v>
+        <v>10.737</v>
       </c>
       <c r="ET2" t="n">
-        <v>30.142</v>
+        <v>31.335</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.4194</v>
+        <v>0.6541</v>
       </c>
       <c r="EV2" t="n">
-        <v>2.0593</v>
+        <v>1.8779</v>
       </c>
       <c r="EW2" t="n">
-        <v>0</v>
+        <v>0.1486</v>
       </c>
       <c r="EX2" t="n">
-        <v>22.46</v>
+        <v>23.87</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>4</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.14</v>
+        <v>63.43</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.6</v>
+        <v>30.5</v>
       </c>
       <c r="FD2" t="n">
-        <v>75.43000000000001</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>62.195</v>
+        <v>61.875</v>
       </c>
       <c r="FF2" t="n">
-        <v>25.23</v>
+        <v>27.235</v>
       </c>
       <c r="FG2" t="n">
-        <v>19.7172</v>
+        <v>19.5202</v>
       </c>
       <c r="FH2" t="n">
-        <v>56.351</v>
+        <v>56.751</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.445</v>
+        <v>38.415</v>
       </c>
       <c r="FJ2" t="n">
-        <v>61.36</v>
+        <v>60.57</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,28 +2322,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>68.64</v>
+        <v>59.37</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.64</v>
+        <v>56.2</v>
       </c>
       <c r="FP2" t="n">
-        <v>51.34</v>
+        <v>40.04</v>
       </c>
       <c r="FQ2" t="n">
-        <v>73.70999999999999</v>
+        <v>61.12</v>
       </c>
       <c r="FR2" t="n">
-        <v>76.26000000000001</v>
+        <v>66</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.2381</v>
+        <v>72.7273</v>
       </c>
       <c r="FT2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2351,21 +2351,21 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.8355</v>
+        <v>56.6385</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260904_133217</t>
+          <t>20260904_194927</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46269.56409637652</v>
+        <v>46269.82601482474</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46269.56408564815</v>
+        <v>46269.82600694444</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1843.9</v>
+        <v>1840</v>
       </c>
       <c r="L2" t="n">
         <v>1855</v>
@@ -2676,37 +2676,37 @@
         <v>1871.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1841</v>
+        <v>1835.2</v>
       </c>
       <c r="O2" t="n">
-        <v>1843.9</v>
+        <v>1840</v>
       </c>
       <c r="P2" t="n">
-        <v>634328</v>
+        <v>1074891</v>
       </c>
       <c r="Q2" t="n">
-        <v>1843.9</v>
+        <v>1840</v>
       </c>
       <c r="R2" t="n">
-        <v>2023.13</v>
+        <v>2020.89</v>
       </c>
       <c r="S2" t="n">
-        <v>1754.29</v>
+        <v>1749.56</v>
       </c>
       <c r="T2" t="n">
-        <v>9.72015835999783</v>
+        <v>9.830978260869569</v>
       </c>
       <c r="U2" t="n">
-        <v>179.23</v>
+        <v>180.8900000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.859808015619075</v>
+        <v>4.915217391304351</v>
       </c>
       <c r="W2" t="n">
-        <v>89.61000000000013</v>
+        <v>90.44000000000005</v>
       </c>
       <c r="X2" t="n">
-        <v>2.00011159468809</v>
+        <v>2.000110570544007</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.72015835999783</v>
+        <v>9.830978260869569</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.859808015619075</v>
+        <v>4.915217391304351</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02053686013661902</v>
+        <v>0.02052433265811339</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3260125477896594</v>
+        <v>0.3258136802335757</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909857256287051</v>
+        <v>0.02909853027070199</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266354522577397</v>
+        <v>0.04266353895739713</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.92</v>
+        <v>38.93</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-04 13:32:17.954310+05:30</t>
+          <t>2026-09-04 19:49:27.718391+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.72015835999783, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001115946880903}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.83097826086957, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000110570544007}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-07 08:23 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.99</v>
+        <v>48.96</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1855</v>
+        <v>1840</v>
       </c>
       <c r="V2" t="n">
-        <v>1871.8</v>
+        <v>1866.7</v>
       </c>
       <c r="W2" t="n">
-        <v>1835.2</v>
+        <v>1832.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1840</v>
+        <v>1861</v>
       </c>
       <c r="Y2" t="n">
-        <v>1840</v>
+        <v>1861</v>
       </c>
       <c r="Z2" t="n">
-        <v>1074891</v>
+        <v>763354</v>
       </c>
       <c r="AA2" t="n">
-        <v>3480851</v>
+        <v>3449742</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.53</v>
+        <v>1.14</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.72</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>36.6</v>
+        <v>34</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.99</v>
+        <v>1.83</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.22</v>
+        <v>44.42</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.22</v>
+        <v>44.42</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.46</v>
+        <v>2.39</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.61</v>
+        <v>0.51</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.21</v>
+        <v>7.98</v>
       </c>
       <c r="AN2" t="n">
-        <v>44.75</v>
+        <v>45.9</v>
       </c>
       <c r="AO2" t="n">
-        <v>54.19</v>
+        <v>57.26</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.11</v>
+        <v>3.33</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.18</v>
+        <v>34.3</v>
       </c>
       <c r="AR2" t="n">
-        <v>1840</v>
+        <v>1861</v>
       </c>
       <c r="AS2" t="n">
-        <v>2020.89</v>
+        <v>2038.68</v>
       </c>
       <c r="AT2" t="n">
-        <v>1749.56</v>
+        <v>1772.16</v>
       </c>
       <c r="AU2" t="n">
-        <v>1840</v>
+        <v>1861</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.83</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>180.89</v>
+        <v>177.68</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.92</v>
+        <v>4.77</v>
       </c>
       <c r="BA2" t="n">
-        <v>90.44</v>
+        <v>88.84</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>67.54000000000001</v>
+        <v>75.86</v>
       </c>
       <c r="CO2" t="n">
-        <v>30.6</v>
+        <v>28.29</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2100,7 +2100,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>90.90909090909091</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2115,10 @@
         <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.831</v>
+        <v>9.547599999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6553</v>
+        <v>0.6367</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.328</v>
+        <v>0.318</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0983</v>
+        <v>0.0955</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2.0021</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.157</v>
+        <v>1.124</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9959</v>
+        <v>3.9958</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9152</v>
+        <v>4.7738</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.15</v>
+        <v>36.81</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9152</v>
+        <v>4.7738</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9958</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9959</v>
+        <v>3.9958</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>2.0022</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8122</v>
+        <v>0.8377</v>
       </c>
       <c r="DQ2" t="n">
-        <v>90.44</v>
+        <v>88.84</v>
       </c>
       <c r="DR2" t="n">
-        <v>39.68</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,90 +2187,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.8577</v>
+        <v>1.3933</v>
       </c>
       <c r="DX2" t="n">
-        <v>85.47499999999999</v>
+        <v>93.14999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>15.5</v>
+        <v>11</v>
       </c>
       <c r="DZ2" t="n">
-        <v>66.8</v>
+        <v>77.001</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>51.88</v>
+        <v>78.58</v>
       </c>
       <c r="ED2" t="n">
-        <v>82.88</v>
+        <v>95.72</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.8577</v>
+        <v>1.3933</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2483</v>
+        <v>0.3919</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9963</v>
+        <v>3.9948</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0292</v>
+        <v>0.0461</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6751</v>
+        <v>0.6923</v>
       </c>
       <c r="EK2" t="n">
-        <v>56.21</v>
+        <v>63.87</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>0.22</v>
+        <v>1.13</v>
       </c>
       <c r="EP2" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="EQ2" t="n">
         <v>0.0259</v>
       </c>
-      <c r="EQ2" t="n">
-        <v>0.0365</v>
-      </c>
       <c r="ER2" t="n">
-        <v>31.7097</v>
+        <v>43.4091</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.737</v>
+        <v>10.8584</v>
       </c>
       <c r="ET2" t="n">
-        <v>31.335</v>
+        <v>30.717</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.6541</v>
+        <v>0.7326</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8779</v>
+        <v>1.959</v>
       </c>
       <c r="EW2" t="n">
-        <v>0.1486</v>
+        <v>0.8572</v>
       </c>
       <c r="EX2" t="n">
-        <v>23.87</v>
+        <v>20.09</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2278,37 +2278,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.43</v>
+        <v>63.54</v>
       </c>
       <c r="FC2" t="n">
-        <v>30.5</v>
+        <v>29.97</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.84999999999999</v>
+        <v>73.77</v>
       </c>
       <c r="FE2" t="n">
-        <v>61.875</v>
+        <v>69.86499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>27.235</v>
+        <v>24.19</v>
       </c>
       <c r="FG2" t="n">
-        <v>19.5202</v>
+        <v>22.3776</v>
       </c>
       <c r="FH2" t="n">
-        <v>56.751</v>
+        <v>58.546</v>
       </c>
       <c r="FI2" t="n">
-        <v>38.415</v>
+        <v>51.605</v>
       </c>
       <c r="FJ2" t="n">
-        <v>60.57</v>
+        <v>62.48</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,50 +2322,50 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>59.37</v>
+        <v>71.18000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>56.2</v>
+        <v>59.32</v>
       </c>
       <c r="FP2" t="n">
-        <v>40.04</v>
+        <v>52.37</v>
       </c>
       <c r="FQ2" t="n">
-        <v>61.12</v>
+        <v>77.23</v>
       </c>
       <c r="FR2" t="n">
-        <v>66</v>
+        <v>80.54000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>72.7273</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>56.6385</v>
+        <v>68.2475</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260904_194927</t>
+          <t>20260907_135353</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46269.82601482474</v>
+        <v>46272.57908569172</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46269.82600694444</v>
+        <v>46272.57908564815</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
+        <v>1861</v>
+      </c>
+      <c r="L2" t="n">
         <v>1840</v>
       </c>
-      <c r="L2" t="n">
-        <v>1855</v>
-      </c>
       <c r="M2" t="n">
-        <v>1871.8</v>
+        <v>1866.7</v>
       </c>
       <c r="N2" t="n">
-        <v>1835.2</v>
+        <v>1832.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1840</v>
+        <v>1861</v>
       </c>
       <c r="P2" t="n">
-        <v>1074891</v>
+        <v>763354</v>
       </c>
       <c r="Q2" t="n">
-        <v>1840</v>
+        <v>1861</v>
       </c>
       <c r="R2" t="n">
-        <v>2020.89</v>
+        <v>2038.68</v>
       </c>
       <c r="S2" t="n">
-        <v>1749.56</v>
+        <v>1772.16</v>
       </c>
       <c r="T2" t="n">
-        <v>9.830978260869569</v>
+        <v>9.547555077915103</v>
       </c>
       <c r="U2" t="n">
-        <v>180.8900000000001</v>
+        <v>177.6800000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.915217391304351</v>
+        <v>4.773777538957545</v>
       </c>
       <c r="W2" t="n">
-        <v>90.44000000000005</v>
+        <v>88.83999999999992</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000110570544007</v>
+        <v>2.000000000000003</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.830978260869569</v>
+        <v>9.547555077915103</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.915217391304351</v>
+        <v>4.773777538957545</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02052433265811339</v>
+        <v>0.02051214052536761</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3258136802335757</v>
+        <v>0.3256201361263948</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909853027070199</v>
+        <v>0.0290984710642187</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353895739713</v>
+        <v>0.04266352464159216</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.93</v>
+        <v>38.95</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-04 19:49:27.718391+05:30</t>
+          <t>2026-09-07 13:53:53.042992+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.83097826086957, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000110570544007}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.547555077915103, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-07 15:49 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.96</v>
+        <v>49</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1872,46 +1872,46 @@
         <v>1840</v>
       </c>
       <c r="V2" t="n">
-        <v>1866.7</v>
+        <v>1876.7</v>
       </c>
       <c r="W2" t="n">
         <v>1832.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1861</v>
+        <v>1876.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>1861</v>
+        <v>1876.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>763354</v>
+        <v>1148595</v>
       </c>
       <c r="AA2" t="n">
-        <v>3449742</v>
+        <v>3469004</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.14</v>
+        <v>1.99</v>
       </c>
       <c r="AD2" t="n">
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.83</v>
+        <v>2.34</v>
       </c>
       <c r="AG2" t="n">
-        <v>44.42</v>
+        <v>45.13</v>
       </c>
       <c r="AH2" t="n">
-        <v>44.42</v>
+        <v>45.13</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.39</v>
+        <v>2.4</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.51</v>
+        <v>1.31</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.98</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.9</v>
+        <v>47.12</v>
       </c>
       <c r="AO2" t="n">
-        <v>57.26</v>
+        <v>59.3</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.33</v>
+        <v>4.2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.3</v>
+        <v>35.43</v>
       </c>
       <c r="AR2" t="n">
-        <v>1861</v>
+        <v>1876.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>2038.68</v>
+        <v>2057.24</v>
       </c>
       <c r="AT2" t="n">
-        <v>1772.16</v>
+        <v>1786.43</v>
       </c>
       <c r="AU2" t="n">
-        <v>1861</v>
+        <v>1876.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.550000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>177.68</v>
+        <v>180.54</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.77</v>
+        <v>4.81</v>
       </c>
       <c r="BA2" t="n">
-        <v>88.84</v>
+        <v>90.27</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.86</v>
+        <v>78.52</v>
       </c>
       <c r="CO2" t="n">
-        <v>28.29</v>
+        <v>29.7</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.547599999999999</v>
+        <v>9.620100000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6367</v>
+        <v>0.6413</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.318</v>
+        <v>0.3207</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0955</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.124</v>
+        <v>1.1323</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9958</v>
+        <v>4.0083</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7738</v>
+        <v>4.81</v>
       </c>
       <c r="DJ2" t="n">
-        <v>36.81</v>
+        <v>37.47</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7738</v>
+        <v>4.81</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9958</v>
+        <v>2.0042</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9958</v>
+        <v>4.0083</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0022</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8377</v>
+        <v>0.8333</v>
       </c>
       <c r="DQ2" t="n">
-        <v>88.84</v>
+        <v>90.27</v>
       </c>
       <c r="DR2" t="n">
-        <v>66.40000000000001</v>
+        <v>54.68</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.3933</v>
+        <v>1.75</v>
       </c>
       <c r="DX2" t="n">
-        <v>93.14999999999999</v>
+        <v>98.25</v>
       </c>
       <c r="DY2" t="n">
-        <v>11</v>
+        <v>16.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>77.001</v>
+        <v>80.306</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>78.58</v>
+        <v>86.43000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>95.72</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.3933</v>
+        <v>1.75</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3919</v>
+        <v>0.4943</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9948</v>
+        <v>4.0084</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0461</v>
+        <v>0.0582</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6923</v>
+        <v>0.6899</v>
       </c>
       <c r="EK2" t="n">
-        <v>63.87</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>1.13</v>
+        <v>1.47</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.133</v>
+        <v>0.173</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0259</v>
+        <v>0.0388</v>
       </c>
       <c r="ER2" t="n">
-        <v>43.4091</v>
+        <v>29.1515</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.8584</v>
+        <v>11.0206</v>
       </c>
       <c r="ET2" t="n">
-        <v>30.717</v>
+        <v>31.455</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.7326</v>
+        <v>1.386</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.959</v>
+        <v>1.8045</v>
       </c>
       <c r="EW2" t="n">
-        <v>0.8572</v>
+        <v>1.1542</v>
       </c>
       <c r="EX2" t="n">
-        <v>20.09</v>
+        <v>20.34</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>5</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.54</v>
+        <v>63.78</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.97</v>
+        <v>30.7</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.77</v>
+        <v>73.33</v>
       </c>
       <c r="FE2" t="n">
-        <v>69.86499999999999</v>
+        <v>78.06</v>
       </c>
       <c r="FF2" t="n">
-        <v>24.19</v>
+        <v>25.02</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.3776</v>
+        <v>23.0941</v>
       </c>
       <c r="FH2" t="n">
-        <v>58.546</v>
+        <v>59.514</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.605</v>
+        <v>46.075</v>
       </c>
       <c r="FJ2" t="n">
-        <v>62.48</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.18000000000001</v>
+        <v>68.02</v>
       </c>
       <c r="FO2" t="n">
-        <v>59.32</v>
+        <v>65.52</v>
       </c>
       <c r="FP2" t="n">
-        <v>52.37</v>
+        <v>42.08</v>
       </c>
       <c r="FQ2" t="n">
-        <v>77.23</v>
+        <v>67.48</v>
       </c>
       <c r="FR2" t="n">
-        <v>80.54000000000001</v>
+        <v>74.58</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.2475</v>
+        <v>63.9765</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260907_135353</t>
+          <t>20260907_211905</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46272.57908569172</v>
+        <v>46272.88825544015</v>
       </c>
     </row>
   </sheetData>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46272.57908564815</v>
+        <v>46272.88825231481</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1861</v>
+        <v>1876.7</v>
       </c>
       <c r="L2" t="n">
         <v>1840</v>
       </c>
       <c r="M2" t="n">
-        <v>1866.7</v>
+        <v>1876.7</v>
       </c>
       <c r="N2" t="n">
         <v>1832.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1861</v>
+        <v>1876.7</v>
       </c>
       <c r="P2" t="n">
-        <v>763354</v>
+        <v>1148595</v>
       </c>
       <c r="Q2" t="n">
-        <v>1861</v>
+        <v>1876.7</v>
       </c>
       <c r="R2" t="n">
-        <v>2038.68</v>
+        <v>2057.24</v>
       </c>
       <c r="S2" t="n">
-        <v>1772.16</v>
+        <v>1786.43</v>
       </c>
       <c r="T2" t="n">
-        <v>9.547555077915103</v>
+        <v>9.620077796131493</v>
       </c>
       <c r="U2" t="n">
-        <v>177.6800000000001</v>
+        <v>180.5399999999997</v>
       </c>
       <c r="V2" t="n">
-        <v>4.773777538957545</v>
+        <v>4.810038898065753</v>
       </c>
       <c r="W2" t="n">
-        <v>88.83999999999992</v>
+        <v>90.26999999999998</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000003</v>
+        <v>1.999999999999998</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.547555077915103</v>
+        <v>9.620077796131493</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.773777538957545</v>
+        <v>4.810038898065753</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02051214052536761</v>
+        <v>0.02052010616750097</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3256201361263948</v>
+        <v>0.3257465867751017</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290984710642187</v>
+        <v>0.02909844287369406</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266352464159216</v>
+        <v>0.04266353522846195</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.95</v>
+        <v>38.94</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-07 13:53:53.042992+05:30</t>
+          <t>2026-09-07 21:19:05.306015+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.547555077915103, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000027}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.620077796131493, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999976}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-08 08:09 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49</v>
+        <v>49.04</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1840</v>
+        <v>1870.8</v>
       </c>
       <c r="V2" t="n">
-        <v>1876.7</v>
+        <v>1948.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1832.7</v>
+        <v>1862.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1876.7</v>
+        <v>1941</v>
       </c>
       <c r="Y2" t="n">
-        <v>1876.7</v>
+        <v>1941</v>
       </c>
       <c r="Z2" t="n">
-        <v>1148595</v>
+        <v>1446433</v>
       </c>
       <c r="AA2" t="n">
-        <v>3469004</v>
+        <v>3483896</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.33</v>
+        <v>0.42</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.99</v>
+        <v>5.49</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="AE2" t="n">
-        <v>44</v>
+        <v>86.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.34</v>
+        <v>4.44</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.13</v>
+        <v>49.77</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.13</v>
+        <v>49.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.4</v>
+        <v>2.56</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.31</v>
+        <v>4.6</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.880000000000001</v>
+        <v>12.52</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.12</v>
+        <v>52.13</v>
       </c>
       <c r="AO2" t="n">
-        <v>59.3</v>
+        <v>65.95</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.2</v>
+        <v>7.77</v>
       </c>
       <c r="AQ2" t="n">
-        <v>35.43</v>
+        <v>40.07</v>
       </c>
       <c r="AR2" t="n">
-        <v>1876.7</v>
+        <v>1941</v>
       </c>
       <c r="AS2" t="n">
-        <v>2057.24</v>
+        <v>2140.08</v>
       </c>
       <c r="AT2" t="n">
-        <v>1786.43</v>
+        <v>1841.46</v>
       </c>
       <c r="AU2" t="n">
-        <v>1876.699951171875</v>
+        <v>1941</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.619999999999999</v>
+        <v>10.26</v>
       </c>
       <c r="AY2" t="n">
-        <v>180.54</v>
+        <v>199.08</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.81</v>
+        <v>5.13</v>
       </c>
       <c r="BA2" t="n">
-        <v>90.27</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>78.52</v>
+        <v>82.78</v>
       </c>
       <c r="CO2" t="n">
-        <v>29.7</v>
+        <v>43.43</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2112,13 +2112,13 @@
         <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.620100000000001</v>
+        <v>10.2566</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6413</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3207</v>
+        <v>0.342</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09619999999999999</v>
+        <v>0.1026</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1323</v>
+        <v>1.2076</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0083</v>
+        <v>4.0078</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.81</v>
+        <v>5.1283</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.47</v>
+        <v>48.35</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.81</v>
+        <v>5.1283</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0042</v>
+        <v>2.0039</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0083</v>
+        <v>4.0078</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8333</v>
+        <v>0.7812</v>
       </c>
       <c r="DQ2" t="n">
-        <v>90.27</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>54.68</v>
+        <v>63.76</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.75</v>
+        <v>3.0352</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.25</v>
+        <v>85.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>16.5</v>
+        <v>21</v>
       </c>
       <c r="DZ2" t="n">
-        <v>80.306</v>
+        <v>88.29300000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>86.43000000000001</v>
+        <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>83.72</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.75</v>
+        <v>3.0352</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.33</v>
+        <v>0.42</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4943</v>
+        <v>0.9145</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0084</v>
+        <v>4.0065</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0582</v>
+        <v>0.1076</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6899</v>
+        <v>0.6536</v>
       </c>
       <c r="EK2" t="n">
-        <v>77.59999999999999</v>
+        <v>76.72</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,72 +2243,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>1.47</v>
+        <v>16.17</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.173</v>
+        <v>1.9032</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0388</v>
+        <v>0.0494</v>
       </c>
       <c r="ER2" t="n">
-        <v>29.1515</v>
+        <v>24.4286</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.0206</v>
+        <v>13.5815</v>
       </c>
       <c r="ET2" t="n">
-        <v>31.455</v>
+        <v>41.357</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.386</v>
+        <v>3.2634</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8045</v>
+        <v>1.8028</v>
       </c>
       <c r="EW2" t="n">
-        <v>1.1542</v>
+        <v>13.3855</v>
       </c>
       <c r="EX2" t="n">
-        <v>20.34</v>
+        <v>43.25</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
         <v>63.78</v>
       </c>
       <c r="FC2" t="n">
-        <v>30.7</v>
+        <v>40.9</v>
       </c>
       <c r="FD2" t="n">
         <v>73.33</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.06</v>
+        <v>79.75</v>
       </c>
       <c r="FF2" t="n">
-        <v>25.02</v>
+        <v>43.34</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.0941</v>
+        <v>23.2528</v>
       </c>
       <c r="FH2" t="n">
-        <v>59.514</v>
+        <v>65.374</v>
       </c>
       <c r="FI2" t="n">
-        <v>46.075</v>
+        <v>56.055</v>
       </c>
       <c r="FJ2" t="n">
-        <v>64.31999999999999</v>
+        <v>70.66</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>68.02</v>
+        <v>78.67</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.52</v>
+        <v>72.52</v>
       </c>
       <c r="FP2" t="n">
-        <v>42.08</v>
+        <v>67.14</v>
       </c>
       <c r="FQ2" t="n">
-        <v>67.48</v>
+        <v>76.06999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.58</v>
+        <v>94.27</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>63.9765</v>
+        <v>78.0835</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260907_211905</t>
+          <t>20260908_133921</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46272.88825544015</v>
+        <v>46273.56899917638</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46272.88825231481</v>
+        <v>46273.56899305555</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1876.7</v>
+        <v>1941</v>
       </c>
       <c r="L2" t="n">
-        <v>1840</v>
+        <v>1870.8</v>
       </c>
       <c r="M2" t="n">
-        <v>1876.7</v>
+        <v>1948.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1832.7</v>
+        <v>1862.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1876.7</v>
+        <v>1941</v>
       </c>
       <c r="P2" t="n">
-        <v>1148595</v>
+        <v>1446433</v>
       </c>
       <c r="Q2" t="n">
-        <v>1876.7</v>
+        <v>1941</v>
       </c>
       <c r="R2" t="n">
-        <v>2057.24</v>
+        <v>2140.08</v>
       </c>
       <c r="S2" t="n">
-        <v>1786.43</v>
+        <v>1841.46</v>
       </c>
       <c r="T2" t="n">
-        <v>9.620077796131493</v>
+        <v>10.2565687789799</v>
       </c>
       <c r="U2" t="n">
-        <v>180.5399999999997</v>
+        <v>199.0799999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.810038898065753</v>
+        <v>5.128284389489952</v>
       </c>
       <c r="W2" t="n">
-        <v>90.26999999999998</v>
+        <v>99.53999999999996</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999998</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.620077796131493</v>
+        <v>10.2565687789799</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.810038898065753</v>
+        <v>5.128284389489952</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02052010616750097</v>
+        <v>0.02060649668265513</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3257465867751017</v>
+        <v>0.3271179936874977</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909844287369406</v>
+        <v>0.0290984710642187</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353522846195</v>
+        <v>0.0426635352331118</v>
       </c>
     </row>
     <row r="13">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.94</v>
+        <v>38.83</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-07 21:19:05.306015+05:30</t>
+          <t>2026-09-08 13:39:21.564483+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.620077796131493, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999976}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.256568778979904, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-08 14:30 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.04</v>
+        <v>49.12</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1872,46 +1872,46 @@
         <v>1870.8</v>
       </c>
       <c r="V2" t="n">
-        <v>1948.9</v>
+        <v>1952</v>
       </c>
       <c r="W2" t="n">
         <v>1862.7</v>
       </c>
       <c r="X2" t="n">
-        <v>1941</v>
+        <v>1946.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>1941</v>
+        <v>1946.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1446433</v>
+        <v>2115303</v>
       </c>
       <c r="AA2" t="n">
-        <v>3483896</v>
+        <v>3517339</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.42</v>
+        <v>0.6</v>
       </c>
       <c r="AC2" t="n">
-        <v>5.49</v>
+        <v>5.81</v>
       </c>
       <c r="AD2" t="n">
         <v>1.67</v>
       </c>
       <c r="AE2" t="n">
-        <v>86.2</v>
+        <v>89.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.44</v>
+        <v>4.59</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.77</v>
+        <v>49.99</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.77</v>
+        <v>49.99</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.56</v>
+        <v>2.57</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.52</v>
+        <v>12.86</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.13</v>
+        <v>52.58</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.95</v>
+        <v>66.45</v>
       </c>
       <c r="AP2" t="n">
-        <v>7.77</v>
+        <v>8.1</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.07</v>
+        <v>40.5</v>
       </c>
       <c r="AR2" t="n">
-        <v>1941</v>
+        <v>1946.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2140.08</v>
+        <v>2146.87</v>
       </c>
       <c r="AT2" t="n">
-        <v>1841.46</v>
+        <v>1846.92</v>
       </c>
       <c r="AU2" t="n">
-        <v>1941</v>
+        <v>1946.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.26</v>
+        <v>10.27</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.08</v>
+        <v>199.97</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.13</v>
+        <v>5.14</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.54000000000001</v>
+        <v>99.98</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.7</v>
+        <v>1480.71</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.78</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.43</v>
+        <v>44.07</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>90.47619047619048</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2566</v>
+        <v>10.2712</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.6847</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.342</v>
+        <v>0.3427</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1026</v>
+        <v>0.1027</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.9981</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.2088</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>3.9961</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>5.1353</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>48.13</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>5.1353</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.2076</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>4.0078</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>5.1283</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>48.35</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>5.1283</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>2</v>
-      </c>
-      <c r="DM2" t="n">
-        <v>2.0039</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0078</v>
+        <v>3.9961</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7812</v>
+        <v>0.7775</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.54000000000001</v>
+        <v>99.98</v>
       </c>
       <c r="DR2" t="n">
-        <v>63.76</v>
+        <v>54.54</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>3.0352</v>
+        <v>3.1518</v>
       </c>
       <c r="DX2" t="n">
-        <v>85.125</v>
+        <v>83.875</v>
       </c>
       <c r="DY2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.29300000000001</v>
+        <v>88.441</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2208,28 +2208,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>83.72</v>
+        <v>83.15000000000001</v>
       </c>
       <c r="EE2" t="n">
-        <v>3.0352</v>
+        <v>3.1518</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.42</v>
+        <v>0.6</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.9145</v>
+        <v>0.9534</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0065</v>
+        <v>3.9966</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1076</v>
+        <v>0.1122</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6536</v>
+        <v>0.6509</v>
       </c>
       <c r="EK2" t="n">
-        <v>76.72</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>16.17</v>
+        <v>17.47</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.9032</v>
+        <v>2.0562</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0494</v>
+        <v>0.0706</v>
       </c>
       <c r="ER2" t="n">
-        <v>24.4286</v>
+        <v>17.1167</v>
       </c>
       <c r="ES2" t="n">
-        <v>13.5815</v>
+        <v>13.4818</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.357</v>
+        <v>41.916</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.2634</v>
+        <v>4.86</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8028</v>
+        <v>1.6062</v>
       </c>
       <c r="EW2" t="n">
-        <v>13.3855</v>
+        <v>14.5944</v>
       </c>
       <c r="EX2" t="n">
-        <v>43.25</v>
+        <v>43.11</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.78</v>
+        <v>63.49</v>
       </c>
       <c r="FC2" t="n">
-        <v>40.9</v>
+        <v>41.32</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.33</v>
+        <v>74.56999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>79.75</v>
+        <v>76.27500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.34</v>
+        <v>43.59</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.2528</v>
+        <v>23.4006</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.374</v>
+        <v>65.429</v>
       </c>
       <c r="FI2" t="n">
-        <v>56.055</v>
+        <v>51.335</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.66</v>
+        <v>70.56</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>78.67</v>
+        <v>74.08</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.52</v>
+        <v>72.69</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.14</v>
+        <v>60.23</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.06999999999999</v>
+        <v>69.17</v>
       </c>
       <c r="FR2" t="n">
-        <v>94.27</v>
+        <v>86.79000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>78.0835</v>
+        <v>72.9075</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260908_133921</t>
+          <t>20260908_200043</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46273.56899917638</v>
+        <v>46273.83384005574</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46273.56899305555</v>
+        <v>46273.83383101852</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1941</v>
+        <v>1946.9</v>
       </c>
       <c r="L2" t="n">
         <v>1870.8</v>
       </c>
       <c r="M2" t="n">
-        <v>1948.9</v>
+        <v>1952</v>
       </c>
       <c r="N2" t="n">
         <v>1862.7</v>
       </c>
       <c r="O2" t="n">
-        <v>1941</v>
+        <v>1946.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1446433</v>
+        <v>2115303</v>
       </c>
       <c r="Q2" t="n">
-        <v>1941</v>
+        <v>1946.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2140.08</v>
+        <v>2146.87</v>
       </c>
       <c r="S2" t="n">
-        <v>1841.46</v>
+        <v>1846.92</v>
       </c>
       <c r="T2" t="n">
-        <v>10.2565687789799</v>
+        <v>10.27120036981868</v>
       </c>
       <c r="U2" t="n">
-        <v>199.0799999999999</v>
+        <v>199.9699999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>5.128284389489952</v>
+        <v>5.135343366377318</v>
       </c>
       <c r="W2" t="n">
-        <v>99.53999999999996</v>
+        <v>99.98000000000002</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000100020003998</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.2565687789799</v>
+        <v>10.27120036981868</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.128284389489952</v>
+        <v>5.135343366377318</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02060649668265513</v>
+        <v>0.02061873646256678</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3271179936874977</v>
+        <v>0.327312294169988</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0426635352331118</v>
+        <v>0.04266353098562824</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.83</v>
+        <v>38.82</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 13:39:21.564483+05:30</t>
+          <t>2026-09-08 20:00:43.820829+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.256568778979904, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.271200369818676, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001000200039982}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-09 08:12 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.12</v>
+        <v>49.02</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1870.8</v>
+        <v>1946.9</v>
       </c>
       <c r="V2" t="n">
-        <v>1952</v>
+        <v>1955</v>
       </c>
       <c r="W2" t="n">
-        <v>1862.7</v>
+        <v>1917.9</v>
       </c>
       <c r="X2" t="n">
-        <v>1946.9</v>
+        <v>1939.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>1946.9</v>
+        <v>1939.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>2115303</v>
+        <v>1320334</v>
       </c>
       <c r="AA2" t="n">
-        <v>3517339</v>
+        <v>3507651</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.6</v>
+        <v>0.38</v>
       </c>
       <c r="AC2" t="n">
-        <v>5.81</v>
+        <v>-0.39</v>
       </c>
       <c r="AD2" t="n">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>89.3</v>
+        <v>37.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.59</v>
+        <v>1.91</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.99</v>
+        <v>49.07</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.99</v>
+        <v>49.07</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.57</v>
+        <v>2.53</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.9</v>
+        <v>4.27</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.86</v>
+        <v>11.87</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.58</v>
+        <v>51.42</v>
       </c>
       <c r="AO2" t="n">
-        <v>66.45</v>
+        <v>65.12</v>
       </c>
       <c r="AP2" t="n">
-        <v>8.1</v>
+        <v>3.92</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.5</v>
+        <v>39.44</v>
       </c>
       <c r="AR2" t="n">
-        <v>1946.9</v>
+        <v>1939.3</v>
       </c>
       <c r="AS2" t="n">
-        <v>2146.87</v>
+        <v>2135.58</v>
       </c>
       <c r="AT2" t="n">
-        <v>1846.92</v>
+        <v>1841.16</v>
       </c>
       <c r="AU2" t="n">
-        <v>1946.900024414062</v>
+        <v>1939.300048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.27</v>
+        <v>10.12</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.97</v>
+        <v>196.28</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.14</v>
+        <v>5.06</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.98</v>
+        <v>98.14</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.71</v>
+        <v>1480.7</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.54000000000001</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.07</v>
+        <v>40.52</v>
       </c>
       <c r="CP2" t="n">
         <v>95.23809523809523</v>
@@ -2094,7 +2094,7 @@
         <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>90.47619047619048</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
@@ -2106,19 +2106,19 @@
         <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>90.47619047619048</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>71.42857142857143</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CX2" t="n">
         <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2712</v>
+        <v>10.1212</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6847</v>
+        <v>0.6747</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3427</v>
+        <v>0.3373</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1027</v>
+        <v>0.1012</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9981</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2088</v>
+        <v>1.1911</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9961</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1353</v>
+        <v>5.0606</v>
       </c>
       <c r="DJ2" t="n">
-        <v>48.13</v>
+        <v>48.72</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1353</v>
+        <v>5.0606</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9961</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.998</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7775</v>
+        <v>0.7905</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.98</v>
+        <v>98.14</v>
       </c>
       <c r="DR2" t="n">
-        <v>54.54</v>
+        <v>64.54000000000001</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>3.1518</v>
+        <v>1.5494</v>
       </c>
       <c r="DX2" t="n">
-        <v>83.875</v>
+        <v>87.19999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.441</v>
+        <v>79.096</v>
       </c>
       <c r="EA2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>100</v>
+        <v>74.20999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>83.15000000000001</v>
+        <v>88.18000000000001</v>
       </c>
       <c r="EE2" t="n">
-        <v>3.1518</v>
+        <v>1.5494</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.6</v>
+        <v>0.38</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.9534</v>
+        <v>0.4614</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9966</v>
+        <v>4.0005</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1122</v>
+        <v>0.0543</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6509</v>
+        <v>0.6601</v>
       </c>
       <c r="EK2" t="n">
-        <v>69.01000000000001</v>
+        <v>62.71</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,75 +2240,75 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>17.47</v>
+        <v>8.99</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.0562</v>
+        <v>1.0581</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0706</v>
+        <v>0.0447</v>
       </c>
       <c r="ER2" t="n">
-        <v>17.1167</v>
+        <v>26.6316</v>
       </c>
       <c r="ES2" t="n">
-        <v>13.4818</v>
+        <v>13.8017</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.916</v>
+        <v>37.952</v>
       </c>
       <c r="EU2" t="n">
-        <v>4.86</v>
+        <v>1.4896</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6062</v>
+        <v>1.8333</v>
       </c>
       <c r="EW2" t="n">
-        <v>14.5944</v>
+        <v>6.6814</v>
       </c>
       <c r="EX2" t="n">
-        <v>43.11</v>
+        <v>29.25</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="FB2" t="n">
         <v>63.49</v>
       </c>
       <c r="FC2" t="n">
-        <v>41.32</v>
+        <v>42.15</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.56999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>76.27500000000001</v>
+        <v>68.515</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.59</v>
+        <v>34.885</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.4006</v>
+        <v>21.0538</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.429</v>
+        <v>59.891</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.335</v>
+        <v>56.63</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.56</v>
+        <v>67.12</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>74.08</v>
+        <v>71.29000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.69</v>
+        <v>67.63</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.23</v>
+        <v>54.15</v>
       </c>
       <c r="FQ2" t="n">
-        <v>69.17</v>
+        <v>73.06</v>
       </c>
       <c r="FR2" t="n">
-        <v>86.79000000000001</v>
+        <v>78.56</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.2381</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.9075</v>
+        <v>69.693</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260908_200043</t>
+          <t>20260909_134240</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46273.83384005574</v>
+        <v>46274.57129689953</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46273.83383101852</v>
+        <v>46274.57129629629</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
+        <v>1939.3</v>
+      </c>
+      <c r="L2" t="n">
         <v>1946.9</v>
       </c>
-      <c r="L2" t="n">
-        <v>1870.8</v>
-      </c>
       <c r="M2" t="n">
-        <v>1952</v>
+        <v>1955</v>
       </c>
       <c r="N2" t="n">
-        <v>1862.7</v>
+        <v>1917.9</v>
       </c>
       <c r="O2" t="n">
-        <v>1946.9</v>
+        <v>1939.3</v>
       </c>
       <c r="P2" t="n">
-        <v>2115303</v>
+        <v>1320334</v>
       </c>
       <c r="Q2" t="n">
-        <v>1946.9</v>
+        <v>1939.3</v>
       </c>
       <c r="R2" t="n">
-        <v>2146.87</v>
+        <v>2135.58</v>
       </c>
       <c r="S2" t="n">
-        <v>1846.92</v>
+        <v>1841.16</v>
       </c>
       <c r="T2" t="n">
-        <v>10.27120036981868</v>
+        <v>10.121177744547</v>
       </c>
       <c r="U2" t="n">
-        <v>199.9699999999998</v>
+        <v>196.28</v>
       </c>
       <c r="V2" t="n">
-        <v>5.135343366377318</v>
+        <v>5.060588872273494</v>
       </c>
       <c r="W2" t="n">
-        <v>99.98000000000002</v>
+        <v>98.13999999999987</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000100020003998</v>
+        <v>2.000000000000002</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.27120036981868</v>
+        <v>10.121177744547</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.135343366377318</v>
+        <v>5.060588872273494</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02061873646256678</v>
+        <v>0.02051082243989397</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.327312294169988</v>
+        <v>0.325599212168175</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353098562824</v>
+        <v>0.04266353092234335</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.82</v>
+        <v>38.95</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 20:00:43.820829+05:30</t>
+          <t>2026-09-09 13:42:40.128866+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.271200369818676, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001000200039982}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.121177744547, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000000000000002}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-09 14:32 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.02</v>
+        <v>49.08</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,22 +1878,22 @@
         <v>1917.9</v>
       </c>
       <c r="X2" t="n">
-        <v>1939.3</v>
+        <v>1937</v>
       </c>
       <c r="Y2" t="n">
-        <v>1939.3</v>
+        <v>1937</v>
       </c>
       <c r="Z2" t="n">
-        <v>1320334</v>
+        <v>1822184</v>
       </c>
       <c r="AA2" t="n">
-        <v>3507651</v>
+        <v>3532744</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.38</v>
+        <v>0.52</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.39</v>
+        <v>-0.51</v>
       </c>
       <c r="AD2" t="n">
         <v>0</v>
@@ -1902,7 +1902,7 @@
         <v>37.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.91</v>
+        <v>1.92</v>
       </c>
       <c r="AG2" t="n">
         <v>49.07</v>
@@ -1920,47 +1920,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.27</v>
+        <v>4.15</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.87</v>
+        <v>11.74</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.42</v>
+        <v>51.24</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.12</v>
+        <v>64.73</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.92</v>
+        <v>3.79</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.44</v>
+        <v>39.27</v>
       </c>
       <c r="AR2" t="n">
-        <v>1939.3</v>
+        <v>1937</v>
       </c>
       <c r="AS2" t="n">
-        <v>2135.58</v>
+        <v>2133.28</v>
       </c>
       <c r="AT2" t="n">
-        <v>1841.16</v>
+        <v>1838.86</v>
       </c>
       <c r="AU2" t="n">
-        <v>1939.300048828125</v>
+        <v>1937</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.12</v>
+        <v>10.13</v>
       </c>
       <c r="AY2" t="n">
         <v>196.28</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.06</v>
+        <v>5.07</v>
       </c>
       <c r="BA2" t="n">
         <v>98.14</v>
@@ -2082,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>74.31999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.52</v>
+        <v>39.67</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>66.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.1212</v>
+        <v>10.1332</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6747</v>
+        <v>0.6753</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3373</v>
+        <v>0.338</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1012</v>
+        <v>0.1013</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1911</v>
+        <v>1.1923</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.004</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0606</v>
+        <v>5.0666</v>
       </c>
       <c r="DJ2" t="n">
-        <v>48.72</v>
+        <v>46.84</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0606</v>
+        <v>5.0666</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.004</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.004</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7905</v>
+        <v>0.7897</v>
       </c>
       <c r="DQ2" t="n">
         <v>98.14</v>
       </c>
       <c r="DR2" t="n">
-        <v>64.54000000000001</v>
+        <v>39.16</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.5494</v>
+        <v>1.498</v>
       </c>
       <c r="DX2" t="n">
-        <v>87.19999999999999</v>
+        <v>88.17499999999998</v>
       </c>
       <c r="DY2" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="DZ2" t="n">
-        <v>79.096</v>
+        <v>81.196</v>
       </c>
       <c r="EA2" t="n">
         <v>4</v>
@@ -2205,31 +2205,31 @@
         <v>8</v>
       </c>
       <c r="EC2" t="n">
-        <v>74.20999999999999</v>
+        <v>77.56</v>
       </c>
       <c r="ED2" t="n">
-        <v>88.18000000000001</v>
+        <v>88.38</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.5494</v>
+        <v>1.498</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.38</v>
+        <v>0.52</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4614</v>
+        <v>0.4461</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0005</v>
+        <v>4.0052</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0543</v>
+        <v>0.0525</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6601</v>
+        <v>0.6598000000000001</v>
       </c>
       <c r="EK2" t="n">
-        <v>62.71</v>
+        <v>67.66</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>8.99</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.0581</v>
+        <v>1.1629</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0447</v>
+        <v>0.0612</v>
       </c>
       <c r="ER2" t="n">
-        <v>26.6316</v>
+        <v>19.4808</v>
       </c>
       <c r="ES2" t="n">
-        <v>13.8017</v>
+        <v>13.2691</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.952</v>
+        <v>37.999</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.4896</v>
+        <v>1.9708</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8333</v>
+        <v>1.6645</v>
       </c>
       <c r="EW2" t="n">
-        <v>6.6814</v>
+        <v>7.4693</v>
       </c>
       <c r="EX2" t="n">
-        <v>29.25</v>
+        <v>30.65</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,28 +2284,28 @@
         <v>6</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.49</v>
+        <v>63.89</v>
       </c>
       <c r="FC2" t="n">
-        <v>42.15</v>
+        <v>40.3</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.93000000000001</v>
+        <v>73.02</v>
       </c>
       <c r="FE2" t="n">
-        <v>68.515</v>
+        <v>71.63</v>
       </c>
       <c r="FF2" t="n">
-        <v>34.885</v>
+        <v>35.16</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.0538</v>
+        <v>21.4164</v>
       </c>
       <c r="FH2" t="n">
-        <v>59.891</v>
+        <v>60.755</v>
       </c>
       <c r="FI2" t="n">
-        <v>56.63</v>
+        <v>43</v>
       </c>
       <c r="FJ2" t="n">
         <v>67.12</v>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.29000000000001</v>
+        <v>65.62</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.63</v>
+        <v>69.88</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.15</v>
+        <v>43.68</v>
       </c>
       <c r="FQ2" t="n">
-        <v>73.06</v>
+        <v>61.59</v>
       </c>
       <c r="FR2" t="n">
-        <v>78.56</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.2381</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.693</v>
+        <v>63.484</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260909_134240</t>
+          <t>20260909_200226</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46274.57129689953</v>
+        <v>46274.83503122582</v>
       </c>
     </row>
   </sheetData>
@@ -2459,8 +2459,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46274.57129629629</v>
+        <v>46274.83502314815</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1939.3</v>
+        <v>1937</v>
       </c>
       <c r="L2" t="n">
         <v>1946.9</v>
@@ -2679,34 +2679,34 @@
         <v>1917.9</v>
       </c>
       <c r="O2" t="n">
-        <v>1939.3</v>
+        <v>1937</v>
       </c>
       <c r="P2" t="n">
-        <v>1320334</v>
+        <v>1822184</v>
       </c>
       <c r="Q2" t="n">
-        <v>1939.3</v>
+        <v>1937</v>
       </c>
       <c r="R2" t="n">
-        <v>2135.58</v>
+        <v>2133.28</v>
       </c>
       <c r="S2" t="n">
-        <v>1841.16</v>
+        <v>1838.86</v>
       </c>
       <c r="T2" t="n">
-        <v>10.121177744547</v>
+        <v>10.13319566339702</v>
       </c>
       <c r="U2" t="n">
-        <v>196.28</v>
+        <v>196.2800000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>5.060588872273494</v>
+        <v>5.066597831698508</v>
       </c>
       <c r="W2" t="n">
-        <v>98.13999999999987</v>
+        <v>98.1400000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000002</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.121177744547</v>
+        <v>10.13319566339702</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.060588872273494</v>
+        <v>5.066597831698508</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02051082243989397</v>
+        <v>0.02060579847487638</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.325599212168175</v>
+        <v>0.3271069099826215</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290984710642187</v>
+        <v>0.02909841185773541</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353092234335</v>
+        <v>0.04266353508262109</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.95</v>
+        <v>38.83</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-09 13:42:40.128866+05:30</t>
+          <t>2026-09-09 20:02:26.738721+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.121177744547, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000000000000002}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.133195663397016, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-10 08:12 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.08</v>
+        <v>48.94</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1946.9</v>
+        <v>1932.6</v>
       </c>
       <c r="V2" t="n">
-        <v>1955</v>
+        <v>1947.5</v>
       </c>
       <c r="W2" t="n">
-        <v>1917.9</v>
+        <v>1920.9</v>
       </c>
       <c r="X2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="Y2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="Z2" t="n">
-        <v>1822184</v>
+        <v>665375</v>
       </c>
       <c r="AA2" t="n">
-        <v>3532744</v>
+        <v>3511587</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.52</v>
+        <v>0.19</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.51</v>
+        <v>0.36</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>-0.23</v>
       </c>
       <c r="AE2" t="n">
-        <v>37.1</v>
+        <v>26.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.92</v>
+        <v>1.37</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.07</v>
+        <v>47.47</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.07</v>
+        <v>47.47</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.53</v>
+        <v>2.44</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.15</v>
+        <v>4.26</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.74</v>
+        <v>11.56</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.24</v>
+        <v>51.22</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.73</v>
+        <v>65.41</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.79</v>
+        <v>3.02</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.27</v>
+        <v>39.42</v>
       </c>
       <c r="AR2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="AS2" t="n">
-        <v>2133.28</v>
+        <v>2133.86</v>
       </c>
       <c r="AT2" t="n">
-        <v>1838.86</v>
+        <v>1849.07</v>
       </c>
       <c r="AU2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.13</v>
+        <v>9.77</v>
       </c>
       <c r="AY2" t="n">
-        <v>196.28</v>
+        <v>189.86</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.07</v>
+        <v>4.88</v>
       </c>
       <c r="BA2" t="n">
-        <v>98.14</v>
+        <v>94.93000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.59999999999999</v>
+        <v>80.02</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.67</v>
+        <v>28.37</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.1332</v>
+        <v>9.766500000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6753</v>
+        <v>0.6513</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.338</v>
+        <v>0.3253</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1013</v>
+        <v>0.0977</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1923</v>
+        <v>1.1499</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.004</v>
+        <v>4.0041</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0666</v>
+        <v>4.8832</v>
       </c>
       <c r="DJ2" t="n">
-        <v>46.84</v>
+        <v>43.82</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0666</v>
+        <v>4.8832</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.004</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.004</v>
+        <v>4.0041</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>2.0022</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7897</v>
+        <v>0.8205</v>
       </c>
       <c r="DQ2" t="n">
-        <v>98.14</v>
+        <v>94.93000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>39.16</v>
+        <v>61.58</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.498</v>
+        <v>1.2377</v>
       </c>
       <c r="DX2" t="n">
-        <v>88.17499999999998</v>
+        <v>86.47500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>26</v>
+        <v>9.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>81.196</v>
+        <v>85.083</v>
       </c>
       <c r="EA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>77.56</v>
+        <v>82.5</v>
       </c>
       <c r="ED2" t="n">
-        <v>88.38</v>
+        <v>89.16</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.498</v>
+        <v>1.2377</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.52</v>
+        <v>0.19</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4461</v>
+        <v>0.3555</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0052</v>
+        <v>4.0027</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0525</v>
+        <v>0.0418</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6598000000000001</v>
+        <v>0.6807</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.66</v>
+        <v>69.53</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,72 +2243,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>9.880000000000001</v>
+        <v>10.33</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.1629</v>
+        <v>1.2158</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0612</v>
+        <v>0.0224</v>
       </c>
       <c r="ER2" t="n">
-        <v>19.4808</v>
+        <v>51.4211</v>
       </c>
       <c r="ES2" t="n">
-        <v>13.2691</v>
+        <v>12.7384</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.999</v>
+        <v>33.614</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.9708</v>
+        <v>0.5738</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6645</v>
+        <v>2.0504</v>
       </c>
       <c r="EW2" t="n">
-        <v>7.4693</v>
+        <v>8.2661</v>
       </c>
       <c r="EX2" t="n">
-        <v>30.65</v>
+        <v>19.66</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Very Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="FA2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="FB2" t="n">
         <v>63.89</v>
       </c>
       <c r="FC2" t="n">
-        <v>40.3</v>
+        <v>37.55</v>
       </c>
       <c r="FD2" t="n">
         <v>73.02</v>
       </c>
       <c r="FE2" t="n">
-        <v>71.63</v>
+        <v>74.77500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>35.16</v>
+        <v>24.015</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.4164</v>
+        <v>23.2616</v>
       </c>
       <c r="FH2" t="n">
-        <v>60.755</v>
+        <v>59.883</v>
       </c>
       <c r="FI2" t="n">
-        <v>43</v>
+        <v>52.7</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.12</v>
+        <v>64.84</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>65.62</v>
+        <v>70.17</v>
       </c>
       <c r="FO2" t="n">
-        <v>69.88</v>
+        <v>64.38</v>
       </c>
       <c r="FP2" t="n">
-        <v>43.68</v>
+        <v>46.48</v>
       </c>
       <c r="FQ2" t="n">
-        <v>61.59</v>
+        <v>75.20999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.31999999999999</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>63.484</v>
+        <v>71.048</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260909_200226</t>
+          <t>20260910_134208</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46274.83503122582</v>
+        <v>46275.5709330755</v>
       </c>
     </row>
   </sheetData>
@@ -2458,8 +2458,8 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46274.83502314815</v>
+        <v>46275.57092592592</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,43 +2667,43 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="L2" t="n">
-        <v>1946.9</v>
+        <v>1932.6</v>
       </c>
       <c r="M2" t="n">
-        <v>1955</v>
+        <v>1947.5</v>
       </c>
       <c r="N2" t="n">
-        <v>1917.9</v>
+        <v>1920.9</v>
       </c>
       <c r="O2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="P2" t="n">
-        <v>1822184</v>
+        <v>665375</v>
       </c>
       <c r="Q2" t="n">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="R2" t="n">
-        <v>2133.28</v>
+        <v>2133.86</v>
       </c>
       <c r="S2" t="n">
-        <v>1838.86</v>
+        <v>1849.07</v>
       </c>
       <c r="T2" t="n">
-        <v>10.13319566339702</v>
+        <v>9.766460905349801</v>
       </c>
       <c r="U2" t="n">
-        <v>196.2800000000002</v>
+        <v>189.8600000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.066597831698508</v>
+        <v>4.8832304526749</v>
       </c>
       <c r="W2" t="n">
-        <v>98.1400000000001</v>
+        <v>94.93000000000006</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.13319566339702</v>
+        <v>9.766460905349801</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.066597831698508</v>
+        <v>4.8832304526749</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02060579847487638</v>
+        <v>0.02060373601318417</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3271069099826215</v>
+        <v>0.3270741694182645</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353508262109</v>
+        <v>0.04266353919774246</v>
       </c>
     </row>
     <row r="13">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-09 20:02:26.738721+05:30</t>
+          <t>2026-09-10 13:42:08.654599+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.133195663397016, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.7664609053498, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-10 14:23 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.94</v>
+        <v>48.99</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1872,46 +1872,46 @@
         <v>1932.6</v>
       </c>
       <c r="V2" t="n">
-        <v>1947.5</v>
+        <v>1950.5</v>
       </c>
       <c r="W2" t="n">
         <v>1920.9</v>
       </c>
       <c r="X2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="Y2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="Z2" t="n">
-        <v>665375</v>
+        <v>1067578</v>
       </c>
       <c r="AA2" t="n">
-        <v>3511587</v>
+        <v>3531697</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.19</v>
+        <v>0.3</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.23</v>
       </c>
       <c r="AE2" t="n">
-        <v>26.6</v>
+        <v>29.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.37</v>
+        <v>1.52</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.47</v>
+        <v>47.68</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.47</v>
+        <v>47.68</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.44</v>
+        <v>2.45</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.26</v>
+        <v>4.31</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.56</v>
+        <v>11.62</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.22</v>
+        <v>51.29</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.41</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.02</v>
+        <v>3.07</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.42</v>
+        <v>39.5</v>
       </c>
       <c r="AR2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="AS2" t="n">
-        <v>2133.86</v>
+        <v>2135.72</v>
       </c>
       <c r="AT2" t="n">
-        <v>1849.07</v>
+        <v>1849.64</v>
       </c>
       <c r="AU2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.77</v>
+        <v>9.81</v>
       </c>
       <c r="AY2" t="n">
-        <v>189.86</v>
+        <v>190.72</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.88</v>
+        <v>4.9</v>
       </c>
       <c r="BA2" t="n">
-        <v>94.93000000000001</v>
+        <v>95.36</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.7</v>
+        <v>1480.71</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>80.02</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>28.37</v>
+        <v>26.97</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.766500000000001</v>
+        <v>9.8057</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2127,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6513</v>
+        <v>0.654</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3253</v>
+        <v>0.3267</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0977</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="DF2" t="n">
         <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1499</v>
+        <v>1.1546</v>
       </c>
       <c r="DH2" t="n">
         <v>4.0041</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8832</v>
+        <v>4.9028</v>
       </c>
       <c r="DJ2" t="n">
-        <v>43.82</v>
+        <v>42.46</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8832</v>
+        <v>4.9028</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2163,16 +2163,16 @@
         <v>4.0041</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0022</v>
+        <v>2.0018</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8205</v>
+        <v>0.8172</v>
       </c>
       <c r="DQ2" t="n">
-        <v>94.93000000000001</v>
+        <v>95.36</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.58</v>
+        <v>68.52</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2377</v>
+        <v>1.2531</v>
       </c>
       <c r="DX2" t="n">
-        <v>86.47500000000001</v>
+        <v>86.22499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>9.5</v>
+        <v>15</v>
       </c>
       <c r="DZ2" t="n">
-        <v>85.083</v>
+        <v>85.54600000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>82.5</v>
+        <v>82.14</v>
       </c>
       <c r="ED2" t="n">
-        <v>89.16</v>
+        <v>91.09</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2377</v>
+        <v>1.2531</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.19</v>
+        <v>0.3</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3555</v>
+        <v>0.3613</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0027</v>
+        <v>4.0023</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0418</v>
+        <v>0.0425</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6807</v>
+        <v>0.6784</v>
       </c>
       <c r="EK2" t="n">
-        <v>69.53</v>
+        <v>70.11</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,72 +2243,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>10.33</v>
+        <v>12.52</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.2158</v>
+        <v>1.4736</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0224</v>
+        <v>0.0353</v>
       </c>
       <c r="ER2" t="n">
-        <v>51.4211</v>
+        <v>32.7</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.7384</v>
+        <v>12.3072</v>
       </c>
       <c r="ET2" t="n">
-        <v>33.614</v>
+        <v>33.711</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.5738</v>
+        <v>0.921</v>
       </c>
       <c r="EV2" t="n">
-        <v>2.0504</v>
+        <v>1.8846</v>
       </c>
       <c r="EW2" t="n">
-        <v>8.2661</v>
+        <v>10.0035</v>
       </c>
       <c r="EX2" t="n">
-        <v>19.66</v>
+        <v>20.66</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FB2" t="n">
         <v>63.89</v>
       </c>
       <c r="FC2" t="n">
-        <v>37.55</v>
+        <v>36.39</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.02</v>
+        <v>73.33</v>
       </c>
       <c r="FE2" t="n">
-        <v>74.77500000000001</v>
+        <v>75.005</v>
       </c>
       <c r="FF2" t="n">
-        <v>24.015</v>
+        <v>23.815</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.2616</v>
+        <v>23.1594</v>
       </c>
       <c r="FH2" t="n">
-        <v>59.883</v>
+        <v>60.047</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.7</v>
+        <v>55.49</v>
       </c>
       <c r="FJ2" t="n">
-        <v>64.84</v>
+        <v>63.97</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.17</v>
+        <v>71.8</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.38</v>
+        <v>62.68</v>
       </c>
       <c r="FP2" t="n">
-        <v>46.48</v>
+        <v>50.75</v>
       </c>
       <c r="FQ2" t="n">
-        <v>75.20999999999999</v>
+        <v>78.48</v>
       </c>
       <c r="FR2" t="n">
-        <v>84.54000000000001</v>
+        <v>82.45999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.048</v>
+        <v>70.67100000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260910_134208</t>
+          <t>20260910_195358</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46275.5709330755</v>
+        <v>46275.82915205924</v>
       </c>
     </row>
   </sheetData>
@@ -2458,8 +2458,8 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46275.57092592592</v>
+        <v>46275.82914351852</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,43 +2667,43 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="L2" t="n">
         <v>1932.6</v>
       </c>
       <c r="M2" t="n">
-        <v>1947.5</v>
+        <v>1950.5</v>
       </c>
       <c r="N2" t="n">
         <v>1920.9</v>
       </c>
       <c r="O2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="P2" t="n">
-        <v>665375</v>
+        <v>1067578</v>
       </c>
       <c r="Q2" t="n">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="R2" t="n">
-        <v>2133.86</v>
+        <v>2135.72</v>
       </c>
       <c r="S2" t="n">
-        <v>1849.07</v>
+        <v>1849.64</v>
       </c>
       <c r="T2" t="n">
-        <v>9.766460905349801</v>
+        <v>9.805655526992279</v>
       </c>
       <c r="U2" t="n">
-        <v>189.8600000000001</v>
+        <v>190.7199999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>4.8832304526749</v>
+        <v>4.902827763496139</v>
       </c>
       <c r="W2" t="n">
-        <v>94.93000000000006</v>
+        <v>95.3599999999999</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.766460905349801</v>
+        <v>9.805655526992279</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.8832304526749</v>
+        <v>4.902827763496139</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02060373601318417</v>
+        <v>0.02059088112828268</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3270741694182645</v>
+        <v>0.3268701044467743</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909841185773541</v>
+        <v>0.02909835265125211</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353919774246</v>
+        <v>0.04266354257276132</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.83</v>
+        <v>38.85</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-10 13:42:08.654599+05:30</t>
+          <t>2026-09-10 19:53:58.779066+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.7664609053498, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.805655526992279, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-11 08:07 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1862,53 +1862,53 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.99</v>
+        <v>49.04</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1932.6</v>
+        <v>1943</v>
       </c>
       <c r="V2" t="n">
-        <v>1950.5</v>
+        <v>1974.7</v>
       </c>
       <c r="W2" t="n">
-        <v>1920.9</v>
+        <v>1918.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1945</v>
+        <v>1971.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>1945</v>
+        <v>1971.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1067578</v>
+        <v>1482497</v>
       </c>
       <c r="AA2" t="n">
-        <v>3531697</v>
+        <v>3538531</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.41</v>
+        <v>1.38</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.23</v>
+        <v>-0.1</v>
       </c>
       <c r="AE2" t="n">
-        <v>29.6</v>
+        <v>56.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.52</v>
+        <v>2.87</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.68</v>
+        <v>48.32</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.68</v>
+        <v>48.32</v>
       </c>
       <c r="AI2" t="n">
         <v>2.45</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.31</v>
+        <v>5.42</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.62</v>
+        <v>12.59</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.29</v>
+        <v>52.79</v>
       </c>
       <c r="AO2" t="n">
-        <v>65.51000000000001</v>
+        <v>68.06999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.07</v>
+        <v>2.2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.5</v>
+        <v>41.96</v>
       </c>
       <c r="AR2" t="n">
-        <v>1945</v>
+        <v>1971.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2135.72</v>
+        <v>2165.17</v>
       </c>
       <c r="AT2" t="n">
-        <v>1849.64</v>
+        <v>1875.27</v>
       </c>
       <c r="AU2" t="n">
-        <v>1945</v>
+        <v>1971.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.81</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>190.72</v>
+        <v>193.27</v>
       </c>
       <c r="AZ2" t="n">
         <v>4.9</v>
       </c>
       <c r="BA2" t="n">
-        <v>95.36</v>
+        <v>96.63</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>79.90000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="CO2" t="n">
-        <v>26.97</v>
+        <v>40.66</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>84.09090909090909</v>
       </c>
       <c r="CW2" t="n">
         <v>68.18181818181817</v>
@@ -2115,10 +2115,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.8057</v>
+        <v>9.8012</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,52 +2127,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.654</v>
+        <v>0.6533</v>
       </c>
       <c r="DD2" t="n">
         <v>0.3267</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.098</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.002</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1546</v>
+        <v>1.1535</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0041</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9028</v>
+        <v>4.9003</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.46</v>
+        <v>43.56</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9028</v>
+        <v>4.9003</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0041</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0018</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8172</v>
+        <v>0.8163</v>
       </c>
       <c r="DQ2" t="n">
-        <v>95.36</v>
+        <v>96.63</v>
       </c>
       <c r="DR2" t="n">
-        <v>68.52</v>
+        <v>57</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2531</v>
+        <v>0.898</v>
       </c>
       <c r="DX2" t="n">
-        <v>86.22499999999999</v>
+        <v>79.82500000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="DZ2" t="n">
-        <v>85.54600000000001</v>
+        <v>83.271</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>82.14</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>91.09</v>
+        <v>90.18000000000001</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2531</v>
+        <v>0.898</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3613</v>
+        <v>0.2589</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0023</v>
+        <v>4.0005</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0425</v>
+        <v>0.0305</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6784</v>
+        <v>0.6781</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.11</v>
+        <v>65.08</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>12.52</v>
+        <v>20.88</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.4736</v>
+        <v>2.4576</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0353</v>
+        <v>0.0494</v>
       </c>
       <c r="ER2" t="n">
-        <v>32.7</v>
+        <v>23.3333</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.3072</v>
+        <v>12.6261</v>
       </c>
       <c r="ET2" t="n">
-        <v>33.711</v>
+        <v>41.737</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.921</v>
+        <v>0.924</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8846</v>
+        <v>1.7254</v>
       </c>
       <c r="EW2" t="n">
-        <v>10.0035</v>
+        <v>15.7644</v>
       </c>
       <c r="EX2" t="n">
-        <v>20.66</v>
+        <v>34.35</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2278,37 +2278,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.89</v>
+        <v>64.03</v>
       </c>
       <c r="FC2" t="n">
-        <v>36.39</v>
+        <v>37.33</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.33</v>
+        <v>73.52</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.005</v>
+        <v>70.29000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>23.815</v>
+        <v>37.505</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.1594</v>
+        <v>21.8841</v>
       </c>
       <c r="FH2" t="n">
-        <v>60.047</v>
+        <v>61.535</v>
       </c>
       <c r="FI2" t="n">
-        <v>55.49</v>
+        <v>50.28</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.97</v>
+        <v>67.3</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.8</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>62.68</v>
+        <v>63.94</v>
       </c>
       <c r="FP2" t="n">
-        <v>50.75</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>78.48</v>
+        <v>81.43000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.45999999999999</v>
+        <v>87.88</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.67100000000001</v>
+        <v>72.48399999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260910_195358</t>
+          <t>20260911_133742</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46275.82915205924</v>
+        <v>46276.56785156037</v>
       </c>
     </row>
   </sheetData>
@@ -2459,8 +2459,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46275.82914351852</v>
+        <v>46276.56784722222</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1945</v>
+        <v>1971.9</v>
       </c>
       <c r="L2" t="n">
-        <v>1932.6</v>
+        <v>1943</v>
       </c>
       <c r="M2" t="n">
-        <v>1950.5</v>
+        <v>1974.7</v>
       </c>
       <c r="N2" t="n">
-        <v>1920.9</v>
+        <v>1918.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1945</v>
+        <v>1971.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1067578</v>
+        <v>1482497</v>
       </c>
       <c r="Q2" t="n">
-        <v>1945</v>
+        <v>1971.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2135.72</v>
+        <v>2165.17</v>
       </c>
       <c r="S2" t="n">
-        <v>1849.64</v>
+        <v>1875.27</v>
       </c>
       <c r="T2" t="n">
-        <v>9.805655526992279</v>
+        <v>9.801206957756477</v>
       </c>
       <c r="U2" t="n">
-        <v>190.7199999999998</v>
+        <v>193.27</v>
       </c>
       <c r="V2" t="n">
-        <v>4.902827763496139</v>
+        <v>4.900349916324362</v>
       </c>
       <c r="W2" t="n">
-        <v>95.3599999999999</v>
+        <v>96.63000000000011</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.00010348752975</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.805655526992279</v>
+        <v>9.801206957756477</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.902827763496139</v>
+        <v>4.900349916324362</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02059088112828268</v>
+        <v>0.0205952379111034</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3268701044467743</v>
+        <v>0.3269392662299339</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266354257276132</v>
+        <v>0.04266353741806376</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645465</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.85</v>
+        <v>38.84</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-10 19:53:58.779066+05:30</t>
+          <t>2026-09-11 13:37:42.414595+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.805655526992279, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.801206957756477, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.00010348752975}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-11 14:24 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.04</v>
+        <v>49.13</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1872,46 +1872,46 @@
         <v>1943</v>
       </c>
       <c r="V2" t="n">
-        <v>1974.7</v>
+        <v>1981.8</v>
       </c>
       <c r="W2" t="n">
         <v>1918.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1971.9</v>
+        <v>1969</v>
       </c>
       <c r="Y2" t="n">
-        <v>1971.9</v>
+        <v>1969</v>
       </c>
       <c r="Z2" t="n">
-        <v>1482497</v>
+        <v>2277186</v>
       </c>
       <c r="AA2" t="n">
-        <v>3538531</v>
+        <v>3578266</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.42</v>
+        <v>0.64</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.38</v>
+        <v>1.23</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.1</v>
       </c>
       <c r="AE2" t="n">
-        <v>56.6</v>
+        <v>63.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.87</v>
+        <v>3.24</v>
       </c>
       <c r="AG2" t="n">
-        <v>48.32</v>
+        <v>48.82</v>
       </c>
       <c r="AH2" t="n">
-        <v>48.32</v>
+        <v>48.82</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.45</v>
+        <v>2.48</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.42</v>
+        <v>5.27</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.59</v>
+        <v>12.43</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.79</v>
+        <v>52.57</v>
       </c>
       <c r="AO2" t="n">
-        <v>68.06999999999999</v>
+        <v>67.81</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.2</v>
+        <v>2.05</v>
       </c>
       <c r="AQ2" t="n">
-        <v>41.96</v>
+        <v>41.75</v>
       </c>
       <c r="AR2" t="n">
-        <v>1971.9</v>
+        <v>1969</v>
       </c>
       <c r="AS2" t="n">
-        <v>2165.17</v>
+        <v>2164.3</v>
       </c>
       <c r="AT2" t="n">
-        <v>1875.27</v>
+        <v>1871.35</v>
       </c>
       <c r="AU2" t="n">
-        <v>1971.900024414062</v>
+        <v>1969</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.800000000000001</v>
+        <v>9.92</v>
       </c>
       <c r="AY2" t="n">
-        <v>193.27</v>
+        <v>195.3</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.9</v>
+        <v>4.96</v>
       </c>
       <c r="BA2" t="n">
-        <v>96.63</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.71</v>
+        <v>1480.7</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.5</v>
+        <v>76.27</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.66</v>
+        <v>38.6</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2112,13 +2112,13 @@
         <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.8012</v>
+        <v>9.918699999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,34 +2127,34 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6533</v>
+        <v>0.6613</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3267</v>
+        <v>0.3307</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.098</v>
+        <v>0.0992</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1535</v>
+        <v>1.1676</v>
       </c>
       <c r="DH2" t="n">
         <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9003</v>
+        <v>4.9594</v>
       </c>
       <c r="DJ2" t="n">
-        <v>43.56</v>
+        <v>42.73</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9003</v>
+        <v>4.9594</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
@@ -2166,19 +2166,19 @@
         <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8163</v>
+        <v>0.8065</v>
       </c>
       <c r="DQ2" t="n">
-        <v>96.63</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>57</v>
+        <v>54.26</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.898</v>
+        <v>0.8266</v>
       </c>
       <c r="DX2" t="n">
-        <v>79.82500000000002</v>
+        <v>80.47499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="DZ2" t="n">
-        <v>83.271</v>
+        <v>82.943</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>73.98999999999999</v>
+        <v>72.83</v>
       </c>
       <c r="ED2" t="n">
-        <v>90.18000000000001</v>
+        <v>82.55</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.898</v>
+        <v>0.8266</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.42</v>
+        <v>0.64</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2589</v>
+        <v>0.2413</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0005</v>
+        <v>3.9995</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0305</v>
+        <v>0.0284</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6781</v>
+        <v>0.6711</v>
       </c>
       <c r="EK2" t="n">
-        <v>65.08</v>
+        <v>63.2</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>20.88</v>
+        <v>22.44</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.4576</v>
+        <v>2.6412</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0494</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="ER2" t="n">
-        <v>23.3333</v>
+        <v>15.5</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.6261</v>
+        <v>12.2787</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.737</v>
+        <v>41.381</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.924</v>
+        <v>1.312</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7254</v>
+        <v>1.5122</v>
       </c>
       <c r="EW2" t="n">
-        <v>15.7644</v>
+        <v>17.115</v>
       </c>
       <c r="EX2" t="n">
-        <v>34.35</v>
+        <v>36.33</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2281,34 +2281,34 @@
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
         <v>64.03</v>
       </c>
       <c r="FC2" t="n">
-        <v>37.33</v>
+        <v>36.03</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.52</v>
+        <v>73.33</v>
       </c>
       <c r="FE2" t="n">
-        <v>70.29000000000001</v>
+        <v>69.735</v>
       </c>
       <c r="FF2" t="n">
-        <v>37.505</v>
+        <v>37.465</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.8841</v>
+        <v>21.9167</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.535</v>
+        <v>62.162</v>
       </c>
       <c r="FI2" t="n">
-        <v>50.28</v>
+        <v>48.495</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.3</v>
+        <v>67.25</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.95999999999999</v>
+        <v>72.92</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.94</v>
+        <v>63.64</v>
       </c>
       <c r="FP2" t="n">
-        <v>66.90000000000001</v>
+        <v>62.01</v>
       </c>
       <c r="FQ2" t="n">
-        <v>81.43000000000001</v>
+        <v>74.93000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.88</v>
+        <v>84.38</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.48399999999999</v>
+        <v>70.1885</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260911_133742</t>
+          <t>20260911_195359</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46276.56785156037</v>
+        <v>46276.82916529106</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46276.56784722222</v>
+        <v>46276.82915509259</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1971.9</v>
+        <v>1969</v>
       </c>
       <c r="L2" t="n">
         <v>1943</v>
       </c>
       <c r="M2" t="n">
-        <v>1974.7</v>
+        <v>1981.8</v>
       </c>
       <c r="N2" t="n">
         <v>1918.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1971.9</v>
+        <v>1969</v>
       </c>
       <c r="P2" t="n">
-        <v>1482497</v>
+        <v>2277186</v>
       </c>
       <c r="Q2" t="n">
-        <v>1971.9</v>
+        <v>1969</v>
       </c>
       <c r="R2" t="n">
-        <v>2165.17</v>
+        <v>2164.3</v>
       </c>
       <c r="S2" t="n">
-        <v>1875.27</v>
+        <v>1871.35</v>
       </c>
       <c r="T2" t="n">
-        <v>9.801206957756477</v>
+        <v>9.918740477399703</v>
       </c>
       <c r="U2" t="n">
-        <v>193.27</v>
+        <v>195.3000000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>4.900349916324362</v>
+        <v>4.959370238699852</v>
       </c>
       <c r="W2" t="n">
-        <v>96.63000000000011</v>
+        <v>97.65000000000009</v>
       </c>
       <c r="X2" t="n">
-        <v>2.00010348752975</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.801206957756477</v>
+        <v>9.918740477399703</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.900349916324362</v>
+        <v>4.959370238699852</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0205952379111034</v>
+        <v>0.02057924365393107</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3269392662299339</v>
+        <v>0.3266853652686347</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909835265125211</v>
+        <v>0.02909829344476882</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353741806376</v>
+        <v>0.04266353895739713</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645465</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.84</v>
+        <v>38.87</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11 13:37:42.414595+05:30</t>
+          <t>2026-09-11 19:53:59.909622+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.801206957756477, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.00010348752975}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.918740477399703, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>